<commit_message>
fix(recipes): regenerate Maida Cake and Vermicelli Kesari photos to match actual dish
Both original Gemini photos were generated from a generic ingredient-list
prompt and didn't match what the recipe instructions actually describe:
Maida Cake is fried diamond-cut pieces, not a baked sponge cake; Vermicelli
Kesari is set and cut into pieces, not a loose spoonable dessert. Corrected
prompts and updated images for both.
</commit_message>
<xml_diff>
--- a/docs/recipe-image-tracker.xlsx
+++ b/docs/recipe-image-tracker.xlsx
@@ -4119,7 +4119,7 @@
       </c>
       <c r="G66" s="3" t="inlineStr">
         <is>
-          <t>Professional food photography of "Vermicelli Kesari" (சேமியா கேசரி), an authentic South Indian Tamil dish. Key visible ingredients: Vermicelli, Sugar, Water, Ghee, Cashew nuts. arranged neatly on a decorative plate or tray. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden or traditional South Indian table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
+          <t>Professional food photography of "Vermicelli Kesari" (சேமியா கேசரி), a South Indian Tamil sweet made from vermicelli, sugar, and ghee, cooked until thick, poured onto a tray, cooled, and cut into firm pieces (like barfi or halwa squares) -- NOT served as a loose, spoonable, wet dessert. Show several bright orange-yellow set pieces/squares of vermicelli kesari with visible vermicelli strands and cashew nuts studded throughout, neatly cut with clean edges, arranged on a plate or tray. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden or traditional South Indian table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
         </is>
       </c>
       <c r="H66" s="9" t="inlineStr">
@@ -4134,12 +4134,12 @@
       </c>
       <c r="J66" s="9" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="K66" s="9" t="inlineStr">
         <is>
-          <t>Gemini image, converted PNG-&gt;JPG, resized to 1600px wide</t>
+          <t>Regenerated: original image mismatched actual dish appearance; corrected prompt to describe finished fried/cut form; converted PNG-&gt;JPG, resized to 1600px wide</t>
         </is>
       </c>
     </row>
@@ -4834,7 +4834,7 @@
       </c>
       <c r="G79" s="5" t="inlineStr">
         <is>
-          <t>Professional food photography of "Maida Cake" (மைதா கேக்), an authentic South Indian Tamil dish. Key visible ingredients: Maida (all-purpose flour), Milk, Egg, Coconut oil, Dalda (hydrogenated vegetable shortening). arranged neatly on a decorative plate or tray. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden or traditional South Indian table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
+          <t>Professional food photography of "Maida Cake" (மைதா கேக்), a traditional South Indian Tamil sweet snack -- NOT a Western baked sponge cake. This is a sweetened maida (all-purpose flour) dough rolled into a slightly thick sheet, cut into diamond/rhombus shapes, and deep-fried until golden-brown and crisp, similar in appearance to a fried maida biscuit or diamond-cut snack. Show several golden-brown diamond-shaped pieces with a slightly glossy, crisp fried surface, piled or arranged on a plate or tray. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden or traditional South Indian table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
         </is>
       </c>
       <c r="H79" s="12" t="inlineStr">
@@ -4849,12 +4849,12 @@
       </c>
       <c r="J79" s="12" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="K79" s="12" t="inlineStr">
         <is>
-          <t>Gemini image, converted PNG-&gt;JPG, resized to 1600px wide</t>
+          <t>Regenerated: original image mismatched actual dish appearance; corrected prompt to describe finished fried/cut form; converted PNG-&gt;JPG, resized to 1600px wide</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
content(recipes): finish fish/seafood metadata+photos; feat(categories): full-bleed tile images
Adds description, timing, servings, difficulty, and a Gemini-generated
photo for all 12 fish/seafood recipes added earlier, completing every
recipe in the site with full content, metadata, and imagery.

Also restyles category tiles (home grid and /categories listing) to show
the representative photo filling the box edge-to-edge, matching the
recipe card treatment, instead of a small circular thumbnail. The
letter-badge fallback for categories without a photo is resized to match.
</commit_message>
<xml_diff>
--- a/docs/recipe-image-tracker.xlsx
+++ b/docs/recipe-image-tracker.xlsx
@@ -88,7 +88,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
@@ -130,6 +130,7 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -495,7 +496,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K140"/>
+  <dimension ref="A1:K152"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -8210,6 +8211,666 @@
       <c r="K140" s="6" t="inlineStr">
         <is>
           <t>Gemini image, converted PNG-&gt;JPG, resized to 1600px wide</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" s="15" t="n">
+        <v>140</v>
+      </c>
+      <c r="B141" s="15" t="inlineStr">
+        <is>
+          <t>Non-Vegetarian</t>
+        </is>
+      </c>
+      <c r="C141" s="15" t="inlineStr">
+        <is>
+          <t>dried-fish-kuzhambu</t>
+        </is>
+      </c>
+      <c r="D141" s="15" t="inlineStr">
+        <is>
+          <t>Dried Fish Kuzhambu for New Mothers</t>
+        </is>
+      </c>
+      <c r="E141" s="15" t="inlineStr">
+        <is>
+          <t>குழந்தை பெற்றவர்க்கு வைக்கும் கருவாட்டுக் குழம்பு</t>
+        </is>
+      </c>
+      <c r="F141" s="15" t="inlineStr">
+        <is>
+          <t>kuzhambu</t>
+        </is>
+      </c>
+      <c r="G141" s="15" t="inlineStr">
+        <is>
+          <t>Professional food photography of "Dried Fish Kuzhambu" (கருவாட்டுக் குழம்பு), a South Indian Tamil dish: dried fish pieces simmered in a thick, dark reddish-brown tamarind-garlic gravy with whole garlic cloves visible, served in a clay bowl. Rustic, home-style South Indian presentation. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden or traditional South Indian table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
+        </is>
+      </c>
+      <c r="H141" s="15" t="inlineStr">
+        <is>
+          <t>public/images/recipes/dried-fish-kuzhambu/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I141" s="15" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J141" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="K141" s="15" t="inlineStr">
+        <is>
+          <t>Gemini image, converted PNG-&gt;JPG, resized to 1600px wide</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" s="15" t="n">
+        <v>141</v>
+      </c>
+      <c r="B142" s="15" t="inlineStr">
+        <is>
+          <t>Non-Vegetarian</t>
+        </is>
+      </c>
+      <c r="C142" s="15" t="inlineStr">
+        <is>
+          <t>prawn-kuzhambu</t>
+        </is>
+      </c>
+      <c r="D142" s="15" t="inlineStr">
+        <is>
+          <t>Prawn Kuzhambu</t>
+        </is>
+      </c>
+      <c r="E142" s="15" t="inlineStr">
+        <is>
+          <t>இறால் மீன் குழம்பு</t>
+        </is>
+      </c>
+      <c r="F142" s="15" t="inlineStr">
+        <is>
+          <t>kuzhambu</t>
+        </is>
+      </c>
+      <c r="G142" s="15" t="inlineStr">
+        <is>
+          <t>Professional food photography of "Prawn Kuzhambu" (இறால் மீன் குழம்பு), a South Indian Tamil dish: prawns simmered in a thick reddish-orange onion-tomato gravy, finished with a light sheen of coconut milk, garnished with curry leaves, served in a clay bowl. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden or traditional South Indian table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
+        </is>
+      </c>
+      <c r="H142" s="15" t="inlineStr">
+        <is>
+          <t>public/images/recipes/prawn-kuzhambu/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I142" s="15" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J142" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="K142" s="15" t="inlineStr">
+        <is>
+          <t>Gemini image, converted PNG-&gt;JPG, resized to 1600px wide</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" s="15" t="n">
+        <v>142</v>
+      </c>
+      <c r="B143" s="15" t="inlineStr">
+        <is>
+          <t>Non-Vegetarian</t>
+        </is>
+      </c>
+      <c r="C143" s="15" t="inlineStr">
+        <is>
+          <t>fish-chips</t>
+        </is>
+      </c>
+      <c r="D143" s="15" t="inlineStr">
+        <is>
+          <t>Fish Chips</t>
+        </is>
+      </c>
+      <c r="E143" s="15" t="inlineStr">
+        <is>
+          <t>சாப்ஸ் மீன்</t>
+        </is>
+      </c>
+      <c r="F143" s="15" t="inlineStr">
+        <is>
+          <t>curry</t>
+        </is>
+      </c>
+      <c r="G143" s="15" t="inlineStr">
+        <is>
+          <t>Professional food photography of "Fish Chips" (சாப்ஸ் மீன்), a South Indian Tamil home-style dish -- NOT fried potato chips or crispy fish chips. This is fish pieces simmered gently in a light, dry mustard-and-cumin tempering with black pepper, glazed with a touch of soy sauce, served on a plate. The fish should look moist and pan-cooked, not deep-fried or breaded. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden or traditional South Indian table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
+        </is>
+      </c>
+      <c r="H143" s="15" t="inlineStr">
+        <is>
+          <t>public/images/recipes/fish-chips/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I143" s="15" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J143" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="K143" s="15" t="inlineStr">
+        <is>
+          <t>Gemini image, converted PNG-&gt;JPG, resized to 1600px wide</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" s="15" t="n">
+        <v>143</v>
+      </c>
+      <c r="B144" s="15" t="inlineStr">
+        <is>
+          <t>Non-Vegetarian</t>
+        </is>
+      </c>
+      <c r="C144" s="15" t="inlineStr">
+        <is>
+          <t>finger-fish</t>
+        </is>
+      </c>
+      <c r="D144" s="15" t="inlineStr">
+        <is>
+          <t>Finger Fish</t>
+        </is>
+      </c>
+      <c r="E144" s="15" t="inlineStr">
+        <is>
+          <t>ஃபிங்கர் ஃபிஷ்</t>
+        </is>
+      </c>
+      <c r="F144" s="15" t="inlineStr">
+        <is>
+          <t>fried-snack</t>
+        </is>
+      </c>
+      <c r="G144" s="15" t="inlineStr">
+        <is>
+          <t>Professional food photography of "Finger Fish" (ஃபிங்கர் ஃபிஷ்), a South Indian Tamil snack: seer fish cut into finger-length strips, marinated and coated in a light corn-flour-and-egg batter, deep-fried until golden and crisp, served piled on a plate. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden or traditional South Indian table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
+        </is>
+      </c>
+      <c r="H144" s="15" t="inlineStr">
+        <is>
+          <t>public/images/recipes/finger-fish/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I144" s="15" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J144" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="K144" s="15" t="inlineStr">
+        <is>
+          <t>Gemini image, converted PNG-&gt;JPG, resized to 1600px wide</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" s="15" t="n">
+        <v>144</v>
+      </c>
+      <c r="B145" s="15" t="inlineStr">
+        <is>
+          <t>Non-Vegetarian</t>
+        </is>
+      </c>
+      <c r="C145" s="15" t="inlineStr">
+        <is>
+          <t>fish-roast</t>
+        </is>
+      </c>
+      <c r="D145" s="15" t="inlineStr">
+        <is>
+          <t>Fish Roast</t>
+        </is>
+      </c>
+      <c r="E145" s="15" t="inlineStr">
+        <is>
+          <t>மீன் ரோஸ்ட்</t>
+        </is>
+      </c>
+      <c r="F145" s="15" t="inlineStr">
+        <is>
+          <t>curry</t>
+        </is>
+      </c>
+      <c r="G145" s="15" t="inlineStr">
+        <is>
+          <t>Professional food photography of "Fish Roast" (மீன் ரோஸ்ட்), a South Indian Tamil dish: fish pieces coated in a dry pepper-coriander-cumin-turmeric rub, shallow-fried in oil until deeply golden-brown and slightly crisp on the outside, served on a plate garnished with onion, coriander leaves, and lemon wedges. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden or traditional South Indian table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
+        </is>
+      </c>
+      <c r="H145" s="15" t="inlineStr">
+        <is>
+          <t>public/images/recipes/fish-roast/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I145" s="15" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J145" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="K145" s="15" t="inlineStr">
+        <is>
+          <t>Gemini image, converted PNG-&gt;JPG, resized to 1600px wide</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" s="15" t="n">
+        <v>145</v>
+      </c>
+      <c r="B146" s="15" t="inlineStr">
+        <is>
+          <t>Non-Vegetarian</t>
+        </is>
+      </c>
+      <c r="C146" s="15" t="inlineStr">
+        <is>
+          <t>boiled-fish</t>
+        </is>
+      </c>
+      <c r="D146" s="15" t="inlineStr">
+        <is>
+          <t>Boiled Fish</t>
+        </is>
+      </c>
+      <c r="E146" s="15" t="inlineStr">
+        <is>
+          <t>வேக வைத்த மீன்</t>
+        </is>
+      </c>
+      <c r="F146" s="15" t="inlineStr">
+        <is>
+          <t>curry</t>
+        </is>
+      </c>
+      <c r="G146" s="15" t="inlineStr">
+        <is>
+          <t>Professional food photography of "Boiled Fish" (வேக வைத்த மீன்), a South Indian Tamil dish: fish pieces coated in a ground turmeric, dried-chili, and mustard seed paste, pressure-cooked in oil until tender, served on a plate -- the fish should look coated in a yellow-orange spice paste, not plain white boiled fish. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden or traditional South Indian table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
+        </is>
+      </c>
+      <c r="H146" s="15" t="inlineStr">
+        <is>
+          <t>public/images/recipes/boiled-fish/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I146" s="15" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J146" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="K146" s="15" t="inlineStr">
+        <is>
+          <t>Gemini image, converted PNG-&gt;JPG, resized to 1600px wide</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" s="15" t="n">
+        <v>146</v>
+      </c>
+      <c r="B147" s="15" t="inlineStr">
+        <is>
+          <t>Non-Vegetarian</t>
+        </is>
+      </c>
+      <c r="C147" s="15" t="inlineStr">
+        <is>
+          <t>kerala-fish-kuzhambu</t>
+        </is>
+      </c>
+      <c r="D147" s="15" t="inlineStr">
+        <is>
+          <t>Kerala-Style Fish Kuzhambu</t>
+        </is>
+      </c>
+      <c r="E147" s="15" t="inlineStr">
+        <is>
+          <t>கேரளா மீன் குழம்பு</t>
+        </is>
+      </c>
+      <c r="F147" s="15" t="inlineStr">
+        <is>
+          <t>kuzhambu</t>
+        </is>
+      </c>
+      <c r="G147" s="15" t="inlineStr">
+        <is>
+          <t>Professional food photography of "Kerala-Style Fish Kuzhambu" (கேரளா மீன் குழம்பு), a South Indian dish: seer fish or shark pieces simmered in a rich reddish-brown onion-tomato gravy with a roasted coconut-and-fennel paste stirred through, garnished with fried curry leaves, served in a clay bowl. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden or traditional South Indian table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
+        </is>
+      </c>
+      <c r="H147" s="15" t="inlineStr">
+        <is>
+          <t>public/images/recipes/kerala-fish-kuzhambu/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I147" s="15" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J147" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="K147" s="15" t="inlineStr">
+        <is>
+          <t>Gemini image, converted PNG-&gt;JPG, resized to 1600px wide</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" s="15" t="n">
+        <v>147</v>
+      </c>
+      <c r="B148" s="15" t="inlineStr">
+        <is>
+          <t>Non-Vegetarian</t>
+        </is>
+      </c>
+      <c r="C148" s="15" t="inlineStr">
+        <is>
+          <t>fish-cutlet</t>
+        </is>
+      </c>
+      <c r="D148" s="15" t="inlineStr">
+        <is>
+          <t>Fish Cutlet</t>
+        </is>
+      </c>
+      <c r="E148" s="15" t="inlineStr">
+        <is>
+          <t>மீன் கட்லெட்</t>
+        </is>
+      </c>
+      <c r="F148" s="15" t="inlineStr">
+        <is>
+          <t>fried-snack</t>
+        </is>
+      </c>
+      <c r="G148" s="15" t="inlineStr">
+        <is>
+          <t>Professional food photography of "Fish Cutlet" (மீன் கட்லெட்), a South Indian Tamil snack: oval-shaped fish croquettes coated in golden breadcrumbs and deep-fried until crisp and golden-brown, served piled on a plate, one cutlet cut in half showing the soft mashed fish-and-onion filling inside. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden or traditional South Indian table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
+        </is>
+      </c>
+      <c r="H148" s="15" t="inlineStr">
+        <is>
+          <t>public/images/recipes/fish-cutlet/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I148" s="15" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J148" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="K148" s="15" t="inlineStr">
+        <is>
+          <t>Gemini image, converted PNG-&gt;JPG, resized to 1600px wide</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" s="15" t="n">
+        <v>148</v>
+      </c>
+      <c r="B149" s="15" t="inlineStr">
+        <is>
+          <t>Non-Vegetarian</t>
+        </is>
+      </c>
+      <c r="C149" s="15" t="inlineStr">
+        <is>
+          <t>fish-bajji</t>
+        </is>
+      </c>
+      <c r="D149" s="15" t="inlineStr">
+        <is>
+          <t>Fish Bajji</t>
+        </is>
+      </c>
+      <c r="E149" s="15" t="inlineStr">
+        <is>
+          <t>மீன் பஜ்ஜி</t>
+        </is>
+      </c>
+      <c r="F149" s="15" t="inlineStr">
+        <is>
+          <t>bajji</t>
+        </is>
+      </c>
+      <c r="G149" s="15" t="inlineStr">
+        <is>
+          <t>Professional food photography of "Fish Bajji" (மீன் பஜ்ஜி), a South Indian Tamil snack: whole small fish coated in a thick golden-brown besan batter and deep-fried until crisp, served piled on a plate. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden or traditional South Indian table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
+        </is>
+      </c>
+      <c r="H149" s="15" t="inlineStr">
+        <is>
+          <t>public/images/recipes/fish-bajji/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I149" s="15" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J149" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="K149" s="15" t="inlineStr">
+        <is>
+          <t>Gemini image, converted PNG-&gt;JPG, resized to 1600px wide</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" s="15" t="n">
+        <v>149</v>
+      </c>
+      <c r="B150" s="15" t="inlineStr">
+        <is>
+          <t>Non-Vegetarian</t>
+        </is>
+      </c>
+      <c r="C150" s="15" t="inlineStr">
+        <is>
+          <t>shark-fish-puttu</t>
+        </is>
+      </c>
+      <c r="D150" s="15" t="inlineStr">
+        <is>
+          <t>Shark Fish Puttu</t>
+        </is>
+      </c>
+      <c r="E150" s="15" t="inlineStr">
+        <is>
+          <t>சுறா மீன் புட்டு</t>
+        </is>
+      </c>
+      <c r="F150" s="15" t="inlineStr">
+        <is>
+          <t>puttu</t>
+        </is>
+      </c>
+      <c r="G150" s="15" t="inlineStr">
+        <is>
+          <t>Professional food photography of "Shark Fish Puttu" (சுறா மீன் புட்டு), a South Indian Tamil dish -- NOT a steamed rice puttu. This is cooked, shredded shark fish stir-fried dry with sauteed onion, green chili, and turmeric, resembling a dry fish thoran/keema-style dish, served on a plate. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden or traditional South Indian table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
+        </is>
+      </c>
+      <c r="H150" s="15" t="inlineStr">
+        <is>
+          <t>public/images/recipes/shark-fish-puttu/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I150" s="15" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J150" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="K150" s="15" t="inlineStr">
+        <is>
+          <t>Gemini image, converted PNG-&gt;JPG, resized to 1600px wide</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" s="15" t="n">
+        <v>150</v>
+      </c>
+      <c r="B151" s="15" t="inlineStr">
+        <is>
+          <t>Non-Vegetarian</t>
+        </is>
+      </c>
+      <c r="C151" s="15" t="inlineStr">
+        <is>
+          <t>pepper-fish-masala</t>
+        </is>
+      </c>
+      <c r="D151" s="15" t="inlineStr">
+        <is>
+          <t>Pepper Fish Masala</t>
+        </is>
+      </c>
+      <c r="E151" s="15" t="inlineStr">
+        <is>
+          <t>பெப்பர் மீன் மசாலா</t>
+        </is>
+      </c>
+      <c r="F151" s="15" t="inlineStr">
+        <is>
+          <t>curry</t>
+        </is>
+      </c>
+      <c r="G151" s="15" t="inlineStr">
+        <is>
+          <t>Professional food photography of "Pepper Fish Masala" (பெப்பர் மீன் மசாலா), a South Indian Tamil dish: fish fillets marinated in lemon juice and black pepper, griddle-cooked in dalda until deeply golden-brown and slightly charred on both sides, served on a plate. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden or traditional South Indian table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
+        </is>
+      </c>
+      <c r="H151" s="15" t="inlineStr">
+        <is>
+          <t>public/images/recipes/pepper-fish-masala/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I151" s="15" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J151" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="K151" s="15" t="inlineStr">
+        <is>
+          <t>Gemini image, converted PNG-&gt;JPG, resized to 1600px wide</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" s="15" t="n">
+        <v>151</v>
+      </c>
+      <c r="B152" s="15" t="inlineStr">
+        <is>
+          <t>Non-Vegetarian</t>
+        </is>
+      </c>
+      <c r="C152" s="15" t="inlineStr">
+        <is>
+          <t>seer-fish-puttu</t>
+        </is>
+      </c>
+      <c r="D152" s="15" t="inlineStr">
+        <is>
+          <t>Seer Fish Puttu</t>
+        </is>
+      </c>
+      <c r="E152" s="15" t="inlineStr">
+        <is>
+          <t>சீலா மீன் புட்டு</t>
+        </is>
+      </c>
+      <c r="F152" s="15" t="inlineStr">
+        <is>
+          <t>puttu</t>
+        </is>
+      </c>
+      <c r="G152" s="15" t="inlineStr">
+        <is>
+          <t>Professional food photography of "Seer Fish Puttu" (சீலா மீன் புட்டு), a South Indian Tamil dish -- NOT a steamed rice puttu. This is steamed, flaked seer fish (a firm, pale, flaky fish, distinct in texture from shark) stir-fried dry with sauteed onion and green chili, with a clearly visible mustard-seed-and-split-urad-dal tempering -- small dark mustard seeds and tiny pale-yellow lentil specks should be visible throughout the dish. Served on a steel plate (not a clay plate). Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden or traditional South Indian table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
+        </is>
+      </c>
+      <c r="H152" s="15" t="inlineStr">
+        <is>
+          <t>public/images/recipes/seer-fish-puttu/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I152" s="15" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J152" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="K152" s="15" t="inlineStr">
+        <is>
+          <t>Prompt revised before first generation: original wording nearly duplicated shark-fish-puttu; now calls out the mustard/urad-dal tempering and steel-plate serving that distinguish this recipe</t>
         </is>
       </c>
     </row>
@@ -8330,7 +8991,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H140"/>
+  <dimension ref="A1:H152"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -13405,6 +14066,426 @@
         </is>
       </c>
     </row>
+    <row r="141">
+      <c r="A141" t="n">
+        <v>140</v>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>kuzhambu</t>
+        </is>
+      </c>
+      <c r="C141" t="inlineStr">
+        <is>
+          <t>dried-fish-kuzhambu</t>
+        </is>
+      </c>
+      <c r="D141" t="inlineStr">
+        <is>
+          <t>Dried Fish Kuzhambu for New Mothers</t>
+        </is>
+      </c>
+      <c r="E141" t="inlineStr">
+        <is>
+          <t>குழந்தை பெற்றவர்க்கு வைக்கும் கருவாட்டுக் குழம்பு</t>
+        </is>
+      </c>
+      <c r="F141" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G141" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="n">
+        <v>141</v>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>kuzhambu</t>
+        </is>
+      </c>
+      <c r="C142" t="inlineStr">
+        <is>
+          <t>prawn-kuzhambu</t>
+        </is>
+      </c>
+      <c r="D142" t="inlineStr">
+        <is>
+          <t>Prawn Kuzhambu</t>
+        </is>
+      </c>
+      <c r="E142" t="inlineStr">
+        <is>
+          <t>இறால் மீன் குழம்பு</t>
+        </is>
+      </c>
+      <c r="F142" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G142" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="n">
+        <v>142</v>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>curry</t>
+        </is>
+      </c>
+      <c r="C143" t="inlineStr">
+        <is>
+          <t>fish-chips</t>
+        </is>
+      </c>
+      <c r="D143" t="inlineStr">
+        <is>
+          <t>Fish Chips</t>
+        </is>
+      </c>
+      <c r="E143" t="inlineStr">
+        <is>
+          <t>சாப்ஸ் மீன்</t>
+        </is>
+      </c>
+      <c r="F143" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G143" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="n">
+        <v>143</v>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>fried-snack</t>
+        </is>
+      </c>
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>finger-fish</t>
+        </is>
+      </c>
+      <c r="D144" t="inlineStr">
+        <is>
+          <t>Finger Fish</t>
+        </is>
+      </c>
+      <c r="E144" t="inlineStr">
+        <is>
+          <t>ஃபிங்கர் ஃபிஷ்</t>
+        </is>
+      </c>
+      <c r="F144" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G144" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="n">
+        <v>144</v>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>curry</t>
+        </is>
+      </c>
+      <c r="C145" t="inlineStr">
+        <is>
+          <t>fish-roast</t>
+        </is>
+      </c>
+      <c r="D145" t="inlineStr">
+        <is>
+          <t>Fish Roast</t>
+        </is>
+      </c>
+      <c r="E145" t="inlineStr">
+        <is>
+          <t>மீன் ரோஸ்ட்</t>
+        </is>
+      </c>
+      <c r="F145" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G145" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="n">
+        <v>145</v>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>curry</t>
+        </is>
+      </c>
+      <c r="C146" t="inlineStr">
+        <is>
+          <t>boiled-fish</t>
+        </is>
+      </c>
+      <c r="D146" t="inlineStr">
+        <is>
+          <t>Boiled Fish</t>
+        </is>
+      </c>
+      <c r="E146" t="inlineStr">
+        <is>
+          <t>வேக வைத்த மீன்</t>
+        </is>
+      </c>
+      <c r="F146" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G146" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="n">
+        <v>146</v>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>kuzhambu</t>
+        </is>
+      </c>
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>kerala-fish-kuzhambu</t>
+        </is>
+      </c>
+      <c r="D147" t="inlineStr">
+        <is>
+          <t>Kerala-Style Fish Kuzhambu</t>
+        </is>
+      </c>
+      <c r="E147" t="inlineStr">
+        <is>
+          <t>கேரளா மீன் குழம்பு</t>
+        </is>
+      </c>
+      <c r="F147" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G147" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="n">
+        <v>147</v>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>fried-snack</t>
+        </is>
+      </c>
+      <c r="C148" t="inlineStr">
+        <is>
+          <t>fish-cutlet</t>
+        </is>
+      </c>
+      <c r="D148" t="inlineStr">
+        <is>
+          <t>Fish Cutlet</t>
+        </is>
+      </c>
+      <c r="E148" t="inlineStr">
+        <is>
+          <t>மீன் கட்லெட்</t>
+        </is>
+      </c>
+      <c r="F148" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G148" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="n">
+        <v>148</v>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>bajji</t>
+        </is>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>fish-bajji</t>
+        </is>
+      </c>
+      <c r="D149" t="inlineStr">
+        <is>
+          <t>Fish Bajji</t>
+        </is>
+      </c>
+      <c r="E149" t="inlineStr">
+        <is>
+          <t>மீன் பஜ்ஜி</t>
+        </is>
+      </c>
+      <c r="F149" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G149" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="n">
+        <v>149</v>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>puttu</t>
+        </is>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>shark-fish-puttu</t>
+        </is>
+      </c>
+      <c r="D150" t="inlineStr">
+        <is>
+          <t>Shark Fish Puttu</t>
+        </is>
+      </c>
+      <c r="E150" t="inlineStr">
+        <is>
+          <t>சுறா மீன் புட்டு</t>
+        </is>
+      </c>
+      <c r="F150" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G150" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="n">
+        <v>150</v>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>curry</t>
+        </is>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>pepper-fish-masala</t>
+        </is>
+      </c>
+      <c r="D151" t="inlineStr">
+        <is>
+          <t>Pepper Fish Masala</t>
+        </is>
+      </c>
+      <c r="E151" t="inlineStr">
+        <is>
+          <t>பெப்பர் மீன் மசாலா</t>
+        </is>
+      </c>
+      <c r="F151" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G151" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="n">
+        <v>151</v>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>puttu</t>
+        </is>
+      </c>
+      <c r="C152" t="inlineStr">
+        <is>
+          <t>seer-fish-puttu</t>
+        </is>
+      </c>
+      <c r="D152" t="inlineStr">
+        <is>
+          <t>Seer Fish Puttu</t>
+        </is>
+      </c>
+      <c r="E152" t="inlineStr">
+        <is>
+          <t>சீலா மீன் புட்டு</t>
+        </is>
+      </c>
+      <c r="F152" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G152" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
content(recipes): add first 50 recipes from the street-food/snacks cookbook
Transcribes recipes 1-50 from recepies1.pdf (book pages 1-66): samosas,
chaat, rolls, rissoles, fritters, puffs/cones, stuffed vegetables, pizza,
Gujarati items, Indo-Chinese fusion snacks, kababs, and the full cutlet
block. Adds 6 new category slugs (roll, kabab, cutlet, bonda, chaat,
sandwich) to categories.json per the agreed taxonomy -- rissoles folded
into cutlet rather than a separate slug. Content only (ingredients and
instructions); description, timing, servings, difficulty, and photos to
follow in a later pass, same as prior batches.
</commit_message>
<xml_diff>
--- a/docs/recipe-image-tracker.xlsx
+++ b/docs/recipe-image-tracker.xlsx
@@ -496,7 +496,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K152"/>
+  <dimension ref="A1:K202"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -8871,6 +8871,2256 @@
       <c r="K152" s="15" t="inlineStr">
         <is>
           <t>Prompt revised before first generation: original wording nearly duplicated shark-fish-puttu; now calls out the mustard/urad-dal tempering and steel-plate serving that distinguish this recipe</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="n">
+        <v>152</v>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>Vegetarian</t>
+        </is>
+      </c>
+      <c r="C153" t="inlineStr">
+        <is>
+          <t>mini-vegetable-samosa</t>
+        </is>
+      </c>
+      <c r="D153" t="inlineStr">
+        <is>
+          <t>Mini Vegetable Samosa</t>
+        </is>
+      </c>
+      <c r="E153" t="inlineStr">
+        <is>
+          <t>சிறிய சமோசா</t>
+        </is>
+      </c>
+      <c r="F153" t="inlineStr">
+        <is>
+          <t>fried-snack</t>
+        </is>
+      </c>
+      <c r="G153" t="inlineStr">
+        <is>
+          <t>Professional food photography of "Mini Vegetable Samosa" (சிறிய சமோசா), an Indian street-food snack: small triangular pastries with a crisp, flaky, deep-fried golden-brown maida crust, filled with a spiced potato-carrot-pea filling (one samosa broken open to show the filling), piled on a plate with mint chutney and tomato sauce on the side. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
+        </is>
+      </c>
+      <c r="H153" t="inlineStr">
+        <is>
+          <t>public/images/recipes/mini-vegetable-samosa/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I153" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="n">
+        <v>153</v>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>Vegetarian</t>
+        </is>
+      </c>
+      <c r="C154" t="inlineStr">
+        <is>
+          <t>punjabi-samosa</t>
+        </is>
+      </c>
+      <c r="D154" t="inlineStr">
+        <is>
+          <t>Punjabi Samosa</t>
+        </is>
+      </c>
+      <c r="E154" t="inlineStr">
+        <is>
+          <t>பஞ்சாபி சமோசா</t>
+        </is>
+      </c>
+      <c r="F154" t="inlineStr">
+        <is>
+          <t>fried-snack</t>
+        </is>
+      </c>
+      <c r="G154" t="inlineStr">
+        <is>
+          <t>Professional food photography of "Punjabi Samosa" (பஞ்சாபி சமோசா), a classic North Indian snack: large triangular pastries with a thick, crisp, deep-fried golden-brown crust, filled with a coarse spiced mashed-potato-and-pea filling studded with visible potato chunks (one samosa broken open to show the filling), served with mint chutney, sweet tamarind chutney, and tomato sauce. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
+        </is>
+      </c>
+      <c r="H154" t="inlineStr">
+        <is>
+          <t>public/images/recipes/punjabi-samosa/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I154" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="n">
+        <v>154</v>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>Vegetarian</t>
+        </is>
+      </c>
+      <c r="C155" t="inlineStr">
+        <is>
+          <t>lentil-kachori</t>
+        </is>
+      </c>
+      <c r="D155" t="inlineStr">
+        <is>
+          <t>Lentil Kachori</t>
+        </is>
+      </c>
+      <c r="E155" t="inlineStr">
+        <is>
+          <t>பருப்பு கசோரிகள்</t>
+        </is>
+      </c>
+      <c r="F155" t="inlineStr">
+        <is>
+          <t>fried-snack</t>
+        </is>
+      </c>
+      <c r="G155" t="inlineStr">
+        <is>
+          <t>Professional food photography of "Lentil Kachori" (பருப்பு கசோரிகள்), an Indian street-food snack: small round, slightly flattened deep-fried pastries with a golden-brown crust, filled with a spiced urad-and-moong-dal filling (one kachori broken open to show the dense lentil filling), served with green coriander chutney and a dark tamarind-jaggery sweet chutney. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
+        </is>
+      </c>
+      <c r="H155" t="inlineStr">
+        <is>
+          <t>public/images/recipes/lentil-kachori/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I155" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="n">
+        <v>155</v>
+      </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>Vegetarian</t>
+        </is>
+      </c>
+      <c r="C156" t="inlineStr">
+        <is>
+          <t>pani-puri</t>
+        </is>
+      </c>
+      <c r="D156" t="inlineStr">
+        <is>
+          <t>Pani Puri</t>
+        </is>
+      </c>
+      <c r="E156" t="inlineStr">
+        <is>
+          <t>பானி பூரி</t>
+        </is>
+      </c>
+      <c r="F156" t="inlineStr">
+        <is>
+          <t>chaat</t>
+        </is>
+      </c>
+      <c r="G156" t="inlineStr">
+        <is>
+          <t>Professional food photography of "Pani Puri" (பானி பூரி), a popular Indian street-food chaat: a plate of small, round, hollow, crisp golden-fried puris, one puri filled with spiced diced potato and moong sprouts and a spoonful of dark tamarind chutney, being filled with bright green mint-coriander spiced water (pani) poured from a small pitcher, with extra puris and a bowl of green pani alongside. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
+        </is>
+      </c>
+      <c r="H156" t="inlineStr">
+        <is>
+          <t>public/images/recipes/pani-puri/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I156" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="n">
+        <v>156</v>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>Vegetarian</t>
+        </is>
+      </c>
+      <c r="C157" t="inlineStr">
+        <is>
+          <t>curd-puri</t>
+        </is>
+      </c>
+      <c r="D157" t="inlineStr">
+        <is>
+          <t>Curd Puri (Dahi Puri)</t>
+        </is>
+      </c>
+      <c r="E157" t="inlineStr">
+        <is>
+          <t>தயிர் பூரி</t>
+        </is>
+      </c>
+      <c r="F157" t="inlineStr">
+        <is>
+          <t>chaat</t>
+        </is>
+      </c>
+      <c r="G157" t="inlineStr">
+        <is>
+          <t>Professional food photography of "Curd Puri" (Dahi Puri) (தயிர் பூரி), an Indian chaat snack: small crisp round puris arranged on a plate, each topped with spiced potato, a generous spoonful of thick whipped curd (yogurt), drizzled with dark tamarind-date sweet chutney, and dusted with red chili powder, roasted cumin powder, and fine sev, garnished with coriander leaves. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
+        </is>
+      </c>
+      <c r="H157" t="inlineStr">
+        <is>
+          <t>public/images/recipes/curd-puri/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I157" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="n">
+        <v>157</v>
+      </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>Vegetarian</t>
+        </is>
+      </c>
+      <c r="C158" t="inlineStr">
+        <is>
+          <t>bel-puri</t>
+        </is>
+      </c>
+      <c r="D158" t="inlineStr">
+        <is>
+          <t>Bhel Puri</t>
+        </is>
+      </c>
+      <c r="E158" t="inlineStr">
+        <is>
+          <t>பேல் பூரி</t>
+        </is>
+      </c>
+      <c r="F158" t="inlineStr">
+        <is>
+          <t>chaat</t>
+        </is>
+      </c>
+      <c r="G158" t="inlineStr">
+        <is>
+          <t>Professional food photography of "Bhel Puri" (பேல் பூரி), a Mumbai-style Indian street-food chaat: a bowl heaped with puffed rice, crushed crisp puris, potato chips, finely chopped onion and tomato, tossed with tangy tamarind chutney, green mint chutney, and garlic chutney, topped generously with crunchy fine sev (chickpea-flour noodles) and fresh coriander leaves. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
+        </is>
+      </c>
+      <c r="H158" t="inlineStr">
+        <is>
+          <t>public/images/recipes/bel-puri/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I158" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="n">
+        <v>158</v>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>Vegetarian</t>
+        </is>
+      </c>
+      <c r="C159" t="inlineStr">
+        <is>
+          <t>vegetable-fingers</t>
+        </is>
+      </c>
+      <c r="D159" t="inlineStr">
+        <is>
+          <t>Vegetable Fingers</t>
+        </is>
+      </c>
+      <c r="E159" t="inlineStr">
+        <is>
+          <t>வெஜிடபிள் ஃபிங்கர்ஸ்</t>
+        </is>
+      </c>
+      <c r="F159" t="inlineStr">
+        <is>
+          <t>fried-snack</t>
+        </is>
+      </c>
+      <c r="G159" t="inlineStr">
+        <is>
+          <t>Professional food photography of "Vegetable Fingers" (வெஜிடபிள் ஃபிங்கர்ஸ்), an Indian snack: golden-brown, deep-fried finger-shaped croquettes with a crisp exterior, made from a steamed moong-dal-and-mixed-vegetable batter, piled on a plate with tomato sauce for dipping. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
+        </is>
+      </c>
+      <c r="H159" t="inlineStr">
+        <is>
+          <t>public/images/recipes/vegetable-fingers/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I159" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="n">
+        <v>159</v>
+      </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>Vegetarian</t>
+        </is>
+      </c>
+      <c r="C160" t="inlineStr">
+        <is>
+          <t>moong-fingers</t>
+        </is>
+      </c>
+      <c r="D160" t="inlineStr">
+        <is>
+          <t>Moong Fingers</t>
+        </is>
+      </c>
+      <c r="E160" t="inlineStr">
+        <is>
+          <t>மூங் ஃபிங்கர்ஸ்</t>
+        </is>
+      </c>
+      <c r="F160" t="inlineStr">
+        <is>
+          <t>fried-snack</t>
+        </is>
+      </c>
+      <c r="G160" t="inlineStr">
+        <is>
+          <t>Professional food photography of "Moong Fingers" (மூங் ஃபிங்கர்ஸ்), an Indian snack: golden-brown, deep-fried finger-shaped croquettes with a crisp exterior, made from cooked moong dal and soaked bread mixed with herbs and spices, piled on a plate with tomato sauce for dipping. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
+        </is>
+      </c>
+      <c r="H160" t="inlineStr">
+        <is>
+          <t>public/images/recipes/moong-fingers/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I160" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="n">
+        <v>160</v>
+      </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>Vegetarian</t>
+        </is>
+      </c>
+      <c r="C161" t="inlineStr">
+        <is>
+          <t>potato-roll</t>
+        </is>
+      </c>
+      <c r="D161" t="inlineStr">
+        <is>
+          <t>Potato Roll</t>
+        </is>
+      </c>
+      <c r="E161" t="inlineStr">
+        <is>
+          <t>உருளைகிழங்கு ரோல்</t>
+        </is>
+      </c>
+      <c r="F161" t="inlineStr">
+        <is>
+          <t>roll</t>
+        </is>
+      </c>
+      <c r="G161" t="inlineStr">
+        <is>
+          <t>Professional food photography of "Potato Roll" (உருளைகிழங்கு ரோல்), an Indian snack: golden-brown deep-fried cylindrical rolls made of thin wheat pastry wrapped tightly around a spiced mashed-potato filling, sliced diagonally into pieces to reveal the potato filling inside, arranged on a plate with tomato sauce. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
+        </is>
+      </c>
+      <c r="H161" t="inlineStr">
+        <is>
+          <t>public/images/recipes/potato-roll/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I161" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="n">
+        <v>161</v>
+      </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>Vegetarian</t>
+        </is>
+      </c>
+      <c r="C162" t="inlineStr">
+        <is>
+          <t>bread-roll</t>
+        </is>
+      </c>
+      <c r="D162" t="inlineStr">
+        <is>
+          <t>Bread Roll</t>
+        </is>
+      </c>
+      <c r="E162" t="inlineStr">
+        <is>
+          <t>பிரட் ரோல்</t>
+        </is>
+      </c>
+      <c r="F162" t="inlineStr">
+        <is>
+          <t>roll</t>
+        </is>
+      </c>
+      <c r="G162" t="inlineStr">
+        <is>
+          <t>Professional food photography of "Bread Roll" (பிரட் ரோல்), an Indian snack: golden-brown deep-fried cylindrical rolls made from softened bread wrapped around a spiced mixed-vegetable-and-potato filling, sliced to show the filling inside, arranged on a plate with tomato sauce. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
+        </is>
+      </c>
+      <c r="H162" t="inlineStr">
+        <is>
+          <t>public/images/recipes/bread-roll/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I162" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="n">
+        <v>162</v>
+      </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>Vegetarian</t>
+        </is>
+      </c>
+      <c r="C163" t="inlineStr">
+        <is>
+          <t>paneer-roll</t>
+        </is>
+      </c>
+      <c r="D163" t="inlineStr">
+        <is>
+          <t>Paneer Roll</t>
+        </is>
+      </c>
+      <c r="E163" t="inlineStr">
+        <is>
+          <t>பனீர் ரோல்</t>
+        </is>
+      </c>
+      <c r="F163" t="inlineStr">
+        <is>
+          <t>roll</t>
+        </is>
+      </c>
+      <c r="G163" t="inlineStr">
+        <is>
+          <t>Professional food photography of "Paneer Roll" (பனீர் ரோல்), an Indian snack: golden-brown deep-fried cylindrical rolls made from a soft paneer-and-bread dough wrapped around a sauteed onion-and-capsicum filling, sliced to show the pale filling inside, arranged on a plate with tomato sauce. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
+        </is>
+      </c>
+      <c r="H163" t="inlineStr">
+        <is>
+          <t>public/images/recipes/paneer-roll/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I163" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="n">
+        <v>163</v>
+      </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>Vegetarian</t>
+        </is>
+      </c>
+      <c r="C164" t="inlineStr">
+        <is>
+          <t>carrot-rissoles</t>
+        </is>
+      </c>
+      <c r="D164" t="inlineStr">
+        <is>
+          <t>Carrot Rissoles</t>
+        </is>
+      </c>
+      <c r="E164" t="inlineStr">
+        <is>
+          <t>கேரட் ரிசோல்ஸ்</t>
+        </is>
+      </c>
+      <c r="F164" t="inlineStr">
+        <is>
+          <t>cutlet</t>
+        </is>
+      </c>
+      <c r="G164" t="inlineStr">
+        <is>
+          <t>Professional food photography of "Carrot Rissoles" (கேரட் ரிசோல்ஸ்), an Indian snack: golden-brown, breadcrumb-coated, deep-fried oval croquettes made from rice, grated carrot, and sauteed onion, with a crisp crumbed exterior, arranged on a plate with tomato sauce. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
+        </is>
+      </c>
+      <c r="H164" t="inlineStr">
+        <is>
+          <t>public/images/recipes/carrot-rissoles/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I164" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="n">
+        <v>164</v>
+      </c>
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>Vegetarian</t>
+        </is>
+      </c>
+      <c r="C165" t="inlineStr">
+        <is>
+          <t>double-beans-rissoles</t>
+        </is>
+      </c>
+      <c r="D165" t="inlineStr">
+        <is>
+          <t>Double Bean Rissoles</t>
+        </is>
+      </c>
+      <c r="E165" t="inlineStr">
+        <is>
+          <t>டபுள் பீன்ஸ் ரிசோல்ஸ்</t>
+        </is>
+      </c>
+      <c r="F165" t="inlineStr">
+        <is>
+          <t>cutlet</t>
+        </is>
+      </c>
+      <c r="G165" t="inlineStr">
+        <is>
+          <t>Professional food photography of "Double Bean Rissoles" (டபுள் பீன்ஸ் ரிசோல்ஸ்), an Indian snack: small round, deep-fried fritters with a rough, textured golden-brown crust, made from a coarsely ground broad-white-bean batter with onion and green chili, similar in look to a vada, piled on a plate. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
+        </is>
+      </c>
+      <c r="H165" t="inlineStr">
+        <is>
+          <t>public/images/recipes/double-beans-rissoles/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I165" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="n">
+        <v>165</v>
+      </c>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>Vegetarian</t>
+        </is>
+      </c>
+      <c r="C166" t="inlineStr">
+        <is>
+          <t>cabbage-steaks</t>
+        </is>
+      </c>
+      <c r="D166" t="inlineStr">
+        <is>
+          <t>Cabbage Steaks</t>
+        </is>
+      </c>
+      <c r="E166" t="inlineStr">
+        <is>
+          <t>முட்டைகோஸ் ஸ்டீக்ஸ்</t>
+        </is>
+      </c>
+      <c r="F166" t="inlineStr">
+        <is>
+          <t>fried-snack</t>
+        </is>
+      </c>
+      <c r="G166" t="inlineStr">
+        <is>
+          <t>Professional food photography of "Cabbage Steaks" (முட்டைகோஸ் ஸ்டீக்ஸ்), an Indian snack: round, flat, pan-fried patties with a golden-brown seared surface, made from a spiced chana-dal-and-grated-cabbage batter that was steamed into a log then sliced into rounds and shallow-fried, arranged on a plate. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
+        </is>
+      </c>
+      <c r="H166" t="inlineStr">
+        <is>
+          <t>public/images/recipes/cabbage-steaks/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I166" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="n">
+        <v>166</v>
+      </c>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>Vegetarian</t>
+        </is>
+      </c>
+      <c r="C167" t="inlineStr">
+        <is>
+          <t>pesalu-kadiyalu</t>
+        </is>
+      </c>
+      <c r="D167" t="inlineStr">
+        <is>
+          <t>Pesalu Kadiyalu</t>
+        </is>
+      </c>
+      <c r="E167" t="inlineStr">
+        <is>
+          <t>பெசலு கடியாலு</t>
+        </is>
+      </c>
+      <c r="F167" t="inlineStr">
+        <is>
+          <t>fried-snack</t>
+        </is>
+      </c>
+      <c r="G167" t="inlineStr">
+        <is>
+          <t>Professional food photography of "Pesalu Kadiyalu" (பெசலு கடியாலு), an Andhra-style South Indian snack: golden-brown deep-fried ring-shaped fritters (like a savory donut), made from a ground moong-and-urad-dal-and-banana batter, with a crisp, slightly bumpy fried surface, served on a plate with white coconut chutney. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
+        </is>
+      </c>
+      <c r="H167" t="inlineStr">
+        <is>
+          <t>public/images/recipes/pesalu-kadiyalu/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I167" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="n">
+        <v>167</v>
+      </c>
+      <c r="B168" t="inlineStr">
+        <is>
+          <t>Vegetarian</t>
+        </is>
+      </c>
+      <c r="C168" t="inlineStr">
+        <is>
+          <t>rice-flour-rings</t>
+        </is>
+      </c>
+      <c r="D168" t="inlineStr">
+        <is>
+          <t>Rice Flour Rings</t>
+        </is>
+      </c>
+      <c r="E168" t="inlineStr">
+        <is>
+          <t>அரிசிமாவு கோடிபேடலு</t>
+        </is>
+      </c>
+      <c r="F168" t="inlineStr">
+        <is>
+          <t>fried-snack</t>
+        </is>
+      </c>
+      <c r="G168" t="inlineStr">
+        <is>
+          <t>Professional food photography of "Rice Flour Rings" (அரிசிமாவு கோடிபேடலு), a South Indian tea-time snack: small golden-brown deep-fried rings shaped like a chain link, made from a cooked rice-flour dough seasoned with pepper and cumin, with a smooth glossy fried crust, piled on a plate with coconut chutney. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
+        </is>
+      </c>
+      <c r="H168" t="inlineStr">
+        <is>
+          <t>public/images/recipes/rice-flour-rings/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I168" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" t="n">
+        <v>168</v>
+      </c>
+      <c r="B169" t="inlineStr">
+        <is>
+          <t>Vegetarian</t>
+        </is>
+      </c>
+      <c r="C169" t="inlineStr">
+        <is>
+          <t>chinese-vegetable-fritters</t>
+        </is>
+      </c>
+      <c r="D169" t="inlineStr">
+        <is>
+          <t>Chinese Vegetable Fritters</t>
+        </is>
+      </c>
+      <c r="E169" t="inlineStr">
+        <is>
+          <t>சீன காய்கறி பகோடா</t>
+        </is>
+      </c>
+      <c r="F169" t="inlineStr">
+        <is>
+          <t>fusion</t>
+        </is>
+      </c>
+      <c r="G169" t="inlineStr">
+        <is>
+          <t>Professional food photography of "Chinese Vegetable Fritters" (சீன காய்கறி பகோடா), an Indo-Chinese street-food snack: irregularly shaped, deep-fried golden-brown fritters made from julienned cabbage, carrot, and capsicum bound in a light batter seasoned with soy sauce and chili sauce, crisp and craggy-textured, piled on a plate. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
+        </is>
+      </c>
+      <c r="H169" t="inlineStr">
+        <is>
+          <t>public/images/recipes/chinese-vegetable-fritters/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I169" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" t="n">
+        <v>169</v>
+      </c>
+      <c r="B170" t="inlineStr">
+        <is>
+          <t>Vegetarian</t>
+        </is>
+      </c>
+      <c r="C170" t="inlineStr">
+        <is>
+          <t>cauliflower-fritters</t>
+        </is>
+      </c>
+      <c r="D170" t="inlineStr">
+        <is>
+          <t>Cauliflower Fritters</t>
+        </is>
+      </c>
+      <c r="E170" t="inlineStr">
+        <is>
+          <t>காலிப்ளவர் ஃபிரிட்டர்ஸ்</t>
+        </is>
+      </c>
+      <c r="F170" t="inlineStr">
+        <is>
+          <t>fried-snack</t>
+        </is>
+      </c>
+      <c r="G170" t="inlineStr">
+        <is>
+          <t>Professional food photography of "Cauliflower Fritters" (காலிப்ளவர் ஃபிரிட்டர்ஸ்), an Indian snack: golden-brown, crisp, batter-coated and breadcrumbed deep-fried cauliflower florets, piled on a plate with tomato sauce for dipping. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
+        </is>
+      </c>
+      <c r="H170" t="inlineStr">
+        <is>
+          <t>public/images/recipes/cauliflower-fritters/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I170" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="n">
+        <v>170</v>
+      </c>
+      <c r="B171" t="inlineStr">
+        <is>
+          <t>Vegetarian</t>
+        </is>
+      </c>
+      <c r="C171" t="inlineStr">
+        <is>
+          <t>chinese-cauliflower-manchurian</t>
+        </is>
+      </c>
+      <c r="D171" t="inlineStr">
+        <is>
+          <t>Chinese Cauliflower Manchurian</t>
+        </is>
+      </c>
+      <c r="E171" t="inlineStr">
+        <is>
+          <t>சீன காலிப்ளவர் மஞ்சூரியன்</t>
+        </is>
+      </c>
+      <c r="F171" t="inlineStr">
+        <is>
+          <t>fusion</t>
+        </is>
+      </c>
+      <c r="G171" t="inlineStr">
+        <is>
+          <t>Professional food photography of "Chinese Cauliflower Manchurian" (சீன காலிப்ளவர் மஞ்சூரியன்), a popular Indo-Chinese dish: deep-fried cauliflower florets coated in a glossy, thick, dark reddish-brown Manchurian sauce (soy, chili, ginger-garlic), served dry-style on a plate, garnished with chopped spring onion greens. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
+        </is>
+      </c>
+      <c r="H171" t="inlineStr">
+        <is>
+          <t>public/images/recipes/chinese-cauliflower-manchurian/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I171" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="n">
+        <v>171</v>
+      </c>
+      <c r="B172" t="inlineStr">
+        <is>
+          <t>Vegetarian</t>
+        </is>
+      </c>
+      <c r="C172" t="inlineStr">
+        <is>
+          <t>potato-fritters</t>
+        </is>
+      </c>
+      <c r="D172" t="inlineStr">
+        <is>
+          <t>Potato Fritters</t>
+        </is>
+      </c>
+      <c r="E172" t="inlineStr">
+        <is>
+          <t>உருளை வறுவல்</t>
+        </is>
+      </c>
+      <c r="F172" t="inlineStr">
+        <is>
+          <t>fried-snack</t>
+        </is>
+      </c>
+      <c r="G172" t="inlineStr">
+        <is>
+          <t>Professional food photography of "Potato Fritters" (உருளை வறுவல்), an Indian snack: thin round potato slices coated in a spiced reddish-orange ground masala paste (fennel, garlic, ginger, dried chili, roasted gram) and shallow-fried until golden and slightly crisp on both sides, arranged overlapping on a plate. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
+        </is>
+      </c>
+      <c r="H172" t="inlineStr">
+        <is>
+          <t>public/images/recipes/potato-fritters/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I172" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" t="n">
+        <v>172</v>
+      </c>
+      <c r="B173" t="inlineStr">
+        <is>
+          <t>Vegetarian</t>
+        </is>
+      </c>
+      <c r="C173" t="inlineStr">
+        <is>
+          <t>banana-fritters</t>
+        </is>
+      </c>
+      <c r="D173" t="inlineStr">
+        <is>
+          <t>Banana Fritters</t>
+        </is>
+      </c>
+      <c r="E173" t="inlineStr">
+        <is>
+          <t>வாழைக்காய் வறுவல்</t>
+        </is>
+      </c>
+      <c r="F173" t="inlineStr">
+        <is>
+          <t>fried-snack</t>
+        </is>
+      </c>
+      <c r="G173" t="inlineStr">
+        <is>
+          <t>Professional food photography of "Banana Fritters" (வாழைக்காய் வறுவல்), an Indian snack: thin round raw-banana slices coated in a spiced reddish-brown ground masala paste (chana dal, dried chili, coriander seeds, shallots) and deep-fried until golden and crisp, arranged overlapping on a plate. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
+        </is>
+      </c>
+      <c r="H173" t="inlineStr">
+        <is>
+          <t>public/images/recipes/banana-fritters/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I173" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="n">
+        <v>173</v>
+      </c>
+      <c r="B174" t="inlineStr">
+        <is>
+          <t>Vegetarian</t>
+        </is>
+      </c>
+      <c r="C174" t="inlineStr">
+        <is>
+          <t>bread-fritters</t>
+        </is>
+      </c>
+      <c r="D174" t="inlineStr">
+        <is>
+          <t>Bread Fritters</t>
+        </is>
+      </c>
+      <c r="E174" t="inlineStr">
+        <is>
+          <t>பிரட் தங்க வறுவல்</t>
+        </is>
+      </c>
+      <c r="F174" t="inlineStr">
+        <is>
+          <t>fried-snack</t>
+        </is>
+      </c>
+      <c r="G174" t="inlineStr">
+        <is>
+          <t>Professional food photography of "Bread Fritters" (பிரட் தங்க வறுவல்), an Indian snack: small bread squares dipped in a spiced gram-flour-and-rice-flour batter and shallow-fried on a griddle until golden-brown and crisp, piled on a plate with tomato sauce. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
+        </is>
+      </c>
+      <c r="H174" t="inlineStr">
+        <is>
+          <t>public/images/recipes/bread-fritters/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I174" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" t="n">
+        <v>174</v>
+      </c>
+      <c r="B175" t="inlineStr">
+        <is>
+          <t>Vegetarian</t>
+        </is>
+      </c>
+      <c r="C175" t="inlineStr">
+        <is>
+          <t>potato-cheese-croquettes</t>
+        </is>
+      </c>
+      <c r="D175" t="inlineStr">
+        <is>
+          <t>Potato Cheese Croquettes</t>
+        </is>
+      </c>
+      <c r="E175" t="inlineStr">
+        <is>
+          <t>உருளைக்கிழங்கு சீஸ் கட்லெட்</t>
+        </is>
+      </c>
+      <c r="F175" t="inlineStr">
+        <is>
+          <t>cutlet</t>
+        </is>
+      </c>
+      <c r="G175" t="inlineStr">
+        <is>
+          <t>Professional food photography of "Potato Cheese Croquettes" (உருளைக்கிழங்கு சீஸ் கட்லெட்), an Indian snack: round, flattened, golden-brown deep-fried patties made from mashed potato and melted cheese with a crisp crumbed crust, one croquette broken in half showing a soft, slightly stringy cheese-flecked interior, served with tomato sauce. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
+        </is>
+      </c>
+      <c r="H175" t="inlineStr">
+        <is>
+          <t>public/images/recipes/potato-cheese-croquettes/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I175" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" t="n">
+        <v>175</v>
+      </c>
+      <c r="B176" t="inlineStr">
+        <is>
+          <t>Vegetarian</t>
+        </is>
+      </c>
+      <c r="C176" t="inlineStr">
+        <is>
+          <t>potato-baskets</t>
+        </is>
+      </c>
+      <c r="D176" t="inlineStr">
+        <is>
+          <t>Potato Baskets</t>
+        </is>
+      </c>
+      <c r="E176" t="inlineStr">
+        <is>
+          <t>உருளைக்கிழங்கு கூடைகள்</t>
+        </is>
+      </c>
+      <c r="F176" t="inlineStr">
+        <is>
+          <t>fried-snack</t>
+        </is>
+      </c>
+      <c r="G176" t="inlineStr">
+        <is>
+          <t>Professional food photography of "Potato Baskets" (உருளைக்கிழங்கு கூடைகள்), an Indian party snack: small golden-brown deep-fried baskets woven from fine shredded potato strands into a crisp, lacy, bird's-nest-like bowl shape, filled with a colorful chopped vegetable salad, arranged on a plate. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
+        </is>
+      </c>
+      <c r="H176" t="inlineStr">
+        <is>
+          <t>public/images/recipes/potato-baskets/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I176" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" t="n">
+        <v>176</v>
+      </c>
+      <c r="B177" t="inlineStr">
+        <is>
+          <t>Vegetarian</t>
+        </is>
+      </c>
+      <c r="C177" t="inlineStr">
+        <is>
+          <t>vegetable-puffs</t>
+        </is>
+      </c>
+      <c r="D177" t="inlineStr">
+        <is>
+          <t>Vegetable Puffs</t>
+        </is>
+      </c>
+      <c r="E177" t="inlineStr">
+        <is>
+          <t>வெஜிடபிள் பஃப்</t>
+        </is>
+      </c>
+      <c r="F177" t="inlineStr">
+        <is>
+          <t>snack</t>
+        </is>
+      </c>
+      <c r="G177" t="inlineStr">
+        <is>
+          <t>Professional food photography of "Vegetable Puffs" (வெஜிடபிள் பஃப்), a bakery-style Indian snack: golden-brown baked triangular puff pastries with a flaky, many-layered crust, one puff broken open to reveal a spiced potato-and-mixed-vegetable filling, arranged on a plate with tomato sauce. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
+        </is>
+      </c>
+      <c r="H177" t="inlineStr">
+        <is>
+          <t>public/images/recipes/vegetable-puffs/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I177" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" t="n">
+        <v>177</v>
+      </c>
+      <c r="B178" t="inlineStr">
+        <is>
+          <t>Vegetarian</t>
+        </is>
+      </c>
+      <c r="C178" t="inlineStr">
+        <is>
+          <t>vegetable-cones</t>
+        </is>
+      </c>
+      <c r="D178" t="inlineStr">
+        <is>
+          <t>Vegetable Cones</t>
+        </is>
+      </c>
+      <c r="E178" t="inlineStr">
+        <is>
+          <t>வெஜிடபிள் கோன்ஸ்</t>
+        </is>
+      </c>
+      <c r="F178" t="inlineStr">
+        <is>
+          <t>snack</t>
+        </is>
+      </c>
+      <c r="G178" t="inlineStr">
+        <is>
+          <t>Professional food photography of "Vegetable Cones" (வெஜிடபிள் கோன்ஸ்), a bakery-style Indian snack: golden-brown baked cone-shaped flaky puff-pastry shells (shaped like small ice-cream cones), filled generously with a spiced potato-and-mixed-vegetable filling, standing upright on a plate. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
+        </is>
+      </c>
+      <c r="H178" t="inlineStr">
+        <is>
+          <t>public/images/recipes/vegetable-cones/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I178" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" t="n">
+        <v>178</v>
+      </c>
+      <c r="B179" t="inlineStr">
+        <is>
+          <t>Vegetarian</t>
+        </is>
+      </c>
+      <c r="C179" t="inlineStr">
+        <is>
+          <t>vol-au-vent-cases</t>
+        </is>
+      </c>
+      <c r="D179" t="inlineStr">
+        <is>
+          <t>Vol-au-vent Cases</t>
+        </is>
+      </c>
+      <c r="E179" t="inlineStr">
+        <is>
+          <t>பஃப் டப்பிகள்</t>
+        </is>
+      </c>
+      <c r="F179" t="inlineStr">
+        <is>
+          <t>snack</t>
+        </is>
+      </c>
+      <c r="G179" t="inlineStr">
+        <is>
+          <t>Professional food photography of "Vol-au-vent Cases" (பஃப் டப்பிகள்), a bakery-style Indian snack: small round, golden-brown baked puff-pastry boxes with tall flaky layered walls, filled with a spiced potato-and-vegetable filling, with a puff-pastry lid resting beside the filled case, arranged on a plate. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
+        </is>
+      </c>
+      <c r="H179" t="inlineStr">
+        <is>
+          <t>public/images/recipes/vol-au-vent-cases/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I179" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="n">
+        <v>179</v>
+      </c>
+      <c r="B180" t="inlineStr">
+        <is>
+          <t>Vegetarian</t>
+        </is>
+      </c>
+      <c r="C180" t="inlineStr">
+        <is>
+          <t>baked-brinjals</t>
+        </is>
+      </c>
+      <c r="D180" t="inlineStr">
+        <is>
+          <t>Baked Brinjals</t>
+        </is>
+      </c>
+      <c r="E180" t="inlineStr">
+        <is>
+          <t>பேக்டு பிரின்ஜால்</t>
+        </is>
+      </c>
+      <c r="F180" t="inlineStr">
+        <is>
+          <t>snack</t>
+        </is>
+      </c>
+      <c r="G180" t="inlineStr">
+        <is>
+          <t>Professional food photography of "Baked Brinjals" (பேக்டு பிரின்ஜால்), an Indian baked dish: a round baking dish layered with crisp fried breaded brinjal rounds, tomato sauce, and melted golden-brown bubbling cheese on top, served warm straight from the oven. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
+        </is>
+      </c>
+      <c r="H180" t="inlineStr">
+        <is>
+          <t>public/images/recipes/baked-brinjals/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I180" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" t="n">
+        <v>180</v>
+      </c>
+      <c r="B181" t="inlineStr">
+        <is>
+          <t>Vegetarian</t>
+        </is>
+      </c>
+      <c r="C181" t="inlineStr">
+        <is>
+          <t>stuffed-capsicum</t>
+        </is>
+      </c>
+      <c r="D181" t="inlineStr">
+        <is>
+          <t>Stuffed Capsicum</t>
+        </is>
+      </c>
+      <c r="E181" t="inlineStr">
+        <is>
+          <t>ஸ்டப் செய்த குடமிளகாய்</t>
+        </is>
+      </c>
+      <c r="F181" t="inlineStr">
+        <is>
+          <t>snack</t>
+        </is>
+      </c>
+      <c r="G181" t="inlineStr">
+        <is>
+          <t>Professional food photography of "Stuffed Capsicum" (ஸ்டப் செய்த குடமிளகாய்), an Indian dish: capsicum halves filled with a spiced mixed-vegetable filling, pan-cooked with a thin golden gram-flour crust on the cut surface, arranged filling-side up on a plate. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
+        </is>
+      </c>
+      <c r="H181" t="inlineStr">
+        <is>
+          <t>public/images/recipes/stuffed-capsicum/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I181" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" t="n">
+        <v>181</v>
+      </c>
+      <c r="B182" t="inlineStr">
+        <is>
+          <t>Vegetarian</t>
+        </is>
+      </c>
+      <c r="C182" t="inlineStr">
+        <is>
+          <t>stuffed-tomatoes</t>
+        </is>
+      </c>
+      <c r="D182" t="inlineStr">
+        <is>
+          <t>Stuffed Tomatoes</t>
+        </is>
+      </c>
+      <c r="E182" t="inlineStr">
+        <is>
+          <t>ஸ்டப் செய்த தக்காளி</t>
+        </is>
+      </c>
+      <c r="F182" t="inlineStr">
+        <is>
+          <t>snack</t>
+        </is>
+      </c>
+      <c r="G182" t="inlineStr">
+        <is>
+          <t>Professional food photography of "Stuffed Tomatoes" (ஸ்டப் செய்த தக்காளி), an Indian baked dish: whole ripe tomatoes with their tops sliced off, hollowed and filled with a spiced mixed-vegetable filling, topped with melted golden-brown cheese, baked and arranged on a plate. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
+        </is>
+      </c>
+      <c r="H182" t="inlineStr">
+        <is>
+          <t>public/images/recipes/stuffed-tomatoes/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I182" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" t="n">
+        <v>182</v>
+      </c>
+      <c r="B183" t="inlineStr">
+        <is>
+          <t>Vegetarian</t>
+        </is>
+      </c>
+      <c r="C183" t="inlineStr">
+        <is>
+          <t>pizza</t>
+        </is>
+      </c>
+      <c r="D183" t="inlineStr">
+        <is>
+          <t>Pizza</t>
+        </is>
+      </c>
+      <c r="E183" t="inlineStr">
+        <is>
+          <t>பிஸ்ஸா</t>
+        </is>
+      </c>
+      <c r="F183" t="inlineStr">
+        <is>
+          <t>fusion</t>
+        </is>
+      </c>
+      <c r="G183" t="inlineStr">
+        <is>
+          <t>Professional food photography of a homemade "Pizza" (பிஸ்ஸா): a round, golden-baked bread crust topped with tomato sauce, sliced rounds of onion, tomato, and capsicum, and a generous layer of melted, lightly browned bubbly cheese, served whole on a wooden board. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
+        </is>
+      </c>
+      <c r="H183" t="inlineStr">
+        <is>
+          <t>public/images/recipes/pizza/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I183" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" t="n">
+        <v>183</v>
+      </c>
+      <c r="B184" t="inlineStr">
+        <is>
+          <t>Vegetarian</t>
+        </is>
+      </c>
+      <c r="C184" t="inlineStr">
+        <is>
+          <t>moong-dal-banzi</t>
+        </is>
+      </c>
+      <c r="D184" t="inlineStr">
+        <is>
+          <t>Moong Dal Banzi</t>
+        </is>
+      </c>
+      <c r="E184" t="inlineStr">
+        <is>
+          <t>பாசிப்பயறு பன்ஸி</t>
+        </is>
+      </c>
+      <c r="F184" t="inlineStr">
+        <is>
+          <t>snack</t>
+        </is>
+      </c>
+      <c r="G184" t="inlineStr">
+        <is>
+          <t>Professional food photography of "Moong Dal Banzi" (பாசிப்பயறு பன்ஸி), an Indian snack: a thick, round, griddle-cooked stuffed flatbread with a lightly charred, leaf-textured surface (cooked between banana leaves), cut into wedges revealing a spiced moong-dal-and-vegetable filling inside, served with chutney. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
+        </is>
+      </c>
+      <c r="H184" t="inlineStr">
+        <is>
+          <t>public/images/recipes/moong-dal-banzi/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I184" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" t="n">
+        <v>184</v>
+      </c>
+      <c r="B185" t="inlineStr">
+        <is>
+          <t>Vegetarian</t>
+        </is>
+      </c>
+      <c r="C185" t="inlineStr">
+        <is>
+          <t>handvo</t>
+        </is>
+      </c>
+      <c r="D185" t="inlineStr">
+        <is>
+          <t>Handvo</t>
+        </is>
+      </c>
+      <c r="E185" t="inlineStr">
+        <is>
+          <t>ஹண்ட்வோ</t>
+        </is>
+      </c>
+      <c r="F185" t="inlineStr">
+        <is>
+          <t>fusion</t>
+        </is>
+      </c>
+      <c r="G185" t="inlineStr">
+        <is>
+          <t>Professional food photography of "Handvo" (ஹண்ட்வோ), a Gujarati savory cake: a thick, golden-brown pan-fried lentil-and-rice cake with a crisp, seed-flecked crust (mustard seeds and sesame visible on top), sliced into squares, arranged on a plate. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
+        </is>
+      </c>
+      <c r="H185" t="inlineStr">
+        <is>
+          <t>public/images/recipes/handvo/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I185" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" t="n">
+        <v>185</v>
+      </c>
+      <c r="B186" t="inlineStr">
+        <is>
+          <t>Vegetarian</t>
+        </is>
+      </c>
+      <c r="C186" t="inlineStr">
+        <is>
+          <t>khandvi</t>
+        </is>
+      </c>
+      <c r="D186" t="inlineStr">
+        <is>
+          <t>Khandvi</t>
+        </is>
+      </c>
+      <c r="E186" t="inlineStr">
+        <is>
+          <t>கண்ட்வி</t>
+        </is>
+      </c>
+      <c r="F186" t="inlineStr">
+        <is>
+          <t>fusion</t>
+        </is>
+      </c>
+      <c r="G186" t="inlineStr">
+        <is>
+          <t>Professional food photography of "Khandvi" (கண்ட்வி), a Gujarati snack: small, tightly rolled, pale-yellow gram-flour spirals (bite-sized pinwheels) arranged on a plate, topped with a mustard-seed tempering, grated coconut, and chopped coriander leaves. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
+        </is>
+      </c>
+      <c r="H186" t="inlineStr">
+        <is>
+          <t>public/images/recipes/khandvi/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I186" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" t="n">
+        <v>186</v>
+      </c>
+      <c r="B187" t="inlineStr">
+        <is>
+          <t>Vegetarian</t>
+        </is>
+      </c>
+      <c r="C187" t="inlineStr">
+        <is>
+          <t>spring-rolls</t>
+        </is>
+      </c>
+      <c r="D187" t="inlineStr">
+        <is>
+          <t>Spring Rolls</t>
+        </is>
+      </c>
+      <c r="E187" t="inlineStr">
+        <is>
+          <t>ஸ்பிரிங் ரோல்</t>
+        </is>
+      </c>
+      <c r="F187" t="inlineStr">
+        <is>
+          <t>fusion</t>
+        </is>
+      </c>
+      <c r="G187" t="inlineStr">
+        <is>
+          <t>Professional food photography of "Spring Rolls" (ஸ்பிரிங் ரோல்), an Indo-Chinese snack: golden-brown deep-fried cylindrical rolls with a thin crisp pastry shell, sliced into rounds showing a colorful julienned cabbage-carrot-capsicum filling inside, arranged on a plate with tomato sauce. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
+        </is>
+      </c>
+      <c r="H187" t="inlineStr">
+        <is>
+          <t>public/images/recipes/spring-rolls/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I187" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" t="n">
+        <v>187</v>
+      </c>
+      <c r="B188" t="inlineStr">
+        <is>
+          <t>Vegetarian</t>
+        </is>
+      </c>
+      <c r="C188" t="inlineStr">
+        <is>
+          <t>wontons</t>
+        </is>
+      </c>
+      <c r="D188" t="inlineStr">
+        <is>
+          <t>Wontons</t>
+        </is>
+      </c>
+      <c r="E188" t="inlineStr">
+        <is>
+          <t>ஒன்டன்ஸ்</t>
+        </is>
+      </c>
+      <c r="F188" t="inlineStr">
+        <is>
+          <t>fusion</t>
+        </is>
+      </c>
+      <c r="G188" t="inlineStr">
+        <is>
+          <t>Professional food photography of "Wontons" (ஒன்டன்ஸ்), an Indo-Chinese snack: small golden-brown deep-fried dumplings with pleated, gathered pastry tops enclosing a vegetable filling, piled on a plate with tomato sauce. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
+        </is>
+      </c>
+      <c r="H188" t="inlineStr">
+        <is>
+          <t>public/images/recipes/wontons/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I188" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" t="n">
+        <v>188</v>
+      </c>
+      <c r="B189" t="inlineStr">
+        <is>
+          <t>Vegetarian</t>
+        </is>
+      </c>
+      <c r="C189" t="inlineStr">
+        <is>
+          <t>crispy-toasts</t>
+        </is>
+      </c>
+      <c r="D189" t="inlineStr">
+        <is>
+          <t>Crispy Toasts</t>
+        </is>
+      </c>
+      <c r="E189" t="inlineStr">
+        <is>
+          <t>சைனீஸ் பொரித்த டோஸ்ட்</t>
+        </is>
+      </c>
+      <c r="F189" t="inlineStr">
+        <is>
+          <t>fusion</t>
+        </is>
+      </c>
+      <c r="G189" t="inlineStr">
+        <is>
+          <t>Professional food photography of "Crispy Toasts" (சைனீஸ் பொரித்த டோஸ்ட்), an Indo-Chinese snack: golden-brown fried bread squares with a spiced mashed-potato-and-vegetable layer pressed onto one side, crisp at the edges, piled on a plate with tomato sauce. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
+        </is>
+      </c>
+      <c r="H189" t="inlineStr">
+        <is>
+          <t>public/images/recipes/crispy-toasts/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I189" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" t="n">
+        <v>189</v>
+      </c>
+      <c r="B190" t="inlineStr">
+        <is>
+          <t>Vegetarian</t>
+        </is>
+      </c>
+      <c r="C190" t="inlineStr">
+        <is>
+          <t>vegetable-pan-cake</t>
+        </is>
+      </c>
+      <c r="D190" t="inlineStr">
+        <is>
+          <t>Vegetable Pan Cake</t>
+        </is>
+      </c>
+      <c r="E190" t="inlineStr">
+        <is>
+          <t>காய்கறி பான் கேக்</t>
+        </is>
+      </c>
+      <c r="F190" t="inlineStr">
+        <is>
+          <t>snack</t>
+        </is>
+      </c>
+      <c r="G190" t="inlineStr">
+        <is>
+          <t>Professional food photography of "Vegetable Pan Cake" (காய்கறி பான் கேக்), an Indian flatbread snack: a round, golden-brown, griddle-cooked spiral flatbread with a crisp seared surface, cut in half to reveal a tight coiled spiral of dough layered with raw chopped vegetables inside, served with tomato-based thokku. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
+        </is>
+      </c>
+      <c r="H190" t="inlineStr">
+        <is>
+          <t>public/images/recipes/vegetable-pan-cake/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I190" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" t="n">
+        <v>190</v>
+      </c>
+      <c r="B191" t="inlineStr">
+        <is>
+          <t>Vegetarian</t>
+        </is>
+      </c>
+      <c r="C191" t="inlineStr">
+        <is>
+          <t>mixed-vegetable-kabab</t>
+        </is>
+      </c>
+      <c r="D191" t="inlineStr">
+        <is>
+          <t>Mixed Vegetable Kabab</t>
+        </is>
+      </c>
+      <c r="E191" t="inlineStr">
+        <is>
+          <t>காய்கறி கபாப்</t>
+        </is>
+      </c>
+      <c r="F191" t="inlineStr">
+        <is>
+          <t>kabab</t>
+        </is>
+      </c>
+      <c r="G191" t="inlineStr">
+        <is>
+          <t>Professional food photography of "Mixed Vegetable Kabab" (காய்கறி கபாப்), an Indian snack: golden-brown deep-fried oblong kabab logs made from a mashed mixed-vegetable dough, arranged on a plate with mint chutney, sweet chutney, and a side of tangy marinated onion strips. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
+        </is>
+      </c>
+      <c r="H191" t="inlineStr">
+        <is>
+          <t>public/images/recipes/mixed-vegetable-kabab/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I191" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" t="n">
+        <v>191</v>
+      </c>
+      <c r="B192" t="inlineStr">
+        <is>
+          <t>Vegetarian</t>
+        </is>
+      </c>
+      <c r="C192" t="inlineStr">
+        <is>
+          <t>potato-kababs</t>
+        </is>
+      </c>
+      <c r="D192" t="inlineStr">
+        <is>
+          <t>Potato Kababs</t>
+        </is>
+      </c>
+      <c r="E192" t="inlineStr">
+        <is>
+          <t>உருளைக்கிழங்கு கபாப்</t>
+        </is>
+      </c>
+      <c r="F192" t="inlineStr">
+        <is>
+          <t>kabab</t>
+        </is>
+      </c>
+      <c r="G192" t="inlineStr">
+        <is>
+          <t>Professional food photography of "Potato Kababs" (உருளைக்கிழங்கு கபாப்), an Indian snack: golden-brown deep-fried oblong kabab logs made from spiced mashed potato studded with fresh herbs, arranged on a plate with mint chutney. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
+        </is>
+      </c>
+      <c r="H192" t="inlineStr">
+        <is>
+          <t>public/images/recipes/potato-kababs/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I192" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" t="n">
+        <v>192</v>
+      </c>
+      <c r="B193" t="inlineStr">
+        <is>
+          <t>Vegetarian</t>
+        </is>
+      </c>
+      <c r="C193" t="inlineStr">
+        <is>
+          <t>bottle-gourd-kababs</t>
+        </is>
+      </c>
+      <c r="D193" t="inlineStr">
+        <is>
+          <t>Bottle Gourd Kababs</t>
+        </is>
+      </c>
+      <c r="E193" t="inlineStr">
+        <is>
+          <t>சுரைக்காய் கபாப்</t>
+        </is>
+      </c>
+      <c r="F193" t="inlineStr">
+        <is>
+          <t>kabab</t>
+        </is>
+      </c>
+      <c r="G193" t="inlineStr">
+        <is>
+          <t>Professional food photography of "Bottle Gourd Kababs" (சுரைக்காய் கபாப்), an Indian snack: golden-brown deep-fried finger-shaped kababs made from a coarse ground bottle-gourd-and-chana-dal mixture, arranged on a plate with tomato sauce. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
+        </is>
+      </c>
+      <c r="H193" t="inlineStr">
+        <is>
+          <t>public/images/recipes/bottle-gourd-kababs/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I193" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" t="n">
+        <v>193</v>
+      </c>
+      <c r="B194" t="inlineStr">
+        <is>
+          <t>Vegetarian</t>
+        </is>
+      </c>
+      <c r="C194" t="inlineStr">
+        <is>
+          <t>minty-kababs</t>
+        </is>
+      </c>
+      <c r="D194" t="inlineStr">
+        <is>
+          <t>Minty Kababs</t>
+        </is>
+      </c>
+      <c r="E194" t="inlineStr">
+        <is>
+          <t>புதினா கபாப்</t>
+        </is>
+      </c>
+      <c r="F194" t="inlineStr">
+        <is>
+          <t>kabab</t>
+        </is>
+      </c>
+      <c r="G194" t="inlineStr">
+        <is>
+          <t>Professional food photography of "Minty Kababs" (புதினா கபாப்), an Indian snack: golden-brown deep-fried oblong kabab logs made from potato, carrot, and sprouted moong beans flecked with green mint and coriander, arranged on a plate with chutney. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
+        </is>
+      </c>
+      <c r="H194" t="inlineStr">
+        <is>
+          <t>public/images/recipes/minty-kababs/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I194" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" t="n">
+        <v>194</v>
+      </c>
+      <c r="B195" t="inlineStr">
+        <is>
+          <t>Vegetarian</t>
+        </is>
+      </c>
+      <c r="C195" t="inlineStr">
+        <is>
+          <t>cauliflower-kababs</t>
+        </is>
+      </c>
+      <c r="D195" t="inlineStr">
+        <is>
+          <t>Cauliflower Kababs</t>
+        </is>
+      </c>
+      <c r="E195" t="inlineStr">
+        <is>
+          <t>காலிப்ளவர் கபாப்</t>
+        </is>
+      </c>
+      <c r="F195" t="inlineStr">
+        <is>
+          <t>kabab</t>
+        </is>
+      </c>
+      <c r="G195" t="inlineStr">
+        <is>
+          <t>Professional food photography of "Cauliflower Kababs" (காலிப்ளவர் கபாப்), an Indian snack: golden-brown deep-fried oblong kabab logs made from ground cauliflower and chana dal, sliced into pieces, arranged on a plate with a side of vinegar-marinated onion rings. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
+        </is>
+      </c>
+      <c r="H195" t="inlineStr">
+        <is>
+          <t>public/images/recipes/cauliflower-kababs/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I195" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" t="n">
+        <v>195</v>
+      </c>
+      <c r="B196" t="inlineStr">
+        <is>
+          <t>Vegetarian</t>
+        </is>
+      </c>
+      <c r="C196" t="inlineStr">
+        <is>
+          <t>vegetable-cutlet</t>
+        </is>
+      </c>
+      <c r="D196" t="inlineStr">
+        <is>
+          <t>Vegetable Cutlet</t>
+        </is>
+      </c>
+      <c r="E196" t="inlineStr">
+        <is>
+          <t>வெஜிடபிள் கட்லெட்</t>
+        </is>
+      </c>
+      <c r="F196" t="inlineStr">
+        <is>
+          <t>cutlet</t>
+        </is>
+      </c>
+      <c r="G196" t="inlineStr">
+        <is>
+          <t>Professional food photography of "Vegetable Cutlet" (வெஜிடபிள் கட்லெட்), an Indian snack: golden-brown pan-fried round patties with a crisp breadcrumb crust, made from mashed potato, carrot, and beetroot, showing a faint reddish tint at the edges, arranged on a plate with tomato sauce and sliced onion, tomato, and cucumber rounds. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
+        </is>
+      </c>
+      <c r="H196" t="inlineStr">
+        <is>
+          <t>public/images/recipes/vegetable-cutlet/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I196" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" t="n">
+        <v>196</v>
+      </c>
+      <c r="B197" t="inlineStr">
+        <is>
+          <t>Vegetarian</t>
+        </is>
+      </c>
+      <c r="C197" t="inlineStr">
+        <is>
+          <t>spicy-cutlet</t>
+        </is>
+      </c>
+      <c r="D197" t="inlineStr">
+        <is>
+          <t>Spicy Cutlet</t>
+        </is>
+      </c>
+      <c r="E197" t="inlineStr">
+        <is>
+          <t>காரக் கட்லெட்</t>
+        </is>
+      </c>
+      <c r="F197" t="inlineStr">
+        <is>
+          <t>cutlet</t>
+        </is>
+      </c>
+      <c r="G197" t="inlineStr">
+        <is>
+          <t>Professional food photography of "Spicy Cutlet" (காரக் கட்லெட்), an Indian snack: golden-brown pan-fried round patties with a crisp breadcrumb crust, made from a spiced mix of potato, carrot, cabbage, and beans, arranged on a plate with tomato sauce. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
+        </is>
+      </c>
+      <c r="H197" t="inlineStr">
+        <is>
+          <t>public/images/recipes/spicy-cutlet/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I197" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" t="n">
+        <v>197</v>
+      </c>
+      <c r="B198" t="inlineStr">
+        <is>
+          <t>Vegetarian</t>
+        </is>
+      </c>
+      <c r="C198" t="inlineStr">
+        <is>
+          <t>beetroot-cutlets</t>
+        </is>
+      </c>
+      <c r="D198" t="inlineStr">
+        <is>
+          <t>Beetroot Cutlets</t>
+        </is>
+      </c>
+      <c r="E198" t="inlineStr">
+        <is>
+          <t>பீட்ரூட் கட்லெட்</t>
+        </is>
+      </c>
+      <c r="F198" t="inlineStr">
+        <is>
+          <t>cutlet</t>
+        </is>
+      </c>
+      <c r="G198" t="inlineStr">
+        <is>
+          <t>Professional food photography of "Beetroot Cutlets" (பீட்ரூட் கட்லெட்), an Indian snack: golden-brown pan-fried round patties with a crisp breadcrumb crust and a vivid magenta-pink hue showing through from the beetroot filling, arranged on a plate with tomato sauce. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
+        </is>
+      </c>
+      <c r="H198" t="inlineStr">
+        <is>
+          <t>public/images/recipes/beetroot-cutlets/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I198" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" t="n">
+        <v>198</v>
+      </c>
+      <c r="B199" t="inlineStr">
+        <is>
+          <t>Vegetarian</t>
+        </is>
+      </c>
+      <c r="C199" t="inlineStr">
+        <is>
+          <t>aloo-tikki</t>
+        </is>
+      </c>
+      <c r="D199" t="inlineStr">
+        <is>
+          <t>Aloo Tikki</t>
+        </is>
+      </c>
+      <c r="E199" t="inlineStr">
+        <is>
+          <t>ஆலூ டிக்கி</t>
+        </is>
+      </c>
+      <c r="F199" t="inlineStr">
+        <is>
+          <t>cutlet</t>
+        </is>
+      </c>
+      <c r="G199" t="inlineStr">
+        <is>
+          <t>Professional food photography of "Aloo Tikki" (ஆலூ டிக்கி), a North Indian street-food snack: round, flattened, golden-brown pan-fried potato patties with a crisp crust, one tikki broken open to reveal a bright green spiced-pea filling inside, topped with chopped onion, tomato chutney, and mint chutney. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
+        </is>
+      </c>
+      <c r="H199" t="inlineStr">
+        <is>
+          <t>public/images/recipes/aloo-tikki/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I199" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" t="n">
+        <v>199</v>
+      </c>
+      <c r="B200" t="inlineStr">
+        <is>
+          <t>Vegetarian</t>
+        </is>
+      </c>
+      <c r="C200" t="inlineStr">
+        <is>
+          <t>cheese-cutlets</t>
+        </is>
+      </c>
+      <c r="D200" t="inlineStr">
+        <is>
+          <t>Cheese Cutlets</t>
+        </is>
+      </c>
+      <c r="E200" t="inlineStr">
+        <is>
+          <t>சீஸ் கட்லெட்</t>
+        </is>
+      </c>
+      <c r="F200" t="inlineStr">
+        <is>
+          <t>cutlet</t>
+        </is>
+      </c>
+      <c r="G200" t="inlineStr">
+        <is>
+          <t>Professional food photography of "Cheese Cutlets" (சீஸ் கட்லெட்), an Indian snack: golden-brown pan-fried round patties with a crisp breadcrumb crust, made from potato, cabbage, and capsicum mixed with melted cheese, one cutlet broken in half showing a soft, slightly stringy cheese-flecked interior, arranged on a plate with tomato sauce. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
+        </is>
+      </c>
+      <c r="H200" t="inlineStr">
+        <is>
+          <t>public/images/recipes/cheese-cutlets/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I200" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" t="n">
+        <v>200</v>
+      </c>
+      <c r="B201" t="inlineStr">
+        <is>
+          <t>Vegetarian</t>
+        </is>
+      </c>
+      <c r="C201" t="inlineStr">
+        <is>
+          <t>green-cutlets</t>
+        </is>
+      </c>
+      <c r="D201" t="inlineStr">
+        <is>
+          <t>Green Cutlets</t>
+        </is>
+      </c>
+      <c r="E201" t="inlineStr">
+        <is>
+          <t>கீரை கட்லெட்</t>
+        </is>
+      </c>
+      <c r="F201" t="inlineStr">
+        <is>
+          <t>cutlet</t>
+        </is>
+      </c>
+      <c r="G201" t="inlineStr">
+        <is>
+          <t>Professional food photography of "Green Cutlets" (கீரை கட்லெட்), an Indian snack: golden-brown pan-fried round patties with a crisp breadcrumb crust, the interior visibly flecked with dark green sauteed leafy greens mixed into a lentil base, arranged on a plate with tomato sauce. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
+        </is>
+      </c>
+      <c r="H201" t="inlineStr">
+        <is>
+          <t>public/images/recipes/green-cutlets/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I201" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" t="n">
+        <v>201</v>
+      </c>
+      <c r="B202" t="inlineStr">
+        <is>
+          <t>Vegetarian</t>
+        </is>
+      </c>
+      <c r="C202" t="inlineStr">
+        <is>
+          <t>sago-cutlets</t>
+        </is>
+      </c>
+      <c r="D202" t="inlineStr">
+        <is>
+          <t>Sago Cutlets</t>
+        </is>
+      </c>
+      <c r="E202" t="inlineStr">
+        <is>
+          <t>ஜவ்வரிசி கட்லெட்</t>
+        </is>
+      </c>
+      <c r="F202" t="inlineStr">
+        <is>
+          <t>cutlet</t>
+        </is>
+      </c>
+      <c r="G202" t="inlineStr">
+        <is>
+          <t>Professional food photography of "Sago Cutlets" (ஜவ்வரிசி கட்லெட்), an Indian snack: golden-brown pan-fried round patties with a crisp breadcrumb crust, the surface and interior studded with small translucent soaked sago pearls mixed into the mashed-potato base, arranged on a plate with tomato sauce and mint chutney. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
+        </is>
+      </c>
+      <c r="H202" t="inlineStr">
+        <is>
+          <t>public/images/recipes/sago-cutlets/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I202" t="inlineStr">
+        <is>
+          <t>Not Started</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
content(images): wire featured images for street-food cookbook batch 1 (50 recipes)
Add Gemini-generated featured.jpg for all 50 recipes from the street-food/
snacks cookbook, wired into featured_image_url/alt_ta/alt_en. Update the
image tracker to Done for S.No 152-201.
</commit_message>
<xml_diff>
--- a/docs/recipe-image-tracker.xlsx
+++ b/docs/recipe-image-tracker.xlsx
@@ -8875,2254 +8875,2554 @@
       </c>
     </row>
     <row r="153">
-      <c r="A153" t="n">
+      <c r="A153" s="15" t="n">
         <v>152</v>
       </c>
-      <c r="B153" t="inlineStr">
+      <c r="B153" s="15" t="inlineStr">
         <is>
           <t>Vegetarian</t>
         </is>
       </c>
-      <c r="C153" t="inlineStr">
+      <c r="C153" s="15" t="inlineStr">
         <is>
           <t>mini-vegetable-samosa</t>
         </is>
       </c>
-      <c r="D153" t="inlineStr">
+      <c r="D153" s="15" t="inlineStr">
         <is>
           <t>Mini Vegetable Samosa</t>
         </is>
       </c>
-      <c r="E153" t="inlineStr">
+      <c r="E153" s="15" t="inlineStr">
         <is>
           <t>சிறிய சமோசா</t>
         </is>
       </c>
-      <c r="F153" t="inlineStr">
+      <c r="F153" s="15" t="inlineStr">
         <is>
           <t>fried-snack</t>
         </is>
       </c>
-      <c r="G153" t="inlineStr">
+      <c r="G153" s="15" t="inlineStr">
         <is>
           <t>Professional food photography of "Mini Vegetable Samosa" (சிறிய சமோசா), an Indian street-food snack: small triangular pastries with a crisp, flaky, deep-fried golden-brown maida crust, filled with a spiced potato-carrot-pea filling (one samosa broken open to show the filling), piled on a plate with mint chutney and tomato sauce on the side. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
         </is>
       </c>
-      <c r="H153" t="inlineStr">
+      <c r="H153" s="15" t="inlineStr">
         <is>
           <t>public/images/recipes/mini-vegetable-samosa/featured.jpg</t>
         </is>
       </c>
-      <c r="I153" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
+      <c r="I153" s="15" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J153" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="K153" s="15" t="n"/>
     </row>
     <row r="154">
-      <c r="A154" t="n">
+      <c r="A154" s="15" t="n">
         <v>153</v>
       </c>
-      <c r="B154" t="inlineStr">
+      <c r="B154" s="15" t="inlineStr">
         <is>
           <t>Vegetarian</t>
         </is>
       </c>
-      <c r="C154" t="inlineStr">
+      <c r="C154" s="15" t="inlineStr">
         <is>
           <t>punjabi-samosa</t>
         </is>
       </c>
-      <c r="D154" t="inlineStr">
+      <c r="D154" s="15" t="inlineStr">
         <is>
           <t>Punjabi Samosa</t>
         </is>
       </c>
-      <c r="E154" t="inlineStr">
+      <c r="E154" s="15" t="inlineStr">
         <is>
           <t>பஞ்சாபி சமோசா</t>
         </is>
       </c>
-      <c r="F154" t="inlineStr">
+      <c r="F154" s="15" t="inlineStr">
         <is>
           <t>fried-snack</t>
         </is>
       </c>
-      <c r="G154" t="inlineStr">
+      <c r="G154" s="15" t="inlineStr">
         <is>
           <t>Professional food photography of "Punjabi Samosa" (பஞ்சாபி சமோசா), a classic North Indian snack: large triangular pastries with a thick, crisp, deep-fried golden-brown crust, filled with a coarse spiced mashed-potato-and-pea filling studded with visible potato chunks (one samosa broken open to show the filling), served with mint chutney, sweet tamarind chutney, and tomato sauce. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
         </is>
       </c>
-      <c r="H154" t="inlineStr">
+      <c r="H154" s="15" t="inlineStr">
         <is>
           <t>public/images/recipes/punjabi-samosa/featured.jpg</t>
         </is>
       </c>
-      <c r="I154" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
+      <c r="I154" s="15" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J154" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="K154" s="15" t="n"/>
     </row>
     <row r="155">
-      <c r="A155" t="n">
+      <c r="A155" s="15" t="n">
         <v>154</v>
       </c>
-      <c r="B155" t="inlineStr">
+      <c r="B155" s="15" t="inlineStr">
         <is>
           <t>Vegetarian</t>
         </is>
       </c>
-      <c r="C155" t="inlineStr">
+      <c r="C155" s="15" t="inlineStr">
         <is>
           <t>lentil-kachori</t>
         </is>
       </c>
-      <c r="D155" t="inlineStr">
+      <c r="D155" s="15" t="inlineStr">
         <is>
           <t>Lentil Kachori</t>
         </is>
       </c>
-      <c r="E155" t="inlineStr">
+      <c r="E155" s="15" t="inlineStr">
         <is>
           <t>பருப்பு கசோரிகள்</t>
         </is>
       </c>
-      <c r="F155" t="inlineStr">
+      <c r="F155" s="15" t="inlineStr">
         <is>
           <t>fried-snack</t>
         </is>
       </c>
-      <c r="G155" t="inlineStr">
+      <c r="G155" s="15" t="inlineStr">
         <is>
           <t>Professional food photography of "Lentil Kachori" (பருப்பு கசோரிகள்), an Indian street-food snack: small round, slightly flattened deep-fried pastries with a golden-brown crust, filled with a spiced urad-and-moong-dal filling (one kachori broken open to show the dense lentil filling), served with green coriander chutney and a dark tamarind-jaggery sweet chutney. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
         </is>
       </c>
-      <c r="H155" t="inlineStr">
+      <c r="H155" s="15" t="inlineStr">
         <is>
           <t>public/images/recipes/lentil-kachori/featured.jpg</t>
         </is>
       </c>
-      <c r="I155" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
+      <c r="I155" s="15" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J155" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="K155" s="15" t="n"/>
     </row>
     <row r="156">
-      <c r="A156" t="n">
+      <c r="A156" s="15" t="n">
         <v>155</v>
       </c>
-      <c r="B156" t="inlineStr">
+      <c r="B156" s="15" t="inlineStr">
         <is>
           <t>Vegetarian</t>
         </is>
       </c>
-      <c r="C156" t="inlineStr">
+      <c r="C156" s="15" t="inlineStr">
         <is>
           <t>pani-puri</t>
         </is>
       </c>
-      <c r="D156" t="inlineStr">
+      <c r="D156" s="15" t="inlineStr">
         <is>
           <t>Pani Puri</t>
         </is>
       </c>
-      <c r="E156" t="inlineStr">
+      <c r="E156" s="15" t="inlineStr">
         <is>
           <t>பானி பூரி</t>
         </is>
       </c>
-      <c r="F156" t="inlineStr">
+      <c r="F156" s="15" t="inlineStr">
         <is>
           <t>chaat</t>
         </is>
       </c>
-      <c r="G156" t="inlineStr">
+      <c r="G156" s="15" t="inlineStr">
         <is>
           <t>Professional food photography of "Pani Puri" (பானி பூரி), a popular Indian street-food chaat: a plate of small, round, hollow, crisp golden-fried puris, one puri filled with spiced diced potato and moong sprouts and a spoonful of dark tamarind chutney, being filled with bright green mint-coriander spiced water (pani) poured from a small pitcher, with extra puris and a bowl of green pani alongside. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
         </is>
       </c>
-      <c r="H156" t="inlineStr">
+      <c r="H156" s="15" t="inlineStr">
         <is>
           <t>public/images/recipes/pani-puri/featured.jpg</t>
         </is>
       </c>
-      <c r="I156" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
+      <c r="I156" s="15" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J156" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="K156" s="15" t="n"/>
     </row>
     <row r="157">
-      <c r="A157" t="n">
+      <c r="A157" s="15" t="n">
         <v>156</v>
       </c>
-      <c r="B157" t="inlineStr">
+      <c r="B157" s="15" t="inlineStr">
         <is>
           <t>Vegetarian</t>
         </is>
       </c>
-      <c r="C157" t="inlineStr">
+      <c r="C157" s="15" t="inlineStr">
         <is>
           <t>curd-puri</t>
         </is>
       </c>
-      <c r="D157" t="inlineStr">
+      <c r="D157" s="15" t="inlineStr">
         <is>
           <t>Curd Puri (Dahi Puri)</t>
         </is>
       </c>
-      <c r="E157" t="inlineStr">
+      <c r="E157" s="15" t="inlineStr">
         <is>
           <t>தயிர் பூரி</t>
         </is>
       </c>
-      <c r="F157" t="inlineStr">
+      <c r="F157" s="15" t="inlineStr">
         <is>
           <t>chaat</t>
         </is>
       </c>
-      <c r="G157" t="inlineStr">
+      <c r="G157" s="15" t="inlineStr">
         <is>
           <t>Professional food photography of "Curd Puri" (Dahi Puri) (தயிர் பூரி), an Indian chaat snack: small crisp round puris arranged on a plate, each topped with spiced potato, a generous spoonful of thick whipped curd (yogurt), drizzled with dark tamarind-date sweet chutney, and dusted with red chili powder, roasted cumin powder, and fine sev, garnished with coriander leaves. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
         </is>
       </c>
-      <c r="H157" t="inlineStr">
+      <c r="H157" s="15" t="inlineStr">
         <is>
           <t>public/images/recipes/curd-puri/featured.jpg</t>
         </is>
       </c>
-      <c r="I157" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
+      <c r="I157" s="15" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J157" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="K157" s="15" t="n"/>
     </row>
     <row r="158">
-      <c r="A158" t="n">
+      <c r="A158" s="15" t="n">
         <v>157</v>
       </c>
-      <c r="B158" t="inlineStr">
+      <c r="B158" s="15" t="inlineStr">
         <is>
           <t>Vegetarian</t>
         </is>
       </c>
-      <c r="C158" t="inlineStr">
+      <c r="C158" s="15" t="inlineStr">
         <is>
           <t>bel-puri</t>
         </is>
       </c>
-      <c r="D158" t="inlineStr">
+      <c r="D158" s="15" t="inlineStr">
         <is>
           <t>Bhel Puri</t>
         </is>
       </c>
-      <c r="E158" t="inlineStr">
+      <c r="E158" s="15" t="inlineStr">
         <is>
           <t>பேல் பூரி</t>
         </is>
       </c>
-      <c r="F158" t="inlineStr">
+      <c r="F158" s="15" t="inlineStr">
         <is>
           <t>chaat</t>
         </is>
       </c>
-      <c r="G158" t="inlineStr">
+      <c r="G158" s="15" t="inlineStr">
         <is>
           <t>Professional food photography of "Bhel Puri" (பேல் பூரி), a Mumbai-style Indian street-food chaat: a bowl heaped with puffed rice, crushed crisp puris, potato chips, finely chopped onion and tomato, tossed with tangy tamarind chutney, green mint chutney, and garlic chutney, topped generously with crunchy fine sev (chickpea-flour noodles) and fresh coriander leaves. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
         </is>
       </c>
-      <c r="H158" t="inlineStr">
+      <c r="H158" s="15" t="inlineStr">
         <is>
           <t>public/images/recipes/bel-puri/featured.jpg</t>
         </is>
       </c>
-      <c r="I158" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
+      <c r="I158" s="15" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J158" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="K158" s="15" t="n"/>
     </row>
     <row r="159">
-      <c r="A159" t="n">
+      <c r="A159" s="15" t="n">
         <v>158</v>
       </c>
-      <c r="B159" t="inlineStr">
+      <c r="B159" s="15" t="inlineStr">
         <is>
           <t>Vegetarian</t>
         </is>
       </c>
-      <c r="C159" t="inlineStr">
+      <c r="C159" s="15" t="inlineStr">
         <is>
           <t>vegetable-fingers</t>
         </is>
       </c>
-      <c r="D159" t="inlineStr">
+      <c r="D159" s="15" t="inlineStr">
         <is>
           <t>Vegetable Fingers</t>
         </is>
       </c>
-      <c r="E159" t="inlineStr">
+      <c r="E159" s="15" t="inlineStr">
         <is>
           <t>வெஜிடபிள் ஃபிங்கர்ஸ்</t>
         </is>
       </c>
-      <c r="F159" t="inlineStr">
+      <c r="F159" s="15" t="inlineStr">
         <is>
           <t>fried-snack</t>
         </is>
       </c>
-      <c r="G159" t="inlineStr">
+      <c r="G159" s="15" t="inlineStr">
         <is>
           <t>Professional food photography of "Vegetable Fingers" (வெஜிடபிள் ஃபிங்கர்ஸ்), an Indian snack: golden-brown, deep-fried finger-shaped croquettes with a crisp exterior, made from a steamed moong-dal-and-mixed-vegetable batter, piled on a plate with tomato sauce for dipping. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
         </is>
       </c>
-      <c r="H159" t="inlineStr">
+      <c r="H159" s="15" t="inlineStr">
         <is>
           <t>public/images/recipes/vegetable-fingers/featured.jpg</t>
         </is>
       </c>
-      <c r="I159" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
+      <c r="I159" s="15" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J159" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="K159" s="15" t="n"/>
     </row>
     <row r="160">
-      <c r="A160" t="n">
+      <c r="A160" s="15" t="n">
         <v>159</v>
       </c>
-      <c r="B160" t="inlineStr">
+      <c r="B160" s="15" t="inlineStr">
         <is>
           <t>Vegetarian</t>
         </is>
       </c>
-      <c r="C160" t="inlineStr">
+      <c r="C160" s="15" t="inlineStr">
         <is>
           <t>moong-fingers</t>
         </is>
       </c>
-      <c r="D160" t="inlineStr">
+      <c r="D160" s="15" t="inlineStr">
         <is>
           <t>Moong Fingers</t>
         </is>
       </c>
-      <c r="E160" t="inlineStr">
+      <c r="E160" s="15" t="inlineStr">
         <is>
           <t>மூங் ஃபிங்கர்ஸ்</t>
         </is>
       </c>
-      <c r="F160" t="inlineStr">
+      <c r="F160" s="15" t="inlineStr">
         <is>
           <t>fried-snack</t>
         </is>
       </c>
-      <c r="G160" t="inlineStr">
+      <c r="G160" s="15" t="inlineStr">
         <is>
           <t>Professional food photography of "Moong Fingers" (மூங் ஃபிங்கர்ஸ்), an Indian snack: golden-brown, deep-fried finger-shaped croquettes with a crisp exterior, made from cooked moong dal and soaked bread mixed with herbs and spices, piled on a plate with tomato sauce for dipping. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
         </is>
       </c>
-      <c r="H160" t="inlineStr">
+      <c r="H160" s="15" t="inlineStr">
         <is>
           <t>public/images/recipes/moong-fingers/featured.jpg</t>
         </is>
       </c>
-      <c r="I160" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
+      <c r="I160" s="15" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J160" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="K160" s="15" t="n"/>
     </row>
     <row r="161">
-      <c r="A161" t="n">
+      <c r="A161" s="15" t="n">
         <v>160</v>
       </c>
-      <c r="B161" t="inlineStr">
+      <c r="B161" s="15" t="inlineStr">
         <is>
           <t>Vegetarian</t>
         </is>
       </c>
-      <c r="C161" t="inlineStr">
+      <c r="C161" s="15" t="inlineStr">
         <is>
           <t>potato-roll</t>
         </is>
       </c>
-      <c r="D161" t="inlineStr">
+      <c r="D161" s="15" t="inlineStr">
         <is>
           <t>Potato Roll</t>
         </is>
       </c>
-      <c r="E161" t="inlineStr">
+      <c r="E161" s="15" t="inlineStr">
         <is>
           <t>உருளைகிழங்கு ரோல்</t>
         </is>
       </c>
-      <c r="F161" t="inlineStr">
+      <c r="F161" s="15" t="inlineStr">
         <is>
           <t>roll</t>
         </is>
       </c>
-      <c r="G161" t="inlineStr">
+      <c r="G161" s="15" t="inlineStr">
         <is>
           <t>Professional food photography of "Potato Roll" (உருளைகிழங்கு ரோல்), an Indian snack: golden-brown deep-fried cylindrical rolls made of thin wheat pastry wrapped tightly around a spiced mashed-potato filling, sliced diagonally into pieces to reveal the potato filling inside, arranged on a plate with tomato sauce. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
         </is>
       </c>
-      <c r="H161" t="inlineStr">
+      <c r="H161" s="15" t="inlineStr">
         <is>
           <t>public/images/recipes/potato-roll/featured.jpg</t>
         </is>
       </c>
-      <c r="I161" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
+      <c r="I161" s="15" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J161" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="K161" s="15" t="n"/>
     </row>
     <row r="162">
-      <c r="A162" t="n">
+      <c r="A162" s="15" t="n">
         <v>161</v>
       </c>
-      <c r="B162" t="inlineStr">
+      <c r="B162" s="15" t="inlineStr">
         <is>
           <t>Vegetarian</t>
         </is>
       </c>
-      <c r="C162" t="inlineStr">
+      <c r="C162" s="15" t="inlineStr">
         <is>
           <t>bread-roll</t>
         </is>
       </c>
-      <c r="D162" t="inlineStr">
+      <c r="D162" s="15" t="inlineStr">
         <is>
           <t>Bread Roll</t>
         </is>
       </c>
-      <c r="E162" t="inlineStr">
+      <c r="E162" s="15" t="inlineStr">
         <is>
           <t>பிரட் ரோல்</t>
         </is>
       </c>
-      <c r="F162" t="inlineStr">
+      <c r="F162" s="15" t="inlineStr">
         <is>
           <t>roll</t>
         </is>
       </c>
-      <c r="G162" t="inlineStr">
+      <c r="G162" s="15" t="inlineStr">
         <is>
           <t>Professional food photography of "Bread Roll" (பிரட் ரோல்), an Indian snack: golden-brown deep-fried cylindrical rolls made from softened bread wrapped around a spiced mixed-vegetable-and-potato filling, sliced to show the filling inside, arranged on a plate with tomato sauce. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
         </is>
       </c>
-      <c r="H162" t="inlineStr">
+      <c r="H162" s="15" t="inlineStr">
         <is>
           <t>public/images/recipes/bread-roll/featured.jpg</t>
         </is>
       </c>
-      <c r="I162" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
+      <c r="I162" s="15" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J162" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="K162" s="15" t="n"/>
     </row>
     <row r="163">
-      <c r="A163" t="n">
+      <c r="A163" s="15" t="n">
         <v>162</v>
       </c>
-      <c r="B163" t="inlineStr">
+      <c r="B163" s="15" t="inlineStr">
         <is>
           <t>Vegetarian</t>
         </is>
       </c>
-      <c r="C163" t="inlineStr">
+      <c r="C163" s="15" t="inlineStr">
         <is>
           <t>paneer-roll</t>
         </is>
       </c>
-      <c r="D163" t="inlineStr">
+      <c r="D163" s="15" t="inlineStr">
         <is>
           <t>Paneer Roll</t>
         </is>
       </c>
-      <c r="E163" t="inlineStr">
+      <c r="E163" s="15" t="inlineStr">
         <is>
           <t>பனீர் ரோல்</t>
         </is>
       </c>
-      <c r="F163" t="inlineStr">
+      <c r="F163" s="15" t="inlineStr">
         <is>
           <t>roll</t>
         </is>
       </c>
-      <c r="G163" t="inlineStr">
+      <c r="G163" s="15" t="inlineStr">
         <is>
           <t>Professional food photography of "Paneer Roll" (பனீர் ரோல்), an Indian snack: golden-brown deep-fried cylindrical rolls made from a soft paneer-and-bread dough wrapped around a sauteed onion-and-capsicum filling, sliced to show the pale filling inside, arranged on a plate with tomato sauce. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
         </is>
       </c>
-      <c r="H163" t="inlineStr">
+      <c r="H163" s="15" t="inlineStr">
         <is>
           <t>public/images/recipes/paneer-roll/featured.jpg</t>
         </is>
       </c>
-      <c r="I163" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
+      <c r="I163" s="15" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J163" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="K163" s="15" t="n"/>
     </row>
     <row r="164">
-      <c r="A164" t="n">
+      <c r="A164" s="15" t="n">
         <v>163</v>
       </c>
-      <c r="B164" t="inlineStr">
+      <c r="B164" s="15" t="inlineStr">
         <is>
           <t>Vegetarian</t>
         </is>
       </c>
-      <c r="C164" t="inlineStr">
+      <c r="C164" s="15" t="inlineStr">
         <is>
           <t>carrot-rissoles</t>
         </is>
       </c>
-      <c r="D164" t="inlineStr">
+      <c r="D164" s="15" t="inlineStr">
         <is>
           <t>Carrot Rissoles</t>
         </is>
       </c>
-      <c r="E164" t="inlineStr">
+      <c r="E164" s="15" t="inlineStr">
         <is>
           <t>கேரட் ரிசோல்ஸ்</t>
         </is>
       </c>
-      <c r="F164" t="inlineStr">
+      <c r="F164" s="15" t="inlineStr">
         <is>
           <t>cutlet</t>
         </is>
       </c>
-      <c r="G164" t="inlineStr">
+      <c r="G164" s="15" t="inlineStr">
         <is>
           <t>Professional food photography of "Carrot Rissoles" (கேரட் ரிசோல்ஸ்), an Indian snack: golden-brown, breadcrumb-coated, deep-fried oval croquettes made from rice, grated carrot, and sauteed onion, with a crisp crumbed exterior, arranged on a plate with tomato sauce. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
         </is>
       </c>
-      <c r="H164" t="inlineStr">
+      <c r="H164" s="15" t="inlineStr">
         <is>
           <t>public/images/recipes/carrot-rissoles/featured.jpg</t>
         </is>
       </c>
-      <c r="I164" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
+      <c r="I164" s="15" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J164" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="K164" s="15" t="n"/>
     </row>
     <row r="165">
-      <c r="A165" t="n">
+      <c r="A165" s="15" t="n">
         <v>164</v>
       </c>
-      <c r="B165" t="inlineStr">
+      <c r="B165" s="15" t="inlineStr">
         <is>
           <t>Vegetarian</t>
         </is>
       </c>
-      <c r="C165" t="inlineStr">
+      <c r="C165" s="15" t="inlineStr">
         <is>
           <t>double-beans-rissoles</t>
         </is>
       </c>
-      <c r="D165" t="inlineStr">
+      <c r="D165" s="15" t="inlineStr">
         <is>
           <t>Double Bean Rissoles</t>
         </is>
       </c>
-      <c r="E165" t="inlineStr">
+      <c r="E165" s="15" t="inlineStr">
         <is>
           <t>டபுள் பீன்ஸ் ரிசோல்ஸ்</t>
         </is>
       </c>
-      <c r="F165" t="inlineStr">
+      <c r="F165" s="15" t="inlineStr">
         <is>
           <t>cutlet</t>
         </is>
       </c>
-      <c r="G165" t="inlineStr">
+      <c r="G165" s="15" t="inlineStr">
         <is>
           <t>Professional food photography of "Double Bean Rissoles" (டபுள் பீன்ஸ் ரிசோல்ஸ்), an Indian snack: small round, deep-fried fritters with a rough, textured golden-brown crust, made from a coarsely ground broad-white-bean batter with onion and green chili, similar in look to a vada, piled on a plate. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
         </is>
       </c>
-      <c r="H165" t="inlineStr">
+      <c r="H165" s="15" t="inlineStr">
         <is>
           <t>public/images/recipes/double-beans-rissoles/featured.jpg</t>
         </is>
       </c>
-      <c r="I165" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
+      <c r="I165" s="15" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J165" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="K165" s="15" t="n"/>
     </row>
     <row r="166">
-      <c r="A166" t="n">
+      <c r="A166" s="15" t="n">
         <v>165</v>
       </c>
-      <c r="B166" t="inlineStr">
+      <c r="B166" s="15" t="inlineStr">
         <is>
           <t>Vegetarian</t>
         </is>
       </c>
-      <c r="C166" t="inlineStr">
+      <c r="C166" s="15" t="inlineStr">
         <is>
           <t>cabbage-steaks</t>
         </is>
       </c>
-      <c r="D166" t="inlineStr">
+      <c r="D166" s="15" t="inlineStr">
         <is>
           <t>Cabbage Steaks</t>
         </is>
       </c>
-      <c r="E166" t="inlineStr">
+      <c r="E166" s="15" t="inlineStr">
         <is>
           <t>முட்டைகோஸ் ஸ்டீக்ஸ்</t>
         </is>
       </c>
-      <c r="F166" t="inlineStr">
+      <c r="F166" s="15" t="inlineStr">
         <is>
           <t>fried-snack</t>
         </is>
       </c>
-      <c r="G166" t="inlineStr">
+      <c r="G166" s="15" t="inlineStr">
         <is>
           <t>Professional food photography of "Cabbage Steaks" (முட்டைகோஸ் ஸ்டீக்ஸ்), an Indian snack: round, flat, pan-fried patties with a golden-brown seared surface, made from a spiced chana-dal-and-grated-cabbage batter that was steamed into a log then sliced into rounds and shallow-fried, arranged on a plate. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
         </is>
       </c>
-      <c r="H166" t="inlineStr">
+      <c r="H166" s="15" t="inlineStr">
         <is>
           <t>public/images/recipes/cabbage-steaks/featured.jpg</t>
         </is>
       </c>
-      <c r="I166" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
+      <c r="I166" s="15" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J166" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="K166" s="15" t="n"/>
     </row>
     <row r="167">
-      <c r="A167" t="n">
+      <c r="A167" s="15" t="n">
         <v>166</v>
       </c>
-      <c r="B167" t="inlineStr">
+      <c r="B167" s="15" t="inlineStr">
         <is>
           <t>Vegetarian</t>
         </is>
       </c>
-      <c r="C167" t="inlineStr">
+      <c r="C167" s="15" t="inlineStr">
         <is>
           <t>pesalu-kadiyalu</t>
         </is>
       </c>
-      <c r="D167" t="inlineStr">
+      <c r="D167" s="15" t="inlineStr">
         <is>
           <t>Pesalu Kadiyalu</t>
         </is>
       </c>
-      <c r="E167" t="inlineStr">
+      <c r="E167" s="15" t="inlineStr">
         <is>
           <t>பெசலு கடியாலு</t>
         </is>
       </c>
-      <c r="F167" t="inlineStr">
+      <c r="F167" s="15" t="inlineStr">
         <is>
           <t>fried-snack</t>
         </is>
       </c>
-      <c r="G167" t="inlineStr">
+      <c r="G167" s="15" t="inlineStr">
         <is>
           <t>Professional food photography of "Pesalu Kadiyalu" (பெசலு கடியாலு), an Andhra-style South Indian snack: golden-brown deep-fried ring-shaped fritters (like a savory donut), made from a ground moong-and-urad-dal-and-banana batter, with a crisp, slightly bumpy fried surface, served on a plate with white coconut chutney. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
         </is>
       </c>
-      <c r="H167" t="inlineStr">
+      <c r="H167" s="15" t="inlineStr">
         <is>
           <t>public/images/recipes/pesalu-kadiyalu/featured.jpg</t>
         </is>
       </c>
-      <c r="I167" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
+      <c r="I167" s="15" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J167" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="K167" s="15" t="n"/>
     </row>
     <row r="168">
-      <c r="A168" t="n">
+      <c r="A168" s="15" t="n">
         <v>167</v>
       </c>
-      <c r="B168" t="inlineStr">
+      <c r="B168" s="15" t="inlineStr">
         <is>
           <t>Vegetarian</t>
         </is>
       </c>
-      <c r="C168" t="inlineStr">
+      <c r="C168" s="15" t="inlineStr">
         <is>
           <t>rice-flour-rings</t>
         </is>
       </c>
-      <c r="D168" t="inlineStr">
+      <c r="D168" s="15" t="inlineStr">
         <is>
           <t>Rice Flour Rings</t>
         </is>
       </c>
-      <c r="E168" t="inlineStr">
+      <c r="E168" s="15" t="inlineStr">
         <is>
           <t>அரிசிமாவு கோடிபேடலு</t>
         </is>
       </c>
-      <c r="F168" t="inlineStr">
+      <c r="F168" s="15" t="inlineStr">
         <is>
           <t>fried-snack</t>
         </is>
       </c>
-      <c r="G168" t="inlineStr">
+      <c r="G168" s="15" t="inlineStr">
         <is>
           <t>Professional food photography of "Rice Flour Rings" (அரிசிமாவு கோடிபேடலு), a South Indian tea-time snack: small golden-brown deep-fried rings shaped like a chain link, made from a cooked rice-flour dough seasoned with pepper and cumin, with a smooth glossy fried crust, piled on a plate with coconut chutney. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
         </is>
       </c>
-      <c r="H168" t="inlineStr">
+      <c r="H168" s="15" t="inlineStr">
         <is>
           <t>public/images/recipes/rice-flour-rings/featured.jpg</t>
         </is>
       </c>
-      <c r="I168" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
+      <c r="I168" s="15" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J168" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="K168" s="15" t="n"/>
     </row>
     <row r="169">
-      <c r="A169" t="n">
+      <c r="A169" s="15" t="n">
         <v>168</v>
       </c>
-      <c r="B169" t="inlineStr">
+      <c r="B169" s="15" t="inlineStr">
         <is>
           <t>Vegetarian</t>
         </is>
       </c>
-      <c r="C169" t="inlineStr">
+      <c r="C169" s="15" t="inlineStr">
         <is>
           <t>chinese-vegetable-fritters</t>
         </is>
       </c>
-      <c r="D169" t="inlineStr">
+      <c r="D169" s="15" t="inlineStr">
         <is>
           <t>Chinese Vegetable Fritters</t>
         </is>
       </c>
-      <c r="E169" t="inlineStr">
+      <c r="E169" s="15" t="inlineStr">
         <is>
           <t>சீன காய்கறி பகோடா</t>
         </is>
       </c>
-      <c r="F169" t="inlineStr">
+      <c r="F169" s="15" t="inlineStr">
         <is>
           <t>fusion</t>
         </is>
       </c>
-      <c r="G169" t="inlineStr">
+      <c r="G169" s="15" t="inlineStr">
         <is>
           <t>Professional food photography of "Chinese Vegetable Fritters" (சீன காய்கறி பகோடா), an Indo-Chinese street-food snack: irregularly shaped, deep-fried golden-brown fritters made from julienned cabbage, carrot, and capsicum bound in a light batter seasoned with soy sauce and chili sauce, crisp and craggy-textured, piled on a plate. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
         </is>
       </c>
-      <c r="H169" t="inlineStr">
+      <c r="H169" s="15" t="inlineStr">
         <is>
           <t>public/images/recipes/chinese-vegetable-fritters/featured.jpg</t>
         </is>
       </c>
-      <c r="I169" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
+      <c r="I169" s="15" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J169" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="K169" s="15" t="n"/>
     </row>
     <row r="170">
-      <c r="A170" t="n">
+      <c r="A170" s="15" t="n">
         <v>169</v>
       </c>
-      <c r="B170" t="inlineStr">
+      <c r="B170" s="15" t="inlineStr">
         <is>
           <t>Vegetarian</t>
         </is>
       </c>
-      <c r="C170" t="inlineStr">
+      <c r="C170" s="15" t="inlineStr">
         <is>
           <t>cauliflower-fritters</t>
         </is>
       </c>
-      <c r="D170" t="inlineStr">
+      <c r="D170" s="15" t="inlineStr">
         <is>
           <t>Cauliflower Fritters</t>
         </is>
       </c>
-      <c r="E170" t="inlineStr">
+      <c r="E170" s="15" t="inlineStr">
         <is>
           <t>காலிப்ளவர் ஃபிரிட்டர்ஸ்</t>
         </is>
       </c>
-      <c r="F170" t="inlineStr">
+      <c r="F170" s="15" t="inlineStr">
         <is>
           <t>fried-snack</t>
         </is>
       </c>
-      <c r="G170" t="inlineStr">
+      <c r="G170" s="15" t="inlineStr">
         <is>
           <t>Professional food photography of "Cauliflower Fritters" (காலிப்ளவர் ஃபிரிட்டர்ஸ்), an Indian snack: golden-brown, crisp, batter-coated and breadcrumbed deep-fried cauliflower florets, piled on a plate with tomato sauce for dipping. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
         </is>
       </c>
-      <c r="H170" t="inlineStr">
+      <c r="H170" s="15" t="inlineStr">
         <is>
           <t>public/images/recipes/cauliflower-fritters/featured.jpg</t>
         </is>
       </c>
-      <c r="I170" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
+      <c r="I170" s="15" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J170" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="K170" s="15" t="n"/>
     </row>
     <row r="171">
-      <c r="A171" t="n">
+      <c r="A171" s="15" t="n">
         <v>170</v>
       </c>
-      <c r="B171" t="inlineStr">
+      <c r="B171" s="15" t="inlineStr">
         <is>
           <t>Vegetarian</t>
         </is>
       </c>
-      <c r="C171" t="inlineStr">
+      <c r="C171" s="15" t="inlineStr">
         <is>
           <t>chinese-cauliflower-manchurian</t>
         </is>
       </c>
-      <c r="D171" t="inlineStr">
+      <c r="D171" s="15" t="inlineStr">
         <is>
           <t>Chinese Cauliflower Manchurian</t>
         </is>
       </c>
-      <c r="E171" t="inlineStr">
+      <c r="E171" s="15" t="inlineStr">
         <is>
           <t>சீன காலிப்ளவர் மஞ்சூரியன்</t>
         </is>
       </c>
-      <c r="F171" t="inlineStr">
+      <c r="F171" s="15" t="inlineStr">
         <is>
           <t>fusion</t>
         </is>
       </c>
-      <c r="G171" t="inlineStr">
+      <c r="G171" s="15" t="inlineStr">
         <is>
           <t>Professional food photography of "Chinese Cauliflower Manchurian" (சீன காலிப்ளவர் மஞ்சூரியன்), a popular Indo-Chinese dish: deep-fried cauliflower florets coated in a glossy, thick, dark reddish-brown Manchurian sauce (soy, chili, ginger-garlic), served dry-style on a plate, garnished with chopped spring onion greens. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
         </is>
       </c>
-      <c r="H171" t="inlineStr">
+      <c r="H171" s="15" t="inlineStr">
         <is>
           <t>public/images/recipes/chinese-cauliflower-manchurian/featured.jpg</t>
         </is>
       </c>
-      <c r="I171" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
+      <c r="I171" s="15" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J171" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="K171" s="15" t="n"/>
     </row>
     <row r="172">
-      <c r="A172" t="n">
+      <c r="A172" s="15" t="n">
         <v>171</v>
       </c>
-      <c r="B172" t="inlineStr">
+      <c r="B172" s="15" t="inlineStr">
         <is>
           <t>Vegetarian</t>
         </is>
       </c>
-      <c r="C172" t="inlineStr">
+      <c r="C172" s="15" t="inlineStr">
         <is>
           <t>potato-fritters</t>
         </is>
       </c>
-      <c r="D172" t="inlineStr">
+      <c r="D172" s="15" t="inlineStr">
         <is>
           <t>Potato Fritters</t>
         </is>
       </c>
-      <c r="E172" t="inlineStr">
+      <c r="E172" s="15" t="inlineStr">
         <is>
           <t>உருளை வறுவல்</t>
         </is>
       </c>
-      <c r="F172" t="inlineStr">
+      <c r="F172" s="15" t="inlineStr">
         <is>
           <t>fried-snack</t>
         </is>
       </c>
-      <c r="G172" t="inlineStr">
+      <c r="G172" s="15" t="inlineStr">
         <is>
           <t>Professional food photography of "Potato Fritters" (உருளை வறுவல்), an Indian snack: thin round potato slices coated in a spiced reddish-orange ground masala paste (fennel, garlic, ginger, dried chili, roasted gram) and shallow-fried until golden and slightly crisp on both sides, arranged overlapping on a plate. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
         </is>
       </c>
-      <c r="H172" t="inlineStr">
+      <c r="H172" s="15" t="inlineStr">
         <is>
           <t>public/images/recipes/potato-fritters/featured.jpg</t>
         </is>
       </c>
-      <c r="I172" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
+      <c r="I172" s="15" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J172" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="K172" s="15" t="n"/>
     </row>
     <row r="173">
-      <c r="A173" t="n">
+      <c r="A173" s="15" t="n">
         <v>172</v>
       </c>
-      <c r="B173" t="inlineStr">
+      <c r="B173" s="15" t="inlineStr">
         <is>
           <t>Vegetarian</t>
         </is>
       </c>
-      <c r="C173" t="inlineStr">
+      <c r="C173" s="15" t="inlineStr">
         <is>
           <t>banana-fritters</t>
         </is>
       </c>
-      <c r="D173" t="inlineStr">
+      <c r="D173" s="15" t="inlineStr">
         <is>
           <t>Banana Fritters</t>
         </is>
       </c>
-      <c r="E173" t="inlineStr">
+      <c r="E173" s="15" t="inlineStr">
         <is>
           <t>வாழைக்காய் வறுவல்</t>
         </is>
       </c>
-      <c r="F173" t="inlineStr">
+      <c r="F173" s="15" t="inlineStr">
         <is>
           <t>fried-snack</t>
         </is>
       </c>
-      <c r="G173" t="inlineStr">
+      <c r="G173" s="15" t="inlineStr">
         <is>
           <t>Professional food photography of "Banana Fritters" (வாழைக்காய் வறுவல்), an Indian snack: thin round raw-banana slices coated in a spiced reddish-brown ground masala paste (chana dal, dried chili, coriander seeds, shallots) and deep-fried until golden and crisp, arranged overlapping on a plate. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
         </is>
       </c>
-      <c r="H173" t="inlineStr">
+      <c r="H173" s="15" t="inlineStr">
         <is>
           <t>public/images/recipes/banana-fritters/featured.jpg</t>
         </is>
       </c>
-      <c r="I173" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
+      <c r="I173" s="15" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J173" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="K173" s="15" t="n"/>
     </row>
     <row r="174">
-      <c r="A174" t="n">
+      <c r="A174" s="15" t="n">
         <v>173</v>
       </c>
-      <c r="B174" t="inlineStr">
+      <c r="B174" s="15" t="inlineStr">
         <is>
           <t>Vegetarian</t>
         </is>
       </c>
-      <c r="C174" t="inlineStr">
+      <c r="C174" s="15" t="inlineStr">
         <is>
           <t>bread-fritters</t>
         </is>
       </c>
-      <c r="D174" t="inlineStr">
+      <c r="D174" s="15" t="inlineStr">
         <is>
           <t>Bread Fritters</t>
         </is>
       </c>
-      <c r="E174" t="inlineStr">
+      <c r="E174" s="15" t="inlineStr">
         <is>
           <t>பிரட் தங்க வறுவல்</t>
         </is>
       </c>
-      <c r="F174" t="inlineStr">
+      <c r="F174" s="15" t="inlineStr">
         <is>
           <t>fried-snack</t>
         </is>
       </c>
-      <c r="G174" t="inlineStr">
+      <c r="G174" s="15" t="inlineStr">
         <is>
           <t>Professional food photography of "Bread Fritters" (பிரட் தங்க வறுவல்), an Indian snack: small bread squares dipped in a spiced gram-flour-and-rice-flour batter and shallow-fried on a griddle until golden-brown and crisp, piled on a plate with tomato sauce. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
         </is>
       </c>
-      <c r="H174" t="inlineStr">
+      <c r="H174" s="15" t="inlineStr">
         <is>
           <t>public/images/recipes/bread-fritters/featured.jpg</t>
         </is>
       </c>
-      <c r="I174" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
+      <c r="I174" s="15" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J174" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="K174" s="15" t="n"/>
     </row>
     <row r="175">
-      <c r="A175" t="n">
+      <c r="A175" s="15" t="n">
         <v>174</v>
       </c>
-      <c r="B175" t="inlineStr">
+      <c r="B175" s="15" t="inlineStr">
         <is>
           <t>Vegetarian</t>
         </is>
       </c>
-      <c r="C175" t="inlineStr">
+      <c r="C175" s="15" t="inlineStr">
         <is>
           <t>potato-cheese-croquettes</t>
         </is>
       </c>
-      <c r="D175" t="inlineStr">
+      <c r="D175" s="15" t="inlineStr">
         <is>
           <t>Potato Cheese Croquettes</t>
         </is>
       </c>
-      <c r="E175" t="inlineStr">
+      <c r="E175" s="15" t="inlineStr">
         <is>
           <t>உருளைக்கிழங்கு சீஸ் கட்லெட்</t>
         </is>
       </c>
-      <c r="F175" t="inlineStr">
+      <c r="F175" s="15" t="inlineStr">
         <is>
           <t>cutlet</t>
         </is>
       </c>
-      <c r="G175" t="inlineStr">
+      <c r="G175" s="15" t="inlineStr">
         <is>
           <t>Professional food photography of "Potato Cheese Croquettes" (உருளைக்கிழங்கு சீஸ் கட்லெட்), an Indian snack: round, flattened, golden-brown deep-fried patties made from mashed potato and melted cheese with a crisp crumbed crust, one croquette broken in half showing a soft, slightly stringy cheese-flecked interior, served with tomato sauce. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
         </is>
       </c>
-      <c r="H175" t="inlineStr">
+      <c r="H175" s="15" t="inlineStr">
         <is>
           <t>public/images/recipes/potato-cheese-croquettes/featured.jpg</t>
         </is>
       </c>
-      <c r="I175" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
+      <c r="I175" s="15" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J175" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="K175" s="15" t="n"/>
     </row>
     <row r="176">
-      <c r="A176" t="n">
+      <c r="A176" s="15" t="n">
         <v>175</v>
       </c>
-      <c r="B176" t="inlineStr">
+      <c r="B176" s="15" t="inlineStr">
         <is>
           <t>Vegetarian</t>
         </is>
       </c>
-      <c r="C176" t="inlineStr">
+      <c r="C176" s="15" t="inlineStr">
         <is>
           <t>potato-baskets</t>
         </is>
       </c>
-      <c r="D176" t="inlineStr">
+      <c r="D176" s="15" t="inlineStr">
         <is>
           <t>Potato Baskets</t>
         </is>
       </c>
-      <c r="E176" t="inlineStr">
+      <c r="E176" s="15" t="inlineStr">
         <is>
           <t>உருளைக்கிழங்கு கூடைகள்</t>
         </is>
       </c>
-      <c r="F176" t="inlineStr">
+      <c r="F176" s="15" t="inlineStr">
         <is>
           <t>fried-snack</t>
         </is>
       </c>
-      <c r="G176" t="inlineStr">
+      <c r="G176" s="15" t="inlineStr">
         <is>
           <t>Professional food photography of "Potato Baskets" (உருளைக்கிழங்கு கூடைகள்), an Indian party snack: small golden-brown deep-fried baskets woven from fine shredded potato strands into a crisp, lacy, bird's-nest-like bowl shape, filled with a colorful chopped vegetable salad, arranged on a plate. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
         </is>
       </c>
-      <c r="H176" t="inlineStr">
+      <c r="H176" s="15" t="inlineStr">
         <is>
           <t>public/images/recipes/potato-baskets/featured.jpg</t>
         </is>
       </c>
-      <c r="I176" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
+      <c r="I176" s="15" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J176" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="K176" s="15" t="n"/>
     </row>
     <row r="177">
-      <c r="A177" t="n">
+      <c r="A177" s="15" t="n">
         <v>176</v>
       </c>
-      <c r="B177" t="inlineStr">
+      <c r="B177" s="15" t="inlineStr">
         <is>
           <t>Vegetarian</t>
         </is>
       </c>
-      <c r="C177" t="inlineStr">
+      <c r="C177" s="15" t="inlineStr">
         <is>
           <t>vegetable-puffs</t>
         </is>
       </c>
-      <c r="D177" t="inlineStr">
+      <c r="D177" s="15" t="inlineStr">
         <is>
           <t>Vegetable Puffs</t>
         </is>
       </c>
-      <c r="E177" t="inlineStr">
+      <c r="E177" s="15" t="inlineStr">
         <is>
           <t>வெஜிடபிள் பஃப்</t>
         </is>
       </c>
-      <c r="F177" t="inlineStr">
+      <c r="F177" s="15" t="inlineStr">
         <is>
           <t>snack</t>
         </is>
       </c>
-      <c r="G177" t="inlineStr">
+      <c r="G177" s="15" t="inlineStr">
         <is>
           <t>Professional food photography of "Vegetable Puffs" (வெஜிடபிள் பஃப்), a bakery-style Indian snack: golden-brown baked triangular puff pastries with a flaky, many-layered crust, one puff broken open to reveal a spiced potato-and-mixed-vegetable filling, arranged on a plate with tomato sauce. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
         </is>
       </c>
-      <c r="H177" t="inlineStr">
+      <c r="H177" s="15" t="inlineStr">
         <is>
           <t>public/images/recipes/vegetable-puffs/featured.jpg</t>
         </is>
       </c>
-      <c r="I177" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
+      <c r="I177" s="15" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J177" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="K177" s="15" t="n"/>
     </row>
     <row r="178">
-      <c r="A178" t="n">
+      <c r="A178" s="15" t="n">
         <v>177</v>
       </c>
-      <c r="B178" t="inlineStr">
+      <c r="B178" s="15" t="inlineStr">
         <is>
           <t>Vegetarian</t>
         </is>
       </c>
-      <c r="C178" t="inlineStr">
+      <c r="C178" s="15" t="inlineStr">
         <is>
           <t>vegetable-cones</t>
         </is>
       </c>
-      <c r="D178" t="inlineStr">
+      <c r="D178" s="15" t="inlineStr">
         <is>
           <t>Vegetable Cones</t>
         </is>
       </c>
-      <c r="E178" t="inlineStr">
+      <c r="E178" s="15" t="inlineStr">
         <is>
           <t>வெஜிடபிள் கோன்ஸ்</t>
         </is>
       </c>
-      <c r="F178" t="inlineStr">
+      <c r="F178" s="15" t="inlineStr">
         <is>
           <t>snack</t>
         </is>
       </c>
-      <c r="G178" t="inlineStr">
+      <c r="G178" s="15" t="inlineStr">
         <is>
           <t>Professional food photography of "Vegetable Cones" (வெஜிடபிள் கோன்ஸ்), a bakery-style Indian snack: golden-brown baked cone-shaped flaky puff-pastry shells (shaped like small ice-cream cones), filled generously with a spiced potato-and-mixed-vegetable filling, standing upright on a plate. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
         </is>
       </c>
-      <c r="H178" t="inlineStr">
+      <c r="H178" s="15" t="inlineStr">
         <is>
           <t>public/images/recipes/vegetable-cones/featured.jpg</t>
         </is>
       </c>
-      <c r="I178" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
+      <c r="I178" s="15" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J178" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="K178" s="15" t="n"/>
     </row>
     <row r="179">
-      <c r="A179" t="n">
+      <c r="A179" s="15" t="n">
         <v>178</v>
       </c>
-      <c r="B179" t="inlineStr">
+      <c r="B179" s="15" t="inlineStr">
         <is>
           <t>Vegetarian</t>
         </is>
       </c>
-      <c r="C179" t="inlineStr">
+      <c r="C179" s="15" t="inlineStr">
         <is>
           <t>vol-au-vent-cases</t>
         </is>
       </c>
-      <c r="D179" t="inlineStr">
+      <c r="D179" s="15" t="inlineStr">
         <is>
           <t>Vol-au-vent Cases</t>
         </is>
       </c>
-      <c r="E179" t="inlineStr">
+      <c r="E179" s="15" t="inlineStr">
         <is>
           <t>பஃப் டப்பிகள்</t>
         </is>
       </c>
-      <c r="F179" t="inlineStr">
+      <c r="F179" s="15" t="inlineStr">
         <is>
           <t>snack</t>
         </is>
       </c>
-      <c r="G179" t="inlineStr">
+      <c r="G179" s="15" t="inlineStr">
         <is>
           <t>Professional food photography of "Vol-au-vent Cases" (பஃப் டப்பிகள்), a bakery-style Indian snack: small round, golden-brown baked puff-pastry boxes with tall flaky layered walls, filled with a spiced potato-and-vegetable filling, with a puff-pastry lid resting beside the filled case, arranged on a plate. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
         </is>
       </c>
-      <c r="H179" t="inlineStr">
+      <c r="H179" s="15" t="inlineStr">
         <is>
           <t>public/images/recipes/vol-au-vent-cases/featured.jpg</t>
         </is>
       </c>
-      <c r="I179" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
+      <c r="I179" s="15" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J179" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="K179" s="15" t="n"/>
     </row>
     <row r="180">
-      <c r="A180" t="n">
+      <c r="A180" s="15" t="n">
         <v>179</v>
       </c>
-      <c r="B180" t="inlineStr">
+      <c r="B180" s="15" t="inlineStr">
         <is>
           <t>Vegetarian</t>
         </is>
       </c>
-      <c r="C180" t="inlineStr">
+      <c r="C180" s="15" t="inlineStr">
         <is>
           <t>baked-brinjals</t>
         </is>
       </c>
-      <c r="D180" t="inlineStr">
+      <c r="D180" s="15" t="inlineStr">
         <is>
           <t>Baked Brinjals</t>
         </is>
       </c>
-      <c r="E180" t="inlineStr">
+      <c r="E180" s="15" t="inlineStr">
         <is>
           <t>பேக்டு பிரின்ஜால்</t>
         </is>
       </c>
-      <c r="F180" t="inlineStr">
+      <c r="F180" s="15" t="inlineStr">
         <is>
           <t>snack</t>
         </is>
       </c>
-      <c r="G180" t="inlineStr">
+      <c r="G180" s="15" t="inlineStr">
         <is>
           <t>Professional food photography of "Baked Brinjals" (பேக்டு பிரின்ஜால்), an Indian baked dish: a round baking dish layered with crisp fried breaded brinjal rounds, tomato sauce, and melted golden-brown bubbling cheese on top, served warm straight from the oven. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
         </is>
       </c>
-      <c r="H180" t="inlineStr">
+      <c r="H180" s="15" t="inlineStr">
         <is>
           <t>public/images/recipes/baked-brinjals/featured.jpg</t>
         </is>
       </c>
-      <c r="I180" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
+      <c r="I180" s="15" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J180" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="K180" s="15" t="n"/>
     </row>
     <row r="181">
-      <c r="A181" t="n">
+      <c r="A181" s="15" t="n">
         <v>180</v>
       </c>
-      <c r="B181" t="inlineStr">
+      <c r="B181" s="15" t="inlineStr">
         <is>
           <t>Vegetarian</t>
         </is>
       </c>
-      <c r="C181" t="inlineStr">
+      <c r="C181" s="15" t="inlineStr">
         <is>
           <t>stuffed-capsicum</t>
         </is>
       </c>
-      <c r="D181" t="inlineStr">
+      <c r="D181" s="15" t="inlineStr">
         <is>
           <t>Stuffed Capsicum</t>
         </is>
       </c>
-      <c r="E181" t="inlineStr">
+      <c r="E181" s="15" t="inlineStr">
         <is>
           <t>ஸ்டப் செய்த குடமிளகாய்</t>
         </is>
       </c>
-      <c r="F181" t="inlineStr">
+      <c r="F181" s="15" t="inlineStr">
         <is>
           <t>snack</t>
         </is>
       </c>
-      <c r="G181" t="inlineStr">
+      <c r="G181" s="15" t="inlineStr">
         <is>
           <t>Professional food photography of "Stuffed Capsicum" (ஸ்டப் செய்த குடமிளகாய்), an Indian dish: capsicum halves filled with a spiced mixed-vegetable filling, pan-cooked with a thin golden gram-flour crust on the cut surface, arranged filling-side up on a plate. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
         </is>
       </c>
-      <c r="H181" t="inlineStr">
+      <c r="H181" s="15" t="inlineStr">
         <is>
           <t>public/images/recipes/stuffed-capsicum/featured.jpg</t>
         </is>
       </c>
-      <c r="I181" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
+      <c r="I181" s="15" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J181" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="K181" s="15" t="n"/>
     </row>
     <row r="182">
-      <c r="A182" t="n">
+      <c r="A182" s="15" t="n">
         <v>181</v>
       </c>
-      <c r="B182" t="inlineStr">
+      <c r="B182" s="15" t="inlineStr">
         <is>
           <t>Vegetarian</t>
         </is>
       </c>
-      <c r="C182" t="inlineStr">
+      <c r="C182" s="15" t="inlineStr">
         <is>
           <t>stuffed-tomatoes</t>
         </is>
       </c>
-      <c r="D182" t="inlineStr">
+      <c r="D182" s="15" t="inlineStr">
         <is>
           <t>Stuffed Tomatoes</t>
         </is>
       </c>
-      <c r="E182" t="inlineStr">
+      <c r="E182" s="15" t="inlineStr">
         <is>
           <t>ஸ்டப் செய்த தக்காளி</t>
         </is>
       </c>
-      <c r="F182" t="inlineStr">
+      <c r="F182" s="15" t="inlineStr">
         <is>
           <t>snack</t>
         </is>
       </c>
-      <c r="G182" t="inlineStr">
+      <c r="G182" s="15" t="inlineStr">
         <is>
           <t>Professional food photography of "Stuffed Tomatoes" (ஸ்டப் செய்த தக்காளி), an Indian baked dish: whole ripe tomatoes with their tops sliced off, hollowed and filled with a spiced mixed-vegetable filling, topped with melted golden-brown cheese, baked and arranged on a plate. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
         </is>
       </c>
-      <c r="H182" t="inlineStr">
+      <c r="H182" s="15" t="inlineStr">
         <is>
           <t>public/images/recipes/stuffed-tomatoes/featured.jpg</t>
         </is>
       </c>
-      <c r="I182" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
+      <c r="I182" s="15" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J182" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="K182" s="15" t="n"/>
     </row>
     <row r="183">
-      <c r="A183" t="n">
+      <c r="A183" s="15" t="n">
         <v>182</v>
       </c>
-      <c r="B183" t="inlineStr">
+      <c r="B183" s="15" t="inlineStr">
         <is>
           <t>Vegetarian</t>
         </is>
       </c>
-      <c r="C183" t="inlineStr">
+      <c r="C183" s="15" t="inlineStr">
         <is>
           <t>pizza</t>
         </is>
       </c>
-      <c r="D183" t="inlineStr">
+      <c r="D183" s="15" t="inlineStr">
         <is>
           <t>Pizza</t>
         </is>
       </c>
-      <c r="E183" t="inlineStr">
+      <c r="E183" s="15" t="inlineStr">
         <is>
           <t>பிஸ்ஸா</t>
         </is>
       </c>
-      <c r="F183" t="inlineStr">
+      <c r="F183" s="15" t="inlineStr">
         <is>
           <t>fusion</t>
         </is>
       </c>
-      <c r="G183" t="inlineStr">
+      <c r="G183" s="15" t="inlineStr">
         <is>
           <t>Professional food photography of a homemade "Pizza" (பிஸ்ஸா): a round, golden-baked bread crust topped with tomato sauce, sliced rounds of onion, tomato, and capsicum, and a generous layer of melted, lightly browned bubbly cheese, served whole on a wooden board. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
         </is>
       </c>
-      <c r="H183" t="inlineStr">
+      <c r="H183" s="15" t="inlineStr">
         <is>
           <t>public/images/recipes/pizza/featured.jpg</t>
         </is>
       </c>
-      <c r="I183" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
+      <c r="I183" s="15" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J183" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="K183" s="15" t="n"/>
     </row>
     <row r="184">
-      <c r="A184" t="n">
+      <c r="A184" s="15" t="n">
         <v>183</v>
       </c>
-      <c r="B184" t="inlineStr">
+      <c r="B184" s="15" t="inlineStr">
         <is>
           <t>Vegetarian</t>
         </is>
       </c>
-      <c r="C184" t="inlineStr">
+      <c r="C184" s="15" t="inlineStr">
         <is>
           <t>moong-dal-banzi</t>
         </is>
       </c>
-      <c r="D184" t="inlineStr">
+      <c r="D184" s="15" t="inlineStr">
         <is>
           <t>Moong Dal Banzi</t>
         </is>
       </c>
-      <c r="E184" t="inlineStr">
+      <c r="E184" s="15" t="inlineStr">
         <is>
           <t>பாசிப்பயறு பன்ஸி</t>
         </is>
       </c>
-      <c r="F184" t="inlineStr">
+      <c r="F184" s="15" t="inlineStr">
         <is>
           <t>snack</t>
         </is>
       </c>
-      <c r="G184" t="inlineStr">
+      <c r="G184" s="15" t="inlineStr">
         <is>
           <t>Professional food photography of "Moong Dal Banzi" (பாசிப்பயறு பன்ஸி), an Indian snack: a thick, round, griddle-cooked stuffed flatbread with a lightly charred, leaf-textured surface (cooked between banana leaves), cut into wedges revealing a spiced moong-dal-and-vegetable filling inside, served with chutney. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
         </is>
       </c>
-      <c r="H184" t="inlineStr">
+      <c r="H184" s="15" t="inlineStr">
         <is>
           <t>public/images/recipes/moong-dal-banzi/featured.jpg</t>
         </is>
       </c>
-      <c r="I184" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
+      <c r="I184" s="15" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J184" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="K184" s="15" t="n"/>
     </row>
     <row r="185">
-      <c r="A185" t="n">
+      <c r="A185" s="15" t="n">
         <v>184</v>
       </c>
-      <c r="B185" t="inlineStr">
+      <c r="B185" s="15" t="inlineStr">
         <is>
           <t>Vegetarian</t>
         </is>
       </c>
-      <c r="C185" t="inlineStr">
+      <c r="C185" s="15" t="inlineStr">
         <is>
           <t>handvo</t>
         </is>
       </c>
-      <c r="D185" t="inlineStr">
+      <c r="D185" s="15" t="inlineStr">
         <is>
           <t>Handvo</t>
         </is>
       </c>
-      <c r="E185" t="inlineStr">
+      <c r="E185" s="15" t="inlineStr">
         <is>
           <t>ஹண்ட்வோ</t>
         </is>
       </c>
-      <c r="F185" t="inlineStr">
+      <c r="F185" s="15" t="inlineStr">
         <is>
           <t>fusion</t>
         </is>
       </c>
-      <c r="G185" t="inlineStr">
+      <c r="G185" s="15" t="inlineStr">
         <is>
           <t>Professional food photography of "Handvo" (ஹண்ட்வோ), a Gujarati savory cake: a thick, golden-brown pan-fried lentil-and-rice cake with a crisp, seed-flecked crust (mustard seeds and sesame visible on top), sliced into squares, arranged on a plate. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
         </is>
       </c>
-      <c r="H185" t="inlineStr">
+      <c r="H185" s="15" t="inlineStr">
         <is>
           <t>public/images/recipes/handvo/featured.jpg</t>
         </is>
       </c>
-      <c r="I185" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
+      <c r="I185" s="15" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J185" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="K185" s="15" t="n"/>
     </row>
     <row r="186">
-      <c r="A186" t="n">
+      <c r="A186" s="15" t="n">
         <v>185</v>
       </c>
-      <c r="B186" t="inlineStr">
+      <c r="B186" s="15" t="inlineStr">
         <is>
           <t>Vegetarian</t>
         </is>
       </c>
-      <c r="C186" t="inlineStr">
+      <c r="C186" s="15" t="inlineStr">
         <is>
           <t>khandvi</t>
         </is>
       </c>
-      <c r="D186" t="inlineStr">
+      <c r="D186" s="15" t="inlineStr">
         <is>
           <t>Khandvi</t>
         </is>
       </c>
-      <c r="E186" t="inlineStr">
+      <c r="E186" s="15" t="inlineStr">
         <is>
           <t>கண்ட்வி</t>
         </is>
       </c>
-      <c r="F186" t="inlineStr">
+      <c r="F186" s="15" t="inlineStr">
         <is>
           <t>fusion</t>
         </is>
       </c>
-      <c r="G186" t="inlineStr">
+      <c r="G186" s="15" t="inlineStr">
         <is>
           <t>Professional food photography of "Khandvi" (கண்ட்வி), a Gujarati snack: small, tightly rolled, pale-yellow gram-flour spirals (bite-sized pinwheels) arranged on a plate, topped with a mustard-seed tempering, grated coconut, and chopped coriander leaves. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
         </is>
       </c>
-      <c r="H186" t="inlineStr">
+      <c r="H186" s="15" t="inlineStr">
         <is>
           <t>public/images/recipes/khandvi/featured.jpg</t>
         </is>
       </c>
-      <c r="I186" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
+      <c r="I186" s="15" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J186" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="K186" s="15" t="n"/>
     </row>
     <row r="187">
-      <c r="A187" t="n">
+      <c r="A187" s="15" t="n">
         <v>186</v>
       </c>
-      <c r="B187" t="inlineStr">
+      <c r="B187" s="15" t="inlineStr">
         <is>
           <t>Vegetarian</t>
         </is>
       </c>
-      <c r="C187" t="inlineStr">
+      <c r="C187" s="15" t="inlineStr">
         <is>
           <t>spring-rolls</t>
         </is>
       </c>
-      <c r="D187" t="inlineStr">
+      <c r="D187" s="15" t="inlineStr">
         <is>
           <t>Spring Rolls</t>
         </is>
       </c>
-      <c r="E187" t="inlineStr">
+      <c r="E187" s="15" t="inlineStr">
         <is>
           <t>ஸ்பிரிங் ரோல்</t>
         </is>
       </c>
-      <c r="F187" t="inlineStr">
+      <c r="F187" s="15" t="inlineStr">
         <is>
           <t>fusion</t>
         </is>
       </c>
-      <c r="G187" t="inlineStr">
+      <c r="G187" s="15" t="inlineStr">
         <is>
           <t>Professional food photography of "Spring Rolls" (ஸ்பிரிங் ரோல்), an Indo-Chinese snack: golden-brown deep-fried cylindrical rolls with a thin crisp pastry shell, sliced into rounds showing a colorful julienned cabbage-carrot-capsicum filling inside, arranged on a plate with tomato sauce. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
         </is>
       </c>
-      <c r="H187" t="inlineStr">
+      <c r="H187" s="15" t="inlineStr">
         <is>
           <t>public/images/recipes/spring-rolls/featured.jpg</t>
         </is>
       </c>
-      <c r="I187" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
+      <c r="I187" s="15" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J187" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="K187" s="15" t="n"/>
     </row>
     <row r="188">
-      <c r="A188" t="n">
+      <c r="A188" s="15" t="n">
         <v>187</v>
       </c>
-      <c r="B188" t="inlineStr">
+      <c r="B188" s="15" t="inlineStr">
         <is>
           <t>Vegetarian</t>
         </is>
       </c>
-      <c r="C188" t="inlineStr">
+      <c r="C188" s="15" t="inlineStr">
         <is>
           <t>wontons</t>
         </is>
       </c>
-      <c r="D188" t="inlineStr">
+      <c r="D188" s="15" t="inlineStr">
         <is>
           <t>Wontons</t>
         </is>
       </c>
-      <c r="E188" t="inlineStr">
+      <c r="E188" s="15" t="inlineStr">
         <is>
           <t>ஒன்டன்ஸ்</t>
         </is>
       </c>
-      <c r="F188" t="inlineStr">
+      <c r="F188" s="15" t="inlineStr">
         <is>
           <t>fusion</t>
         </is>
       </c>
-      <c r="G188" t="inlineStr">
+      <c r="G188" s="15" t="inlineStr">
         <is>
           <t>Professional food photography of "Wontons" (ஒன்டன்ஸ்), an Indo-Chinese snack: small golden-brown deep-fried dumplings with pleated, gathered pastry tops enclosing a vegetable filling, piled on a plate with tomato sauce. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
         </is>
       </c>
-      <c r="H188" t="inlineStr">
+      <c r="H188" s="15" t="inlineStr">
         <is>
           <t>public/images/recipes/wontons/featured.jpg</t>
         </is>
       </c>
-      <c r="I188" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
+      <c r="I188" s="15" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J188" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="K188" s="15" t="n"/>
     </row>
     <row r="189">
-      <c r="A189" t="n">
+      <c r="A189" s="15" t="n">
         <v>188</v>
       </c>
-      <c r="B189" t="inlineStr">
+      <c r="B189" s="15" t="inlineStr">
         <is>
           <t>Vegetarian</t>
         </is>
       </c>
-      <c r="C189" t="inlineStr">
+      <c r="C189" s="15" t="inlineStr">
         <is>
           <t>crispy-toasts</t>
         </is>
       </c>
-      <c r="D189" t="inlineStr">
+      <c r="D189" s="15" t="inlineStr">
         <is>
           <t>Crispy Toasts</t>
         </is>
       </c>
-      <c r="E189" t="inlineStr">
+      <c r="E189" s="15" t="inlineStr">
         <is>
           <t>சைனீஸ் பொரித்த டோஸ்ட்</t>
         </is>
       </c>
-      <c r="F189" t="inlineStr">
+      <c r="F189" s="15" t="inlineStr">
         <is>
           <t>fusion</t>
         </is>
       </c>
-      <c r="G189" t="inlineStr">
+      <c r="G189" s="15" t="inlineStr">
         <is>
           <t>Professional food photography of "Crispy Toasts" (சைனீஸ் பொரித்த டோஸ்ட்), an Indo-Chinese snack: golden-brown fried bread squares with a spiced mashed-potato-and-vegetable layer pressed onto one side, crisp at the edges, piled on a plate with tomato sauce. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
         </is>
       </c>
-      <c r="H189" t="inlineStr">
+      <c r="H189" s="15" t="inlineStr">
         <is>
           <t>public/images/recipes/crispy-toasts/featured.jpg</t>
         </is>
       </c>
-      <c r="I189" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
+      <c r="I189" s="15" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J189" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="K189" s="15" t="n"/>
     </row>
     <row r="190">
-      <c r="A190" t="n">
+      <c r="A190" s="15" t="n">
         <v>189</v>
       </c>
-      <c r="B190" t="inlineStr">
+      <c r="B190" s="15" t="inlineStr">
         <is>
           <t>Vegetarian</t>
         </is>
       </c>
-      <c r="C190" t="inlineStr">
+      <c r="C190" s="15" t="inlineStr">
         <is>
           <t>vegetable-pan-cake</t>
         </is>
       </c>
-      <c r="D190" t="inlineStr">
+      <c r="D190" s="15" t="inlineStr">
         <is>
           <t>Vegetable Pan Cake</t>
         </is>
       </c>
-      <c r="E190" t="inlineStr">
+      <c r="E190" s="15" t="inlineStr">
         <is>
           <t>காய்கறி பான் கேக்</t>
         </is>
       </c>
-      <c r="F190" t="inlineStr">
+      <c r="F190" s="15" t="inlineStr">
         <is>
           <t>snack</t>
         </is>
       </c>
-      <c r="G190" t="inlineStr">
+      <c r="G190" s="15" t="inlineStr">
         <is>
           <t>Professional food photography of "Vegetable Pan Cake" (காய்கறி பான் கேக்), an Indian flatbread snack: a round, golden-brown, griddle-cooked spiral flatbread with a crisp seared surface, cut in half to reveal a tight coiled spiral of dough layered with raw chopped vegetables inside, served with tomato-based thokku. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
         </is>
       </c>
-      <c r="H190" t="inlineStr">
+      <c r="H190" s="15" t="inlineStr">
         <is>
           <t>public/images/recipes/vegetable-pan-cake/featured.jpg</t>
         </is>
       </c>
-      <c r="I190" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
+      <c r="I190" s="15" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J190" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="K190" s="15" t="n"/>
     </row>
     <row r="191">
-      <c r="A191" t="n">
+      <c r="A191" s="15" t="n">
         <v>190</v>
       </c>
-      <c r="B191" t="inlineStr">
+      <c r="B191" s="15" t="inlineStr">
         <is>
           <t>Vegetarian</t>
         </is>
       </c>
-      <c r="C191" t="inlineStr">
+      <c r="C191" s="15" t="inlineStr">
         <is>
           <t>mixed-vegetable-kabab</t>
         </is>
       </c>
-      <c r="D191" t="inlineStr">
+      <c r="D191" s="15" t="inlineStr">
         <is>
           <t>Mixed Vegetable Kabab</t>
         </is>
       </c>
-      <c r="E191" t="inlineStr">
+      <c r="E191" s="15" t="inlineStr">
         <is>
           <t>காய்கறி கபாப்</t>
         </is>
       </c>
-      <c r="F191" t="inlineStr">
+      <c r="F191" s="15" t="inlineStr">
         <is>
           <t>kabab</t>
         </is>
       </c>
-      <c r="G191" t="inlineStr">
+      <c r="G191" s="15" t="inlineStr">
         <is>
           <t>Professional food photography of "Mixed Vegetable Kabab" (காய்கறி கபாப்), an Indian snack: golden-brown deep-fried oblong kabab logs made from a mashed mixed-vegetable dough, arranged on a plate with mint chutney, sweet chutney, and a side of tangy marinated onion strips. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
         </is>
       </c>
-      <c r="H191" t="inlineStr">
+      <c r="H191" s="15" t="inlineStr">
         <is>
           <t>public/images/recipes/mixed-vegetable-kabab/featured.jpg</t>
         </is>
       </c>
-      <c r="I191" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
+      <c r="I191" s="15" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J191" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="K191" s="15" t="n"/>
     </row>
     <row r="192">
-      <c r="A192" t="n">
+      <c r="A192" s="15" t="n">
         <v>191</v>
       </c>
-      <c r="B192" t="inlineStr">
+      <c r="B192" s="15" t="inlineStr">
         <is>
           <t>Vegetarian</t>
         </is>
       </c>
-      <c r="C192" t="inlineStr">
+      <c r="C192" s="15" t="inlineStr">
         <is>
           <t>potato-kababs</t>
         </is>
       </c>
-      <c r="D192" t="inlineStr">
+      <c r="D192" s="15" t="inlineStr">
         <is>
           <t>Potato Kababs</t>
         </is>
       </c>
-      <c r="E192" t="inlineStr">
+      <c r="E192" s="15" t="inlineStr">
         <is>
           <t>உருளைக்கிழங்கு கபாப்</t>
         </is>
       </c>
-      <c r="F192" t="inlineStr">
+      <c r="F192" s="15" t="inlineStr">
         <is>
           <t>kabab</t>
         </is>
       </c>
-      <c r="G192" t="inlineStr">
+      <c r="G192" s="15" t="inlineStr">
         <is>
           <t>Professional food photography of "Potato Kababs" (உருளைக்கிழங்கு கபாப்), an Indian snack: golden-brown deep-fried oblong kabab logs made from spiced mashed potato studded with fresh herbs, arranged on a plate with mint chutney. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
         </is>
       </c>
-      <c r="H192" t="inlineStr">
+      <c r="H192" s="15" t="inlineStr">
         <is>
           <t>public/images/recipes/potato-kababs/featured.jpg</t>
         </is>
       </c>
-      <c r="I192" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
+      <c r="I192" s="15" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J192" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="K192" s="15" t="n"/>
     </row>
     <row r="193">
-      <c r="A193" t="n">
+      <c r="A193" s="15" t="n">
         <v>192</v>
       </c>
-      <c r="B193" t="inlineStr">
+      <c r="B193" s="15" t="inlineStr">
         <is>
           <t>Vegetarian</t>
         </is>
       </c>
-      <c r="C193" t="inlineStr">
+      <c r="C193" s="15" t="inlineStr">
         <is>
           <t>bottle-gourd-kababs</t>
         </is>
       </c>
-      <c r="D193" t="inlineStr">
+      <c r="D193" s="15" t="inlineStr">
         <is>
           <t>Bottle Gourd Kababs</t>
         </is>
       </c>
-      <c r="E193" t="inlineStr">
+      <c r="E193" s="15" t="inlineStr">
         <is>
           <t>சுரைக்காய் கபாப்</t>
         </is>
       </c>
-      <c r="F193" t="inlineStr">
+      <c r="F193" s="15" t="inlineStr">
         <is>
           <t>kabab</t>
         </is>
       </c>
-      <c r="G193" t="inlineStr">
+      <c r="G193" s="15" t="inlineStr">
         <is>
           <t>Professional food photography of "Bottle Gourd Kababs" (சுரைக்காய் கபாப்), an Indian snack: golden-brown deep-fried finger-shaped kababs made from a coarse ground bottle-gourd-and-chana-dal mixture, arranged on a plate with tomato sauce. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
         </is>
       </c>
-      <c r="H193" t="inlineStr">
+      <c r="H193" s="15" t="inlineStr">
         <is>
           <t>public/images/recipes/bottle-gourd-kababs/featured.jpg</t>
         </is>
       </c>
-      <c r="I193" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
+      <c r="I193" s="15" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J193" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="K193" s="15" t="n"/>
     </row>
     <row r="194">
-      <c r="A194" t="n">
+      <c r="A194" s="15" t="n">
         <v>193</v>
       </c>
-      <c r="B194" t="inlineStr">
+      <c r="B194" s="15" t="inlineStr">
         <is>
           <t>Vegetarian</t>
         </is>
       </c>
-      <c r="C194" t="inlineStr">
+      <c r="C194" s="15" t="inlineStr">
         <is>
           <t>minty-kababs</t>
         </is>
       </c>
-      <c r="D194" t="inlineStr">
+      <c r="D194" s="15" t="inlineStr">
         <is>
           <t>Minty Kababs</t>
         </is>
       </c>
-      <c r="E194" t="inlineStr">
+      <c r="E194" s="15" t="inlineStr">
         <is>
           <t>புதினா கபாப்</t>
         </is>
       </c>
-      <c r="F194" t="inlineStr">
+      <c r="F194" s="15" t="inlineStr">
         <is>
           <t>kabab</t>
         </is>
       </c>
-      <c r="G194" t="inlineStr">
+      <c r="G194" s="15" t="inlineStr">
         <is>
           <t>Professional food photography of "Minty Kababs" (புதினா கபாப்), an Indian snack: golden-brown deep-fried oblong kabab logs made from potato, carrot, and sprouted moong beans flecked with green mint and coriander, arranged on a plate with chutney. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
         </is>
       </c>
-      <c r="H194" t="inlineStr">
+      <c r="H194" s="15" t="inlineStr">
         <is>
           <t>public/images/recipes/minty-kababs/featured.jpg</t>
         </is>
       </c>
-      <c r="I194" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
+      <c r="I194" s="15" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J194" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="K194" s="15" t="n"/>
     </row>
     <row r="195">
-      <c r="A195" t="n">
+      <c r="A195" s="15" t="n">
         <v>194</v>
       </c>
-      <c r="B195" t="inlineStr">
+      <c r="B195" s="15" t="inlineStr">
         <is>
           <t>Vegetarian</t>
         </is>
       </c>
-      <c r="C195" t="inlineStr">
+      <c r="C195" s="15" t="inlineStr">
         <is>
           <t>cauliflower-kababs</t>
         </is>
       </c>
-      <c r="D195" t="inlineStr">
+      <c r="D195" s="15" t="inlineStr">
         <is>
           <t>Cauliflower Kababs</t>
         </is>
       </c>
-      <c r="E195" t="inlineStr">
+      <c r="E195" s="15" t="inlineStr">
         <is>
           <t>காலிப்ளவர் கபாப்</t>
         </is>
       </c>
-      <c r="F195" t="inlineStr">
+      <c r="F195" s="15" t="inlineStr">
         <is>
           <t>kabab</t>
         </is>
       </c>
-      <c r="G195" t="inlineStr">
+      <c r="G195" s="15" t="inlineStr">
         <is>
           <t>Professional food photography of "Cauliflower Kababs" (காலிப்ளவர் கபாப்), an Indian snack: golden-brown deep-fried oblong kabab logs made from ground cauliflower and chana dal, sliced into pieces, arranged on a plate with a side of vinegar-marinated onion rings. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
         </is>
       </c>
-      <c r="H195" t="inlineStr">
+      <c r="H195" s="15" t="inlineStr">
         <is>
           <t>public/images/recipes/cauliflower-kababs/featured.jpg</t>
         </is>
       </c>
-      <c r="I195" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
+      <c r="I195" s="15" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J195" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="K195" s="15" t="n"/>
     </row>
     <row r="196">
-      <c r="A196" t="n">
+      <c r="A196" s="15" t="n">
         <v>195</v>
       </c>
-      <c r="B196" t="inlineStr">
+      <c r="B196" s="15" t="inlineStr">
         <is>
           <t>Vegetarian</t>
         </is>
       </c>
-      <c r="C196" t="inlineStr">
+      <c r="C196" s="15" t="inlineStr">
         <is>
           <t>vegetable-cutlet</t>
         </is>
       </c>
-      <c r="D196" t="inlineStr">
+      <c r="D196" s="15" t="inlineStr">
         <is>
           <t>Vegetable Cutlet</t>
         </is>
       </c>
-      <c r="E196" t="inlineStr">
+      <c r="E196" s="15" t="inlineStr">
         <is>
           <t>வெஜிடபிள் கட்லெட்</t>
         </is>
       </c>
-      <c r="F196" t="inlineStr">
+      <c r="F196" s="15" t="inlineStr">
         <is>
           <t>cutlet</t>
         </is>
       </c>
-      <c r="G196" t="inlineStr">
+      <c r="G196" s="15" t="inlineStr">
         <is>
           <t>Professional food photography of "Vegetable Cutlet" (வெஜிடபிள் கட்லெட்), an Indian snack: golden-brown pan-fried round patties with a crisp breadcrumb crust, made from mashed potato, carrot, and beetroot, showing a faint reddish tint at the edges, arranged on a plate with tomato sauce and sliced onion, tomato, and cucumber rounds. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
         </is>
       </c>
-      <c r="H196" t="inlineStr">
+      <c r="H196" s="15" t="inlineStr">
         <is>
           <t>public/images/recipes/vegetable-cutlet/featured.jpg</t>
         </is>
       </c>
-      <c r="I196" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
+      <c r="I196" s="15" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J196" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="K196" s="15" t="n"/>
     </row>
     <row r="197">
-      <c r="A197" t="n">
+      <c r="A197" s="15" t="n">
         <v>196</v>
       </c>
-      <c r="B197" t="inlineStr">
+      <c r="B197" s="15" t="inlineStr">
         <is>
           <t>Vegetarian</t>
         </is>
       </c>
-      <c r="C197" t="inlineStr">
+      <c r="C197" s="15" t="inlineStr">
         <is>
           <t>spicy-cutlet</t>
         </is>
       </c>
-      <c r="D197" t="inlineStr">
+      <c r="D197" s="15" t="inlineStr">
         <is>
           <t>Spicy Cutlet</t>
         </is>
       </c>
-      <c r="E197" t="inlineStr">
+      <c r="E197" s="15" t="inlineStr">
         <is>
           <t>காரக் கட்லெட்</t>
         </is>
       </c>
-      <c r="F197" t="inlineStr">
+      <c r="F197" s="15" t="inlineStr">
         <is>
           <t>cutlet</t>
         </is>
       </c>
-      <c r="G197" t="inlineStr">
+      <c r="G197" s="15" t="inlineStr">
         <is>
           <t>Professional food photography of "Spicy Cutlet" (காரக் கட்லெட்), an Indian snack: golden-brown pan-fried round patties with a crisp breadcrumb crust, made from a spiced mix of potato, carrot, cabbage, and beans, arranged on a plate with tomato sauce. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
         </is>
       </c>
-      <c r="H197" t="inlineStr">
+      <c r="H197" s="15" t="inlineStr">
         <is>
           <t>public/images/recipes/spicy-cutlet/featured.jpg</t>
         </is>
       </c>
-      <c r="I197" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
+      <c r="I197" s="15" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J197" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="K197" s="15" t="n"/>
     </row>
     <row r="198">
-      <c r="A198" t="n">
+      <c r="A198" s="15" t="n">
         <v>197</v>
       </c>
-      <c r="B198" t="inlineStr">
+      <c r="B198" s="15" t="inlineStr">
         <is>
           <t>Vegetarian</t>
         </is>
       </c>
-      <c r="C198" t="inlineStr">
+      <c r="C198" s="15" t="inlineStr">
         <is>
           <t>beetroot-cutlets</t>
         </is>
       </c>
-      <c r="D198" t="inlineStr">
+      <c r="D198" s="15" t="inlineStr">
         <is>
           <t>Beetroot Cutlets</t>
         </is>
       </c>
-      <c r="E198" t="inlineStr">
+      <c r="E198" s="15" t="inlineStr">
         <is>
           <t>பீட்ரூட் கட்லெட்</t>
         </is>
       </c>
-      <c r="F198" t="inlineStr">
+      <c r="F198" s="15" t="inlineStr">
         <is>
           <t>cutlet</t>
         </is>
       </c>
-      <c r="G198" t="inlineStr">
+      <c r="G198" s="15" t="inlineStr">
         <is>
           <t>Professional food photography of "Beetroot Cutlets" (பீட்ரூட் கட்லெட்), an Indian snack: golden-brown pan-fried round patties with a crisp breadcrumb crust and a vivid magenta-pink hue showing through from the beetroot filling, arranged on a plate with tomato sauce. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
         </is>
       </c>
-      <c r="H198" t="inlineStr">
+      <c r="H198" s="15" t="inlineStr">
         <is>
           <t>public/images/recipes/beetroot-cutlets/featured.jpg</t>
         </is>
       </c>
-      <c r="I198" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
+      <c r="I198" s="15" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J198" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="K198" s="15" t="n"/>
     </row>
     <row r="199">
-      <c r="A199" t="n">
+      <c r="A199" s="15" t="n">
         <v>198</v>
       </c>
-      <c r="B199" t="inlineStr">
+      <c r="B199" s="15" t="inlineStr">
         <is>
           <t>Vegetarian</t>
         </is>
       </c>
-      <c r="C199" t="inlineStr">
+      <c r="C199" s="15" t="inlineStr">
         <is>
           <t>aloo-tikki</t>
         </is>
       </c>
-      <c r="D199" t="inlineStr">
+      <c r="D199" s="15" t="inlineStr">
         <is>
           <t>Aloo Tikki</t>
         </is>
       </c>
-      <c r="E199" t="inlineStr">
+      <c r="E199" s="15" t="inlineStr">
         <is>
           <t>ஆலூ டிக்கி</t>
         </is>
       </c>
-      <c r="F199" t="inlineStr">
+      <c r="F199" s="15" t="inlineStr">
         <is>
           <t>cutlet</t>
         </is>
       </c>
-      <c r="G199" t="inlineStr">
+      <c r="G199" s="15" t="inlineStr">
         <is>
           <t>Professional food photography of "Aloo Tikki" (ஆலூ டிக்கி), a North Indian street-food snack: round, flattened, golden-brown pan-fried potato patties with a crisp crust, one tikki broken open to reveal a bright green spiced-pea filling inside, topped with chopped onion, tomato chutney, and mint chutney. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
         </is>
       </c>
-      <c r="H199" t="inlineStr">
+      <c r="H199" s="15" t="inlineStr">
         <is>
           <t>public/images/recipes/aloo-tikki/featured.jpg</t>
         </is>
       </c>
-      <c r="I199" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
+      <c r="I199" s="15" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J199" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="K199" s="15" t="n"/>
     </row>
     <row r="200">
-      <c r="A200" t="n">
+      <c r="A200" s="15" t="n">
         <v>199</v>
       </c>
-      <c r="B200" t="inlineStr">
+      <c r="B200" s="15" t="inlineStr">
         <is>
           <t>Vegetarian</t>
         </is>
       </c>
-      <c r="C200" t="inlineStr">
+      <c r="C200" s="15" t="inlineStr">
         <is>
           <t>cheese-cutlets</t>
         </is>
       </c>
-      <c r="D200" t="inlineStr">
+      <c r="D200" s="15" t="inlineStr">
         <is>
           <t>Cheese Cutlets</t>
         </is>
       </c>
-      <c r="E200" t="inlineStr">
+      <c r="E200" s="15" t="inlineStr">
         <is>
           <t>சீஸ் கட்லெட்</t>
         </is>
       </c>
-      <c r="F200" t="inlineStr">
+      <c r="F200" s="15" t="inlineStr">
         <is>
           <t>cutlet</t>
         </is>
       </c>
-      <c r="G200" t="inlineStr">
+      <c r="G200" s="15" t="inlineStr">
         <is>
           <t>Professional food photography of "Cheese Cutlets" (சீஸ் கட்லெட்), an Indian snack: golden-brown pan-fried round patties with a crisp breadcrumb crust, made from potato, cabbage, and capsicum mixed with melted cheese, one cutlet broken in half showing a soft, slightly stringy cheese-flecked interior, arranged on a plate with tomato sauce. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
         </is>
       </c>
-      <c r="H200" t="inlineStr">
+      <c r="H200" s="15" t="inlineStr">
         <is>
           <t>public/images/recipes/cheese-cutlets/featured.jpg</t>
         </is>
       </c>
-      <c r="I200" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
+      <c r="I200" s="15" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J200" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="K200" s="15" t="n"/>
     </row>
     <row r="201">
-      <c r="A201" t="n">
+      <c r="A201" s="15" t="n">
         <v>200</v>
       </c>
-      <c r="B201" t="inlineStr">
+      <c r="B201" s="15" t="inlineStr">
         <is>
           <t>Vegetarian</t>
         </is>
       </c>
-      <c r="C201" t="inlineStr">
+      <c r="C201" s="15" t="inlineStr">
         <is>
           <t>green-cutlets</t>
         </is>
       </c>
-      <c r="D201" t="inlineStr">
+      <c r="D201" s="15" t="inlineStr">
         <is>
           <t>Green Cutlets</t>
         </is>
       </c>
-      <c r="E201" t="inlineStr">
+      <c r="E201" s="15" t="inlineStr">
         <is>
           <t>கீரை கட்லெட்</t>
         </is>
       </c>
-      <c r="F201" t="inlineStr">
+      <c r="F201" s="15" t="inlineStr">
         <is>
           <t>cutlet</t>
         </is>
       </c>
-      <c r="G201" t="inlineStr">
+      <c r="G201" s="15" t="inlineStr">
         <is>
           <t>Professional food photography of "Green Cutlets" (கீரை கட்லெட்), an Indian snack: golden-brown pan-fried round patties with a crisp breadcrumb crust, the interior visibly flecked with dark green sauteed leafy greens mixed into a lentil base, arranged on a plate with tomato sauce. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
         </is>
       </c>
-      <c r="H201" t="inlineStr">
+      <c r="H201" s="15" t="inlineStr">
         <is>
           <t>public/images/recipes/green-cutlets/featured.jpg</t>
         </is>
       </c>
-      <c r="I201" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
+      <c r="I201" s="15" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J201" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="K201" s="15" t="n"/>
     </row>
     <row r="202">
-      <c r="A202" t="n">
+      <c r="A202" s="15" t="n">
         <v>201</v>
       </c>
-      <c r="B202" t="inlineStr">
+      <c r="B202" s="15" t="inlineStr">
         <is>
           <t>Vegetarian</t>
         </is>
       </c>
-      <c r="C202" t="inlineStr">
+      <c r="C202" s="15" t="inlineStr">
         <is>
           <t>sago-cutlets</t>
         </is>
       </c>
-      <c r="D202" t="inlineStr">
+      <c r="D202" s="15" t="inlineStr">
         <is>
           <t>Sago Cutlets</t>
         </is>
       </c>
-      <c r="E202" t="inlineStr">
+      <c r="E202" s="15" t="inlineStr">
         <is>
           <t>ஜவ்வரிசி கட்லெட்</t>
         </is>
       </c>
-      <c r="F202" t="inlineStr">
+      <c r="F202" s="15" t="inlineStr">
         <is>
           <t>cutlet</t>
         </is>
       </c>
-      <c r="G202" t="inlineStr">
+      <c r="G202" s="15" t="inlineStr">
         <is>
           <t>Professional food photography of "Sago Cutlets" (ஜவ்வரிசி கட்லெட்), an Indian snack: golden-brown pan-fried round patties with a crisp breadcrumb crust, the surface and interior studded with small translucent soaked sago pearls mixed into the mashed-potato base, arranged on a plate with tomato sauce and mint chutney. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
         </is>
       </c>
-      <c r="H202" t="inlineStr">
+      <c r="H202" s="15" t="inlineStr">
         <is>
           <t>public/images/recipes/sago-cutlets/featured.jpg</t>
         </is>
       </c>
-      <c r="I202" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
+      <c r="I202" s="15" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J202" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="K202" s="15" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Fill 21 missing recipes from Vegetarian Cooking Tips cookbook
Cross-checked all 85 recipes across cooking tips.pdf + cooking tips2.pdf
against already-transcribed content and found 21 genuine gaps (egg dosai,
masala idli, vegetable sambar, idiyappam, sweet appam, chapati, patrora,
tomato kurma, kathirikkai kosu, masala sundal, kuzhai puttu, pan cake,
milk basundi, cashew pakoda, potato chips, sweet raw mango, kinch mosara,
pirattu kari, chinese sooce, boat egg, fish fry roast). Also adds Gemini
image prompts for these 21 to the tracker.
</commit_message>
<xml_diff>
--- a/docs/recipe-image-tracker.xlsx
+++ b/docs/recipe-image-tracker.xlsx
@@ -496,7 +496,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K202"/>
+  <dimension ref="A1:K294"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -11423,6 +11423,4146 @@
         </is>
       </c>
       <c r="K202" s="15" t="n"/>
+    </row>
+    <row r="203">
+      <c r="A203" t="n">
+        <v>202</v>
+      </c>
+      <c r="B203" t="inlineStr">
+        <is>
+          <t>Vegetarian</t>
+        </is>
+      </c>
+      <c r="C203" t="inlineStr">
+        <is>
+          <t>banana-cutlets</t>
+        </is>
+      </c>
+      <c r="D203" t="inlineStr">
+        <is>
+          <t>Banana Cutlets</t>
+        </is>
+      </c>
+      <c r="E203" t="inlineStr">
+        <is>
+          <t>வாழைக்காய் கட்லெட்</t>
+        </is>
+      </c>
+      <c r="F203" t="inlineStr">
+        <is>
+          <t>cutlet</t>
+        </is>
+      </c>
+      <c r="G203" t="inlineStr">
+        <is>
+          <t>A close-up photorealistic food photo of golden-brown oval cutlets with a crisp breadcrumb crust, plated on a white ceramic plate, garnished with a wedge of lemon and a small bowl of tomato ketchup, one cutlet broken open to reveal a soft reddish-brown banana-potato filling flecked with green coriander, warm natural lighting, shallow depth of field.</t>
+        </is>
+      </c>
+      <c r="H203" t="inlineStr">
+        <is>
+          <t>public/images/recipes/banana-cutlets/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I203" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" t="n">
+        <v>203</v>
+      </c>
+      <c r="B204" t="inlineStr">
+        <is>
+          <t>Vegetarian</t>
+        </is>
+      </c>
+      <c r="C204" t="inlineStr">
+        <is>
+          <t>vegetable-sizzlers</t>
+        </is>
+      </c>
+      <c r="D204" t="inlineStr">
+        <is>
+          <t>Vegetable Sizzlers</t>
+        </is>
+      </c>
+      <c r="E204" t="inlineStr">
+        <is>
+          <t>வெஜிடபிள் சிஸ்லர்ஸ்</t>
+        </is>
+      </c>
+      <c r="F204" t="inlineStr">
+        <is>
+          <t>fusion</t>
+        </is>
+      </c>
+      <c r="G204" t="inlineStr">
+        <is>
+          <t>A dramatic photorealistic photo of a cast-iron sizzler plate on a wooden board, visibly smoking with steam rising, holding a golden fried cutlet in the center surrounded by charred grilled carrot rounds, cabbage wedges, capsicum rings, and potato slices, glossy with butter and reddish sauce, dark moody restaurant lighting.</t>
+        </is>
+      </c>
+      <c r="H204" t="inlineStr">
+        <is>
+          <t>public/images/recipes/vegetable-sizzlers/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I204" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" t="n">
+        <v>204</v>
+      </c>
+      <c r="B205" t="inlineStr">
+        <is>
+          <t>Vegetarian</t>
+        </is>
+      </c>
+      <c r="C205" t="inlineStr">
+        <is>
+          <t>vegetable-burgers</t>
+        </is>
+      </c>
+      <c r="D205" t="inlineStr">
+        <is>
+          <t>Vegetable Burgers</t>
+        </is>
+      </c>
+      <c r="E205" t="inlineStr">
+        <is>
+          <t>வெஜிடபிள் பர்கர்ஸ்</t>
+        </is>
+      </c>
+      <c r="F205" t="inlineStr">
+        <is>
+          <t>fusion</t>
+        </is>
+      </c>
+      <c r="G205" t="inlineStr">
+        <is>
+          <t>A photorealistic close-up of a round golden-brown vegetable burger patty inside a soft bun, layered with a crisp cabbage leaf, thin onion rings, beetroot slices, and tomato, skewered with a small toothpick, plated with crinkle-cut potato fries and ketchup, bright appetizing lighting.</t>
+        </is>
+      </c>
+      <c r="H205" t="inlineStr">
+        <is>
+          <t>public/images/recipes/vegetable-burgers/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I205" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" t="n">
+        <v>205</v>
+      </c>
+      <c r="B206" t="inlineStr">
+        <is>
+          <t>Vegetarian</t>
+        </is>
+      </c>
+      <c r="C206" t="inlineStr">
+        <is>
+          <t>sago-bonda</t>
+        </is>
+      </c>
+      <c r="D206" t="inlineStr">
+        <is>
+          <t>Sago Bonda</t>
+        </is>
+      </c>
+      <c r="E206" t="inlineStr">
+        <is>
+          <t>ஜவ்வரிசி போண்டா</t>
+        </is>
+      </c>
+      <c r="F206" t="inlineStr">
+        <is>
+          <t>bonda</t>
+        </is>
+      </c>
+      <c r="G206" t="inlineStr">
+        <is>
+          <t>A photorealistic close-up of small round golden-brown bondas with a translucent, pearly, slightly bumpy sago texture visible on the fried crust, piled on a steel plate lined with paper, garnished with coriander leaves, a small bowl of green chutney beside them, warm kitchen lighting.</t>
+        </is>
+      </c>
+      <c r="H206" t="inlineStr">
+        <is>
+          <t>public/images/recipes/sago-bonda/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I206" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" t="n">
+        <v>206</v>
+      </c>
+      <c r="B207" t="inlineStr">
+        <is>
+          <t>Vegetarian</t>
+        </is>
+      </c>
+      <c r="C207" t="inlineStr">
+        <is>
+          <t>vegetable-bonda</t>
+        </is>
+      </c>
+      <c r="D207" t="inlineStr">
+        <is>
+          <t>Vegetable Bonda</t>
+        </is>
+      </c>
+      <c r="E207" t="inlineStr">
+        <is>
+          <t>வெஜிடபிள் போண்டா</t>
+        </is>
+      </c>
+      <c r="F207" t="inlineStr">
+        <is>
+          <t>bonda</t>
+        </is>
+      </c>
+      <c r="G207" t="inlineStr">
+        <is>
+          <t>A photorealistic photo of golden fried round bondas with a slightly bumpy, craggy batter surface, one bonda broken in half to show a moist mixed-vegetable filling of carrot, peas, and potato, served on a steel plate with mint chutney and tomato sauce, natural daylight.</t>
+        </is>
+      </c>
+      <c r="H207" t="inlineStr">
+        <is>
+          <t>public/images/recipes/vegetable-bonda/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I207" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" t="n">
+        <v>207</v>
+      </c>
+      <c r="B208" t="inlineStr">
+        <is>
+          <t>Vegetarian</t>
+        </is>
+      </c>
+      <c r="C208" t="inlineStr">
+        <is>
+          <t>aloo-bonda</t>
+        </is>
+      </c>
+      <c r="D208" t="inlineStr">
+        <is>
+          <t>Aloo Bonda</t>
+        </is>
+      </c>
+      <c r="E208" t="inlineStr">
+        <is>
+          <t>உருளைக்கிழங்கு போண்டா</t>
+        </is>
+      </c>
+      <c r="F208" t="inlineStr">
+        <is>
+          <t>bonda</t>
+        </is>
+      </c>
+      <c r="G208" t="inlineStr">
+        <is>
+          <t>A photorealistic image of golden-brown round bondas with a smooth thin batter coating, arranged on a banana leaf, one cut open to reveal a soft yellow mashed-potato filling flecked with onion and coriander, served with coconut chutney, warm South Indian tea-stall lighting.</t>
+        </is>
+      </c>
+      <c r="H208" t="inlineStr">
+        <is>
+          <t>public/images/recipes/aloo-bonda/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I208" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" t="n">
+        <v>208</v>
+      </c>
+      <c r="B209" t="inlineStr">
+        <is>
+          <t>Vegetarian</t>
+        </is>
+      </c>
+      <c r="C209" t="inlineStr">
+        <is>
+          <t>mysore-bonda</t>
+        </is>
+      </c>
+      <c r="D209" t="inlineStr">
+        <is>
+          <t>Mysore Bonda</t>
+        </is>
+      </c>
+      <c r="E209" t="inlineStr">
+        <is>
+          <t>மைசூர் போண்டா</t>
+        </is>
+      </c>
+      <c r="F209" t="inlineStr">
+        <is>
+          <t>bonda</t>
+        </is>
+      </c>
+      <c r="G209" t="inlineStr">
+        <is>
+          <t>A photorealistic close-up of fluffy, irregularly round golden-brown bondas with a light, airy fried crust, stacked in a steel plate, one broken open showing a soft white lentil interior studded with coconut bits, served with coconut chutney in a small bowl, bright natural light.</t>
+        </is>
+      </c>
+      <c r="H209" t="inlineStr">
+        <is>
+          <t>public/images/recipes/mysore-bonda/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I209" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" t="n">
+        <v>209</v>
+      </c>
+      <c r="B210" t="inlineStr">
+        <is>
+          <t>Vegetarian</t>
+        </is>
+      </c>
+      <c r="C210" t="inlineStr">
+        <is>
+          <t>pullani-vunta</t>
+        </is>
+      </c>
+      <c r="D210" t="inlineStr">
+        <is>
+          <t>Pullani Vunta</t>
+        </is>
+      </c>
+      <c r="E210" t="inlineStr">
+        <is>
+          <t>தோசைமாவு போண்டா</t>
+        </is>
+      </c>
+      <c r="F210" t="inlineStr">
+        <is>
+          <t>bonda</t>
+        </is>
+      </c>
+      <c r="G210" t="inlineStr">
+        <is>
+          <t>A photorealistic photo of small irregular golden-brown fried dumplings made from fermented dosa batter, slightly craggy surface with visible onion and coriander flecks, piled on a steel plate with coconut chutney on the side, cozy kitchen lighting.</t>
+        </is>
+      </c>
+      <c r="H210" t="inlineStr">
+        <is>
+          <t>public/images/recipes/pullani-vunta/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I210" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" t="n">
+        <v>210</v>
+      </c>
+      <c r="B211" t="inlineStr">
+        <is>
+          <t>Vegetarian</t>
+        </is>
+      </c>
+      <c r="C211" t="inlineStr">
+        <is>
+          <t>mangalore-bonda</t>
+        </is>
+      </c>
+      <c r="D211" t="inlineStr">
+        <is>
+          <t>Mangalore Bonda</t>
+        </is>
+      </c>
+      <c r="E211" t="inlineStr">
+        <is>
+          <t>மங்களூர் போண்டா</t>
+        </is>
+      </c>
+      <c r="F211" t="inlineStr">
+        <is>
+          <t>bonda</t>
+        </is>
+      </c>
+      <c r="G211" t="inlineStr">
+        <is>
+          <t>A photorealistic close-up of soft, puffy golden-brown fried bondas with a slightly wrinkled curd-based batter texture, arranged on a plate, one broken open to reveal a soft white interior, served with coconut chutney, warm ambient lighting.</t>
+        </is>
+      </c>
+      <c r="H211" t="inlineStr">
+        <is>
+          <t>public/images/recipes/mangalore-bonda/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I211" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" t="n">
+        <v>211</v>
+      </c>
+      <c r="B212" t="inlineStr">
+        <is>
+          <t>Vegetarian</t>
+        </is>
+      </c>
+      <c r="C212" t="inlineStr">
+        <is>
+          <t>cheese-bonda</t>
+        </is>
+      </c>
+      <c r="D212" t="inlineStr">
+        <is>
+          <t>Cheese Bonda</t>
+        </is>
+      </c>
+      <c r="E212" t="inlineStr">
+        <is>
+          <t>சீஸ் போண்டா</t>
+        </is>
+      </c>
+      <c r="F212" t="inlineStr">
+        <is>
+          <t>bonda</t>
+        </is>
+      </c>
+      <c r="G212" t="inlineStr">
+        <is>
+          <t>A photorealistic close-up of small golden fried bondas glistening with oil, one cut in half to reveal a stretchy, melted golden-yellow cheese pull, plated on a white dish, steam rising, cozy warm lighting.</t>
+        </is>
+      </c>
+      <c r="H212" t="inlineStr">
+        <is>
+          <t>public/images/recipes/cheese-bonda/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I212" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" t="n">
+        <v>212</v>
+      </c>
+      <c r="B213" t="inlineStr">
+        <is>
+          <t>Vegetarian</t>
+        </is>
+      </c>
+      <c r="C213" t="inlineStr">
+        <is>
+          <t>palak-dumplings</t>
+        </is>
+      </c>
+      <c r="D213" t="inlineStr">
+        <is>
+          <t>Palak Dumplings</t>
+        </is>
+      </c>
+      <c r="E213" t="inlineStr">
+        <is>
+          <t>பாலக் மெதுபக்கோடா</t>
+        </is>
+      </c>
+      <c r="F213" t="inlineStr">
+        <is>
+          <t>fried-snack</t>
+        </is>
+      </c>
+      <c r="G213" t="inlineStr">
+        <is>
+          <t>A photorealistic photo of small dark-green-flecked golden fried dumplings, irregular round shape, piled on a plate, showing visible bits of dark green spinach and chili in the crisp fried crust, served with ketchup, natural daylight.</t>
+        </is>
+      </c>
+      <c r="H213" t="inlineStr">
+        <is>
+          <t>public/images/recipes/palak-dumplings/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I213" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" t="n">
+        <v>213</v>
+      </c>
+      <c r="B214" t="inlineStr">
+        <is>
+          <t>Vegetarian</t>
+        </is>
+      </c>
+      <c r="C214" t="inlineStr">
+        <is>
+          <t>ridge-gourd-dumplings</t>
+        </is>
+      </c>
+      <c r="D214" t="inlineStr">
+        <is>
+          <t>Ridge Gourd Dumplings</t>
+        </is>
+      </c>
+      <c r="E214" t="inlineStr">
+        <is>
+          <t>பீர்க்கங்காய் மெதுபக்கோடா</t>
+        </is>
+      </c>
+      <c r="F214" t="inlineStr">
+        <is>
+          <t>fried-snack</t>
+        </is>
+      </c>
+      <c r="G214" t="inlineStr">
+        <is>
+          <t>A photorealistic close-up of small golden fried dumplings with pale green ridge-gourd flecks visible through the thin gram-flour crust, piled on a steel plate, served hot with tomato sauce, warm kitchen lighting.</t>
+        </is>
+      </c>
+      <c r="H214" t="inlineStr">
+        <is>
+          <t>public/images/recipes/ridge-gourd-dumplings/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I214" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" t="n">
+        <v>214</v>
+      </c>
+      <c r="B215" t="inlineStr">
+        <is>
+          <t>Vegetarian</t>
+        </is>
+      </c>
+      <c r="C215" t="inlineStr">
+        <is>
+          <t>mint-pakodas</t>
+        </is>
+      </c>
+      <c r="D215" t="inlineStr">
+        <is>
+          <t>Mint Pakodas</t>
+        </is>
+      </c>
+      <c r="E215" t="inlineStr">
+        <is>
+          <t>புதினா பக்கோடா</t>
+        </is>
+      </c>
+      <c r="F215" t="inlineStr">
+        <is>
+          <t>bajji</t>
+        </is>
+      </c>
+      <c r="G215" t="inlineStr">
+        <is>
+          <t>A photorealistic photo of dark green-brown irregular fried pakodas with visible mint and coriander leaf flecks throughout the crumbly, coarse lentil texture, piled high on a plate, steam rising, natural light.</t>
+        </is>
+      </c>
+      <c r="H215" t="inlineStr">
+        <is>
+          <t>public/images/recipes/mint-pakodas/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I215" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" t="n">
+        <v>215</v>
+      </c>
+      <c r="B216" t="inlineStr">
+        <is>
+          <t>Vegetarian</t>
+        </is>
+      </c>
+      <c r="C216" t="inlineStr">
+        <is>
+          <t>potato-nest</t>
+        </is>
+      </c>
+      <c r="D216" t="inlineStr">
+        <is>
+          <t>Potato Nest</t>
+        </is>
+      </c>
+      <c r="E216" t="inlineStr">
+        <is>
+          <t>உருளைக்கிழங்கு கூடுகள்</t>
+        </is>
+      </c>
+      <c r="F216" t="inlineStr">
+        <is>
+          <t>fried-snack</t>
+        </is>
+      </c>
+      <c r="G216" t="inlineStr">
+        <is>
+          <t>A photorealistic close-up of round golden fried balls coated entirely in crisp, spiky strands of fried vermicelli giving a bird's-nest texture, one cut in half to reveal a bright yellow mashed-potato interior with green peas, plated elegantly with lettuce and tomato sauce, bright studio food photography lighting.</t>
+        </is>
+      </c>
+      <c r="H216" t="inlineStr">
+        <is>
+          <t>public/images/recipes/potato-nest/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I216" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" t="n">
+        <v>216</v>
+      </c>
+      <c r="B217" t="inlineStr">
+        <is>
+          <t>Vegetarian</t>
+        </is>
+      </c>
+      <c r="C217" t="inlineStr">
+        <is>
+          <t>garam-pakodas</t>
+        </is>
+      </c>
+      <c r="D217" t="inlineStr">
+        <is>
+          <t>Garam Pakodas</t>
+        </is>
+      </c>
+      <c r="E217" t="inlineStr">
+        <is>
+          <t>வெங்காய பக்கோடா</t>
+        </is>
+      </c>
+      <c r="F217" t="inlineStr">
+        <is>
+          <t>bajji</t>
+        </is>
+      </c>
+      <c r="G217" t="inlineStr">
+        <is>
+          <t>A photorealistic photo of a heaping pile of irregular, craggy, deep-golden fried pakoda chunks with visible long strands of onion and green chili baked into the crisp crust, on a steel plate, chai glass beside it, warm evening tea-stall lighting.</t>
+        </is>
+      </c>
+      <c r="H217" t="inlineStr">
+        <is>
+          <t>public/images/recipes/garam-pakodas/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I217" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" t="n">
+        <v>217</v>
+      </c>
+      <c r="B218" t="inlineStr">
+        <is>
+          <t>Vegetarian</t>
+        </is>
+      </c>
+      <c r="C218" t="inlineStr">
+        <is>
+          <t>paneer-pakodas</t>
+        </is>
+      </c>
+      <c r="D218" t="inlineStr">
+        <is>
+          <t>Paneer Pakodas</t>
+        </is>
+      </c>
+      <c r="E218" t="inlineStr">
+        <is>
+          <t>பனீர் பக்கோடா</t>
+        </is>
+      </c>
+      <c r="F218" t="inlineStr">
+        <is>
+          <t>bajji</t>
+        </is>
+      </c>
+      <c r="G218" t="inlineStr">
+        <is>
+          <t>A photorealistic close-up of irregular golden fried pakoda chunks with visible crumbly white paneer and pink cashew pieces embedded in the crust, piled on a plate with mint garnish, warm kitchen lighting.</t>
+        </is>
+      </c>
+      <c r="H218" t="inlineStr">
+        <is>
+          <t>public/images/recipes/paneer-pakodas/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I218" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" t="n">
+        <v>218</v>
+      </c>
+      <c r="B219" t="inlineStr">
+        <is>
+          <t>Vegetarian</t>
+        </is>
+      </c>
+      <c r="C219" t="inlineStr">
+        <is>
+          <t>bread-pakodas</t>
+        </is>
+      </c>
+      <c r="D219" t="inlineStr">
+        <is>
+          <t>Bread Pakodas</t>
+        </is>
+      </c>
+      <c r="E219" t="inlineStr">
+        <is>
+          <t>பிரட் பக்கோடா</t>
+        </is>
+      </c>
+      <c r="F219" t="inlineStr">
+        <is>
+          <t>bajji</t>
+        </is>
+      </c>
+      <c r="G219" t="inlineStr">
+        <is>
+          <t>A photorealistic photo of golden-brown irregular fried pakoda pieces with a soft doughy bread interior visible at the torn edges, piled on a plate, served with tomato ketchup, natural daylight.</t>
+        </is>
+      </c>
+      <c r="H219" t="inlineStr">
+        <is>
+          <t>public/images/recipes/bread-pakodas/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I219" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" t="n">
+        <v>219</v>
+      </c>
+      <c r="B220" t="inlineStr">
+        <is>
+          <t>Vegetarian</t>
+        </is>
+      </c>
+      <c r="C220" t="inlineStr">
+        <is>
+          <t>vermicelli-pakodas</t>
+        </is>
+      </c>
+      <c r="D220" t="inlineStr">
+        <is>
+          <t>Vermicelli Pakodas</t>
+        </is>
+      </c>
+      <c r="E220" t="inlineStr">
+        <is>
+          <t>சேமியா பக்கோடா</t>
+        </is>
+      </c>
+      <c r="F220" t="inlineStr">
+        <is>
+          <t>bajji</t>
+        </is>
+      </c>
+      <c r="G220" t="inlineStr">
+        <is>
+          <t>A photorealistic close-up of golden fried pakodas with fine strands of crisp vermicelli visible on the textured surface, piled on a steel plate with mint chutney, warm ambient lighting.</t>
+        </is>
+      </c>
+      <c r="H220" t="inlineStr">
+        <is>
+          <t>public/images/recipes/vermicelli-pakodas/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I220" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" t="n">
+        <v>220</v>
+      </c>
+      <c r="B221" t="inlineStr">
+        <is>
+          <t>Vegetarian</t>
+        </is>
+      </c>
+      <c r="C221" t="inlineStr">
+        <is>
+          <t>layered-sandwich-bajji</t>
+        </is>
+      </c>
+      <c r="D221" t="inlineStr">
+        <is>
+          <t>Layered Sandwich Bajji</t>
+        </is>
+      </c>
+      <c r="E221" t="inlineStr">
+        <is>
+          <t>பிரட் சாண்ட்விட்ச் பஜ்ஜி</t>
+        </is>
+      </c>
+      <c r="F221" t="inlineStr">
+        <is>
+          <t>bajji,sandwich</t>
+        </is>
+      </c>
+      <c r="G221" t="inlineStr">
+        <is>
+          <t>A photorealistic close-up of a golden fried rectangular sandwich bajji cut in half, showing three layers of white bread with visible green mint chutney and red tomato chutney filling between the layers, crisp golden batter coating on the outside, served with tomato sauce, bright natural lighting.</t>
+        </is>
+      </c>
+      <c r="H221" t="inlineStr">
+        <is>
+          <t>public/images/recipes/layered-sandwich-bajji/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I221" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" t="n">
+        <v>221</v>
+      </c>
+      <c r="B222" t="inlineStr">
+        <is>
+          <t>Vegetarian</t>
+        </is>
+      </c>
+      <c r="C222" t="inlineStr">
+        <is>
+          <t>capsicum-bajji</t>
+        </is>
+      </c>
+      <c r="D222" t="inlineStr">
+        <is>
+          <t>Capsicum Bajji</t>
+        </is>
+      </c>
+      <c r="E222" t="inlineStr">
+        <is>
+          <t>குடமிளகாய் பஜ்ஜி</t>
+        </is>
+      </c>
+      <c r="F222" t="inlineStr">
+        <is>
+          <t>bajji</t>
+        </is>
+      </c>
+      <c r="G222" t="inlineStr">
+        <is>
+          <t>A photorealistic photo of whole small green capsicums coated in a golden fried batter, one sliced open at the top showing chopped onion tucked inside with a wedge of lemon on the side, plated attractively, warm lighting.</t>
+        </is>
+      </c>
+      <c r="H222" t="inlineStr">
+        <is>
+          <t>public/images/recipes/capsicum-bajji/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I222" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" t="n">
+        <v>222</v>
+      </c>
+      <c r="B223" t="inlineStr">
+        <is>
+          <t>Vegetarian</t>
+        </is>
+      </c>
+      <c r="C223" t="inlineStr">
+        <is>
+          <t>stuffed-chilli-bajji</t>
+        </is>
+      </c>
+      <c r="D223" t="inlineStr">
+        <is>
+          <t>Stuffed Chilli Bajji</t>
+        </is>
+      </c>
+      <c r="E223" t="inlineStr">
+        <is>
+          <t>மிளகாய் பஜ்ஜி</t>
+        </is>
+      </c>
+      <c r="F223" t="inlineStr">
+        <is>
+          <t>bajji</t>
+        </is>
+      </c>
+      <c r="G223" t="inlineStr">
+        <is>
+          <t>A photorealistic close-up of long green bajji chilies coated in golden fried batter, one split open lengthwise to reveal a pale coconut-and-gram filling inside, garnished with chopped onion and a drizzle of sweet brown chutney, plated on a steel dish, warm tea-stall lighting.</t>
+        </is>
+      </c>
+      <c r="H223" t="inlineStr">
+        <is>
+          <t>public/images/recipes/stuffed-chilli-bajji/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I223" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" t="n">
+        <v>223</v>
+      </c>
+      <c r="B224" t="inlineStr">
+        <is>
+          <t>Vegetarian</t>
+        </is>
+      </c>
+      <c r="C224" t="inlineStr">
+        <is>
+          <t>lasania</t>
+        </is>
+      </c>
+      <c r="D224" t="inlineStr">
+        <is>
+          <t>Lasania (Stuffed Potato Bajji)</t>
+        </is>
+      </c>
+      <c r="E224" t="inlineStr">
+        <is>
+          <t>உருளைகிழங்கு ஸ்டப் பஜ்ஜி</t>
+        </is>
+      </c>
+      <c r="F224" t="inlineStr">
+        <is>
+          <t>bajji</t>
+        </is>
+      </c>
+      <c r="G224" t="inlineStr">
+        <is>
+          <t>A photorealistic photo of small whole potatoes coated in golden fried batter, one sliced partway open showing a reddish garlic-spice paste inside, piled on a plate, warm lighting.</t>
+        </is>
+      </c>
+      <c r="H224" t="inlineStr">
+        <is>
+          <t>public/images/recipes/lasania/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I224" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" t="n">
+        <v>224</v>
+      </c>
+      <c r="B225" t="inlineStr">
+        <is>
+          <t>Vegetarian</t>
+        </is>
+      </c>
+      <c r="C225" t="inlineStr">
+        <is>
+          <t>medu-vadai</t>
+        </is>
+      </c>
+      <c r="D225" t="inlineStr">
+        <is>
+          <t>Medu Vadai</t>
+        </is>
+      </c>
+      <c r="E225" t="inlineStr">
+        <is>
+          <t>மெதுவடை</t>
+        </is>
+      </c>
+      <c r="F225" t="inlineStr">
+        <is>
+          <t>vadai</t>
+        </is>
+      </c>
+      <c r="G225" t="inlineStr">
+        <is>
+          <t>A photorealistic close-up of classic golden-brown ring-shaped vadais with a lacy, crisp textured surface, stacked on a banana leaf, served with sambar in a small steel bowl and coconut chutney, warm South Indian breakfast table lighting.</t>
+        </is>
+      </c>
+      <c r="H225" t="inlineStr">
+        <is>
+          <t>public/images/recipes/medu-vadai/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I225" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" t="n">
+        <v>225</v>
+      </c>
+      <c r="B226" t="inlineStr">
+        <is>
+          <t>Vegetarian</t>
+        </is>
+      </c>
+      <c r="C226" t="inlineStr">
+        <is>
+          <t>curd-vadai</t>
+        </is>
+      </c>
+      <c r="D226" t="inlineStr">
+        <is>
+          <t>Thair Vadai</t>
+        </is>
+      </c>
+      <c r="E226" t="inlineStr">
+        <is>
+          <t>தயிர் வடை</t>
+        </is>
+      </c>
+      <c r="F226" t="inlineStr">
+        <is>
+          <t>vadai</t>
+        </is>
+      </c>
+      <c r="G226" t="inlineStr">
+        <is>
+          <t>A photorealistic close-up of soft, pale golden vadais submerged in thick white curd on a steel plate, garnished with a drizzle of tempered mustard seeds, chopped coriander leaves, and a light dusting of red chili powder on top, bright natural lighting.</t>
+        </is>
+      </c>
+      <c r="H226" t="inlineStr">
+        <is>
+          <t>public/images/recipes/curd-vadai/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I226" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" t="n">
+        <v>226</v>
+      </c>
+      <c r="B227" t="inlineStr">
+        <is>
+          <t>Vegetarian</t>
+        </is>
+      </c>
+      <c r="C227" t="inlineStr">
+        <is>
+          <t>special-curd-vadai-1</t>
+        </is>
+      </c>
+      <c r="D227" t="inlineStr">
+        <is>
+          <t>Special Curd Vadai 1</t>
+        </is>
+      </c>
+      <c r="E227" t="inlineStr">
+        <is>
+          <t>ஸ்பெஷல் தயிர் வடை (1)</t>
+        </is>
+      </c>
+      <c r="F227" t="inlineStr">
+        <is>
+          <t>vadai</t>
+        </is>
+      </c>
+      <c r="G227" t="inlineStr">
+        <is>
+          <t>A photorealistic close-up of a curd-soaked vadai cut open on a plate revealing a colorful filling of chopped cashews, almonds, raisins, and coconut inside the soft white lentil dough, surrounded by thick curd, garnished with fried spicy boondi on top, bright lighting.</t>
+        </is>
+      </c>
+      <c r="H227" t="inlineStr">
+        <is>
+          <t>public/images/recipes/special-curd-vadai-1/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I227" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" t="n">
+        <v>227</v>
+      </c>
+      <c r="B228" t="inlineStr">
+        <is>
+          <t>Vegetarian</t>
+        </is>
+      </c>
+      <c r="C228" t="inlineStr">
+        <is>
+          <t>special-curd-vadai-2</t>
+        </is>
+      </c>
+      <c r="D228" t="inlineStr">
+        <is>
+          <t>Special Curd Vadai 2</t>
+        </is>
+      </c>
+      <c r="E228" t="inlineStr">
+        <is>
+          <t>ஸ்பெஷல் தயிர் வடை (2)</t>
+        </is>
+      </c>
+      <c r="F228" t="inlineStr">
+        <is>
+          <t>vadai</t>
+        </is>
+      </c>
+      <c r="G228" t="inlineStr">
+        <is>
+          <t>A photorealistic close-up of a half-moon, samosa-shaped curd vadai on a plate, soaked in white curd, with visible green herb flecks along the folded edge, garnished with grated carrot and coriander, natural lighting.</t>
+        </is>
+      </c>
+      <c r="H228" t="inlineStr">
+        <is>
+          <t>public/images/recipes/special-curd-vadai-2/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I228" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" t="n">
+        <v>228</v>
+      </c>
+      <c r="B229" t="inlineStr">
+        <is>
+          <t>Vegetarian</t>
+        </is>
+      </c>
+      <c r="C229" t="inlineStr">
+        <is>
+          <t>pattani-curd-vadai</t>
+        </is>
+      </c>
+      <c r="D229" t="inlineStr">
+        <is>
+          <t>Pattani Curd Vadai</t>
+        </is>
+      </c>
+      <c r="E229" t="inlineStr">
+        <is>
+          <t>பட்டாணி தயிர் வடை</t>
+        </is>
+      </c>
+      <c r="F229" t="inlineStr">
+        <is>
+          <t>vadai</t>
+        </is>
+      </c>
+      <c r="G229" t="inlineStr">
+        <is>
+          <t>A photorealistic close-up of a curd-soaked vadai cut in half showing a bright green mashed-pea filling inside the soft white lentil exterior, surrounded by thick curd on a steel plate, garnished with coriander, natural lighting.</t>
+        </is>
+      </c>
+      <c r="H229" t="inlineStr">
+        <is>
+          <t>public/images/recipes/pattani-curd-vadai/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I229" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" t="n">
+        <v>229</v>
+      </c>
+      <c r="B230" t="inlineStr">
+        <is>
+          <t>Vegetarian</t>
+        </is>
+      </c>
+      <c r="C230" t="inlineStr">
+        <is>
+          <t>mor-kuzhambu-vadai</t>
+        </is>
+      </c>
+      <c r="D230" t="inlineStr">
+        <is>
+          <t>Mor Kuzhambu Vadai</t>
+        </is>
+      </c>
+      <c r="E230" t="inlineStr">
+        <is>
+          <t>மோர்க்குழம்பு வடை</t>
+        </is>
+      </c>
+      <c r="F230" t="inlineStr">
+        <is>
+          <t>vadai</t>
+        </is>
+      </c>
+      <c r="G230" t="inlineStr">
+        <is>
+          <t>A photorealistic close-up of pale golden vadais submerged in a thick, pale-yellow spiced buttermilk gravy flecked with coconut and curry leaves, served in a steel bowl, garnished with coriander leaves, warm home-style lighting.</t>
+        </is>
+      </c>
+      <c r="H230" t="inlineStr">
+        <is>
+          <t>public/images/recipes/mor-kuzhambu-vadai/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I230" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" t="n">
+        <v>230</v>
+      </c>
+      <c r="B231" t="inlineStr">
+        <is>
+          <t>Vegetarian</t>
+        </is>
+      </c>
+      <c r="C231" t="inlineStr">
+        <is>
+          <t>aamai-vadai</t>
+        </is>
+      </c>
+      <c r="D231" t="inlineStr">
+        <is>
+          <t>Aamai Vadai</t>
+        </is>
+      </c>
+      <c r="E231" t="inlineStr">
+        <is>
+          <t>ஆமை வடை</t>
+        </is>
+      </c>
+      <c r="F231" t="inlineStr">
+        <is>
+          <t>vadai</t>
+        </is>
+      </c>
+      <c r="G231" t="inlineStr">
+        <is>
+          <t>A photorealistic photo of torn half-moon pieces of coarse-textured urad-toor dal vadai, soaked briefly in curd, plated with a light garnish, rustic table lighting.</t>
+        </is>
+      </c>
+      <c r="H231" t="inlineStr">
+        <is>
+          <t>public/images/recipes/aamai-vadai/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I231" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" t="n">
+        <v>231</v>
+      </c>
+      <c r="B232" t="inlineStr">
+        <is>
+          <t>Vegetarian</t>
+        </is>
+      </c>
+      <c r="C232" t="inlineStr">
+        <is>
+          <t>bread-dahi-vadai</t>
+        </is>
+      </c>
+      <c r="D232" t="inlineStr">
+        <is>
+          <t>Bread Dahi Vadai</t>
+        </is>
+      </c>
+      <c r="E232" t="inlineStr">
+        <is>
+          <t>திடீர் பிரட் தயிர்வடை</t>
+        </is>
+      </c>
+      <c r="F232" t="inlineStr">
+        <is>
+          <t>vadai</t>
+        </is>
+      </c>
+      <c r="G232" t="inlineStr">
+        <is>
+          <t>A photorealistic close-up of small round bread-dough vadais topped generously with white curd, dusted with black salt, roasted cumin powder, and red chili powder, drizzled with brown sweet chutney and garnished with coriander leaves, bright appetizing lighting.</t>
+        </is>
+      </c>
+      <c r="H232" t="inlineStr">
+        <is>
+          <t>public/images/recipes/bread-dahi-vadai/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I232" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" t="n">
+        <v>232</v>
+      </c>
+      <c r="B233" t="inlineStr">
+        <is>
+          <t>Vegetarian</t>
+        </is>
+      </c>
+      <c r="C233" t="inlineStr">
+        <is>
+          <t>moong-dhal-curd-pakoda</t>
+        </is>
+      </c>
+      <c r="D233" t="inlineStr">
+        <is>
+          <t>Moong Dhal Curd Pakoda</t>
+        </is>
+      </c>
+      <c r="E233" t="inlineStr">
+        <is>
+          <t>பயத்தம் பருப்பு தயிர் பக்கோடா</t>
+        </is>
+      </c>
+      <c r="F233" t="inlineStr">
+        <is>
+          <t>bajji</t>
+        </is>
+      </c>
+      <c r="G233" t="inlineStr">
+        <is>
+          <t>A photorealistic close-up of small golden fried lentil pakodas arranged on a plate, topped with a generous pour of white whisked curd, dusted with a dark spice powder and tomato sauce drizzle, bright lighting.</t>
+        </is>
+      </c>
+      <c r="H233" t="inlineStr">
+        <is>
+          <t>public/images/recipes/moong-dhal-curd-pakoda/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I233" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" t="n">
+        <v>233</v>
+      </c>
+      <c r="B234" t="inlineStr">
+        <is>
+          <t>Vegetarian</t>
+        </is>
+      </c>
+      <c r="C234" t="inlineStr">
+        <is>
+          <t>mysore-vadai</t>
+        </is>
+      </c>
+      <c r="D234" t="inlineStr">
+        <is>
+          <t>Mysore Vadai</t>
+        </is>
+      </c>
+      <c r="E234" t="inlineStr">
+        <is>
+          <t>மைசூர் வடை</t>
+        </is>
+      </c>
+      <c r="F234" t="inlineStr">
+        <is>
+          <t>vadai</t>
+        </is>
+      </c>
+      <c r="G234" t="inlineStr">
+        <is>
+          <t>A photorealistic close-up of textured, coarse golden-brown vadais studded with visible cashew pieces and melon seeds, stacked on a plate, served with thokku, warm lighting.</t>
+        </is>
+      </c>
+      <c r="H234" t="inlineStr">
+        <is>
+          <t>public/images/recipes/mysore-vadai/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I234" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" t="n">
+        <v>234</v>
+      </c>
+      <c r="B235" t="inlineStr">
+        <is>
+          <t>Vegetarian</t>
+        </is>
+      </c>
+      <c r="C235" t="inlineStr">
+        <is>
+          <t>madhur-vadai</t>
+        </is>
+      </c>
+      <c r="D235" t="inlineStr">
+        <is>
+          <t>Madhur Vadai</t>
+        </is>
+      </c>
+      <c r="E235" t="inlineStr">
+        <is>
+          <t>மதுர் வடை</t>
+        </is>
+      </c>
+      <c r="F235" t="inlineStr">
+        <is>
+          <t>vadai</t>
+        </is>
+      </c>
+      <c r="G235" t="inlineStr">
+        <is>
+          <t>A photorealistic photo of thin, flat, deep reddish-brown crispy discs with visible onion flecks, stacked in a glass jar and also arranged on a plate, matte crunchy texture, natural light.</t>
+        </is>
+      </c>
+      <c r="H235" t="inlineStr">
+        <is>
+          <t>public/images/recipes/madhur-vadai/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I235" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" t="n">
+        <v>235</v>
+      </c>
+      <c r="B236" t="inlineStr">
+        <is>
+          <t>Vegetarian</t>
+        </is>
+      </c>
+      <c r="C236" t="inlineStr">
+        <is>
+          <t>masal-vadai</t>
+        </is>
+      </c>
+      <c r="D236" t="inlineStr">
+        <is>
+          <t>Masal Vadai</t>
+        </is>
+      </c>
+      <c r="E236" t="inlineStr">
+        <is>
+          <t>மசால் வடை</t>
+        </is>
+      </c>
+      <c r="F236" t="inlineStr">
+        <is>
+          <t>vadai</t>
+        </is>
+      </c>
+      <c r="G236" t="inlineStr">
+        <is>
+          <t>A photorealistic close-up of flat, coarse-textured golden-brown vadais with visible chana dal grains, onion, and curry leaf flecks, stacked on a banana leaf, served with coconut chutney, warm lighting.</t>
+        </is>
+      </c>
+      <c r="H236" t="inlineStr">
+        <is>
+          <t>public/images/recipes/masal-vadai/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I236" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" t="n">
+        <v>236</v>
+      </c>
+      <c r="B237" t="inlineStr">
+        <is>
+          <t>Vegetarian</t>
+        </is>
+      </c>
+      <c r="C237" t="inlineStr">
+        <is>
+          <t>gherugu-vadai</t>
+        </is>
+      </c>
+      <c r="D237" t="inlineStr">
+        <is>
+          <t>Gherugu Vadai</t>
+        </is>
+      </c>
+      <c r="E237" t="inlineStr">
+        <is>
+          <t>கெருகு வடை</t>
+        </is>
+      </c>
+      <c r="F237" t="inlineStr">
+        <is>
+          <t>vadai</t>
+        </is>
+      </c>
+      <c r="G237" t="inlineStr">
+        <is>
+          <t>A photorealistic photo of thin, flat, pale golden crispy discs with a slightly speckled sesame-seed texture, stacked on a plate, rustic homely lighting.</t>
+        </is>
+      </c>
+      <c r="H237" t="inlineStr">
+        <is>
+          <t>public/images/recipes/gherugu-vadai/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I237" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238" t="n">
+        <v>237</v>
+      </c>
+      <c r="B238" t="inlineStr">
+        <is>
+          <t>Vegetarian</t>
+        </is>
+      </c>
+      <c r="C238" t="inlineStr">
+        <is>
+          <t>mullangi-vadai</t>
+        </is>
+      </c>
+      <c r="D238" t="inlineStr">
+        <is>
+          <t>Mullangi Vadai</t>
+        </is>
+      </c>
+      <c r="E238" t="inlineStr">
+        <is>
+          <t>முள்ளங்கி வடை</t>
+        </is>
+      </c>
+      <c r="F238" t="inlineStr">
+        <is>
+          <t>vadai</t>
+        </is>
+      </c>
+      <c r="G238" t="inlineStr">
+        <is>
+          <t>A photorealistic close-up of thin, flat, pale golden-brown vadais with visible shreds of white radish embedded in the crisp exterior, stacked on a steel plate, natural daylight.</t>
+        </is>
+      </c>
+      <c r="H238" t="inlineStr">
+        <is>
+          <t>public/images/recipes/mullangi-vadai/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I238" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" t="n">
+        <v>238</v>
+      </c>
+      <c r="B239" t="inlineStr">
+        <is>
+          <t>Vegetarian</t>
+        </is>
+      </c>
+      <c r="C239" t="inlineStr">
+        <is>
+          <t>pulusu-vadai</t>
+        </is>
+      </c>
+      <c r="D239" t="inlineStr">
+        <is>
+          <t>Pulusu Vadai</t>
+        </is>
+      </c>
+      <c r="E239" t="inlineStr">
+        <is>
+          <t>புளி வடை அல்லது புலுசு வடை</t>
+        </is>
+      </c>
+      <c r="F239" t="inlineStr">
+        <is>
+          <t>vadai</t>
+        </is>
+      </c>
+      <c r="G239" t="inlineStr">
+        <is>
+          <t>A photorealistic photo of flat reddish-orange vadais with a speckled texture from ground red chili and pumpkin, stacked on a plate, tangy glossy sheen, warm lighting.</t>
+        </is>
+      </c>
+      <c r="H239" t="inlineStr">
+        <is>
+          <t>public/images/recipes/pulusu-vadai/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I239" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" t="n">
+        <v>239</v>
+      </c>
+      <c r="B240" t="inlineStr">
+        <is>
+          <t>Vegetarian</t>
+        </is>
+      </c>
+      <c r="C240" t="inlineStr">
+        <is>
+          <t>milagu-vadai</t>
+        </is>
+      </c>
+      <c r="D240" t="inlineStr">
+        <is>
+          <t>Milagu Vadai</t>
+        </is>
+      </c>
+      <c r="E240" t="inlineStr">
+        <is>
+          <t>மிளகு வடை</t>
+        </is>
+      </c>
+      <c r="F240" t="inlineStr">
+        <is>
+          <t>vadai</t>
+        </is>
+      </c>
+      <c r="G240" t="inlineStr">
+        <is>
+          <t>A photorealistic close-up of small pale golden vadais with visible flecks of cracked black pepper, some strung together on a thread like a garland, others piled on a plate, temple-offering style presentation, warm devotional lighting.</t>
+        </is>
+      </c>
+      <c r="H240" t="inlineStr">
+        <is>
+          <t>public/images/recipes/milagu-vadai/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I240" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="241">
+      <c r="A241" t="n">
+        <v>240</v>
+      </c>
+      <c r="B241" t="inlineStr">
+        <is>
+          <t>Vegetarian</t>
+        </is>
+      </c>
+      <c r="C241" t="inlineStr">
+        <is>
+          <t>drumstick-vadai</t>
+        </is>
+      </c>
+      <c r="D241" t="inlineStr">
+        <is>
+          <t>Drumstick Vadai</t>
+        </is>
+      </c>
+      <c r="E241" t="inlineStr">
+        <is>
+          <t>முருங்கைக்காய் வடை</t>
+        </is>
+      </c>
+      <c r="F241" t="inlineStr">
+        <is>
+          <t>vadai</t>
+        </is>
+      </c>
+      <c r="G241" t="inlineStr">
+        <is>
+          <t>A photorealistic close-up of coarse, flat golden-brown vadais with a slightly speckled surface, stacked on a plate, served with vinegar-tossed onion rings on the side, warm lighting.</t>
+        </is>
+      </c>
+      <c r="H241" t="inlineStr">
+        <is>
+          <t>public/images/recipes/drumstick-vadai/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I241" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="242">
+      <c r="A242" t="n">
+        <v>241</v>
+      </c>
+      <c r="B242" t="inlineStr">
+        <is>
+          <t>Vegetarian</t>
+        </is>
+      </c>
+      <c r="C242" t="inlineStr">
+        <is>
+          <t>perugu-vadai</t>
+        </is>
+      </c>
+      <c r="D242" t="inlineStr">
+        <is>
+          <t>Perugu Vadai</t>
+        </is>
+      </c>
+      <c r="E242" t="inlineStr">
+        <is>
+          <t>பெருகு வடை</t>
+        </is>
+      </c>
+      <c r="F242" t="inlineStr">
+        <is>
+          <t>vadai</t>
+        </is>
+      </c>
+      <c r="G242" t="inlineStr">
+        <is>
+          <t>A photorealistic photo of soft, pale, lightly golden flat discs with a matte soft surface (not deeply fried), stacked on a plate, gentle lighting emphasizing their softness.</t>
+        </is>
+      </c>
+      <c r="H242" t="inlineStr">
+        <is>
+          <t>public/images/recipes/perugu-vadai/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I242" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="243">
+      <c r="A243" t="n">
+        <v>242</v>
+      </c>
+      <c r="B243" t="inlineStr">
+        <is>
+          <t>Vegetarian</t>
+        </is>
+      </c>
+      <c r="C243" t="inlineStr">
+        <is>
+          <t>moong-dhal-toast</t>
+        </is>
+      </c>
+      <c r="D243" t="inlineStr">
+        <is>
+          <t>Moong Dhal Toast</t>
+        </is>
+      </c>
+      <c r="E243" t="inlineStr">
+        <is>
+          <t>பயத்தம்பருப்பு டோஸ்ட்</t>
+        </is>
+      </c>
+      <c r="F243" t="inlineStr">
+        <is>
+          <t>sandwich</t>
+        </is>
+      </c>
+      <c r="G243" t="inlineStr">
+        <is>
+          <t>A photorealistic close-up of a golden-brown fried bread toast cut diagonally, showing a thin green mint chutney layer and a yellow lentil paste layer between the crisp bread surface and the crust, plated with tomato sauce, bright lighting.</t>
+        </is>
+      </c>
+      <c r="H243" t="inlineStr">
+        <is>
+          <t>public/images/recipes/moong-dhal-toast/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I243" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="244">
+      <c r="A244" t="n">
+        <v>243</v>
+      </c>
+      <c r="B244" t="inlineStr">
+        <is>
+          <t>Vegetarian</t>
+        </is>
+      </c>
+      <c r="C244" t="inlineStr">
+        <is>
+          <t>masala-toast</t>
+        </is>
+      </c>
+      <c r="D244" t="inlineStr">
+        <is>
+          <t>Masala Toast</t>
+        </is>
+      </c>
+      <c r="E244" t="inlineStr">
+        <is>
+          <t>மசாலா டோஸ்ட்</t>
+        </is>
+      </c>
+      <c r="F244" t="inlineStr">
+        <is>
+          <t>sandwich</t>
+        </is>
+      </c>
+      <c r="G244" t="inlineStr">
+        <is>
+          <t>A photorealistic photo of golden-brown toasted bread slices with a thin reddish-brown spice chutney visible on the surface, griddle-toasted with light char marks, stacked on a plate, warm lighting.</t>
+        </is>
+      </c>
+      <c r="H244" t="inlineStr">
+        <is>
+          <t>public/images/recipes/masala-toast/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I244" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="245">
+      <c r="A245" t="n">
+        <v>244</v>
+      </c>
+      <c r="B245" t="inlineStr">
+        <is>
+          <t>Vegetarian</t>
+        </is>
+      </c>
+      <c r="C245" t="inlineStr">
+        <is>
+          <t>tomato-toast</t>
+        </is>
+      </c>
+      <c r="D245" t="inlineStr">
+        <is>
+          <t>Tomato Toast</t>
+        </is>
+      </c>
+      <c r="E245" t="inlineStr">
+        <is>
+          <t>தக்காளி டோஸ்ட்</t>
+        </is>
+      </c>
+      <c r="F245" t="inlineStr">
+        <is>
+          <t>sandwich</t>
+        </is>
+      </c>
+      <c r="G245" t="inlineStr">
+        <is>
+          <t>A photorealistic close-up of a golden-toasted bread slice topped with a glossy reddish-orange cooked tomato-onion masala spread evenly across the surface, slightly caramelized edges, plated hot, warm kitchen lighting.</t>
+        </is>
+      </c>
+      <c r="H245" t="inlineStr">
+        <is>
+          <t>public/images/recipes/tomato-toast/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I245" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="246">
+      <c r="A246" t="n">
+        <v>245</v>
+      </c>
+      <c r="B246" t="inlineStr">
+        <is>
+          <t>Vegetarian</t>
+        </is>
+      </c>
+      <c r="C246" t="inlineStr">
+        <is>
+          <t>potato-sandwich</t>
+        </is>
+      </c>
+      <c r="D246" t="inlineStr">
+        <is>
+          <t>Potato Sandwich</t>
+        </is>
+      </c>
+      <c r="E246" t="inlineStr">
+        <is>
+          <t>உருளைக்கிழங்கு பிரட் சாண்ட்விச்</t>
+        </is>
+      </c>
+      <c r="F246" t="inlineStr">
+        <is>
+          <t>sandwich</t>
+        </is>
+      </c>
+      <c r="G246" t="inlineStr">
+        <is>
+          <t>A photorealistic close-up of a golden-brown griddle-fried sandwich cut diagonally, showing a thick yellow spiced-potato filling coated in crisp bread crumbs between the toasted bread layers, plated with ketchup, bright appetizing lighting.</t>
+        </is>
+      </c>
+      <c r="H246" t="inlineStr">
+        <is>
+          <t>public/images/recipes/potato-sandwich/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I246" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="247">
+      <c r="A247" t="n">
+        <v>246</v>
+      </c>
+      <c r="B247" t="inlineStr">
+        <is>
+          <t>Vegetarian</t>
+        </is>
+      </c>
+      <c r="C247" t="inlineStr">
+        <is>
+          <t>corn-sandwich</t>
+        </is>
+      </c>
+      <c r="D247" t="inlineStr">
+        <is>
+          <t>Corn Sandwich</t>
+        </is>
+      </c>
+      <c r="E247" t="inlineStr">
+        <is>
+          <t>மக்காச்சோள சாண்ட்விச்</t>
+        </is>
+      </c>
+      <c r="F247" t="inlineStr">
+        <is>
+          <t>sandwich</t>
+        </is>
+      </c>
+      <c r="G247" t="inlineStr">
+        <is>
+          <t>A photorealistic photo of an open-faced toast topped with golden corn kernels mixed with cream, and a layer of melted golden cheese bubbling on top, baked and lightly browned, warm oven-fresh lighting.</t>
+        </is>
+      </c>
+      <c r="H247" t="inlineStr">
+        <is>
+          <t>public/images/recipes/corn-sandwich/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I247" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="248">
+      <c r="A248" t="n">
+        <v>247</v>
+      </c>
+      <c r="B248" t="inlineStr">
+        <is>
+          <t>Vegetarian</t>
+        </is>
+      </c>
+      <c r="C248" t="inlineStr">
+        <is>
+          <t>tomato-ketchup</t>
+        </is>
+      </c>
+      <c r="D248" t="inlineStr">
+        <is>
+          <t>Tomato Ketchup</t>
+        </is>
+      </c>
+      <c r="E248" t="inlineStr">
+        <is>
+          <t>தக்காளி கெட்ச்அப்</t>
+        </is>
+      </c>
+      <c r="F248" t="inlineStr">
+        <is>
+          <t>chutney</t>
+        </is>
+      </c>
+      <c r="G248" t="inlineStr">
+        <is>
+          <t>A photorealistic close-up of a clear glass bottle filled with thick, deep-red glossy homemade tomato ketchup, a spoonful pooled beside it on a white plate showing its smooth, thick consistency, bright clean lighting.</t>
+        </is>
+      </c>
+      <c r="H248" t="inlineStr">
+        <is>
+          <t>public/images/recipes/tomato-ketchup/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I248" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="249">
+      <c r="A249" t="n">
+        <v>248</v>
+      </c>
+      <c r="B249" t="inlineStr">
+        <is>
+          <t>Vegetarian</t>
+        </is>
+      </c>
+      <c r="C249" t="inlineStr">
+        <is>
+          <t>vegetable-sandwich</t>
+        </is>
+      </c>
+      <c r="D249" t="inlineStr">
+        <is>
+          <t>Vegetable Sandwich</t>
+        </is>
+      </c>
+      <c r="E249" t="inlineStr">
+        <is>
+          <t>காய்கறி சாண்ட்விச்</t>
+        </is>
+      </c>
+      <c r="F249" t="inlineStr">
+        <is>
+          <t>sandwich</t>
+        </is>
+      </c>
+      <c r="G249" t="inlineStr">
+        <is>
+          <t>A photorealistic close-up of a triangle-cut sandwich showing distinct colorful layers of thin cucumber, carrot, tomato, and onion rounds between green mint-chutney-spread bread, fresh and vibrant, natural bright lighting.</t>
+        </is>
+      </c>
+      <c r="H249" t="inlineStr">
+        <is>
+          <t>public/images/recipes/vegetable-sandwich/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I249" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="250">
+      <c r="A250" t="n">
+        <v>249</v>
+      </c>
+      <c r="B250" t="inlineStr">
+        <is>
+          <t>Vegetarian</t>
+        </is>
+      </c>
+      <c r="C250" t="inlineStr">
+        <is>
+          <t>chilli-cheese-sandwich</t>
+        </is>
+      </c>
+      <c r="D250" t="inlineStr">
+        <is>
+          <t>Chilli Cheese Sandwich</t>
+        </is>
+      </c>
+      <c r="E250" t="inlineStr">
+        <is>
+          <t>சில்லி சீஸ் சாண்ட்விச்</t>
+        </is>
+      </c>
+      <c r="F250" t="inlineStr">
+        <is>
+          <t>sandwich</t>
+        </is>
+      </c>
+      <c r="G250" t="inlineStr">
+        <is>
+          <t>A photorealistic close-up of a golden toasted sandwich cut in half, oozing melted golden cheese mixed with visible flecks of green chili and onion between the crisp bread layers, warm appetizing lighting.</t>
+        </is>
+      </c>
+      <c r="H250" t="inlineStr">
+        <is>
+          <t>public/images/recipes/chilli-cheese-sandwich/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I250" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="251">
+      <c r="A251" t="n">
+        <v>250</v>
+      </c>
+      <c r="B251" t="inlineStr">
+        <is>
+          <t>Vegetarian</t>
+        </is>
+      </c>
+      <c r="C251" t="inlineStr">
+        <is>
+          <t>paneer-sandwich</t>
+        </is>
+      </c>
+      <c r="D251" t="inlineStr">
+        <is>
+          <t>Paneer Sandwich</t>
+        </is>
+      </c>
+      <c r="E251" t="inlineStr">
+        <is>
+          <t>பாலாடைக்கட்டி சாண்ட்விச்</t>
+        </is>
+      </c>
+      <c r="F251" t="inlineStr">
+        <is>
+          <t>sandwich</t>
+        </is>
+      </c>
+      <c r="G251" t="inlineStr">
+        <is>
+          <t>A photorealistic close-up of a golden toasted sandwich cut diagonally, showing a crumbly white paneer filling studded with green sprouts and herbs between the bread layers, plated with ketchup, bright lighting.</t>
+        </is>
+      </c>
+      <c r="H251" t="inlineStr">
+        <is>
+          <t>public/images/recipes/paneer-sandwich/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I251" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="252">
+      <c r="A252" t="n">
+        <v>251</v>
+      </c>
+      <c r="B252" t="inlineStr">
+        <is>
+          <t>Vegetarian</t>
+        </is>
+      </c>
+      <c r="C252" t="inlineStr">
+        <is>
+          <t>sandwich-roll</t>
+        </is>
+      </c>
+      <c r="D252" t="inlineStr">
+        <is>
+          <t>Sandwich Roll</t>
+        </is>
+      </c>
+      <c r="E252" t="inlineStr">
+        <is>
+          <t>சாண்ட்விட்ச் ரோல்</t>
+        </is>
+      </c>
+      <c r="F252" t="inlineStr">
+        <is>
+          <t>sandwich</t>
+        </is>
+      </c>
+      <c r="G252" t="inlineStr">
+        <is>
+          <t>A photorealistic close-up of pinwheel-shaped bread roll slices arranged on a plate, showing a spiral of white bread with thin green and red chutney swirls visible in the layers, elegant party-platter presentation, bright clean lighting.</t>
+        </is>
+      </c>
+      <c r="H252" t="inlineStr">
+        <is>
+          <t>public/images/recipes/sandwich-roll/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I252" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="253">
+      <c r="A253" t="n">
+        <v>252</v>
+      </c>
+      <c r="B253" t="inlineStr">
+        <is>
+          <t>Vegetarian</t>
+        </is>
+      </c>
+      <c r="C253" t="inlineStr">
+        <is>
+          <t>aloo-chat-1</t>
+        </is>
+      </c>
+      <c r="D253" t="inlineStr">
+        <is>
+          <t>Aloo Chat 1</t>
+        </is>
+      </c>
+      <c r="E253" t="inlineStr">
+        <is>
+          <t>ஆலு சாட் - 1</t>
+        </is>
+      </c>
+      <c r="F253" t="inlineStr">
+        <is>
+          <t>chaat</t>
+        </is>
+      </c>
+      <c r="G253" t="inlineStr">
+        <is>
+          <t>A photorealistic close-up of a boiled potato stuffed and topped generously with white whisked curd, drizzled with dark brown tangy tamarind sauce, dusted with red chili powder and dark chat masala, garnished with coriander leaves, served on a decorative plate, vibrant street-food lighting.</t>
+        </is>
+      </c>
+      <c r="H253" t="inlineStr">
+        <is>
+          <t>public/images/recipes/aloo-chat-1/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I253" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="254">
+      <c r="A254" t="n">
+        <v>253</v>
+      </c>
+      <c r="B254" t="inlineStr">
+        <is>
+          <t>Vegetarian</t>
+        </is>
+      </c>
+      <c r="C254" t="inlineStr">
+        <is>
+          <t>aloo-chat-2</t>
+        </is>
+      </c>
+      <c r="D254" t="inlineStr">
+        <is>
+          <t>Aloo Chat 2</t>
+        </is>
+      </c>
+      <c r="E254" t="inlineStr">
+        <is>
+          <t>ஆலு சாட் - 2</t>
+        </is>
+      </c>
+      <c r="F254" t="inlineStr">
+        <is>
+          <t>chaat</t>
+        </is>
+      </c>
+      <c r="G254" t="inlineStr">
+        <is>
+          <t>A photorealistic photo of diced potato mixed with golden fried diamond-shaped crisps, tossed in a chat bowl with dark tangy sauce, chopped onion, and a scattering of thin crispy sev on top, colorful street-food presentation, bright lighting.</t>
+        </is>
+      </c>
+      <c r="H254" t="inlineStr">
+        <is>
+          <t>public/images/recipes/aloo-chat-2/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I254" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="255">
+      <c r="A255" t="n">
+        <v>254</v>
+      </c>
+      <c r="B255" t="inlineStr">
+        <is>
+          <t>Vegetarian</t>
+        </is>
+      </c>
+      <c r="C255" t="inlineStr">
+        <is>
+          <t>chat-masala-powder</t>
+        </is>
+      </c>
+      <c r="D255" t="inlineStr">
+        <is>
+          <t>Chat Masala Powder</t>
+        </is>
+      </c>
+      <c r="E255" t="inlineStr">
+        <is>
+          <t>சாட் மசாலா பவுடர்</t>
+        </is>
+      </c>
+      <c r="F255" t="inlineStr">
+        <is>
+          <t>chaat</t>
+        </is>
+      </c>
+      <c r="G255" t="inlineStr">
+        <is>
+          <t>A photorealistic close-up of a small glass jar filled with reddish-brown aromatic spice powder, a small mound of the powder spilled beside it on a wooden surface with whole dried red chilies and cardamom pods scattered around, warm spice-market lighting.</t>
+        </is>
+      </c>
+      <c r="H255" t="inlineStr">
+        <is>
+          <t>public/images/recipes/chat-masala-powder/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I255" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="256">
+      <c r="A256" t="n">
+        <v>255</v>
+      </c>
+      <c r="B256" t="inlineStr">
+        <is>
+          <t>Vegetarian</t>
+        </is>
+      </c>
+      <c r="C256" t="inlineStr">
+        <is>
+          <t>aloo-pappad-chat</t>
+        </is>
+      </c>
+      <c r="D256" t="inlineStr">
+        <is>
+          <t>Aloo Pappad Chat</t>
+        </is>
+      </c>
+      <c r="E256" t="inlineStr">
+        <is>
+          <t>ஆலு பப்பட் சாட்</t>
+        </is>
+      </c>
+      <c r="F256" t="inlineStr">
+        <is>
+          <t>chaat</t>
+        </is>
+      </c>
+      <c r="G256" t="inlineStr">
+        <is>
+          <t>A photorealistic close-up of a plate layered with crushed golden fried papad pieces, topped with diced potato, a generous pour of white curd, dark brown sweet chutney drizzle, and a dusting of spices with fresh coriander on top, vibrant street-food lighting.</t>
+        </is>
+      </c>
+      <c r="H256" t="inlineStr">
+        <is>
+          <t>public/images/recipes/aloo-pappad-chat/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I256" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="257">
+      <c r="A257" t="n">
+        <v>256</v>
+      </c>
+      <c r="B257" t="inlineStr">
+        <is>
+          <t>Vegetarian</t>
+        </is>
+      </c>
+      <c r="C257" t="inlineStr">
+        <is>
+          <t>mattar-chat</t>
+        </is>
+      </c>
+      <c r="D257" t="inlineStr">
+        <is>
+          <t>Mattar Chat</t>
+        </is>
+      </c>
+      <c r="E257" t="inlineStr">
+        <is>
+          <t>பச்சைப் பட்டாணி சாட்</t>
+        </is>
+      </c>
+      <c r="F257" t="inlineStr">
+        <is>
+          <t>chaat</t>
+        </is>
+      </c>
+      <c r="G257" t="inlineStr">
+        <is>
+          <t>A photorealistic close-up of a bowl of cooked green peas topped with crushed golden puri pieces, white curd, dark tamarind chutney, chopped onion, and fine crispy sev, colorful layered presentation, bright lighting.</t>
+        </is>
+      </c>
+      <c r="H257" t="inlineStr">
+        <is>
+          <t>public/images/recipes/mattar-chat/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I257" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="258">
+      <c r="A258" t="n">
+        <v>257</v>
+      </c>
+      <c r="B258" t="inlineStr">
+        <is>
+          <t>Vegetarian</t>
+        </is>
+      </c>
+      <c r="C258" t="inlineStr">
+        <is>
+          <t>fruit-vegetable-chat</t>
+        </is>
+      </c>
+      <c r="D258" t="inlineStr">
+        <is>
+          <t>Fruit &amp; Vegetable Chat</t>
+        </is>
+      </c>
+      <c r="E258" t="inlineStr">
+        <is>
+          <t>காய்கறி, பழக்கலவை சாட்</t>
+        </is>
+      </c>
+      <c r="F258" t="inlineStr">
+        <is>
+          <t>chaat</t>
+        </is>
+      </c>
+      <c r="G258" t="inlineStr">
+        <is>
+          <t>A photorealistic photo of a colorful bowl mix of diced banana, orange segments, tomato, potato, and guava tossed together, garnished with coriander leaves and a light dusting of chat masala, fresh and vibrant, bright natural lighting.</t>
+        </is>
+      </c>
+      <c r="H258" t="inlineStr">
+        <is>
+          <t>public/images/recipes/fruit-vegetable-chat/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I258" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="259">
+      <c r="A259" t="n">
+        <v>258</v>
+      </c>
+      <c r="B259" t="inlineStr">
+        <is>
+          <t>Vegetarian</t>
+        </is>
+      </c>
+      <c r="C259" t="inlineStr">
+        <is>
+          <t>finger-chips</t>
+        </is>
+      </c>
+      <c r="D259" t="inlineStr">
+        <is>
+          <t>Finger Chips</t>
+        </is>
+      </c>
+      <c r="E259" t="inlineStr">
+        <is>
+          <t>ஃபிங்கர் சிப்ஸ்</t>
+        </is>
+      </c>
+      <c r="F259" t="inlineStr">
+        <is>
+          <t>snack</t>
+        </is>
+      </c>
+      <c r="G259" t="inlineStr">
+        <is>
+          <t>A photorealistic close-up of golden-brown crispy potato finger chips piled high on a plate, lightly dusted with salt and pepper, served with tomato ketchup, bright appetizing lighting.</t>
+        </is>
+      </c>
+      <c r="H259" t="inlineStr">
+        <is>
+          <t>public/images/recipes/finger-chips/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I259" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="260">
+      <c r="A260" t="n">
+        <v>259</v>
+      </c>
+      <c r="B260" t="inlineStr">
+        <is>
+          <t>Vegetarian</t>
+        </is>
+      </c>
+      <c r="C260" t="inlineStr">
+        <is>
+          <t>crisp-groundnuts</t>
+        </is>
+      </c>
+      <c r="D260" t="inlineStr">
+        <is>
+          <t>Crisp Groundnuts</t>
+        </is>
+      </c>
+      <c r="E260" t="inlineStr">
+        <is>
+          <t>வறுகடலை</t>
+        </is>
+      </c>
+      <c r="F260" t="inlineStr">
+        <is>
+          <t>snack</t>
+        </is>
+      </c>
+      <c r="G260" t="inlineStr">
+        <is>
+          <t>A photorealistic close-up of small glossy, deep golden-brown fried groundnuts piled in a bowl, with a visible shiny sheen, some scattered on a napkin, warm snack-time lighting.</t>
+        </is>
+      </c>
+      <c r="H260" t="inlineStr">
+        <is>
+          <t>public/images/recipes/crisp-groundnuts/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I260" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="261">
+      <c r="A261" t="n">
+        <v>260</v>
+      </c>
+      <c r="B261" t="inlineStr">
+        <is>
+          <t>Vegetarian</t>
+        </is>
+      </c>
+      <c r="C261" t="inlineStr">
+        <is>
+          <t>pop-corn</t>
+        </is>
+      </c>
+      <c r="D261" t="inlineStr">
+        <is>
+          <t>Pop Corn</t>
+        </is>
+      </c>
+      <c r="E261" t="inlineStr">
+        <is>
+          <t>பாப் கார்ன்</t>
+        </is>
+      </c>
+      <c r="F261" t="inlineStr">
+        <is>
+          <t>snack</t>
+        </is>
+      </c>
+      <c r="G261" t="inlineStr">
+        <is>
+          <t>A photorealistic close-up of a bowl overflowing with fluffy white popcorn lightly dusted with orange-red spice seasoning, warm cozy lighting.</t>
+        </is>
+      </c>
+      <c r="H261" t="inlineStr">
+        <is>
+          <t>public/images/recipes/pop-corn/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I261" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="262">
+      <c r="A262" t="n">
+        <v>261</v>
+      </c>
+      <c r="B262" t="inlineStr">
+        <is>
+          <t>Vegetarian</t>
+        </is>
+      </c>
+      <c r="C262" t="inlineStr">
+        <is>
+          <t>masala-pori-1</t>
+        </is>
+      </c>
+      <c r="D262" t="inlineStr">
+        <is>
+          <t>Masala Pori 1 (Instant Bhel)</t>
+        </is>
+      </c>
+      <c r="E262" t="inlineStr">
+        <is>
+          <t>மசாலா பொரி - 1</t>
+        </is>
+      </c>
+      <c r="F262" t="inlineStr">
+        <is>
+          <t>chaat</t>
+        </is>
+      </c>
+      <c r="G262" t="inlineStr">
+        <is>
+          <t>A photorealistic photo of a colorful bowl of puffed rice mixed with roasted gram, small dice of mango, tomato, carrot, and beetroot, garnished with coriander leaves, bright vibrant street-food lighting.</t>
+        </is>
+      </c>
+      <c r="H262" t="inlineStr">
+        <is>
+          <t>public/images/recipes/masala-pori-1/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I262" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="263">
+      <c r="A263" t="n">
+        <v>262</v>
+      </c>
+      <c r="B263" t="inlineStr">
+        <is>
+          <t>Vegetarian</t>
+        </is>
+      </c>
+      <c r="C263" t="inlineStr">
+        <is>
+          <t>masala-pori-2</t>
+        </is>
+      </c>
+      <c r="D263" t="inlineStr">
+        <is>
+          <t>Masala Pori 2 (Instant Bhel)</t>
+        </is>
+      </c>
+      <c r="E263" t="inlineStr">
+        <is>
+          <t>மசாலா பொரி - 2</t>
+        </is>
+      </c>
+      <c r="F263" t="inlineStr">
+        <is>
+          <t>chaat</t>
+        </is>
+      </c>
+      <c r="G263" t="inlineStr">
+        <is>
+          <t>A photorealistic photo of a bowl of puffed rice mixed with roasted gram and groundnuts, tossed with pink-tinged marinated onion and a drizzle of dark green chutney, colorful and fresh, bright lighting.</t>
+        </is>
+      </c>
+      <c r="H263" t="inlineStr">
+        <is>
+          <t>public/images/recipes/masala-pori-2/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I263" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="264">
+      <c r="A264" t="n">
+        <v>263</v>
+      </c>
+      <c r="B264" t="inlineStr">
+        <is>
+          <t>Vegetarian</t>
+        </is>
+      </c>
+      <c r="C264" t="inlineStr">
+        <is>
+          <t>mint-coriander-chutney-cutlets</t>
+        </is>
+      </c>
+      <c r="D264" t="inlineStr">
+        <is>
+          <t>Mint-Coriander Chutney (for Cutlets)</t>
+        </is>
+      </c>
+      <c r="E264" t="inlineStr">
+        <is>
+          <t>புதினா, கொத்தமல்லி சட்னி (கட்லெட்டிற்கு)</t>
+        </is>
+      </c>
+      <c r="F264" t="inlineStr">
+        <is>
+          <t>chutney</t>
+        </is>
+      </c>
+      <c r="G264" t="inlineStr">
+        <is>
+          <t>A photorealistic close-up of a small bowl of smooth, vivid green chutney with a glossy sheen, served beside golden fried cutlets, garnished with a mint sprig, bright fresh lighting.</t>
+        </is>
+      </c>
+      <c r="H264" t="inlineStr">
+        <is>
+          <t>public/images/recipes/mint-coriander-chutney-cutlets/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I264" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="265">
+      <c r="A265" t="n">
+        <v>264</v>
+      </c>
+      <c r="B265" t="inlineStr">
+        <is>
+          <t>Vegetarian</t>
+        </is>
+      </c>
+      <c r="C265" t="inlineStr">
+        <is>
+          <t>mint-chutney-cutlets</t>
+        </is>
+      </c>
+      <c r="D265" t="inlineStr">
+        <is>
+          <t>Mint Chutney (for Cutlets)</t>
+        </is>
+      </c>
+      <c r="E265" t="inlineStr">
+        <is>
+          <t>புதினா சட்னி (கட்லெட்டிற்கு)</t>
+        </is>
+      </c>
+      <c r="F265" t="inlineStr">
+        <is>
+          <t>chutney</t>
+        </is>
+      </c>
+      <c r="G265" t="inlineStr">
+        <is>
+          <t>A photorealistic close-up of a small bowl of dark green, thick chutney with a tempered mustard-seed garnish floating on top, bright natural lighting.</t>
+        </is>
+      </c>
+      <c r="H265" t="inlineStr">
+        <is>
+          <t>public/images/recipes/mint-chutney-cutlets/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I265" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="266">
+      <c r="A266" t="n">
+        <v>265</v>
+      </c>
+      <c r="B266" t="inlineStr">
+        <is>
+          <t>Vegetarian</t>
+        </is>
+      </c>
+      <c r="C266" t="inlineStr">
+        <is>
+          <t>mint-onion-chutney</t>
+        </is>
+      </c>
+      <c r="D266" t="inlineStr">
+        <is>
+          <t>Mint-Onion Chutney</t>
+        </is>
+      </c>
+      <c r="E266" t="inlineStr">
+        <is>
+          <t>புதினா வெங்காயச் சட்னி</t>
+        </is>
+      </c>
+      <c r="F266" t="inlineStr">
+        <is>
+          <t>chutney</t>
+        </is>
+      </c>
+      <c r="G266" t="inlineStr">
+        <is>
+          <t>A photorealistic close-up of a bowl of textured dark green chutney flecked with white coconut, garnished with a tempering of mustard seeds and curry leaves on top, warm lighting.</t>
+        </is>
+      </c>
+      <c r="H266" t="inlineStr">
+        <is>
+          <t>public/images/recipes/mint-onion-chutney/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I266" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="267">
+      <c r="A267" t="n">
+        <v>266</v>
+      </c>
+      <c r="B267" t="inlineStr">
+        <is>
+          <t>Vegetarian</t>
+        </is>
+      </c>
+      <c r="C267" t="inlineStr">
+        <is>
+          <t>coriander-chutney-sandwiches</t>
+        </is>
+      </c>
+      <c r="D267" t="inlineStr">
+        <is>
+          <t>Coriander Chutney (for Sandwiches)</t>
+        </is>
+      </c>
+      <c r="E267" t="inlineStr">
+        <is>
+          <t>கொத்தமல்லி சட்னி (சாண்ட்விச்சிற்கு)</t>
+        </is>
+      </c>
+      <c r="F267" t="inlineStr">
+        <is>
+          <t>chutney</t>
+        </is>
+      </c>
+      <c r="G267" t="inlineStr">
+        <is>
+          <t>A photorealistic close-up of a small bowl of deep green-red chutney with a thick, spreadable texture, a butter knife resting beside it with chutney on the blade, bright kitchen lighting.</t>
+        </is>
+      </c>
+      <c r="H267" t="inlineStr">
+        <is>
+          <t>public/images/recipes/coriander-chutney-sandwiches/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I267" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="268">
+      <c r="A268" t="n">
+        <v>267</v>
+      </c>
+      <c r="B268" t="inlineStr">
+        <is>
+          <t>Vegetarian</t>
+        </is>
+      </c>
+      <c r="C268" t="inlineStr">
+        <is>
+          <t>garlic-chutney-sandwiches</t>
+        </is>
+      </c>
+      <c r="D268" t="inlineStr">
+        <is>
+          <t>Garlic Chutney (for Sandwiches)</t>
+        </is>
+      </c>
+      <c r="E268" t="inlineStr">
+        <is>
+          <t>பூண்டு சட்னி (சாண்ட்விச்சிற்கு)</t>
+        </is>
+      </c>
+      <c r="F268" t="inlineStr">
+        <is>
+          <t>chutney</t>
+        </is>
+      </c>
+      <c r="G268" t="inlineStr">
+        <is>
+          <t>A photorealistic close-up of a bowl of reddish-brown chutney with visible garlic and chili flecks, thick and glossy, served beside buttered bread slices, warm lighting.</t>
+        </is>
+      </c>
+      <c r="H268" t="inlineStr">
+        <is>
+          <t>public/images/recipes/garlic-chutney-sandwiches/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I268" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="269">
+      <c r="A269" t="n">
+        <v>268</v>
+      </c>
+      <c r="B269" t="inlineStr">
+        <is>
+          <t>Vegetarian</t>
+        </is>
+      </c>
+      <c r="C269" t="inlineStr">
+        <is>
+          <t>coconut-ginger-chutney-sandwiches</t>
+        </is>
+      </c>
+      <c r="D269" t="inlineStr">
+        <is>
+          <t>Coconut-Ginger Chutney (for Sandwiches)</t>
+        </is>
+      </c>
+      <c r="E269" t="inlineStr">
+        <is>
+          <t>தேங்காய், இஞ்சி சட்னி (சாண்ட்விச்சிற்கு)</t>
+        </is>
+      </c>
+      <c r="F269" t="inlineStr">
+        <is>
+          <t>chutney</t>
+        </is>
+      </c>
+      <c r="G269" t="inlineStr">
+        <is>
+          <t>A photorealistic close-up of a bowl of coarse, off-white coconut chutney with visible ginger and red chili flecks, glossy texture, natural bright lighting.</t>
+        </is>
+      </c>
+      <c r="H269" t="inlineStr">
+        <is>
+          <t>public/images/recipes/coconut-ginger-chutney-sandwiches/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I269" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="270">
+      <c r="A270" t="n">
+        <v>269</v>
+      </c>
+      <c r="B270" t="inlineStr">
+        <is>
+          <t>Vegetarian</t>
+        </is>
+      </c>
+      <c r="C270" t="inlineStr">
+        <is>
+          <t>mint-chutney-sandwiches</t>
+        </is>
+      </c>
+      <c r="D270" t="inlineStr">
+        <is>
+          <t>Mint Chutney (for Sandwiches)</t>
+        </is>
+      </c>
+      <c r="E270" t="inlineStr">
+        <is>
+          <t>புதினா சட்னி (சாண்ட்விச்சிற்கு)</t>
+        </is>
+      </c>
+      <c r="F270" t="inlineStr">
+        <is>
+          <t>chutney</t>
+        </is>
+      </c>
+      <c r="G270" t="inlineStr">
+        <is>
+          <t>A photorealistic close-up of a small bowl of smooth bright green mint chutney, glossy sheen, served beside a stack of white bread slices, fresh vibrant lighting.</t>
+        </is>
+      </c>
+      <c r="H270" t="inlineStr">
+        <is>
+          <t>public/images/recipes/mint-chutney-sandwiches/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I270" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="271">
+      <c r="A271" t="n">
+        <v>270</v>
+      </c>
+      <c r="B271" t="inlineStr">
+        <is>
+          <t>Vegetarian</t>
+        </is>
+      </c>
+      <c r="C271" t="inlineStr">
+        <is>
+          <t>onion-bajji</t>
+        </is>
+      </c>
+      <c r="D271" t="inlineStr">
+        <is>
+          <t>Onion Bajji</t>
+        </is>
+      </c>
+      <c r="E271" t="inlineStr">
+        <is>
+          <t>வெங்காயப் பஜ்ஜி</t>
+        </is>
+      </c>
+      <c r="F271" t="inlineStr">
+        <is>
+          <t>bajji</t>
+        </is>
+      </c>
+      <c r="G271" t="inlineStr">
+        <is>
+          <t>A photorealistic close-up of golden fried onion bajjis with a distinctive ring-shaped, batter-coated onion visible inside the crisp fried coating, piled on a plate, served with coconut chutney, warm tea-stall lighting.</t>
+        </is>
+      </c>
+      <c r="H271" t="inlineStr">
+        <is>
+          <t>public/images/recipes/onion-bajji/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I271" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="272">
+      <c r="A272" t="n">
+        <v>271</v>
+      </c>
+      <c r="B272" t="inlineStr">
+        <is>
+          <t>Vegetarian</t>
+        </is>
+      </c>
+      <c r="C272" t="inlineStr">
+        <is>
+          <t>vendaikkai-pakoda</t>
+        </is>
+      </c>
+      <c r="D272" t="inlineStr">
+        <is>
+          <t>Deep Fried Ladies Fingers</t>
+        </is>
+      </c>
+      <c r="E272" t="inlineStr">
+        <is>
+          <t>வெண்டைக்காய் பக்கோடா</t>
+        </is>
+      </c>
+      <c r="F272" t="inlineStr">
+        <is>
+          <t>bajji</t>
+        </is>
+      </c>
+      <c r="G272" t="inlineStr">
+        <is>
+          <t>A photorealistic close-up of whole okra pieces coated in a crisp golden fried batter with visible bread-crumb texture, arranged on a plate with tomato sauce, natural daylight.</t>
+        </is>
+      </c>
+      <c r="H272" t="inlineStr">
+        <is>
+          <t>public/images/recipes/vendaikkai-pakoda/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I272" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="273">
+      <c r="A273" t="n">
+        <v>272</v>
+      </c>
+      <c r="B273" t="inlineStr">
+        <is>
+          <t>Vegetarian</t>
+        </is>
+      </c>
+      <c r="C273" t="inlineStr">
+        <is>
+          <t>carrot-sandwich</t>
+        </is>
+      </c>
+      <c r="D273" t="inlineStr">
+        <is>
+          <t>Carrot Sandwich</t>
+        </is>
+      </c>
+      <c r="E273" t="inlineStr">
+        <is>
+          <t>கேரட் சாண்ட்விச்</t>
+        </is>
+      </c>
+      <c r="F273" t="inlineStr">
+        <is>
+          <t>sandwich</t>
+        </is>
+      </c>
+      <c r="G273" t="inlineStr">
+        <is>
+          <t>A photorealistic close-up of a pressed golden-toasted sandwich cut in half, showing a bright orange sauteed carrot-tomato filling between the bread layers, plated with tomato sauce, warm appetizing lighting.</t>
+        </is>
+      </c>
+      <c r="H273" t="inlineStr">
+        <is>
+          <t>public/images/recipes/carrot-sandwich/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I273" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="274">
+      <c r="A274" t="n">
+        <v>273</v>
+      </c>
+      <c r="B274" t="inlineStr">
+        <is>
+          <t>Vegetarian Cooking Tips - Gap Fill</t>
+        </is>
+      </c>
+      <c r="C274" t="inlineStr">
+        <is>
+          <t>egg-dosai</t>
+        </is>
+      </c>
+      <c r="D274" t="inlineStr">
+        <is>
+          <t>Egg Dosai</t>
+        </is>
+      </c>
+      <c r="E274" t="inlineStr">
+        <is>
+          <t>முட்டைத் தோசை</t>
+        </is>
+      </c>
+      <c r="F274" t="inlineStr">
+        <is>
+          <t>dosa</t>
+        </is>
+      </c>
+      <c r="G274" t="inlineStr">
+        <is>
+          <t>A close-up photorealistic food photo of a thin, golden-brown crepe-like dosa on a black stone griddle, a thin layer of beaten egg cooked into its surface giving it a mottled yellow-and-brown speckled texture, folded in half on a steel plate, a wedge of onion and a small bowl of coconut chutney beside it, warm kitchen lighting, shallow depth of field.</t>
+        </is>
+      </c>
+      <c r="H274" t="inlineStr">
+        <is>
+          <t>public/images/recipes/egg-dosai/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I274" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="275">
+      <c r="A275" t="n">
+        <v>274</v>
+      </c>
+      <c r="B275" t="inlineStr">
+        <is>
+          <t>Vegetarian Cooking Tips - Gap Fill</t>
+        </is>
+      </c>
+      <c r="C275" t="inlineStr">
+        <is>
+          <t>masala-idli</t>
+        </is>
+      </c>
+      <c r="D275" t="inlineStr">
+        <is>
+          <t>Masala Idli</t>
+        </is>
+      </c>
+      <c r="E275" t="inlineStr">
+        <is>
+          <t>மசாலா இட்லி</t>
+        </is>
+      </c>
+      <c r="F275" t="inlineStr">
+        <is>
+          <t>idli</t>
+        </is>
+      </c>
+      <c r="G275" t="inlineStr">
+        <is>
+          <t>A close-up photorealistic food photo of a soft white idli cut in half on a steel plate, revealing a spiced reddish-orange vegetable filling layered through its center, steam rising gently, a small bowl of sambar and coconut chutney alongside, natural morning light.</t>
+        </is>
+      </c>
+      <c r="H275" t="inlineStr">
+        <is>
+          <t>public/images/recipes/masala-idli/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I275" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="276">
+      <c r="A276" t="n">
+        <v>275</v>
+      </c>
+      <c r="B276" t="inlineStr">
+        <is>
+          <t>Vegetarian Cooking Tips - Gap Fill</t>
+        </is>
+      </c>
+      <c r="C276" t="inlineStr">
+        <is>
+          <t>vegetable-sambar</t>
+        </is>
+      </c>
+      <c r="D276" t="inlineStr">
+        <is>
+          <t>Vegetable Sambar</t>
+        </is>
+      </c>
+      <c r="E276" t="inlineStr">
+        <is>
+          <t>காய்கறி சாம்பார்</t>
+        </is>
+      </c>
+      <c r="F276" t="inlineStr">
+        <is>
+          <t>sambar</t>
+        </is>
+      </c>
+      <c r="G276" t="inlineStr">
+        <is>
+          <t>A close-up photorealistic food photo of steaming orange-yellow vegetable sambar in a steel bowl, chunks of drumstick and brinjal visible in the thick lentil gravy, a mustard-and-curry-leaf tempering glistening on top, garnished with fresh coriander leaves, warm natural lighting.</t>
+        </is>
+      </c>
+      <c r="H276" t="inlineStr">
+        <is>
+          <t>public/images/recipes/vegetable-sambar/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I276" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="277">
+      <c r="A277" t="n">
+        <v>276</v>
+      </c>
+      <c r="B277" t="inlineStr">
+        <is>
+          <t>Vegetarian Cooking Tips - Gap Fill</t>
+        </is>
+      </c>
+      <c r="C277" t="inlineStr">
+        <is>
+          <t>idiyappam</t>
+        </is>
+      </c>
+      <c r="D277" t="inlineStr">
+        <is>
+          <t>Idiyappam (String Hoppers)</t>
+        </is>
+      </c>
+      <c r="E277" t="inlineStr">
+        <is>
+          <t>இடியாப்பம்</t>
+        </is>
+      </c>
+      <c r="F277" t="inlineStr">
+        <is>
+          <t>steamed-tiffin</t>
+        </is>
+      </c>
+      <c r="G277" t="inlineStr">
+        <is>
+          <t>A close-up photorealistic food photo of a neat coiled disc of thin white rice-flour string hoppers on a banana leaf, delicate steamed strands visible, served beside a small bowl of coconut milk and a wedge of lime, soft natural daylight, shallow depth of field.</t>
+        </is>
+      </c>
+      <c r="H277" t="inlineStr">
+        <is>
+          <t>public/images/recipes/idiyappam/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I277" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="278">
+      <c r="A278" t="n">
+        <v>277</v>
+      </c>
+      <c r="B278" t="inlineStr">
+        <is>
+          <t>Vegetarian Cooking Tips - Gap Fill</t>
+        </is>
+      </c>
+      <c r="C278" t="inlineStr">
+        <is>
+          <t>sweet-appam</t>
+        </is>
+      </c>
+      <c r="D278" t="inlineStr">
+        <is>
+          <t>Sweet Appam</t>
+        </is>
+      </c>
+      <c r="E278" t="inlineStr">
+        <is>
+          <t>இனிப்பு ஆப்பம்</t>
+        </is>
+      </c>
+      <c r="F278" t="inlineStr">
+        <is>
+          <t>steamed-tiffin, sweet</t>
+        </is>
+      </c>
+      <c r="G278" t="inlineStr">
+        <is>
+          <t>A close-up photorealistic food photo of a golden-brown bowl-shaped appam with a thick spongy center and lacy crisp edges, resting on a steel plate, its jaggery-sweetened surface glistening slightly, warm kitchen lighting, shallow depth of field.</t>
+        </is>
+      </c>
+      <c r="H278" t="inlineStr">
+        <is>
+          <t>public/images/recipes/sweet-appam/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I278" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="279">
+      <c r="A279" t="n">
+        <v>278</v>
+      </c>
+      <c r="B279" t="inlineStr">
+        <is>
+          <t>Vegetarian Cooking Tips - Gap Fill</t>
+        </is>
+      </c>
+      <c r="C279" t="inlineStr">
+        <is>
+          <t>chapati</t>
+        </is>
+      </c>
+      <c r="D279" t="inlineStr">
+        <is>
+          <t>Chapati</t>
+        </is>
+      </c>
+      <c r="E279" t="inlineStr">
+        <is>
+          <t>சப்பாத்தி</t>
+        </is>
+      </c>
+      <c r="F279" t="inlineStr">
+        <is>
+          <t>flatbread</t>
+        </is>
+      </c>
+      <c r="G279" t="inlineStr">
+        <is>
+          <t>A close-up photorealistic food photo of a puffed, golden-brown round chapati fresh off the griddle, a light sheen of ghee brushed on top, stacked slightly with one leaning against the pile on a steel plate, warm kitchen lighting.</t>
+        </is>
+      </c>
+      <c r="H279" t="inlineStr">
+        <is>
+          <t>public/images/recipes/chapati/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I279" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="280">
+      <c r="A280" t="n">
+        <v>279</v>
+      </c>
+      <c r="B280" t="inlineStr">
+        <is>
+          <t>Vegetarian Cooking Tips - Gap Fill</t>
+        </is>
+      </c>
+      <c r="C280" t="inlineStr">
+        <is>
+          <t>patrora</t>
+        </is>
+      </c>
+      <c r="D280" t="inlineStr">
+        <is>
+          <t>Patrora (or Curd Poori)</t>
+        </is>
+      </c>
+      <c r="E280" t="inlineStr">
+        <is>
+          <t>பட்ரோரா (அல்லது) தயிர் பூரி</t>
+        </is>
+      </c>
+      <c r="F280" t="inlineStr">
+        <is>
+          <t>fried-bread</t>
+        </is>
+      </c>
+      <c r="G280" t="inlineStr">
+        <is>
+          <t>A close-up photorealistic food photo of a thick, golden-brown deep-fried round bread with a slightly puffed naan-like texture, served on a steel plate with a side of chana masala gravy, warm kitchen lighting, shallow depth of field.</t>
+        </is>
+      </c>
+      <c r="H280" t="inlineStr">
+        <is>
+          <t>public/images/recipes/patrora/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I280" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="281">
+      <c r="A281" t="n">
+        <v>280</v>
+      </c>
+      <c r="B281" t="inlineStr">
+        <is>
+          <t>Vegetarian Cooking Tips - Gap Fill</t>
+        </is>
+      </c>
+      <c r="C281" t="inlineStr">
+        <is>
+          <t>tomato-kurma</t>
+        </is>
+      </c>
+      <c r="D281" t="inlineStr">
+        <is>
+          <t>Tomato Kurma</t>
+        </is>
+      </c>
+      <c r="E281" t="inlineStr">
+        <is>
+          <t>தக்காளி குருமா</t>
+        </is>
+      </c>
+      <c r="F281" t="inlineStr">
+        <is>
+          <t>kuzhambu</t>
+        </is>
+      </c>
+      <c r="G281" t="inlineStr">
+        <is>
+          <t>A close-up photorealistic food photo of a thick reddish-orange tomato kurma gravy in a steel bowl, chunks of potato visible in the glossy sauce, garnished with fresh coriander leaves, warm natural lighting, shallow depth of field.</t>
+        </is>
+      </c>
+      <c r="H281" t="inlineStr">
+        <is>
+          <t>public/images/recipes/tomato-kurma/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I281" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="282">
+      <c r="A282" t="n">
+        <v>281</v>
+      </c>
+      <c r="B282" t="inlineStr">
+        <is>
+          <t>Vegetarian Cooking Tips - Gap Fill</t>
+        </is>
+      </c>
+      <c r="C282" t="inlineStr">
+        <is>
+          <t>kathirikkai-kosu</t>
+        </is>
+      </c>
+      <c r="D282" t="inlineStr">
+        <is>
+          <t>Kathirikkai Kosu (Brinjal Kosu)</t>
+        </is>
+      </c>
+      <c r="E282" t="inlineStr">
+        <is>
+          <t>கத்தரிக்காய் கொச்சு</t>
+        </is>
+      </c>
+      <c r="F282" t="inlineStr">
+        <is>
+          <t>kuzhambu</t>
+        </is>
+      </c>
+      <c r="G282" t="inlineStr">
+        <is>
+          <t>A close-up photorealistic food photo of a dark reddish-brown mashed brinjal side dish in a small steel bowl, thick and glossy with visible flecks of tempered mustard seeds, served beside plain rice, warm natural lighting.</t>
+        </is>
+      </c>
+      <c r="H282" t="inlineStr">
+        <is>
+          <t>public/images/recipes/kathirikkai-kosu/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I282" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="283">
+      <c r="A283" t="n">
+        <v>282</v>
+      </c>
+      <c r="B283" t="inlineStr">
+        <is>
+          <t>Vegetarian Cooking Tips - Gap Fill</t>
+        </is>
+      </c>
+      <c r="C283" t="inlineStr">
+        <is>
+          <t>masala-sundal</t>
+        </is>
+      </c>
+      <c r="D283" t="inlineStr">
+        <is>
+          <t>Masala Sundal</t>
+        </is>
+      </c>
+      <c r="E283" t="inlineStr">
+        <is>
+          <t>மசால் சுண்டல்</t>
+        </is>
+      </c>
+      <c r="F283" t="inlineStr">
+        <is>
+          <t>sundal</t>
+        </is>
+      </c>
+      <c r="G283" t="inlineStr">
+        <is>
+          <t>A close-up photorealistic food photo of a bowl of golden-brown spiced chickpea sundal, garnished generously with grated coconut and chopped coriander leaves, curry leaves visible throughout, natural daylight, shallow depth of field.</t>
+        </is>
+      </c>
+      <c r="H283" t="inlineStr">
+        <is>
+          <t>public/images/recipes/masala-sundal/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I283" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="284">
+      <c r="A284" t="n">
+        <v>283</v>
+      </c>
+      <c r="B284" t="inlineStr">
+        <is>
+          <t>Vegetarian Cooking Tips - Gap Fill</t>
+        </is>
+      </c>
+      <c r="C284" t="inlineStr">
+        <is>
+          <t>kuzhai-puttu</t>
+        </is>
+      </c>
+      <c r="D284" t="inlineStr">
+        <is>
+          <t>Kuzhai Puttu (Tube Puttu)</t>
+        </is>
+      </c>
+      <c r="E284" t="inlineStr">
+        <is>
+          <t>குழாய்ப்புட்டு</t>
+        </is>
+      </c>
+      <c r="F284" t="inlineStr">
+        <is>
+          <t>puttu, sweet</t>
+        </is>
+      </c>
+      <c r="G284" t="inlineStr">
+        <is>
+          <t>A close-up photorealistic food photo of a cylindrical steamed puttu on a plate, cut into thick discs revealing alternating white rice-flour and grated-coconut layers studded with sugar, steam still rising, warm morning light.</t>
+        </is>
+      </c>
+      <c r="H284" t="inlineStr">
+        <is>
+          <t>public/images/recipes/kuzhai-puttu/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I284" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="285">
+      <c r="A285" t="n">
+        <v>284</v>
+      </c>
+      <c r="B285" t="inlineStr">
+        <is>
+          <t>Vegetarian Cooking Tips - Gap Fill</t>
+        </is>
+      </c>
+      <c r="C285" t="inlineStr">
+        <is>
+          <t>egg-pan-cake</t>
+        </is>
+      </c>
+      <c r="D285" t="inlineStr">
+        <is>
+          <t>Pan Cake</t>
+        </is>
+      </c>
+      <c r="E285" t="inlineStr">
+        <is>
+          <t>பான் கேக்</t>
+        </is>
+      </c>
+      <c r="F285" t="inlineStr">
+        <is>
+          <t>sweet</t>
+        </is>
+      </c>
+      <c r="G285" t="inlineStr">
+        <is>
+          <t>A close-up photorealistic food photo of a thin, pale golden egg-and-maida pancake folded in half on a plate, a slightly glossy surface from ghee, dusted lightly with sugar, soft warm lighting, shallow depth of field.</t>
+        </is>
+      </c>
+      <c r="H285" t="inlineStr">
+        <is>
+          <t>public/images/recipes/egg-pan-cake/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I285" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="286">
+      <c r="A286" t="n">
+        <v>285</v>
+      </c>
+      <c r="B286" t="inlineStr">
+        <is>
+          <t>Vegetarian Cooking Tips - Gap Fill</t>
+        </is>
+      </c>
+      <c r="C286" t="inlineStr">
+        <is>
+          <t>milk-basundi</t>
+        </is>
+      </c>
+      <c r="D286" t="inlineStr">
+        <is>
+          <t>Milk Basundi</t>
+        </is>
+      </c>
+      <c r="E286" t="inlineStr">
+        <is>
+          <t>பால் பாஸந்தி</t>
+        </is>
+      </c>
+      <c r="F286" t="inlineStr">
+        <is>
+          <t>sweet</t>
+        </is>
+      </c>
+      <c r="G286" t="inlineStr">
+        <is>
+          <t>A close-up photorealistic food photo of thick, creamy off-white basundi in a small clay bowl, slivers of pistachio and cashew scattered on top with a few golden saffron strands, condensation on the bowl suggesting it's chilled, soft natural lighting.</t>
+        </is>
+      </c>
+      <c r="H286" t="inlineStr">
+        <is>
+          <t>public/images/recipes/milk-basundi/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I286" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="287">
+      <c r="A287" t="n">
+        <v>286</v>
+      </c>
+      <c r="B287" t="inlineStr">
+        <is>
+          <t>Vegetarian Cooking Tips - Gap Fill</t>
+        </is>
+      </c>
+      <c r="C287" t="inlineStr">
+        <is>
+          <t>cashew-pakoda</t>
+        </is>
+      </c>
+      <c r="D287" t="inlineStr">
+        <is>
+          <t>Cashew Pakoda</t>
+        </is>
+      </c>
+      <c r="E287" t="inlineStr">
+        <is>
+          <t>முந்திரி பருப்பு பகோடா</t>
+        </is>
+      </c>
+      <c r="F287" t="inlineStr">
+        <is>
+          <t>bajji</t>
+        </is>
+      </c>
+      <c r="G287" t="inlineStr">
+        <is>
+          <t>A close-up photorealistic food photo of golden-brown irregular-shaped fritters piled on a steel plate, whole cashew nuts and flecks of onion visible embedded in the crisp fried batter, a small bowl of ketchup beside it, warm kitchen lighting.</t>
+        </is>
+      </c>
+      <c r="H287" t="inlineStr">
+        <is>
+          <t>public/images/recipes/cashew-pakoda/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I287" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="288">
+      <c r="A288" t="n">
+        <v>287</v>
+      </c>
+      <c r="B288" t="inlineStr">
+        <is>
+          <t>Vegetarian Cooking Tips - Gap Fill</t>
+        </is>
+      </c>
+      <c r="C288" t="inlineStr">
+        <is>
+          <t>potato-chips</t>
+        </is>
+      </c>
+      <c r="D288" t="inlineStr">
+        <is>
+          <t>Potato Chips</t>
+        </is>
+      </c>
+      <c r="E288" t="inlineStr">
+        <is>
+          <t>உருளைக் கிழங்கு சிப்ஸ்</t>
+        </is>
+      </c>
+      <c r="F288" t="inlineStr">
+        <is>
+          <t>snack</t>
+        </is>
+      </c>
+      <c r="G288" t="inlineStr">
+        <is>
+          <t>A close-up photorealistic food photo of thin, golden potato chip rounds piled in a steel bowl, dusted lightly with red chilli powder, glossy from frying oil, warm natural lighting, shallow depth of field.</t>
+        </is>
+      </c>
+      <c r="H288" t="inlineStr">
+        <is>
+          <t>public/images/recipes/potato-chips/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I288" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="289">
+      <c r="A289" t="n">
+        <v>288</v>
+      </c>
+      <c r="B289" t="inlineStr">
+        <is>
+          <t>Vegetarian Cooking Tips - Gap Fill</t>
+        </is>
+      </c>
+      <c r="C289" t="inlineStr">
+        <is>
+          <t>sweet-raw-mango</t>
+        </is>
+      </c>
+      <c r="D289" t="inlineStr">
+        <is>
+          <t>Sweet Raw Mango</t>
+        </is>
+      </c>
+      <c r="E289" t="inlineStr">
+        <is>
+          <t>இனிப்பு மாங்காய்</t>
+        </is>
+      </c>
+      <c r="F289" t="inlineStr">
+        <is>
+          <t>curry</t>
+        </is>
+      </c>
+      <c r="G289" t="inlineStr">
+        <is>
+          <t>A close-up photorealistic food photo of a thick, glossy amber-colored mashed raw mango curry in a steel bowl, flecks of curry leaves and mustard seeds visible, served beside plain rice, warm natural lighting.</t>
+        </is>
+      </c>
+      <c r="H289" t="inlineStr">
+        <is>
+          <t>public/images/recipes/sweet-raw-mango/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I289" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="290">
+      <c r="A290" t="n">
+        <v>289</v>
+      </c>
+      <c r="B290" t="inlineStr">
+        <is>
+          <t>Vegetarian Cooking Tips - Gap Fill</t>
+        </is>
+      </c>
+      <c r="C290" t="inlineStr">
+        <is>
+          <t>kinch-mosara</t>
+        </is>
+      </c>
+      <c r="D290" t="inlineStr">
+        <is>
+          <t>Kinch Mosara (Stuffed Potato Cones)</t>
+        </is>
+      </c>
+      <c r="E290" t="inlineStr">
+        <is>
+          <t>கிஞ்ச மோசரா</t>
+        </is>
+      </c>
+      <c r="F290" t="inlineStr">
+        <is>
+          <t>fried-snack</t>
+        </is>
+      </c>
+      <c r="G290" t="inlineStr">
+        <is>
+          <t>A close-up photorealistic food photo of golden-brown deep-fried cone-shaped pastries on a steel plate, one broken open to reveal a spiced mashed-potato-and-green-pea filling studded with raisins and cashews, warm kitchen lighting, shallow depth of field.</t>
+        </is>
+      </c>
+      <c r="H290" t="inlineStr">
+        <is>
+          <t>public/images/recipes/kinch-mosara/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I290" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="291">
+      <c r="A291" t="n">
+        <v>290</v>
+      </c>
+      <c r="B291" t="inlineStr">
+        <is>
+          <t>Vegetarian Cooking Tips - Gap Fill</t>
+        </is>
+      </c>
+      <c r="C291" t="inlineStr">
+        <is>
+          <t>pirattu-kari</t>
+        </is>
+      </c>
+      <c r="D291" t="inlineStr">
+        <is>
+          <t>Pirattu Kari (Braised Mutton)</t>
+        </is>
+      </c>
+      <c r="E291" t="inlineStr">
+        <is>
+          <t>பிறட்டுக்கறி</t>
+        </is>
+      </c>
+      <c r="F291" t="inlineStr">
+        <is>
+          <t>curry</t>
+        </is>
+      </c>
+      <c r="G291" t="inlineStr">
+        <is>
+          <t>A close-up photorealistic food photo of dark reddish-brown braised mutton pieces in a thick, dry-ish onion masala coating, glistening slightly with oil, served in a steel bowl garnished with curry leaves, warm dramatic lighting, shallow depth of field.</t>
+        </is>
+      </c>
+      <c r="H291" t="inlineStr">
+        <is>
+          <t>public/images/recipes/pirattu-kari/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I291" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="292">
+      <c r="A292" t="n">
+        <v>291</v>
+      </c>
+      <c r="B292" t="inlineStr">
+        <is>
+          <t>Vegetarian Cooking Tips - Gap Fill</t>
+        </is>
+      </c>
+      <c r="C292" t="inlineStr">
+        <is>
+          <t>chinese-sooce</t>
+        </is>
+      </c>
+      <c r="D292" t="inlineStr">
+        <is>
+          <t>Chinese Sooce (Cashew-Date Bars)</t>
+        </is>
+      </c>
+      <c r="E292" t="inlineStr">
+        <is>
+          <t>சைனீஸ் சூஸ்</t>
+        </is>
+      </c>
+      <c r="F292" t="inlineStr">
+        <is>
+          <t>sweet</t>
+        </is>
+      </c>
+      <c r="G292" t="inlineStr">
+        <is>
+          <t>A close-up photorealistic food photo of rectangular golden-brown baked bars studded with chopped cashews and dates, dusted with white icing sugar, stacked on a plate, soft natural lighting, shallow depth of field.</t>
+        </is>
+      </c>
+      <c r="H292" t="inlineStr">
+        <is>
+          <t>public/images/recipes/chinese-sooce/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I292" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="293">
+      <c r="A293" t="n">
+        <v>292</v>
+      </c>
+      <c r="B293" t="inlineStr">
+        <is>
+          <t>Vegetarian Cooking Tips - Gap Fill</t>
+        </is>
+      </c>
+      <c r="C293" t="inlineStr">
+        <is>
+          <t>boat-egg</t>
+        </is>
+      </c>
+      <c r="D293" t="inlineStr">
+        <is>
+          <t>Boat Egg</t>
+        </is>
+      </c>
+      <c r="E293" t="inlineStr">
+        <is>
+          <t>படகு முட்டை</t>
+        </is>
+      </c>
+      <c r="F293" t="inlineStr">
+        <is>
+          <t>snack</t>
+        </is>
+      </c>
+      <c r="G293" t="inlineStr">
+        <is>
+          <t>A close-up photorealistic food photo of small boiled-egg-white boat shapes arranged on a platter, each filled with pale yellow mashed egg yolk and topped with a small triangular bread-slice sail propped upright, playful party-snack styling, bright even lighting.</t>
+        </is>
+      </c>
+      <c r="H293" t="inlineStr">
+        <is>
+          <t>public/images/recipes/boat-egg/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I293" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="294">
+      <c r="A294" t="n">
+        <v>293</v>
+      </c>
+      <c r="B294" t="inlineStr">
+        <is>
+          <t>Vegetarian Cooking Tips - Gap Fill</t>
+        </is>
+      </c>
+      <c r="C294" t="inlineStr">
+        <is>
+          <t>fish-fry-roast</t>
+        </is>
+      </c>
+      <c r="D294" t="inlineStr">
+        <is>
+          <t>Fish Fry Roast</t>
+        </is>
+      </c>
+      <c r="E294" t="inlineStr">
+        <is>
+          <t>மீன் ஃபிராஸ்ட்</t>
+        </is>
+      </c>
+      <c r="F294" t="inlineStr">
+        <is>
+          <t>curry</t>
+        </is>
+      </c>
+      <c r="G294" t="inlineStr">
+        <is>
+          <t>A close-up photorealistic food photo of golden-brown shallow-fried fish steaks on a steel plate, a red-orange spice crust visible on the surface, garnished with sliced onion, coriander leaves, and a lemon wedge, warm kitchen lighting, shallow depth of field.</t>
+        </is>
+      </c>
+      <c r="H294" t="inlineStr">
+        <is>
+          <t>public/images/recipes/fish-fry-roast/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I294" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Revert "Fill 21 missing recipes from Vegetarian Cooking Tips cookbook"
This reverts commit db43fffd284510f1f3b4ff31f698944ef55722e0.
</commit_message>
<xml_diff>
--- a/docs/recipe-image-tracker.xlsx
+++ b/docs/recipe-image-tracker.xlsx
@@ -496,7 +496,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K294"/>
+  <dimension ref="A1:K202"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -11423,4146 +11423,6 @@
         </is>
       </c>
       <c r="K202" s="15" t="n"/>
-    </row>
-    <row r="203">
-      <c r="A203" t="n">
-        <v>202</v>
-      </c>
-      <c r="B203" t="inlineStr">
-        <is>
-          <t>Vegetarian</t>
-        </is>
-      </c>
-      <c r="C203" t="inlineStr">
-        <is>
-          <t>banana-cutlets</t>
-        </is>
-      </c>
-      <c r="D203" t="inlineStr">
-        <is>
-          <t>Banana Cutlets</t>
-        </is>
-      </c>
-      <c r="E203" t="inlineStr">
-        <is>
-          <t>வாழைக்காய் கட்லெட்</t>
-        </is>
-      </c>
-      <c r="F203" t="inlineStr">
-        <is>
-          <t>cutlet</t>
-        </is>
-      </c>
-      <c r="G203" t="inlineStr">
-        <is>
-          <t>A close-up photorealistic food photo of golden-brown oval cutlets with a crisp breadcrumb crust, plated on a white ceramic plate, garnished with a wedge of lemon and a small bowl of tomato ketchup, one cutlet broken open to reveal a soft reddish-brown banana-potato filling flecked with green coriander, warm natural lighting, shallow depth of field.</t>
-        </is>
-      </c>
-      <c r="H203" t="inlineStr">
-        <is>
-          <t>public/images/recipes/banana-cutlets/featured.jpg</t>
-        </is>
-      </c>
-      <c r="I203" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="204">
-      <c r="A204" t="n">
-        <v>203</v>
-      </c>
-      <c r="B204" t="inlineStr">
-        <is>
-          <t>Vegetarian</t>
-        </is>
-      </c>
-      <c r="C204" t="inlineStr">
-        <is>
-          <t>vegetable-sizzlers</t>
-        </is>
-      </c>
-      <c r="D204" t="inlineStr">
-        <is>
-          <t>Vegetable Sizzlers</t>
-        </is>
-      </c>
-      <c r="E204" t="inlineStr">
-        <is>
-          <t>வெஜிடபிள் சிஸ்லர்ஸ்</t>
-        </is>
-      </c>
-      <c r="F204" t="inlineStr">
-        <is>
-          <t>fusion</t>
-        </is>
-      </c>
-      <c r="G204" t="inlineStr">
-        <is>
-          <t>A dramatic photorealistic photo of a cast-iron sizzler plate on a wooden board, visibly smoking with steam rising, holding a golden fried cutlet in the center surrounded by charred grilled carrot rounds, cabbage wedges, capsicum rings, and potato slices, glossy with butter and reddish sauce, dark moody restaurant lighting.</t>
-        </is>
-      </c>
-      <c r="H204" t="inlineStr">
-        <is>
-          <t>public/images/recipes/vegetable-sizzlers/featured.jpg</t>
-        </is>
-      </c>
-      <c r="I204" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="205">
-      <c r="A205" t="n">
-        <v>204</v>
-      </c>
-      <c r="B205" t="inlineStr">
-        <is>
-          <t>Vegetarian</t>
-        </is>
-      </c>
-      <c r="C205" t="inlineStr">
-        <is>
-          <t>vegetable-burgers</t>
-        </is>
-      </c>
-      <c r="D205" t="inlineStr">
-        <is>
-          <t>Vegetable Burgers</t>
-        </is>
-      </c>
-      <c r="E205" t="inlineStr">
-        <is>
-          <t>வெஜிடபிள் பர்கர்ஸ்</t>
-        </is>
-      </c>
-      <c r="F205" t="inlineStr">
-        <is>
-          <t>fusion</t>
-        </is>
-      </c>
-      <c r="G205" t="inlineStr">
-        <is>
-          <t>A photorealistic close-up of a round golden-brown vegetable burger patty inside a soft bun, layered with a crisp cabbage leaf, thin onion rings, beetroot slices, and tomato, skewered with a small toothpick, plated with crinkle-cut potato fries and ketchup, bright appetizing lighting.</t>
-        </is>
-      </c>
-      <c r="H205" t="inlineStr">
-        <is>
-          <t>public/images/recipes/vegetable-burgers/featured.jpg</t>
-        </is>
-      </c>
-      <c r="I205" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="206">
-      <c r="A206" t="n">
-        <v>205</v>
-      </c>
-      <c r="B206" t="inlineStr">
-        <is>
-          <t>Vegetarian</t>
-        </is>
-      </c>
-      <c r="C206" t="inlineStr">
-        <is>
-          <t>sago-bonda</t>
-        </is>
-      </c>
-      <c r="D206" t="inlineStr">
-        <is>
-          <t>Sago Bonda</t>
-        </is>
-      </c>
-      <c r="E206" t="inlineStr">
-        <is>
-          <t>ஜவ்வரிசி போண்டா</t>
-        </is>
-      </c>
-      <c r="F206" t="inlineStr">
-        <is>
-          <t>bonda</t>
-        </is>
-      </c>
-      <c r="G206" t="inlineStr">
-        <is>
-          <t>A photorealistic close-up of small round golden-brown bondas with a translucent, pearly, slightly bumpy sago texture visible on the fried crust, piled on a steel plate lined with paper, garnished with coriander leaves, a small bowl of green chutney beside them, warm kitchen lighting.</t>
-        </is>
-      </c>
-      <c r="H206" t="inlineStr">
-        <is>
-          <t>public/images/recipes/sago-bonda/featured.jpg</t>
-        </is>
-      </c>
-      <c r="I206" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="207">
-      <c r="A207" t="n">
-        <v>206</v>
-      </c>
-      <c r="B207" t="inlineStr">
-        <is>
-          <t>Vegetarian</t>
-        </is>
-      </c>
-      <c r="C207" t="inlineStr">
-        <is>
-          <t>vegetable-bonda</t>
-        </is>
-      </c>
-      <c r="D207" t="inlineStr">
-        <is>
-          <t>Vegetable Bonda</t>
-        </is>
-      </c>
-      <c r="E207" t="inlineStr">
-        <is>
-          <t>வெஜிடபிள் போண்டா</t>
-        </is>
-      </c>
-      <c r="F207" t="inlineStr">
-        <is>
-          <t>bonda</t>
-        </is>
-      </c>
-      <c r="G207" t="inlineStr">
-        <is>
-          <t>A photorealistic photo of golden fried round bondas with a slightly bumpy, craggy batter surface, one bonda broken in half to show a moist mixed-vegetable filling of carrot, peas, and potato, served on a steel plate with mint chutney and tomato sauce, natural daylight.</t>
-        </is>
-      </c>
-      <c r="H207" t="inlineStr">
-        <is>
-          <t>public/images/recipes/vegetable-bonda/featured.jpg</t>
-        </is>
-      </c>
-      <c r="I207" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="208">
-      <c r="A208" t="n">
-        <v>207</v>
-      </c>
-      <c r="B208" t="inlineStr">
-        <is>
-          <t>Vegetarian</t>
-        </is>
-      </c>
-      <c r="C208" t="inlineStr">
-        <is>
-          <t>aloo-bonda</t>
-        </is>
-      </c>
-      <c r="D208" t="inlineStr">
-        <is>
-          <t>Aloo Bonda</t>
-        </is>
-      </c>
-      <c r="E208" t="inlineStr">
-        <is>
-          <t>உருளைக்கிழங்கு போண்டா</t>
-        </is>
-      </c>
-      <c r="F208" t="inlineStr">
-        <is>
-          <t>bonda</t>
-        </is>
-      </c>
-      <c r="G208" t="inlineStr">
-        <is>
-          <t>A photorealistic image of golden-brown round bondas with a smooth thin batter coating, arranged on a banana leaf, one cut open to reveal a soft yellow mashed-potato filling flecked with onion and coriander, served with coconut chutney, warm South Indian tea-stall lighting.</t>
-        </is>
-      </c>
-      <c r="H208" t="inlineStr">
-        <is>
-          <t>public/images/recipes/aloo-bonda/featured.jpg</t>
-        </is>
-      </c>
-      <c r="I208" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="209">
-      <c r="A209" t="n">
-        <v>208</v>
-      </c>
-      <c r="B209" t="inlineStr">
-        <is>
-          <t>Vegetarian</t>
-        </is>
-      </c>
-      <c r="C209" t="inlineStr">
-        <is>
-          <t>mysore-bonda</t>
-        </is>
-      </c>
-      <c r="D209" t="inlineStr">
-        <is>
-          <t>Mysore Bonda</t>
-        </is>
-      </c>
-      <c r="E209" t="inlineStr">
-        <is>
-          <t>மைசூர் போண்டா</t>
-        </is>
-      </c>
-      <c r="F209" t="inlineStr">
-        <is>
-          <t>bonda</t>
-        </is>
-      </c>
-      <c r="G209" t="inlineStr">
-        <is>
-          <t>A photorealistic close-up of fluffy, irregularly round golden-brown bondas with a light, airy fried crust, stacked in a steel plate, one broken open showing a soft white lentil interior studded with coconut bits, served with coconut chutney in a small bowl, bright natural light.</t>
-        </is>
-      </c>
-      <c r="H209" t="inlineStr">
-        <is>
-          <t>public/images/recipes/mysore-bonda/featured.jpg</t>
-        </is>
-      </c>
-      <c r="I209" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="210">
-      <c r="A210" t="n">
-        <v>209</v>
-      </c>
-      <c r="B210" t="inlineStr">
-        <is>
-          <t>Vegetarian</t>
-        </is>
-      </c>
-      <c r="C210" t="inlineStr">
-        <is>
-          <t>pullani-vunta</t>
-        </is>
-      </c>
-      <c r="D210" t="inlineStr">
-        <is>
-          <t>Pullani Vunta</t>
-        </is>
-      </c>
-      <c r="E210" t="inlineStr">
-        <is>
-          <t>தோசைமாவு போண்டா</t>
-        </is>
-      </c>
-      <c r="F210" t="inlineStr">
-        <is>
-          <t>bonda</t>
-        </is>
-      </c>
-      <c r="G210" t="inlineStr">
-        <is>
-          <t>A photorealistic photo of small irregular golden-brown fried dumplings made from fermented dosa batter, slightly craggy surface with visible onion and coriander flecks, piled on a steel plate with coconut chutney on the side, cozy kitchen lighting.</t>
-        </is>
-      </c>
-      <c r="H210" t="inlineStr">
-        <is>
-          <t>public/images/recipes/pullani-vunta/featured.jpg</t>
-        </is>
-      </c>
-      <c r="I210" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="211">
-      <c r="A211" t="n">
-        <v>210</v>
-      </c>
-      <c r="B211" t="inlineStr">
-        <is>
-          <t>Vegetarian</t>
-        </is>
-      </c>
-      <c r="C211" t="inlineStr">
-        <is>
-          <t>mangalore-bonda</t>
-        </is>
-      </c>
-      <c r="D211" t="inlineStr">
-        <is>
-          <t>Mangalore Bonda</t>
-        </is>
-      </c>
-      <c r="E211" t="inlineStr">
-        <is>
-          <t>மங்களூர் போண்டா</t>
-        </is>
-      </c>
-      <c r="F211" t="inlineStr">
-        <is>
-          <t>bonda</t>
-        </is>
-      </c>
-      <c r="G211" t="inlineStr">
-        <is>
-          <t>A photorealistic close-up of soft, puffy golden-brown fried bondas with a slightly wrinkled curd-based batter texture, arranged on a plate, one broken open to reveal a soft white interior, served with coconut chutney, warm ambient lighting.</t>
-        </is>
-      </c>
-      <c r="H211" t="inlineStr">
-        <is>
-          <t>public/images/recipes/mangalore-bonda/featured.jpg</t>
-        </is>
-      </c>
-      <c r="I211" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="212">
-      <c r="A212" t="n">
-        <v>211</v>
-      </c>
-      <c r="B212" t="inlineStr">
-        <is>
-          <t>Vegetarian</t>
-        </is>
-      </c>
-      <c r="C212" t="inlineStr">
-        <is>
-          <t>cheese-bonda</t>
-        </is>
-      </c>
-      <c r="D212" t="inlineStr">
-        <is>
-          <t>Cheese Bonda</t>
-        </is>
-      </c>
-      <c r="E212" t="inlineStr">
-        <is>
-          <t>சீஸ் போண்டா</t>
-        </is>
-      </c>
-      <c r="F212" t="inlineStr">
-        <is>
-          <t>bonda</t>
-        </is>
-      </c>
-      <c r="G212" t="inlineStr">
-        <is>
-          <t>A photorealistic close-up of small golden fried bondas glistening with oil, one cut in half to reveal a stretchy, melted golden-yellow cheese pull, plated on a white dish, steam rising, cozy warm lighting.</t>
-        </is>
-      </c>
-      <c r="H212" t="inlineStr">
-        <is>
-          <t>public/images/recipes/cheese-bonda/featured.jpg</t>
-        </is>
-      </c>
-      <c r="I212" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="213">
-      <c r="A213" t="n">
-        <v>212</v>
-      </c>
-      <c r="B213" t="inlineStr">
-        <is>
-          <t>Vegetarian</t>
-        </is>
-      </c>
-      <c r="C213" t="inlineStr">
-        <is>
-          <t>palak-dumplings</t>
-        </is>
-      </c>
-      <c r="D213" t="inlineStr">
-        <is>
-          <t>Palak Dumplings</t>
-        </is>
-      </c>
-      <c r="E213" t="inlineStr">
-        <is>
-          <t>பாலக் மெதுபக்கோடா</t>
-        </is>
-      </c>
-      <c r="F213" t="inlineStr">
-        <is>
-          <t>fried-snack</t>
-        </is>
-      </c>
-      <c r="G213" t="inlineStr">
-        <is>
-          <t>A photorealistic photo of small dark-green-flecked golden fried dumplings, irregular round shape, piled on a plate, showing visible bits of dark green spinach and chili in the crisp fried crust, served with ketchup, natural daylight.</t>
-        </is>
-      </c>
-      <c r="H213" t="inlineStr">
-        <is>
-          <t>public/images/recipes/palak-dumplings/featured.jpg</t>
-        </is>
-      </c>
-      <c r="I213" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="214">
-      <c r="A214" t="n">
-        <v>213</v>
-      </c>
-      <c r="B214" t="inlineStr">
-        <is>
-          <t>Vegetarian</t>
-        </is>
-      </c>
-      <c r="C214" t="inlineStr">
-        <is>
-          <t>ridge-gourd-dumplings</t>
-        </is>
-      </c>
-      <c r="D214" t="inlineStr">
-        <is>
-          <t>Ridge Gourd Dumplings</t>
-        </is>
-      </c>
-      <c r="E214" t="inlineStr">
-        <is>
-          <t>பீர்க்கங்காய் மெதுபக்கோடா</t>
-        </is>
-      </c>
-      <c r="F214" t="inlineStr">
-        <is>
-          <t>fried-snack</t>
-        </is>
-      </c>
-      <c r="G214" t="inlineStr">
-        <is>
-          <t>A photorealistic close-up of small golden fried dumplings with pale green ridge-gourd flecks visible through the thin gram-flour crust, piled on a steel plate, served hot with tomato sauce, warm kitchen lighting.</t>
-        </is>
-      </c>
-      <c r="H214" t="inlineStr">
-        <is>
-          <t>public/images/recipes/ridge-gourd-dumplings/featured.jpg</t>
-        </is>
-      </c>
-      <c r="I214" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="215">
-      <c r="A215" t="n">
-        <v>214</v>
-      </c>
-      <c r="B215" t="inlineStr">
-        <is>
-          <t>Vegetarian</t>
-        </is>
-      </c>
-      <c r="C215" t="inlineStr">
-        <is>
-          <t>mint-pakodas</t>
-        </is>
-      </c>
-      <c r="D215" t="inlineStr">
-        <is>
-          <t>Mint Pakodas</t>
-        </is>
-      </c>
-      <c r="E215" t="inlineStr">
-        <is>
-          <t>புதினா பக்கோடா</t>
-        </is>
-      </c>
-      <c r="F215" t="inlineStr">
-        <is>
-          <t>bajji</t>
-        </is>
-      </c>
-      <c r="G215" t="inlineStr">
-        <is>
-          <t>A photorealistic photo of dark green-brown irregular fried pakodas with visible mint and coriander leaf flecks throughout the crumbly, coarse lentil texture, piled high on a plate, steam rising, natural light.</t>
-        </is>
-      </c>
-      <c r="H215" t="inlineStr">
-        <is>
-          <t>public/images/recipes/mint-pakodas/featured.jpg</t>
-        </is>
-      </c>
-      <c r="I215" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="216">
-      <c r="A216" t="n">
-        <v>215</v>
-      </c>
-      <c r="B216" t="inlineStr">
-        <is>
-          <t>Vegetarian</t>
-        </is>
-      </c>
-      <c r="C216" t="inlineStr">
-        <is>
-          <t>potato-nest</t>
-        </is>
-      </c>
-      <c r="D216" t="inlineStr">
-        <is>
-          <t>Potato Nest</t>
-        </is>
-      </c>
-      <c r="E216" t="inlineStr">
-        <is>
-          <t>உருளைக்கிழங்கு கூடுகள்</t>
-        </is>
-      </c>
-      <c r="F216" t="inlineStr">
-        <is>
-          <t>fried-snack</t>
-        </is>
-      </c>
-      <c r="G216" t="inlineStr">
-        <is>
-          <t>A photorealistic close-up of round golden fried balls coated entirely in crisp, spiky strands of fried vermicelli giving a bird's-nest texture, one cut in half to reveal a bright yellow mashed-potato interior with green peas, plated elegantly with lettuce and tomato sauce, bright studio food photography lighting.</t>
-        </is>
-      </c>
-      <c r="H216" t="inlineStr">
-        <is>
-          <t>public/images/recipes/potato-nest/featured.jpg</t>
-        </is>
-      </c>
-      <c r="I216" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="217">
-      <c r="A217" t="n">
-        <v>216</v>
-      </c>
-      <c r="B217" t="inlineStr">
-        <is>
-          <t>Vegetarian</t>
-        </is>
-      </c>
-      <c r="C217" t="inlineStr">
-        <is>
-          <t>garam-pakodas</t>
-        </is>
-      </c>
-      <c r="D217" t="inlineStr">
-        <is>
-          <t>Garam Pakodas</t>
-        </is>
-      </c>
-      <c r="E217" t="inlineStr">
-        <is>
-          <t>வெங்காய பக்கோடா</t>
-        </is>
-      </c>
-      <c r="F217" t="inlineStr">
-        <is>
-          <t>bajji</t>
-        </is>
-      </c>
-      <c r="G217" t="inlineStr">
-        <is>
-          <t>A photorealistic photo of a heaping pile of irregular, craggy, deep-golden fried pakoda chunks with visible long strands of onion and green chili baked into the crisp crust, on a steel plate, chai glass beside it, warm evening tea-stall lighting.</t>
-        </is>
-      </c>
-      <c r="H217" t="inlineStr">
-        <is>
-          <t>public/images/recipes/garam-pakodas/featured.jpg</t>
-        </is>
-      </c>
-      <c r="I217" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="218">
-      <c r="A218" t="n">
-        <v>217</v>
-      </c>
-      <c r="B218" t="inlineStr">
-        <is>
-          <t>Vegetarian</t>
-        </is>
-      </c>
-      <c r="C218" t="inlineStr">
-        <is>
-          <t>paneer-pakodas</t>
-        </is>
-      </c>
-      <c r="D218" t="inlineStr">
-        <is>
-          <t>Paneer Pakodas</t>
-        </is>
-      </c>
-      <c r="E218" t="inlineStr">
-        <is>
-          <t>பனீர் பக்கோடா</t>
-        </is>
-      </c>
-      <c r="F218" t="inlineStr">
-        <is>
-          <t>bajji</t>
-        </is>
-      </c>
-      <c r="G218" t="inlineStr">
-        <is>
-          <t>A photorealistic close-up of irregular golden fried pakoda chunks with visible crumbly white paneer and pink cashew pieces embedded in the crust, piled on a plate with mint garnish, warm kitchen lighting.</t>
-        </is>
-      </c>
-      <c r="H218" t="inlineStr">
-        <is>
-          <t>public/images/recipes/paneer-pakodas/featured.jpg</t>
-        </is>
-      </c>
-      <c r="I218" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="219">
-      <c r="A219" t="n">
-        <v>218</v>
-      </c>
-      <c r="B219" t="inlineStr">
-        <is>
-          <t>Vegetarian</t>
-        </is>
-      </c>
-      <c r="C219" t="inlineStr">
-        <is>
-          <t>bread-pakodas</t>
-        </is>
-      </c>
-      <c r="D219" t="inlineStr">
-        <is>
-          <t>Bread Pakodas</t>
-        </is>
-      </c>
-      <c r="E219" t="inlineStr">
-        <is>
-          <t>பிரட் பக்கோடா</t>
-        </is>
-      </c>
-      <c r="F219" t="inlineStr">
-        <is>
-          <t>bajji</t>
-        </is>
-      </c>
-      <c r="G219" t="inlineStr">
-        <is>
-          <t>A photorealistic photo of golden-brown irregular fried pakoda pieces with a soft doughy bread interior visible at the torn edges, piled on a plate, served with tomato ketchup, natural daylight.</t>
-        </is>
-      </c>
-      <c r="H219" t="inlineStr">
-        <is>
-          <t>public/images/recipes/bread-pakodas/featured.jpg</t>
-        </is>
-      </c>
-      <c r="I219" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="220">
-      <c r="A220" t="n">
-        <v>219</v>
-      </c>
-      <c r="B220" t="inlineStr">
-        <is>
-          <t>Vegetarian</t>
-        </is>
-      </c>
-      <c r="C220" t="inlineStr">
-        <is>
-          <t>vermicelli-pakodas</t>
-        </is>
-      </c>
-      <c r="D220" t="inlineStr">
-        <is>
-          <t>Vermicelli Pakodas</t>
-        </is>
-      </c>
-      <c r="E220" t="inlineStr">
-        <is>
-          <t>சேமியா பக்கோடா</t>
-        </is>
-      </c>
-      <c r="F220" t="inlineStr">
-        <is>
-          <t>bajji</t>
-        </is>
-      </c>
-      <c r="G220" t="inlineStr">
-        <is>
-          <t>A photorealistic close-up of golden fried pakodas with fine strands of crisp vermicelli visible on the textured surface, piled on a steel plate with mint chutney, warm ambient lighting.</t>
-        </is>
-      </c>
-      <c r="H220" t="inlineStr">
-        <is>
-          <t>public/images/recipes/vermicelli-pakodas/featured.jpg</t>
-        </is>
-      </c>
-      <c r="I220" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="221">
-      <c r="A221" t="n">
-        <v>220</v>
-      </c>
-      <c r="B221" t="inlineStr">
-        <is>
-          <t>Vegetarian</t>
-        </is>
-      </c>
-      <c r="C221" t="inlineStr">
-        <is>
-          <t>layered-sandwich-bajji</t>
-        </is>
-      </c>
-      <c r="D221" t="inlineStr">
-        <is>
-          <t>Layered Sandwich Bajji</t>
-        </is>
-      </c>
-      <c r="E221" t="inlineStr">
-        <is>
-          <t>பிரட் சாண்ட்விட்ச் பஜ்ஜி</t>
-        </is>
-      </c>
-      <c r="F221" t="inlineStr">
-        <is>
-          <t>bajji,sandwich</t>
-        </is>
-      </c>
-      <c r="G221" t="inlineStr">
-        <is>
-          <t>A photorealistic close-up of a golden fried rectangular sandwich bajji cut in half, showing three layers of white bread with visible green mint chutney and red tomato chutney filling between the layers, crisp golden batter coating on the outside, served with tomato sauce, bright natural lighting.</t>
-        </is>
-      </c>
-      <c r="H221" t="inlineStr">
-        <is>
-          <t>public/images/recipes/layered-sandwich-bajji/featured.jpg</t>
-        </is>
-      </c>
-      <c r="I221" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="222">
-      <c r="A222" t="n">
-        <v>221</v>
-      </c>
-      <c r="B222" t="inlineStr">
-        <is>
-          <t>Vegetarian</t>
-        </is>
-      </c>
-      <c r="C222" t="inlineStr">
-        <is>
-          <t>capsicum-bajji</t>
-        </is>
-      </c>
-      <c r="D222" t="inlineStr">
-        <is>
-          <t>Capsicum Bajji</t>
-        </is>
-      </c>
-      <c r="E222" t="inlineStr">
-        <is>
-          <t>குடமிளகாய் பஜ்ஜி</t>
-        </is>
-      </c>
-      <c r="F222" t="inlineStr">
-        <is>
-          <t>bajji</t>
-        </is>
-      </c>
-      <c r="G222" t="inlineStr">
-        <is>
-          <t>A photorealistic photo of whole small green capsicums coated in a golden fried batter, one sliced open at the top showing chopped onion tucked inside with a wedge of lemon on the side, plated attractively, warm lighting.</t>
-        </is>
-      </c>
-      <c r="H222" t="inlineStr">
-        <is>
-          <t>public/images/recipes/capsicum-bajji/featured.jpg</t>
-        </is>
-      </c>
-      <c r="I222" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="223">
-      <c r="A223" t="n">
-        <v>222</v>
-      </c>
-      <c r="B223" t="inlineStr">
-        <is>
-          <t>Vegetarian</t>
-        </is>
-      </c>
-      <c r="C223" t="inlineStr">
-        <is>
-          <t>stuffed-chilli-bajji</t>
-        </is>
-      </c>
-      <c r="D223" t="inlineStr">
-        <is>
-          <t>Stuffed Chilli Bajji</t>
-        </is>
-      </c>
-      <c r="E223" t="inlineStr">
-        <is>
-          <t>மிளகாய் பஜ்ஜி</t>
-        </is>
-      </c>
-      <c r="F223" t="inlineStr">
-        <is>
-          <t>bajji</t>
-        </is>
-      </c>
-      <c r="G223" t="inlineStr">
-        <is>
-          <t>A photorealistic close-up of long green bajji chilies coated in golden fried batter, one split open lengthwise to reveal a pale coconut-and-gram filling inside, garnished with chopped onion and a drizzle of sweet brown chutney, plated on a steel dish, warm tea-stall lighting.</t>
-        </is>
-      </c>
-      <c r="H223" t="inlineStr">
-        <is>
-          <t>public/images/recipes/stuffed-chilli-bajji/featured.jpg</t>
-        </is>
-      </c>
-      <c r="I223" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="224">
-      <c r="A224" t="n">
-        <v>223</v>
-      </c>
-      <c r="B224" t="inlineStr">
-        <is>
-          <t>Vegetarian</t>
-        </is>
-      </c>
-      <c r="C224" t="inlineStr">
-        <is>
-          <t>lasania</t>
-        </is>
-      </c>
-      <c r="D224" t="inlineStr">
-        <is>
-          <t>Lasania (Stuffed Potato Bajji)</t>
-        </is>
-      </c>
-      <c r="E224" t="inlineStr">
-        <is>
-          <t>உருளைகிழங்கு ஸ்டப் பஜ்ஜி</t>
-        </is>
-      </c>
-      <c r="F224" t="inlineStr">
-        <is>
-          <t>bajji</t>
-        </is>
-      </c>
-      <c r="G224" t="inlineStr">
-        <is>
-          <t>A photorealistic photo of small whole potatoes coated in golden fried batter, one sliced partway open showing a reddish garlic-spice paste inside, piled on a plate, warm lighting.</t>
-        </is>
-      </c>
-      <c r="H224" t="inlineStr">
-        <is>
-          <t>public/images/recipes/lasania/featured.jpg</t>
-        </is>
-      </c>
-      <c r="I224" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="225">
-      <c r="A225" t="n">
-        <v>224</v>
-      </c>
-      <c r="B225" t="inlineStr">
-        <is>
-          <t>Vegetarian</t>
-        </is>
-      </c>
-      <c r="C225" t="inlineStr">
-        <is>
-          <t>medu-vadai</t>
-        </is>
-      </c>
-      <c r="D225" t="inlineStr">
-        <is>
-          <t>Medu Vadai</t>
-        </is>
-      </c>
-      <c r="E225" t="inlineStr">
-        <is>
-          <t>மெதுவடை</t>
-        </is>
-      </c>
-      <c r="F225" t="inlineStr">
-        <is>
-          <t>vadai</t>
-        </is>
-      </c>
-      <c r="G225" t="inlineStr">
-        <is>
-          <t>A photorealistic close-up of classic golden-brown ring-shaped vadais with a lacy, crisp textured surface, stacked on a banana leaf, served with sambar in a small steel bowl and coconut chutney, warm South Indian breakfast table lighting.</t>
-        </is>
-      </c>
-      <c r="H225" t="inlineStr">
-        <is>
-          <t>public/images/recipes/medu-vadai/featured.jpg</t>
-        </is>
-      </c>
-      <c r="I225" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="226">
-      <c r="A226" t="n">
-        <v>225</v>
-      </c>
-      <c r="B226" t="inlineStr">
-        <is>
-          <t>Vegetarian</t>
-        </is>
-      </c>
-      <c r="C226" t="inlineStr">
-        <is>
-          <t>curd-vadai</t>
-        </is>
-      </c>
-      <c r="D226" t="inlineStr">
-        <is>
-          <t>Thair Vadai</t>
-        </is>
-      </c>
-      <c r="E226" t="inlineStr">
-        <is>
-          <t>தயிர் வடை</t>
-        </is>
-      </c>
-      <c r="F226" t="inlineStr">
-        <is>
-          <t>vadai</t>
-        </is>
-      </c>
-      <c r="G226" t="inlineStr">
-        <is>
-          <t>A photorealistic close-up of soft, pale golden vadais submerged in thick white curd on a steel plate, garnished with a drizzle of tempered mustard seeds, chopped coriander leaves, and a light dusting of red chili powder on top, bright natural lighting.</t>
-        </is>
-      </c>
-      <c r="H226" t="inlineStr">
-        <is>
-          <t>public/images/recipes/curd-vadai/featured.jpg</t>
-        </is>
-      </c>
-      <c r="I226" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="227">
-      <c r="A227" t="n">
-        <v>226</v>
-      </c>
-      <c r="B227" t="inlineStr">
-        <is>
-          <t>Vegetarian</t>
-        </is>
-      </c>
-      <c r="C227" t="inlineStr">
-        <is>
-          <t>special-curd-vadai-1</t>
-        </is>
-      </c>
-      <c r="D227" t="inlineStr">
-        <is>
-          <t>Special Curd Vadai 1</t>
-        </is>
-      </c>
-      <c r="E227" t="inlineStr">
-        <is>
-          <t>ஸ்பெஷல் தயிர் வடை (1)</t>
-        </is>
-      </c>
-      <c r="F227" t="inlineStr">
-        <is>
-          <t>vadai</t>
-        </is>
-      </c>
-      <c r="G227" t="inlineStr">
-        <is>
-          <t>A photorealistic close-up of a curd-soaked vadai cut open on a plate revealing a colorful filling of chopped cashews, almonds, raisins, and coconut inside the soft white lentil dough, surrounded by thick curd, garnished with fried spicy boondi on top, bright lighting.</t>
-        </is>
-      </c>
-      <c r="H227" t="inlineStr">
-        <is>
-          <t>public/images/recipes/special-curd-vadai-1/featured.jpg</t>
-        </is>
-      </c>
-      <c r="I227" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="228">
-      <c r="A228" t="n">
-        <v>227</v>
-      </c>
-      <c r="B228" t="inlineStr">
-        <is>
-          <t>Vegetarian</t>
-        </is>
-      </c>
-      <c r="C228" t="inlineStr">
-        <is>
-          <t>special-curd-vadai-2</t>
-        </is>
-      </c>
-      <c r="D228" t="inlineStr">
-        <is>
-          <t>Special Curd Vadai 2</t>
-        </is>
-      </c>
-      <c r="E228" t="inlineStr">
-        <is>
-          <t>ஸ்பெஷல் தயிர் வடை (2)</t>
-        </is>
-      </c>
-      <c r="F228" t="inlineStr">
-        <is>
-          <t>vadai</t>
-        </is>
-      </c>
-      <c r="G228" t="inlineStr">
-        <is>
-          <t>A photorealistic close-up of a half-moon, samosa-shaped curd vadai on a plate, soaked in white curd, with visible green herb flecks along the folded edge, garnished with grated carrot and coriander, natural lighting.</t>
-        </is>
-      </c>
-      <c r="H228" t="inlineStr">
-        <is>
-          <t>public/images/recipes/special-curd-vadai-2/featured.jpg</t>
-        </is>
-      </c>
-      <c r="I228" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="229">
-      <c r="A229" t="n">
-        <v>228</v>
-      </c>
-      <c r="B229" t="inlineStr">
-        <is>
-          <t>Vegetarian</t>
-        </is>
-      </c>
-      <c r="C229" t="inlineStr">
-        <is>
-          <t>pattani-curd-vadai</t>
-        </is>
-      </c>
-      <c r="D229" t="inlineStr">
-        <is>
-          <t>Pattani Curd Vadai</t>
-        </is>
-      </c>
-      <c r="E229" t="inlineStr">
-        <is>
-          <t>பட்டாணி தயிர் வடை</t>
-        </is>
-      </c>
-      <c r="F229" t="inlineStr">
-        <is>
-          <t>vadai</t>
-        </is>
-      </c>
-      <c r="G229" t="inlineStr">
-        <is>
-          <t>A photorealistic close-up of a curd-soaked vadai cut in half showing a bright green mashed-pea filling inside the soft white lentil exterior, surrounded by thick curd on a steel plate, garnished with coriander, natural lighting.</t>
-        </is>
-      </c>
-      <c r="H229" t="inlineStr">
-        <is>
-          <t>public/images/recipes/pattani-curd-vadai/featured.jpg</t>
-        </is>
-      </c>
-      <c r="I229" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="230">
-      <c r="A230" t="n">
-        <v>229</v>
-      </c>
-      <c r="B230" t="inlineStr">
-        <is>
-          <t>Vegetarian</t>
-        </is>
-      </c>
-      <c r="C230" t="inlineStr">
-        <is>
-          <t>mor-kuzhambu-vadai</t>
-        </is>
-      </c>
-      <c r="D230" t="inlineStr">
-        <is>
-          <t>Mor Kuzhambu Vadai</t>
-        </is>
-      </c>
-      <c r="E230" t="inlineStr">
-        <is>
-          <t>மோர்க்குழம்பு வடை</t>
-        </is>
-      </c>
-      <c r="F230" t="inlineStr">
-        <is>
-          <t>vadai</t>
-        </is>
-      </c>
-      <c r="G230" t="inlineStr">
-        <is>
-          <t>A photorealistic close-up of pale golden vadais submerged in a thick, pale-yellow spiced buttermilk gravy flecked with coconut and curry leaves, served in a steel bowl, garnished with coriander leaves, warm home-style lighting.</t>
-        </is>
-      </c>
-      <c r="H230" t="inlineStr">
-        <is>
-          <t>public/images/recipes/mor-kuzhambu-vadai/featured.jpg</t>
-        </is>
-      </c>
-      <c r="I230" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="231">
-      <c r="A231" t="n">
-        <v>230</v>
-      </c>
-      <c r="B231" t="inlineStr">
-        <is>
-          <t>Vegetarian</t>
-        </is>
-      </c>
-      <c r="C231" t="inlineStr">
-        <is>
-          <t>aamai-vadai</t>
-        </is>
-      </c>
-      <c r="D231" t="inlineStr">
-        <is>
-          <t>Aamai Vadai</t>
-        </is>
-      </c>
-      <c r="E231" t="inlineStr">
-        <is>
-          <t>ஆமை வடை</t>
-        </is>
-      </c>
-      <c r="F231" t="inlineStr">
-        <is>
-          <t>vadai</t>
-        </is>
-      </c>
-      <c r="G231" t="inlineStr">
-        <is>
-          <t>A photorealistic photo of torn half-moon pieces of coarse-textured urad-toor dal vadai, soaked briefly in curd, plated with a light garnish, rustic table lighting.</t>
-        </is>
-      </c>
-      <c r="H231" t="inlineStr">
-        <is>
-          <t>public/images/recipes/aamai-vadai/featured.jpg</t>
-        </is>
-      </c>
-      <c r="I231" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="232">
-      <c r="A232" t="n">
-        <v>231</v>
-      </c>
-      <c r="B232" t="inlineStr">
-        <is>
-          <t>Vegetarian</t>
-        </is>
-      </c>
-      <c r="C232" t="inlineStr">
-        <is>
-          <t>bread-dahi-vadai</t>
-        </is>
-      </c>
-      <c r="D232" t="inlineStr">
-        <is>
-          <t>Bread Dahi Vadai</t>
-        </is>
-      </c>
-      <c r="E232" t="inlineStr">
-        <is>
-          <t>திடீர் பிரட் தயிர்வடை</t>
-        </is>
-      </c>
-      <c r="F232" t="inlineStr">
-        <is>
-          <t>vadai</t>
-        </is>
-      </c>
-      <c r="G232" t="inlineStr">
-        <is>
-          <t>A photorealistic close-up of small round bread-dough vadais topped generously with white curd, dusted with black salt, roasted cumin powder, and red chili powder, drizzled with brown sweet chutney and garnished with coriander leaves, bright appetizing lighting.</t>
-        </is>
-      </c>
-      <c r="H232" t="inlineStr">
-        <is>
-          <t>public/images/recipes/bread-dahi-vadai/featured.jpg</t>
-        </is>
-      </c>
-      <c r="I232" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="233">
-      <c r="A233" t="n">
-        <v>232</v>
-      </c>
-      <c r="B233" t="inlineStr">
-        <is>
-          <t>Vegetarian</t>
-        </is>
-      </c>
-      <c r="C233" t="inlineStr">
-        <is>
-          <t>moong-dhal-curd-pakoda</t>
-        </is>
-      </c>
-      <c r="D233" t="inlineStr">
-        <is>
-          <t>Moong Dhal Curd Pakoda</t>
-        </is>
-      </c>
-      <c r="E233" t="inlineStr">
-        <is>
-          <t>பயத்தம் பருப்பு தயிர் பக்கோடா</t>
-        </is>
-      </c>
-      <c r="F233" t="inlineStr">
-        <is>
-          <t>bajji</t>
-        </is>
-      </c>
-      <c r="G233" t="inlineStr">
-        <is>
-          <t>A photorealistic close-up of small golden fried lentil pakodas arranged on a plate, topped with a generous pour of white whisked curd, dusted with a dark spice powder and tomato sauce drizzle, bright lighting.</t>
-        </is>
-      </c>
-      <c r="H233" t="inlineStr">
-        <is>
-          <t>public/images/recipes/moong-dhal-curd-pakoda/featured.jpg</t>
-        </is>
-      </c>
-      <c r="I233" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="234">
-      <c r="A234" t="n">
-        <v>233</v>
-      </c>
-      <c r="B234" t="inlineStr">
-        <is>
-          <t>Vegetarian</t>
-        </is>
-      </c>
-      <c r="C234" t="inlineStr">
-        <is>
-          <t>mysore-vadai</t>
-        </is>
-      </c>
-      <c r="D234" t="inlineStr">
-        <is>
-          <t>Mysore Vadai</t>
-        </is>
-      </c>
-      <c r="E234" t="inlineStr">
-        <is>
-          <t>மைசூர் வடை</t>
-        </is>
-      </c>
-      <c r="F234" t="inlineStr">
-        <is>
-          <t>vadai</t>
-        </is>
-      </c>
-      <c r="G234" t="inlineStr">
-        <is>
-          <t>A photorealistic close-up of textured, coarse golden-brown vadais studded with visible cashew pieces and melon seeds, stacked on a plate, served with thokku, warm lighting.</t>
-        </is>
-      </c>
-      <c r="H234" t="inlineStr">
-        <is>
-          <t>public/images/recipes/mysore-vadai/featured.jpg</t>
-        </is>
-      </c>
-      <c r="I234" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="235">
-      <c r="A235" t="n">
-        <v>234</v>
-      </c>
-      <c r="B235" t="inlineStr">
-        <is>
-          <t>Vegetarian</t>
-        </is>
-      </c>
-      <c r="C235" t="inlineStr">
-        <is>
-          <t>madhur-vadai</t>
-        </is>
-      </c>
-      <c r="D235" t="inlineStr">
-        <is>
-          <t>Madhur Vadai</t>
-        </is>
-      </c>
-      <c r="E235" t="inlineStr">
-        <is>
-          <t>மதுர் வடை</t>
-        </is>
-      </c>
-      <c r="F235" t="inlineStr">
-        <is>
-          <t>vadai</t>
-        </is>
-      </c>
-      <c r="G235" t="inlineStr">
-        <is>
-          <t>A photorealistic photo of thin, flat, deep reddish-brown crispy discs with visible onion flecks, stacked in a glass jar and also arranged on a plate, matte crunchy texture, natural light.</t>
-        </is>
-      </c>
-      <c r="H235" t="inlineStr">
-        <is>
-          <t>public/images/recipes/madhur-vadai/featured.jpg</t>
-        </is>
-      </c>
-      <c r="I235" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="236">
-      <c r="A236" t="n">
-        <v>235</v>
-      </c>
-      <c r="B236" t="inlineStr">
-        <is>
-          <t>Vegetarian</t>
-        </is>
-      </c>
-      <c r="C236" t="inlineStr">
-        <is>
-          <t>masal-vadai</t>
-        </is>
-      </c>
-      <c r="D236" t="inlineStr">
-        <is>
-          <t>Masal Vadai</t>
-        </is>
-      </c>
-      <c r="E236" t="inlineStr">
-        <is>
-          <t>மசால் வடை</t>
-        </is>
-      </c>
-      <c r="F236" t="inlineStr">
-        <is>
-          <t>vadai</t>
-        </is>
-      </c>
-      <c r="G236" t="inlineStr">
-        <is>
-          <t>A photorealistic close-up of flat, coarse-textured golden-brown vadais with visible chana dal grains, onion, and curry leaf flecks, stacked on a banana leaf, served with coconut chutney, warm lighting.</t>
-        </is>
-      </c>
-      <c r="H236" t="inlineStr">
-        <is>
-          <t>public/images/recipes/masal-vadai/featured.jpg</t>
-        </is>
-      </c>
-      <c r="I236" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="237">
-      <c r="A237" t="n">
-        <v>236</v>
-      </c>
-      <c r="B237" t="inlineStr">
-        <is>
-          <t>Vegetarian</t>
-        </is>
-      </c>
-      <c r="C237" t="inlineStr">
-        <is>
-          <t>gherugu-vadai</t>
-        </is>
-      </c>
-      <c r="D237" t="inlineStr">
-        <is>
-          <t>Gherugu Vadai</t>
-        </is>
-      </c>
-      <c r="E237" t="inlineStr">
-        <is>
-          <t>கெருகு வடை</t>
-        </is>
-      </c>
-      <c r="F237" t="inlineStr">
-        <is>
-          <t>vadai</t>
-        </is>
-      </c>
-      <c r="G237" t="inlineStr">
-        <is>
-          <t>A photorealistic photo of thin, flat, pale golden crispy discs with a slightly speckled sesame-seed texture, stacked on a plate, rustic homely lighting.</t>
-        </is>
-      </c>
-      <c r="H237" t="inlineStr">
-        <is>
-          <t>public/images/recipes/gherugu-vadai/featured.jpg</t>
-        </is>
-      </c>
-      <c r="I237" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="238">
-      <c r="A238" t="n">
-        <v>237</v>
-      </c>
-      <c r="B238" t="inlineStr">
-        <is>
-          <t>Vegetarian</t>
-        </is>
-      </c>
-      <c r="C238" t="inlineStr">
-        <is>
-          <t>mullangi-vadai</t>
-        </is>
-      </c>
-      <c r="D238" t="inlineStr">
-        <is>
-          <t>Mullangi Vadai</t>
-        </is>
-      </c>
-      <c r="E238" t="inlineStr">
-        <is>
-          <t>முள்ளங்கி வடை</t>
-        </is>
-      </c>
-      <c r="F238" t="inlineStr">
-        <is>
-          <t>vadai</t>
-        </is>
-      </c>
-      <c r="G238" t="inlineStr">
-        <is>
-          <t>A photorealistic close-up of thin, flat, pale golden-brown vadais with visible shreds of white radish embedded in the crisp exterior, stacked on a steel plate, natural daylight.</t>
-        </is>
-      </c>
-      <c r="H238" t="inlineStr">
-        <is>
-          <t>public/images/recipes/mullangi-vadai/featured.jpg</t>
-        </is>
-      </c>
-      <c r="I238" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="239">
-      <c r="A239" t="n">
-        <v>238</v>
-      </c>
-      <c r="B239" t="inlineStr">
-        <is>
-          <t>Vegetarian</t>
-        </is>
-      </c>
-      <c r="C239" t="inlineStr">
-        <is>
-          <t>pulusu-vadai</t>
-        </is>
-      </c>
-      <c r="D239" t="inlineStr">
-        <is>
-          <t>Pulusu Vadai</t>
-        </is>
-      </c>
-      <c r="E239" t="inlineStr">
-        <is>
-          <t>புளி வடை அல்லது புலுசு வடை</t>
-        </is>
-      </c>
-      <c r="F239" t="inlineStr">
-        <is>
-          <t>vadai</t>
-        </is>
-      </c>
-      <c r="G239" t="inlineStr">
-        <is>
-          <t>A photorealistic photo of flat reddish-orange vadais with a speckled texture from ground red chili and pumpkin, stacked on a plate, tangy glossy sheen, warm lighting.</t>
-        </is>
-      </c>
-      <c r="H239" t="inlineStr">
-        <is>
-          <t>public/images/recipes/pulusu-vadai/featured.jpg</t>
-        </is>
-      </c>
-      <c r="I239" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="240">
-      <c r="A240" t="n">
-        <v>239</v>
-      </c>
-      <c r="B240" t="inlineStr">
-        <is>
-          <t>Vegetarian</t>
-        </is>
-      </c>
-      <c r="C240" t="inlineStr">
-        <is>
-          <t>milagu-vadai</t>
-        </is>
-      </c>
-      <c r="D240" t="inlineStr">
-        <is>
-          <t>Milagu Vadai</t>
-        </is>
-      </c>
-      <c r="E240" t="inlineStr">
-        <is>
-          <t>மிளகு வடை</t>
-        </is>
-      </c>
-      <c r="F240" t="inlineStr">
-        <is>
-          <t>vadai</t>
-        </is>
-      </c>
-      <c r="G240" t="inlineStr">
-        <is>
-          <t>A photorealistic close-up of small pale golden vadais with visible flecks of cracked black pepper, some strung together on a thread like a garland, others piled on a plate, temple-offering style presentation, warm devotional lighting.</t>
-        </is>
-      </c>
-      <c r="H240" t="inlineStr">
-        <is>
-          <t>public/images/recipes/milagu-vadai/featured.jpg</t>
-        </is>
-      </c>
-      <c r="I240" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="241">
-      <c r="A241" t="n">
-        <v>240</v>
-      </c>
-      <c r="B241" t="inlineStr">
-        <is>
-          <t>Vegetarian</t>
-        </is>
-      </c>
-      <c r="C241" t="inlineStr">
-        <is>
-          <t>drumstick-vadai</t>
-        </is>
-      </c>
-      <c r="D241" t="inlineStr">
-        <is>
-          <t>Drumstick Vadai</t>
-        </is>
-      </c>
-      <c r="E241" t="inlineStr">
-        <is>
-          <t>முருங்கைக்காய் வடை</t>
-        </is>
-      </c>
-      <c r="F241" t="inlineStr">
-        <is>
-          <t>vadai</t>
-        </is>
-      </c>
-      <c r="G241" t="inlineStr">
-        <is>
-          <t>A photorealistic close-up of coarse, flat golden-brown vadais with a slightly speckled surface, stacked on a plate, served with vinegar-tossed onion rings on the side, warm lighting.</t>
-        </is>
-      </c>
-      <c r="H241" t="inlineStr">
-        <is>
-          <t>public/images/recipes/drumstick-vadai/featured.jpg</t>
-        </is>
-      </c>
-      <c r="I241" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="242">
-      <c r="A242" t="n">
-        <v>241</v>
-      </c>
-      <c r="B242" t="inlineStr">
-        <is>
-          <t>Vegetarian</t>
-        </is>
-      </c>
-      <c r="C242" t="inlineStr">
-        <is>
-          <t>perugu-vadai</t>
-        </is>
-      </c>
-      <c r="D242" t="inlineStr">
-        <is>
-          <t>Perugu Vadai</t>
-        </is>
-      </c>
-      <c r="E242" t="inlineStr">
-        <is>
-          <t>பெருகு வடை</t>
-        </is>
-      </c>
-      <c r="F242" t="inlineStr">
-        <is>
-          <t>vadai</t>
-        </is>
-      </c>
-      <c r="G242" t="inlineStr">
-        <is>
-          <t>A photorealistic photo of soft, pale, lightly golden flat discs with a matte soft surface (not deeply fried), stacked on a plate, gentle lighting emphasizing their softness.</t>
-        </is>
-      </c>
-      <c r="H242" t="inlineStr">
-        <is>
-          <t>public/images/recipes/perugu-vadai/featured.jpg</t>
-        </is>
-      </c>
-      <c r="I242" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="243">
-      <c r="A243" t="n">
-        <v>242</v>
-      </c>
-      <c r="B243" t="inlineStr">
-        <is>
-          <t>Vegetarian</t>
-        </is>
-      </c>
-      <c r="C243" t="inlineStr">
-        <is>
-          <t>moong-dhal-toast</t>
-        </is>
-      </c>
-      <c r="D243" t="inlineStr">
-        <is>
-          <t>Moong Dhal Toast</t>
-        </is>
-      </c>
-      <c r="E243" t="inlineStr">
-        <is>
-          <t>பயத்தம்பருப்பு டோஸ்ட்</t>
-        </is>
-      </c>
-      <c r="F243" t="inlineStr">
-        <is>
-          <t>sandwich</t>
-        </is>
-      </c>
-      <c r="G243" t="inlineStr">
-        <is>
-          <t>A photorealistic close-up of a golden-brown fried bread toast cut diagonally, showing a thin green mint chutney layer and a yellow lentil paste layer between the crisp bread surface and the crust, plated with tomato sauce, bright lighting.</t>
-        </is>
-      </c>
-      <c r="H243" t="inlineStr">
-        <is>
-          <t>public/images/recipes/moong-dhal-toast/featured.jpg</t>
-        </is>
-      </c>
-      <c r="I243" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="244">
-      <c r="A244" t="n">
-        <v>243</v>
-      </c>
-      <c r="B244" t="inlineStr">
-        <is>
-          <t>Vegetarian</t>
-        </is>
-      </c>
-      <c r="C244" t="inlineStr">
-        <is>
-          <t>masala-toast</t>
-        </is>
-      </c>
-      <c r="D244" t="inlineStr">
-        <is>
-          <t>Masala Toast</t>
-        </is>
-      </c>
-      <c r="E244" t="inlineStr">
-        <is>
-          <t>மசாலா டோஸ்ட்</t>
-        </is>
-      </c>
-      <c r="F244" t="inlineStr">
-        <is>
-          <t>sandwich</t>
-        </is>
-      </c>
-      <c r="G244" t="inlineStr">
-        <is>
-          <t>A photorealistic photo of golden-brown toasted bread slices with a thin reddish-brown spice chutney visible on the surface, griddle-toasted with light char marks, stacked on a plate, warm lighting.</t>
-        </is>
-      </c>
-      <c r="H244" t="inlineStr">
-        <is>
-          <t>public/images/recipes/masala-toast/featured.jpg</t>
-        </is>
-      </c>
-      <c r="I244" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="245">
-      <c r="A245" t="n">
-        <v>244</v>
-      </c>
-      <c r="B245" t="inlineStr">
-        <is>
-          <t>Vegetarian</t>
-        </is>
-      </c>
-      <c r="C245" t="inlineStr">
-        <is>
-          <t>tomato-toast</t>
-        </is>
-      </c>
-      <c r="D245" t="inlineStr">
-        <is>
-          <t>Tomato Toast</t>
-        </is>
-      </c>
-      <c r="E245" t="inlineStr">
-        <is>
-          <t>தக்காளி டோஸ்ட்</t>
-        </is>
-      </c>
-      <c r="F245" t="inlineStr">
-        <is>
-          <t>sandwich</t>
-        </is>
-      </c>
-      <c r="G245" t="inlineStr">
-        <is>
-          <t>A photorealistic close-up of a golden-toasted bread slice topped with a glossy reddish-orange cooked tomato-onion masala spread evenly across the surface, slightly caramelized edges, plated hot, warm kitchen lighting.</t>
-        </is>
-      </c>
-      <c r="H245" t="inlineStr">
-        <is>
-          <t>public/images/recipes/tomato-toast/featured.jpg</t>
-        </is>
-      </c>
-      <c r="I245" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="246">
-      <c r="A246" t="n">
-        <v>245</v>
-      </c>
-      <c r="B246" t="inlineStr">
-        <is>
-          <t>Vegetarian</t>
-        </is>
-      </c>
-      <c r="C246" t="inlineStr">
-        <is>
-          <t>potato-sandwich</t>
-        </is>
-      </c>
-      <c r="D246" t="inlineStr">
-        <is>
-          <t>Potato Sandwich</t>
-        </is>
-      </c>
-      <c r="E246" t="inlineStr">
-        <is>
-          <t>உருளைக்கிழங்கு பிரட் சாண்ட்விச்</t>
-        </is>
-      </c>
-      <c r="F246" t="inlineStr">
-        <is>
-          <t>sandwich</t>
-        </is>
-      </c>
-      <c r="G246" t="inlineStr">
-        <is>
-          <t>A photorealistic close-up of a golden-brown griddle-fried sandwich cut diagonally, showing a thick yellow spiced-potato filling coated in crisp bread crumbs between the toasted bread layers, plated with ketchup, bright appetizing lighting.</t>
-        </is>
-      </c>
-      <c r="H246" t="inlineStr">
-        <is>
-          <t>public/images/recipes/potato-sandwich/featured.jpg</t>
-        </is>
-      </c>
-      <c r="I246" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="247">
-      <c r="A247" t="n">
-        <v>246</v>
-      </c>
-      <c r="B247" t="inlineStr">
-        <is>
-          <t>Vegetarian</t>
-        </is>
-      </c>
-      <c r="C247" t="inlineStr">
-        <is>
-          <t>corn-sandwich</t>
-        </is>
-      </c>
-      <c r="D247" t="inlineStr">
-        <is>
-          <t>Corn Sandwich</t>
-        </is>
-      </c>
-      <c r="E247" t="inlineStr">
-        <is>
-          <t>மக்காச்சோள சாண்ட்விச்</t>
-        </is>
-      </c>
-      <c r="F247" t="inlineStr">
-        <is>
-          <t>sandwich</t>
-        </is>
-      </c>
-      <c r="G247" t="inlineStr">
-        <is>
-          <t>A photorealistic photo of an open-faced toast topped with golden corn kernels mixed with cream, and a layer of melted golden cheese bubbling on top, baked and lightly browned, warm oven-fresh lighting.</t>
-        </is>
-      </c>
-      <c r="H247" t="inlineStr">
-        <is>
-          <t>public/images/recipes/corn-sandwich/featured.jpg</t>
-        </is>
-      </c>
-      <c r="I247" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="248">
-      <c r="A248" t="n">
-        <v>247</v>
-      </c>
-      <c r="B248" t="inlineStr">
-        <is>
-          <t>Vegetarian</t>
-        </is>
-      </c>
-      <c r="C248" t="inlineStr">
-        <is>
-          <t>tomato-ketchup</t>
-        </is>
-      </c>
-      <c r="D248" t="inlineStr">
-        <is>
-          <t>Tomato Ketchup</t>
-        </is>
-      </c>
-      <c r="E248" t="inlineStr">
-        <is>
-          <t>தக்காளி கெட்ச்அப்</t>
-        </is>
-      </c>
-      <c r="F248" t="inlineStr">
-        <is>
-          <t>chutney</t>
-        </is>
-      </c>
-      <c r="G248" t="inlineStr">
-        <is>
-          <t>A photorealistic close-up of a clear glass bottle filled with thick, deep-red glossy homemade tomato ketchup, a spoonful pooled beside it on a white plate showing its smooth, thick consistency, bright clean lighting.</t>
-        </is>
-      </c>
-      <c r="H248" t="inlineStr">
-        <is>
-          <t>public/images/recipes/tomato-ketchup/featured.jpg</t>
-        </is>
-      </c>
-      <c r="I248" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="249">
-      <c r="A249" t="n">
-        <v>248</v>
-      </c>
-      <c r="B249" t="inlineStr">
-        <is>
-          <t>Vegetarian</t>
-        </is>
-      </c>
-      <c r="C249" t="inlineStr">
-        <is>
-          <t>vegetable-sandwich</t>
-        </is>
-      </c>
-      <c r="D249" t="inlineStr">
-        <is>
-          <t>Vegetable Sandwich</t>
-        </is>
-      </c>
-      <c r="E249" t="inlineStr">
-        <is>
-          <t>காய்கறி சாண்ட்விச்</t>
-        </is>
-      </c>
-      <c r="F249" t="inlineStr">
-        <is>
-          <t>sandwich</t>
-        </is>
-      </c>
-      <c r="G249" t="inlineStr">
-        <is>
-          <t>A photorealistic close-up of a triangle-cut sandwich showing distinct colorful layers of thin cucumber, carrot, tomato, and onion rounds between green mint-chutney-spread bread, fresh and vibrant, natural bright lighting.</t>
-        </is>
-      </c>
-      <c r="H249" t="inlineStr">
-        <is>
-          <t>public/images/recipes/vegetable-sandwich/featured.jpg</t>
-        </is>
-      </c>
-      <c r="I249" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="250">
-      <c r="A250" t="n">
-        <v>249</v>
-      </c>
-      <c r="B250" t="inlineStr">
-        <is>
-          <t>Vegetarian</t>
-        </is>
-      </c>
-      <c r="C250" t="inlineStr">
-        <is>
-          <t>chilli-cheese-sandwich</t>
-        </is>
-      </c>
-      <c r="D250" t="inlineStr">
-        <is>
-          <t>Chilli Cheese Sandwich</t>
-        </is>
-      </c>
-      <c r="E250" t="inlineStr">
-        <is>
-          <t>சில்லி சீஸ் சாண்ட்விச்</t>
-        </is>
-      </c>
-      <c r="F250" t="inlineStr">
-        <is>
-          <t>sandwich</t>
-        </is>
-      </c>
-      <c r="G250" t="inlineStr">
-        <is>
-          <t>A photorealistic close-up of a golden toasted sandwich cut in half, oozing melted golden cheese mixed with visible flecks of green chili and onion between the crisp bread layers, warm appetizing lighting.</t>
-        </is>
-      </c>
-      <c r="H250" t="inlineStr">
-        <is>
-          <t>public/images/recipes/chilli-cheese-sandwich/featured.jpg</t>
-        </is>
-      </c>
-      <c r="I250" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="251">
-      <c r="A251" t="n">
-        <v>250</v>
-      </c>
-      <c r="B251" t="inlineStr">
-        <is>
-          <t>Vegetarian</t>
-        </is>
-      </c>
-      <c r="C251" t="inlineStr">
-        <is>
-          <t>paneer-sandwich</t>
-        </is>
-      </c>
-      <c r="D251" t="inlineStr">
-        <is>
-          <t>Paneer Sandwich</t>
-        </is>
-      </c>
-      <c r="E251" t="inlineStr">
-        <is>
-          <t>பாலாடைக்கட்டி சாண்ட்விச்</t>
-        </is>
-      </c>
-      <c r="F251" t="inlineStr">
-        <is>
-          <t>sandwich</t>
-        </is>
-      </c>
-      <c r="G251" t="inlineStr">
-        <is>
-          <t>A photorealistic close-up of a golden toasted sandwich cut diagonally, showing a crumbly white paneer filling studded with green sprouts and herbs between the bread layers, plated with ketchup, bright lighting.</t>
-        </is>
-      </c>
-      <c r="H251" t="inlineStr">
-        <is>
-          <t>public/images/recipes/paneer-sandwich/featured.jpg</t>
-        </is>
-      </c>
-      <c r="I251" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="252">
-      <c r="A252" t="n">
-        <v>251</v>
-      </c>
-      <c r="B252" t="inlineStr">
-        <is>
-          <t>Vegetarian</t>
-        </is>
-      </c>
-      <c r="C252" t="inlineStr">
-        <is>
-          <t>sandwich-roll</t>
-        </is>
-      </c>
-      <c r="D252" t="inlineStr">
-        <is>
-          <t>Sandwich Roll</t>
-        </is>
-      </c>
-      <c r="E252" t="inlineStr">
-        <is>
-          <t>சாண்ட்விட்ச் ரோல்</t>
-        </is>
-      </c>
-      <c r="F252" t="inlineStr">
-        <is>
-          <t>sandwich</t>
-        </is>
-      </c>
-      <c r="G252" t="inlineStr">
-        <is>
-          <t>A photorealistic close-up of pinwheel-shaped bread roll slices arranged on a plate, showing a spiral of white bread with thin green and red chutney swirls visible in the layers, elegant party-platter presentation, bright clean lighting.</t>
-        </is>
-      </c>
-      <c r="H252" t="inlineStr">
-        <is>
-          <t>public/images/recipes/sandwich-roll/featured.jpg</t>
-        </is>
-      </c>
-      <c r="I252" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="253">
-      <c r="A253" t="n">
-        <v>252</v>
-      </c>
-      <c r="B253" t="inlineStr">
-        <is>
-          <t>Vegetarian</t>
-        </is>
-      </c>
-      <c r="C253" t="inlineStr">
-        <is>
-          <t>aloo-chat-1</t>
-        </is>
-      </c>
-      <c r="D253" t="inlineStr">
-        <is>
-          <t>Aloo Chat 1</t>
-        </is>
-      </c>
-      <c r="E253" t="inlineStr">
-        <is>
-          <t>ஆலு சாட் - 1</t>
-        </is>
-      </c>
-      <c r="F253" t="inlineStr">
-        <is>
-          <t>chaat</t>
-        </is>
-      </c>
-      <c r="G253" t="inlineStr">
-        <is>
-          <t>A photorealistic close-up of a boiled potato stuffed and topped generously with white whisked curd, drizzled with dark brown tangy tamarind sauce, dusted with red chili powder and dark chat masala, garnished with coriander leaves, served on a decorative plate, vibrant street-food lighting.</t>
-        </is>
-      </c>
-      <c r="H253" t="inlineStr">
-        <is>
-          <t>public/images/recipes/aloo-chat-1/featured.jpg</t>
-        </is>
-      </c>
-      <c r="I253" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="254">
-      <c r="A254" t="n">
-        <v>253</v>
-      </c>
-      <c r="B254" t="inlineStr">
-        <is>
-          <t>Vegetarian</t>
-        </is>
-      </c>
-      <c r="C254" t="inlineStr">
-        <is>
-          <t>aloo-chat-2</t>
-        </is>
-      </c>
-      <c r="D254" t="inlineStr">
-        <is>
-          <t>Aloo Chat 2</t>
-        </is>
-      </c>
-      <c r="E254" t="inlineStr">
-        <is>
-          <t>ஆலு சாட் - 2</t>
-        </is>
-      </c>
-      <c r="F254" t="inlineStr">
-        <is>
-          <t>chaat</t>
-        </is>
-      </c>
-      <c r="G254" t="inlineStr">
-        <is>
-          <t>A photorealistic photo of diced potato mixed with golden fried diamond-shaped crisps, tossed in a chat bowl with dark tangy sauce, chopped onion, and a scattering of thin crispy sev on top, colorful street-food presentation, bright lighting.</t>
-        </is>
-      </c>
-      <c r="H254" t="inlineStr">
-        <is>
-          <t>public/images/recipes/aloo-chat-2/featured.jpg</t>
-        </is>
-      </c>
-      <c r="I254" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="255">
-      <c r="A255" t="n">
-        <v>254</v>
-      </c>
-      <c r="B255" t="inlineStr">
-        <is>
-          <t>Vegetarian</t>
-        </is>
-      </c>
-      <c r="C255" t="inlineStr">
-        <is>
-          <t>chat-masala-powder</t>
-        </is>
-      </c>
-      <c r="D255" t="inlineStr">
-        <is>
-          <t>Chat Masala Powder</t>
-        </is>
-      </c>
-      <c r="E255" t="inlineStr">
-        <is>
-          <t>சாட் மசாலா பவுடர்</t>
-        </is>
-      </c>
-      <c r="F255" t="inlineStr">
-        <is>
-          <t>chaat</t>
-        </is>
-      </c>
-      <c r="G255" t="inlineStr">
-        <is>
-          <t>A photorealistic close-up of a small glass jar filled with reddish-brown aromatic spice powder, a small mound of the powder spilled beside it on a wooden surface with whole dried red chilies and cardamom pods scattered around, warm spice-market lighting.</t>
-        </is>
-      </c>
-      <c r="H255" t="inlineStr">
-        <is>
-          <t>public/images/recipes/chat-masala-powder/featured.jpg</t>
-        </is>
-      </c>
-      <c r="I255" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="256">
-      <c r="A256" t="n">
-        <v>255</v>
-      </c>
-      <c r="B256" t="inlineStr">
-        <is>
-          <t>Vegetarian</t>
-        </is>
-      </c>
-      <c r="C256" t="inlineStr">
-        <is>
-          <t>aloo-pappad-chat</t>
-        </is>
-      </c>
-      <c r="D256" t="inlineStr">
-        <is>
-          <t>Aloo Pappad Chat</t>
-        </is>
-      </c>
-      <c r="E256" t="inlineStr">
-        <is>
-          <t>ஆலு பப்பட் சாட்</t>
-        </is>
-      </c>
-      <c r="F256" t="inlineStr">
-        <is>
-          <t>chaat</t>
-        </is>
-      </c>
-      <c r="G256" t="inlineStr">
-        <is>
-          <t>A photorealistic close-up of a plate layered with crushed golden fried papad pieces, topped with diced potato, a generous pour of white curd, dark brown sweet chutney drizzle, and a dusting of spices with fresh coriander on top, vibrant street-food lighting.</t>
-        </is>
-      </c>
-      <c r="H256" t="inlineStr">
-        <is>
-          <t>public/images/recipes/aloo-pappad-chat/featured.jpg</t>
-        </is>
-      </c>
-      <c r="I256" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="257">
-      <c r="A257" t="n">
-        <v>256</v>
-      </c>
-      <c r="B257" t="inlineStr">
-        <is>
-          <t>Vegetarian</t>
-        </is>
-      </c>
-      <c r="C257" t="inlineStr">
-        <is>
-          <t>mattar-chat</t>
-        </is>
-      </c>
-      <c r="D257" t="inlineStr">
-        <is>
-          <t>Mattar Chat</t>
-        </is>
-      </c>
-      <c r="E257" t="inlineStr">
-        <is>
-          <t>பச்சைப் பட்டாணி சாட்</t>
-        </is>
-      </c>
-      <c r="F257" t="inlineStr">
-        <is>
-          <t>chaat</t>
-        </is>
-      </c>
-      <c r="G257" t="inlineStr">
-        <is>
-          <t>A photorealistic close-up of a bowl of cooked green peas topped with crushed golden puri pieces, white curd, dark tamarind chutney, chopped onion, and fine crispy sev, colorful layered presentation, bright lighting.</t>
-        </is>
-      </c>
-      <c r="H257" t="inlineStr">
-        <is>
-          <t>public/images/recipes/mattar-chat/featured.jpg</t>
-        </is>
-      </c>
-      <c r="I257" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="258">
-      <c r="A258" t="n">
-        <v>257</v>
-      </c>
-      <c r="B258" t="inlineStr">
-        <is>
-          <t>Vegetarian</t>
-        </is>
-      </c>
-      <c r="C258" t="inlineStr">
-        <is>
-          <t>fruit-vegetable-chat</t>
-        </is>
-      </c>
-      <c r="D258" t="inlineStr">
-        <is>
-          <t>Fruit &amp; Vegetable Chat</t>
-        </is>
-      </c>
-      <c r="E258" t="inlineStr">
-        <is>
-          <t>காய்கறி, பழக்கலவை சாட்</t>
-        </is>
-      </c>
-      <c r="F258" t="inlineStr">
-        <is>
-          <t>chaat</t>
-        </is>
-      </c>
-      <c r="G258" t="inlineStr">
-        <is>
-          <t>A photorealistic photo of a colorful bowl mix of diced banana, orange segments, tomato, potato, and guava tossed together, garnished with coriander leaves and a light dusting of chat masala, fresh and vibrant, bright natural lighting.</t>
-        </is>
-      </c>
-      <c r="H258" t="inlineStr">
-        <is>
-          <t>public/images/recipes/fruit-vegetable-chat/featured.jpg</t>
-        </is>
-      </c>
-      <c r="I258" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="259">
-      <c r="A259" t="n">
-        <v>258</v>
-      </c>
-      <c r="B259" t="inlineStr">
-        <is>
-          <t>Vegetarian</t>
-        </is>
-      </c>
-      <c r="C259" t="inlineStr">
-        <is>
-          <t>finger-chips</t>
-        </is>
-      </c>
-      <c r="D259" t="inlineStr">
-        <is>
-          <t>Finger Chips</t>
-        </is>
-      </c>
-      <c r="E259" t="inlineStr">
-        <is>
-          <t>ஃபிங்கர் சிப்ஸ்</t>
-        </is>
-      </c>
-      <c r="F259" t="inlineStr">
-        <is>
-          <t>snack</t>
-        </is>
-      </c>
-      <c r="G259" t="inlineStr">
-        <is>
-          <t>A photorealistic close-up of golden-brown crispy potato finger chips piled high on a plate, lightly dusted with salt and pepper, served with tomato ketchup, bright appetizing lighting.</t>
-        </is>
-      </c>
-      <c r="H259" t="inlineStr">
-        <is>
-          <t>public/images/recipes/finger-chips/featured.jpg</t>
-        </is>
-      </c>
-      <c r="I259" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="260">
-      <c r="A260" t="n">
-        <v>259</v>
-      </c>
-      <c r="B260" t="inlineStr">
-        <is>
-          <t>Vegetarian</t>
-        </is>
-      </c>
-      <c r="C260" t="inlineStr">
-        <is>
-          <t>crisp-groundnuts</t>
-        </is>
-      </c>
-      <c r="D260" t="inlineStr">
-        <is>
-          <t>Crisp Groundnuts</t>
-        </is>
-      </c>
-      <c r="E260" t="inlineStr">
-        <is>
-          <t>வறுகடலை</t>
-        </is>
-      </c>
-      <c r="F260" t="inlineStr">
-        <is>
-          <t>snack</t>
-        </is>
-      </c>
-      <c r="G260" t="inlineStr">
-        <is>
-          <t>A photorealistic close-up of small glossy, deep golden-brown fried groundnuts piled in a bowl, with a visible shiny sheen, some scattered on a napkin, warm snack-time lighting.</t>
-        </is>
-      </c>
-      <c r="H260" t="inlineStr">
-        <is>
-          <t>public/images/recipes/crisp-groundnuts/featured.jpg</t>
-        </is>
-      </c>
-      <c r="I260" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="261">
-      <c r="A261" t="n">
-        <v>260</v>
-      </c>
-      <c r="B261" t="inlineStr">
-        <is>
-          <t>Vegetarian</t>
-        </is>
-      </c>
-      <c r="C261" t="inlineStr">
-        <is>
-          <t>pop-corn</t>
-        </is>
-      </c>
-      <c r="D261" t="inlineStr">
-        <is>
-          <t>Pop Corn</t>
-        </is>
-      </c>
-      <c r="E261" t="inlineStr">
-        <is>
-          <t>பாப் கார்ன்</t>
-        </is>
-      </c>
-      <c r="F261" t="inlineStr">
-        <is>
-          <t>snack</t>
-        </is>
-      </c>
-      <c r="G261" t="inlineStr">
-        <is>
-          <t>A photorealistic close-up of a bowl overflowing with fluffy white popcorn lightly dusted with orange-red spice seasoning, warm cozy lighting.</t>
-        </is>
-      </c>
-      <c r="H261" t="inlineStr">
-        <is>
-          <t>public/images/recipes/pop-corn/featured.jpg</t>
-        </is>
-      </c>
-      <c r="I261" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="262">
-      <c r="A262" t="n">
-        <v>261</v>
-      </c>
-      <c r="B262" t="inlineStr">
-        <is>
-          <t>Vegetarian</t>
-        </is>
-      </c>
-      <c r="C262" t="inlineStr">
-        <is>
-          <t>masala-pori-1</t>
-        </is>
-      </c>
-      <c r="D262" t="inlineStr">
-        <is>
-          <t>Masala Pori 1 (Instant Bhel)</t>
-        </is>
-      </c>
-      <c r="E262" t="inlineStr">
-        <is>
-          <t>மசாலா பொரி - 1</t>
-        </is>
-      </c>
-      <c r="F262" t="inlineStr">
-        <is>
-          <t>chaat</t>
-        </is>
-      </c>
-      <c r="G262" t="inlineStr">
-        <is>
-          <t>A photorealistic photo of a colorful bowl of puffed rice mixed with roasted gram, small dice of mango, tomato, carrot, and beetroot, garnished with coriander leaves, bright vibrant street-food lighting.</t>
-        </is>
-      </c>
-      <c r="H262" t="inlineStr">
-        <is>
-          <t>public/images/recipes/masala-pori-1/featured.jpg</t>
-        </is>
-      </c>
-      <c r="I262" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="263">
-      <c r="A263" t="n">
-        <v>262</v>
-      </c>
-      <c r="B263" t="inlineStr">
-        <is>
-          <t>Vegetarian</t>
-        </is>
-      </c>
-      <c r="C263" t="inlineStr">
-        <is>
-          <t>masala-pori-2</t>
-        </is>
-      </c>
-      <c r="D263" t="inlineStr">
-        <is>
-          <t>Masala Pori 2 (Instant Bhel)</t>
-        </is>
-      </c>
-      <c r="E263" t="inlineStr">
-        <is>
-          <t>மசாலா பொரி - 2</t>
-        </is>
-      </c>
-      <c r="F263" t="inlineStr">
-        <is>
-          <t>chaat</t>
-        </is>
-      </c>
-      <c r="G263" t="inlineStr">
-        <is>
-          <t>A photorealistic photo of a bowl of puffed rice mixed with roasted gram and groundnuts, tossed with pink-tinged marinated onion and a drizzle of dark green chutney, colorful and fresh, bright lighting.</t>
-        </is>
-      </c>
-      <c r="H263" t="inlineStr">
-        <is>
-          <t>public/images/recipes/masala-pori-2/featured.jpg</t>
-        </is>
-      </c>
-      <c r="I263" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="264">
-      <c r="A264" t="n">
-        <v>263</v>
-      </c>
-      <c r="B264" t="inlineStr">
-        <is>
-          <t>Vegetarian</t>
-        </is>
-      </c>
-      <c r="C264" t="inlineStr">
-        <is>
-          <t>mint-coriander-chutney-cutlets</t>
-        </is>
-      </c>
-      <c r="D264" t="inlineStr">
-        <is>
-          <t>Mint-Coriander Chutney (for Cutlets)</t>
-        </is>
-      </c>
-      <c r="E264" t="inlineStr">
-        <is>
-          <t>புதினா, கொத்தமல்லி சட்னி (கட்லெட்டிற்கு)</t>
-        </is>
-      </c>
-      <c r="F264" t="inlineStr">
-        <is>
-          <t>chutney</t>
-        </is>
-      </c>
-      <c r="G264" t="inlineStr">
-        <is>
-          <t>A photorealistic close-up of a small bowl of smooth, vivid green chutney with a glossy sheen, served beside golden fried cutlets, garnished with a mint sprig, bright fresh lighting.</t>
-        </is>
-      </c>
-      <c r="H264" t="inlineStr">
-        <is>
-          <t>public/images/recipes/mint-coriander-chutney-cutlets/featured.jpg</t>
-        </is>
-      </c>
-      <c r="I264" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="265">
-      <c r="A265" t="n">
-        <v>264</v>
-      </c>
-      <c r="B265" t="inlineStr">
-        <is>
-          <t>Vegetarian</t>
-        </is>
-      </c>
-      <c r="C265" t="inlineStr">
-        <is>
-          <t>mint-chutney-cutlets</t>
-        </is>
-      </c>
-      <c r="D265" t="inlineStr">
-        <is>
-          <t>Mint Chutney (for Cutlets)</t>
-        </is>
-      </c>
-      <c r="E265" t="inlineStr">
-        <is>
-          <t>புதினா சட்னி (கட்லெட்டிற்கு)</t>
-        </is>
-      </c>
-      <c r="F265" t="inlineStr">
-        <is>
-          <t>chutney</t>
-        </is>
-      </c>
-      <c r="G265" t="inlineStr">
-        <is>
-          <t>A photorealistic close-up of a small bowl of dark green, thick chutney with a tempered mustard-seed garnish floating on top, bright natural lighting.</t>
-        </is>
-      </c>
-      <c r="H265" t="inlineStr">
-        <is>
-          <t>public/images/recipes/mint-chutney-cutlets/featured.jpg</t>
-        </is>
-      </c>
-      <c r="I265" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="266">
-      <c r="A266" t="n">
-        <v>265</v>
-      </c>
-      <c r="B266" t="inlineStr">
-        <is>
-          <t>Vegetarian</t>
-        </is>
-      </c>
-      <c r="C266" t="inlineStr">
-        <is>
-          <t>mint-onion-chutney</t>
-        </is>
-      </c>
-      <c r="D266" t="inlineStr">
-        <is>
-          <t>Mint-Onion Chutney</t>
-        </is>
-      </c>
-      <c r="E266" t="inlineStr">
-        <is>
-          <t>புதினா வெங்காயச் சட்னி</t>
-        </is>
-      </c>
-      <c r="F266" t="inlineStr">
-        <is>
-          <t>chutney</t>
-        </is>
-      </c>
-      <c r="G266" t="inlineStr">
-        <is>
-          <t>A photorealistic close-up of a bowl of textured dark green chutney flecked with white coconut, garnished with a tempering of mustard seeds and curry leaves on top, warm lighting.</t>
-        </is>
-      </c>
-      <c r="H266" t="inlineStr">
-        <is>
-          <t>public/images/recipes/mint-onion-chutney/featured.jpg</t>
-        </is>
-      </c>
-      <c r="I266" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="267">
-      <c r="A267" t="n">
-        <v>266</v>
-      </c>
-      <c r="B267" t="inlineStr">
-        <is>
-          <t>Vegetarian</t>
-        </is>
-      </c>
-      <c r="C267" t="inlineStr">
-        <is>
-          <t>coriander-chutney-sandwiches</t>
-        </is>
-      </c>
-      <c r="D267" t="inlineStr">
-        <is>
-          <t>Coriander Chutney (for Sandwiches)</t>
-        </is>
-      </c>
-      <c r="E267" t="inlineStr">
-        <is>
-          <t>கொத்தமல்லி சட்னி (சாண்ட்விச்சிற்கு)</t>
-        </is>
-      </c>
-      <c r="F267" t="inlineStr">
-        <is>
-          <t>chutney</t>
-        </is>
-      </c>
-      <c r="G267" t="inlineStr">
-        <is>
-          <t>A photorealistic close-up of a small bowl of deep green-red chutney with a thick, spreadable texture, a butter knife resting beside it with chutney on the blade, bright kitchen lighting.</t>
-        </is>
-      </c>
-      <c r="H267" t="inlineStr">
-        <is>
-          <t>public/images/recipes/coriander-chutney-sandwiches/featured.jpg</t>
-        </is>
-      </c>
-      <c r="I267" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="268">
-      <c r="A268" t="n">
-        <v>267</v>
-      </c>
-      <c r="B268" t="inlineStr">
-        <is>
-          <t>Vegetarian</t>
-        </is>
-      </c>
-      <c r="C268" t="inlineStr">
-        <is>
-          <t>garlic-chutney-sandwiches</t>
-        </is>
-      </c>
-      <c r="D268" t="inlineStr">
-        <is>
-          <t>Garlic Chutney (for Sandwiches)</t>
-        </is>
-      </c>
-      <c r="E268" t="inlineStr">
-        <is>
-          <t>பூண்டு சட்னி (சாண்ட்விச்சிற்கு)</t>
-        </is>
-      </c>
-      <c r="F268" t="inlineStr">
-        <is>
-          <t>chutney</t>
-        </is>
-      </c>
-      <c r="G268" t="inlineStr">
-        <is>
-          <t>A photorealistic close-up of a bowl of reddish-brown chutney with visible garlic and chili flecks, thick and glossy, served beside buttered bread slices, warm lighting.</t>
-        </is>
-      </c>
-      <c r="H268" t="inlineStr">
-        <is>
-          <t>public/images/recipes/garlic-chutney-sandwiches/featured.jpg</t>
-        </is>
-      </c>
-      <c r="I268" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="269">
-      <c r="A269" t="n">
-        <v>268</v>
-      </c>
-      <c r="B269" t="inlineStr">
-        <is>
-          <t>Vegetarian</t>
-        </is>
-      </c>
-      <c r="C269" t="inlineStr">
-        <is>
-          <t>coconut-ginger-chutney-sandwiches</t>
-        </is>
-      </c>
-      <c r="D269" t="inlineStr">
-        <is>
-          <t>Coconut-Ginger Chutney (for Sandwiches)</t>
-        </is>
-      </c>
-      <c r="E269" t="inlineStr">
-        <is>
-          <t>தேங்காய், இஞ்சி சட்னி (சாண்ட்விச்சிற்கு)</t>
-        </is>
-      </c>
-      <c r="F269" t="inlineStr">
-        <is>
-          <t>chutney</t>
-        </is>
-      </c>
-      <c r="G269" t="inlineStr">
-        <is>
-          <t>A photorealistic close-up of a bowl of coarse, off-white coconut chutney with visible ginger and red chili flecks, glossy texture, natural bright lighting.</t>
-        </is>
-      </c>
-      <c r="H269" t="inlineStr">
-        <is>
-          <t>public/images/recipes/coconut-ginger-chutney-sandwiches/featured.jpg</t>
-        </is>
-      </c>
-      <c r="I269" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="270">
-      <c r="A270" t="n">
-        <v>269</v>
-      </c>
-      <c r="B270" t="inlineStr">
-        <is>
-          <t>Vegetarian</t>
-        </is>
-      </c>
-      <c r="C270" t="inlineStr">
-        <is>
-          <t>mint-chutney-sandwiches</t>
-        </is>
-      </c>
-      <c r="D270" t="inlineStr">
-        <is>
-          <t>Mint Chutney (for Sandwiches)</t>
-        </is>
-      </c>
-      <c r="E270" t="inlineStr">
-        <is>
-          <t>புதினா சட்னி (சாண்ட்விச்சிற்கு)</t>
-        </is>
-      </c>
-      <c r="F270" t="inlineStr">
-        <is>
-          <t>chutney</t>
-        </is>
-      </c>
-      <c r="G270" t="inlineStr">
-        <is>
-          <t>A photorealistic close-up of a small bowl of smooth bright green mint chutney, glossy sheen, served beside a stack of white bread slices, fresh vibrant lighting.</t>
-        </is>
-      </c>
-      <c r="H270" t="inlineStr">
-        <is>
-          <t>public/images/recipes/mint-chutney-sandwiches/featured.jpg</t>
-        </is>
-      </c>
-      <c r="I270" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="271">
-      <c r="A271" t="n">
-        <v>270</v>
-      </c>
-      <c r="B271" t="inlineStr">
-        <is>
-          <t>Vegetarian</t>
-        </is>
-      </c>
-      <c r="C271" t="inlineStr">
-        <is>
-          <t>onion-bajji</t>
-        </is>
-      </c>
-      <c r="D271" t="inlineStr">
-        <is>
-          <t>Onion Bajji</t>
-        </is>
-      </c>
-      <c r="E271" t="inlineStr">
-        <is>
-          <t>வெங்காயப் பஜ்ஜி</t>
-        </is>
-      </c>
-      <c r="F271" t="inlineStr">
-        <is>
-          <t>bajji</t>
-        </is>
-      </c>
-      <c r="G271" t="inlineStr">
-        <is>
-          <t>A photorealistic close-up of golden fried onion bajjis with a distinctive ring-shaped, batter-coated onion visible inside the crisp fried coating, piled on a plate, served with coconut chutney, warm tea-stall lighting.</t>
-        </is>
-      </c>
-      <c r="H271" t="inlineStr">
-        <is>
-          <t>public/images/recipes/onion-bajji/featured.jpg</t>
-        </is>
-      </c>
-      <c r="I271" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="272">
-      <c r="A272" t="n">
-        <v>271</v>
-      </c>
-      <c r="B272" t="inlineStr">
-        <is>
-          <t>Vegetarian</t>
-        </is>
-      </c>
-      <c r="C272" t="inlineStr">
-        <is>
-          <t>vendaikkai-pakoda</t>
-        </is>
-      </c>
-      <c r="D272" t="inlineStr">
-        <is>
-          <t>Deep Fried Ladies Fingers</t>
-        </is>
-      </c>
-      <c r="E272" t="inlineStr">
-        <is>
-          <t>வெண்டைக்காய் பக்கோடா</t>
-        </is>
-      </c>
-      <c r="F272" t="inlineStr">
-        <is>
-          <t>bajji</t>
-        </is>
-      </c>
-      <c r="G272" t="inlineStr">
-        <is>
-          <t>A photorealistic close-up of whole okra pieces coated in a crisp golden fried batter with visible bread-crumb texture, arranged on a plate with tomato sauce, natural daylight.</t>
-        </is>
-      </c>
-      <c r="H272" t="inlineStr">
-        <is>
-          <t>public/images/recipes/vendaikkai-pakoda/featured.jpg</t>
-        </is>
-      </c>
-      <c r="I272" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="273">
-      <c r="A273" t="n">
-        <v>272</v>
-      </c>
-      <c r="B273" t="inlineStr">
-        <is>
-          <t>Vegetarian</t>
-        </is>
-      </c>
-      <c r="C273" t="inlineStr">
-        <is>
-          <t>carrot-sandwich</t>
-        </is>
-      </c>
-      <c r="D273" t="inlineStr">
-        <is>
-          <t>Carrot Sandwich</t>
-        </is>
-      </c>
-      <c r="E273" t="inlineStr">
-        <is>
-          <t>கேரட் சாண்ட்விச்</t>
-        </is>
-      </c>
-      <c r="F273" t="inlineStr">
-        <is>
-          <t>sandwich</t>
-        </is>
-      </c>
-      <c r="G273" t="inlineStr">
-        <is>
-          <t>A photorealistic close-up of a pressed golden-toasted sandwich cut in half, showing a bright orange sauteed carrot-tomato filling between the bread layers, plated with tomato sauce, warm appetizing lighting.</t>
-        </is>
-      </c>
-      <c r="H273" t="inlineStr">
-        <is>
-          <t>public/images/recipes/carrot-sandwich/featured.jpg</t>
-        </is>
-      </c>
-      <c r="I273" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="274">
-      <c r="A274" t="n">
-        <v>273</v>
-      </c>
-      <c r="B274" t="inlineStr">
-        <is>
-          <t>Vegetarian Cooking Tips - Gap Fill</t>
-        </is>
-      </c>
-      <c r="C274" t="inlineStr">
-        <is>
-          <t>egg-dosai</t>
-        </is>
-      </c>
-      <c r="D274" t="inlineStr">
-        <is>
-          <t>Egg Dosai</t>
-        </is>
-      </c>
-      <c r="E274" t="inlineStr">
-        <is>
-          <t>முட்டைத் தோசை</t>
-        </is>
-      </c>
-      <c r="F274" t="inlineStr">
-        <is>
-          <t>dosa</t>
-        </is>
-      </c>
-      <c r="G274" t="inlineStr">
-        <is>
-          <t>A close-up photorealistic food photo of a thin, golden-brown crepe-like dosa on a black stone griddle, a thin layer of beaten egg cooked into its surface giving it a mottled yellow-and-brown speckled texture, folded in half on a steel plate, a wedge of onion and a small bowl of coconut chutney beside it, warm kitchen lighting, shallow depth of field.</t>
-        </is>
-      </c>
-      <c r="H274" t="inlineStr">
-        <is>
-          <t>public/images/recipes/egg-dosai/featured.jpg</t>
-        </is>
-      </c>
-      <c r="I274" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="275">
-      <c r="A275" t="n">
-        <v>274</v>
-      </c>
-      <c r="B275" t="inlineStr">
-        <is>
-          <t>Vegetarian Cooking Tips - Gap Fill</t>
-        </is>
-      </c>
-      <c r="C275" t="inlineStr">
-        <is>
-          <t>masala-idli</t>
-        </is>
-      </c>
-      <c r="D275" t="inlineStr">
-        <is>
-          <t>Masala Idli</t>
-        </is>
-      </c>
-      <c r="E275" t="inlineStr">
-        <is>
-          <t>மசாலா இட்லி</t>
-        </is>
-      </c>
-      <c r="F275" t="inlineStr">
-        <is>
-          <t>idli</t>
-        </is>
-      </c>
-      <c r="G275" t="inlineStr">
-        <is>
-          <t>A close-up photorealistic food photo of a soft white idli cut in half on a steel plate, revealing a spiced reddish-orange vegetable filling layered through its center, steam rising gently, a small bowl of sambar and coconut chutney alongside, natural morning light.</t>
-        </is>
-      </c>
-      <c r="H275" t="inlineStr">
-        <is>
-          <t>public/images/recipes/masala-idli/featured.jpg</t>
-        </is>
-      </c>
-      <c r="I275" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="276">
-      <c r="A276" t="n">
-        <v>275</v>
-      </c>
-      <c r="B276" t="inlineStr">
-        <is>
-          <t>Vegetarian Cooking Tips - Gap Fill</t>
-        </is>
-      </c>
-      <c r="C276" t="inlineStr">
-        <is>
-          <t>vegetable-sambar</t>
-        </is>
-      </c>
-      <c r="D276" t="inlineStr">
-        <is>
-          <t>Vegetable Sambar</t>
-        </is>
-      </c>
-      <c r="E276" t="inlineStr">
-        <is>
-          <t>காய்கறி சாம்பார்</t>
-        </is>
-      </c>
-      <c r="F276" t="inlineStr">
-        <is>
-          <t>sambar</t>
-        </is>
-      </c>
-      <c r="G276" t="inlineStr">
-        <is>
-          <t>A close-up photorealistic food photo of steaming orange-yellow vegetable sambar in a steel bowl, chunks of drumstick and brinjal visible in the thick lentil gravy, a mustard-and-curry-leaf tempering glistening on top, garnished with fresh coriander leaves, warm natural lighting.</t>
-        </is>
-      </c>
-      <c r="H276" t="inlineStr">
-        <is>
-          <t>public/images/recipes/vegetable-sambar/featured.jpg</t>
-        </is>
-      </c>
-      <c r="I276" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="277">
-      <c r="A277" t="n">
-        <v>276</v>
-      </c>
-      <c r="B277" t="inlineStr">
-        <is>
-          <t>Vegetarian Cooking Tips - Gap Fill</t>
-        </is>
-      </c>
-      <c r="C277" t="inlineStr">
-        <is>
-          <t>idiyappam</t>
-        </is>
-      </c>
-      <c r="D277" t="inlineStr">
-        <is>
-          <t>Idiyappam (String Hoppers)</t>
-        </is>
-      </c>
-      <c r="E277" t="inlineStr">
-        <is>
-          <t>இடியாப்பம்</t>
-        </is>
-      </c>
-      <c r="F277" t="inlineStr">
-        <is>
-          <t>steamed-tiffin</t>
-        </is>
-      </c>
-      <c r="G277" t="inlineStr">
-        <is>
-          <t>A close-up photorealistic food photo of a neat coiled disc of thin white rice-flour string hoppers on a banana leaf, delicate steamed strands visible, served beside a small bowl of coconut milk and a wedge of lime, soft natural daylight, shallow depth of field.</t>
-        </is>
-      </c>
-      <c r="H277" t="inlineStr">
-        <is>
-          <t>public/images/recipes/idiyappam/featured.jpg</t>
-        </is>
-      </c>
-      <c r="I277" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="278">
-      <c r="A278" t="n">
-        <v>277</v>
-      </c>
-      <c r="B278" t="inlineStr">
-        <is>
-          <t>Vegetarian Cooking Tips - Gap Fill</t>
-        </is>
-      </c>
-      <c r="C278" t="inlineStr">
-        <is>
-          <t>sweet-appam</t>
-        </is>
-      </c>
-      <c r="D278" t="inlineStr">
-        <is>
-          <t>Sweet Appam</t>
-        </is>
-      </c>
-      <c r="E278" t="inlineStr">
-        <is>
-          <t>இனிப்பு ஆப்பம்</t>
-        </is>
-      </c>
-      <c r="F278" t="inlineStr">
-        <is>
-          <t>steamed-tiffin, sweet</t>
-        </is>
-      </c>
-      <c r="G278" t="inlineStr">
-        <is>
-          <t>A close-up photorealistic food photo of a golden-brown bowl-shaped appam with a thick spongy center and lacy crisp edges, resting on a steel plate, its jaggery-sweetened surface glistening slightly, warm kitchen lighting, shallow depth of field.</t>
-        </is>
-      </c>
-      <c r="H278" t="inlineStr">
-        <is>
-          <t>public/images/recipes/sweet-appam/featured.jpg</t>
-        </is>
-      </c>
-      <c r="I278" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="279">
-      <c r="A279" t="n">
-        <v>278</v>
-      </c>
-      <c r="B279" t="inlineStr">
-        <is>
-          <t>Vegetarian Cooking Tips - Gap Fill</t>
-        </is>
-      </c>
-      <c r="C279" t="inlineStr">
-        <is>
-          <t>chapati</t>
-        </is>
-      </c>
-      <c r="D279" t="inlineStr">
-        <is>
-          <t>Chapati</t>
-        </is>
-      </c>
-      <c r="E279" t="inlineStr">
-        <is>
-          <t>சப்பாத்தி</t>
-        </is>
-      </c>
-      <c r="F279" t="inlineStr">
-        <is>
-          <t>flatbread</t>
-        </is>
-      </c>
-      <c r="G279" t="inlineStr">
-        <is>
-          <t>A close-up photorealistic food photo of a puffed, golden-brown round chapati fresh off the griddle, a light sheen of ghee brushed on top, stacked slightly with one leaning against the pile on a steel plate, warm kitchen lighting.</t>
-        </is>
-      </c>
-      <c r="H279" t="inlineStr">
-        <is>
-          <t>public/images/recipes/chapati/featured.jpg</t>
-        </is>
-      </c>
-      <c r="I279" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="280">
-      <c r="A280" t="n">
-        <v>279</v>
-      </c>
-      <c r="B280" t="inlineStr">
-        <is>
-          <t>Vegetarian Cooking Tips - Gap Fill</t>
-        </is>
-      </c>
-      <c r="C280" t="inlineStr">
-        <is>
-          <t>patrora</t>
-        </is>
-      </c>
-      <c r="D280" t="inlineStr">
-        <is>
-          <t>Patrora (or Curd Poori)</t>
-        </is>
-      </c>
-      <c r="E280" t="inlineStr">
-        <is>
-          <t>பட்ரோரா (அல்லது) தயிர் பூரி</t>
-        </is>
-      </c>
-      <c r="F280" t="inlineStr">
-        <is>
-          <t>fried-bread</t>
-        </is>
-      </c>
-      <c r="G280" t="inlineStr">
-        <is>
-          <t>A close-up photorealistic food photo of a thick, golden-brown deep-fried round bread with a slightly puffed naan-like texture, served on a steel plate with a side of chana masala gravy, warm kitchen lighting, shallow depth of field.</t>
-        </is>
-      </c>
-      <c r="H280" t="inlineStr">
-        <is>
-          <t>public/images/recipes/patrora/featured.jpg</t>
-        </is>
-      </c>
-      <c r="I280" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="281">
-      <c r="A281" t="n">
-        <v>280</v>
-      </c>
-      <c r="B281" t="inlineStr">
-        <is>
-          <t>Vegetarian Cooking Tips - Gap Fill</t>
-        </is>
-      </c>
-      <c r="C281" t="inlineStr">
-        <is>
-          <t>tomato-kurma</t>
-        </is>
-      </c>
-      <c r="D281" t="inlineStr">
-        <is>
-          <t>Tomato Kurma</t>
-        </is>
-      </c>
-      <c r="E281" t="inlineStr">
-        <is>
-          <t>தக்காளி குருமா</t>
-        </is>
-      </c>
-      <c r="F281" t="inlineStr">
-        <is>
-          <t>kuzhambu</t>
-        </is>
-      </c>
-      <c r="G281" t="inlineStr">
-        <is>
-          <t>A close-up photorealistic food photo of a thick reddish-orange tomato kurma gravy in a steel bowl, chunks of potato visible in the glossy sauce, garnished with fresh coriander leaves, warm natural lighting, shallow depth of field.</t>
-        </is>
-      </c>
-      <c r="H281" t="inlineStr">
-        <is>
-          <t>public/images/recipes/tomato-kurma/featured.jpg</t>
-        </is>
-      </c>
-      <c r="I281" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="282">
-      <c r="A282" t="n">
-        <v>281</v>
-      </c>
-      <c r="B282" t="inlineStr">
-        <is>
-          <t>Vegetarian Cooking Tips - Gap Fill</t>
-        </is>
-      </c>
-      <c r="C282" t="inlineStr">
-        <is>
-          <t>kathirikkai-kosu</t>
-        </is>
-      </c>
-      <c r="D282" t="inlineStr">
-        <is>
-          <t>Kathirikkai Kosu (Brinjal Kosu)</t>
-        </is>
-      </c>
-      <c r="E282" t="inlineStr">
-        <is>
-          <t>கத்தரிக்காய் கொச்சு</t>
-        </is>
-      </c>
-      <c r="F282" t="inlineStr">
-        <is>
-          <t>kuzhambu</t>
-        </is>
-      </c>
-      <c r="G282" t="inlineStr">
-        <is>
-          <t>A close-up photorealistic food photo of a dark reddish-brown mashed brinjal side dish in a small steel bowl, thick and glossy with visible flecks of tempered mustard seeds, served beside plain rice, warm natural lighting.</t>
-        </is>
-      </c>
-      <c r="H282" t="inlineStr">
-        <is>
-          <t>public/images/recipes/kathirikkai-kosu/featured.jpg</t>
-        </is>
-      </c>
-      <c r="I282" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="283">
-      <c r="A283" t="n">
-        <v>282</v>
-      </c>
-      <c r="B283" t="inlineStr">
-        <is>
-          <t>Vegetarian Cooking Tips - Gap Fill</t>
-        </is>
-      </c>
-      <c r="C283" t="inlineStr">
-        <is>
-          <t>masala-sundal</t>
-        </is>
-      </c>
-      <c r="D283" t="inlineStr">
-        <is>
-          <t>Masala Sundal</t>
-        </is>
-      </c>
-      <c r="E283" t="inlineStr">
-        <is>
-          <t>மசால் சுண்டல்</t>
-        </is>
-      </c>
-      <c r="F283" t="inlineStr">
-        <is>
-          <t>sundal</t>
-        </is>
-      </c>
-      <c r="G283" t="inlineStr">
-        <is>
-          <t>A close-up photorealistic food photo of a bowl of golden-brown spiced chickpea sundal, garnished generously with grated coconut and chopped coriander leaves, curry leaves visible throughout, natural daylight, shallow depth of field.</t>
-        </is>
-      </c>
-      <c r="H283" t="inlineStr">
-        <is>
-          <t>public/images/recipes/masala-sundal/featured.jpg</t>
-        </is>
-      </c>
-      <c r="I283" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="284">
-      <c r="A284" t="n">
-        <v>283</v>
-      </c>
-      <c r="B284" t="inlineStr">
-        <is>
-          <t>Vegetarian Cooking Tips - Gap Fill</t>
-        </is>
-      </c>
-      <c r="C284" t="inlineStr">
-        <is>
-          <t>kuzhai-puttu</t>
-        </is>
-      </c>
-      <c r="D284" t="inlineStr">
-        <is>
-          <t>Kuzhai Puttu (Tube Puttu)</t>
-        </is>
-      </c>
-      <c r="E284" t="inlineStr">
-        <is>
-          <t>குழாய்ப்புட்டு</t>
-        </is>
-      </c>
-      <c r="F284" t="inlineStr">
-        <is>
-          <t>puttu, sweet</t>
-        </is>
-      </c>
-      <c r="G284" t="inlineStr">
-        <is>
-          <t>A close-up photorealistic food photo of a cylindrical steamed puttu on a plate, cut into thick discs revealing alternating white rice-flour and grated-coconut layers studded with sugar, steam still rising, warm morning light.</t>
-        </is>
-      </c>
-      <c r="H284" t="inlineStr">
-        <is>
-          <t>public/images/recipes/kuzhai-puttu/featured.jpg</t>
-        </is>
-      </c>
-      <c r="I284" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="285">
-      <c r="A285" t="n">
-        <v>284</v>
-      </c>
-      <c r="B285" t="inlineStr">
-        <is>
-          <t>Vegetarian Cooking Tips - Gap Fill</t>
-        </is>
-      </c>
-      <c r="C285" t="inlineStr">
-        <is>
-          <t>egg-pan-cake</t>
-        </is>
-      </c>
-      <c r="D285" t="inlineStr">
-        <is>
-          <t>Pan Cake</t>
-        </is>
-      </c>
-      <c r="E285" t="inlineStr">
-        <is>
-          <t>பான் கேக்</t>
-        </is>
-      </c>
-      <c r="F285" t="inlineStr">
-        <is>
-          <t>sweet</t>
-        </is>
-      </c>
-      <c r="G285" t="inlineStr">
-        <is>
-          <t>A close-up photorealistic food photo of a thin, pale golden egg-and-maida pancake folded in half on a plate, a slightly glossy surface from ghee, dusted lightly with sugar, soft warm lighting, shallow depth of field.</t>
-        </is>
-      </c>
-      <c r="H285" t="inlineStr">
-        <is>
-          <t>public/images/recipes/egg-pan-cake/featured.jpg</t>
-        </is>
-      </c>
-      <c r="I285" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="286">
-      <c r="A286" t="n">
-        <v>285</v>
-      </c>
-      <c r="B286" t="inlineStr">
-        <is>
-          <t>Vegetarian Cooking Tips - Gap Fill</t>
-        </is>
-      </c>
-      <c r="C286" t="inlineStr">
-        <is>
-          <t>milk-basundi</t>
-        </is>
-      </c>
-      <c r="D286" t="inlineStr">
-        <is>
-          <t>Milk Basundi</t>
-        </is>
-      </c>
-      <c r="E286" t="inlineStr">
-        <is>
-          <t>பால் பாஸந்தி</t>
-        </is>
-      </c>
-      <c r="F286" t="inlineStr">
-        <is>
-          <t>sweet</t>
-        </is>
-      </c>
-      <c r="G286" t="inlineStr">
-        <is>
-          <t>A close-up photorealistic food photo of thick, creamy off-white basundi in a small clay bowl, slivers of pistachio and cashew scattered on top with a few golden saffron strands, condensation on the bowl suggesting it's chilled, soft natural lighting.</t>
-        </is>
-      </c>
-      <c r="H286" t="inlineStr">
-        <is>
-          <t>public/images/recipes/milk-basundi/featured.jpg</t>
-        </is>
-      </c>
-      <c r="I286" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="287">
-      <c r="A287" t="n">
-        <v>286</v>
-      </c>
-      <c r="B287" t="inlineStr">
-        <is>
-          <t>Vegetarian Cooking Tips - Gap Fill</t>
-        </is>
-      </c>
-      <c r="C287" t="inlineStr">
-        <is>
-          <t>cashew-pakoda</t>
-        </is>
-      </c>
-      <c r="D287" t="inlineStr">
-        <is>
-          <t>Cashew Pakoda</t>
-        </is>
-      </c>
-      <c r="E287" t="inlineStr">
-        <is>
-          <t>முந்திரி பருப்பு பகோடா</t>
-        </is>
-      </c>
-      <c r="F287" t="inlineStr">
-        <is>
-          <t>bajji</t>
-        </is>
-      </c>
-      <c r="G287" t="inlineStr">
-        <is>
-          <t>A close-up photorealistic food photo of golden-brown irregular-shaped fritters piled on a steel plate, whole cashew nuts and flecks of onion visible embedded in the crisp fried batter, a small bowl of ketchup beside it, warm kitchen lighting.</t>
-        </is>
-      </c>
-      <c r="H287" t="inlineStr">
-        <is>
-          <t>public/images/recipes/cashew-pakoda/featured.jpg</t>
-        </is>
-      </c>
-      <c r="I287" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="288">
-      <c r="A288" t="n">
-        <v>287</v>
-      </c>
-      <c r="B288" t="inlineStr">
-        <is>
-          <t>Vegetarian Cooking Tips - Gap Fill</t>
-        </is>
-      </c>
-      <c r="C288" t="inlineStr">
-        <is>
-          <t>potato-chips</t>
-        </is>
-      </c>
-      <c r="D288" t="inlineStr">
-        <is>
-          <t>Potato Chips</t>
-        </is>
-      </c>
-      <c r="E288" t="inlineStr">
-        <is>
-          <t>உருளைக் கிழங்கு சிப்ஸ்</t>
-        </is>
-      </c>
-      <c r="F288" t="inlineStr">
-        <is>
-          <t>snack</t>
-        </is>
-      </c>
-      <c r="G288" t="inlineStr">
-        <is>
-          <t>A close-up photorealistic food photo of thin, golden potato chip rounds piled in a steel bowl, dusted lightly with red chilli powder, glossy from frying oil, warm natural lighting, shallow depth of field.</t>
-        </is>
-      </c>
-      <c r="H288" t="inlineStr">
-        <is>
-          <t>public/images/recipes/potato-chips/featured.jpg</t>
-        </is>
-      </c>
-      <c r="I288" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="289">
-      <c r="A289" t="n">
-        <v>288</v>
-      </c>
-      <c r="B289" t="inlineStr">
-        <is>
-          <t>Vegetarian Cooking Tips - Gap Fill</t>
-        </is>
-      </c>
-      <c r="C289" t="inlineStr">
-        <is>
-          <t>sweet-raw-mango</t>
-        </is>
-      </c>
-      <c r="D289" t="inlineStr">
-        <is>
-          <t>Sweet Raw Mango</t>
-        </is>
-      </c>
-      <c r="E289" t="inlineStr">
-        <is>
-          <t>இனிப்பு மாங்காய்</t>
-        </is>
-      </c>
-      <c r="F289" t="inlineStr">
-        <is>
-          <t>curry</t>
-        </is>
-      </c>
-      <c r="G289" t="inlineStr">
-        <is>
-          <t>A close-up photorealistic food photo of a thick, glossy amber-colored mashed raw mango curry in a steel bowl, flecks of curry leaves and mustard seeds visible, served beside plain rice, warm natural lighting.</t>
-        </is>
-      </c>
-      <c r="H289" t="inlineStr">
-        <is>
-          <t>public/images/recipes/sweet-raw-mango/featured.jpg</t>
-        </is>
-      </c>
-      <c r="I289" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="290">
-      <c r="A290" t="n">
-        <v>289</v>
-      </c>
-      <c r="B290" t="inlineStr">
-        <is>
-          <t>Vegetarian Cooking Tips - Gap Fill</t>
-        </is>
-      </c>
-      <c r="C290" t="inlineStr">
-        <is>
-          <t>kinch-mosara</t>
-        </is>
-      </c>
-      <c r="D290" t="inlineStr">
-        <is>
-          <t>Kinch Mosara (Stuffed Potato Cones)</t>
-        </is>
-      </c>
-      <c r="E290" t="inlineStr">
-        <is>
-          <t>கிஞ்ச மோசரா</t>
-        </is>
-      </c>
-      <c r="F290" t="inlineStr">
-        <is>
-          <t>fried-snack</t>
-        </is>
-      </c>
-      <c r="G290" t="inlineStr">
-        <is>
-          <t>A close-up photorealistic food photo of golden-brown deep-fried cone-shaped pastries on a steel plate, one broken open to reveal a spiced mashed-potato-and-green-pea filling studded with raisins and cashews, warm kitchen lighting, shallow depth of field.</t>
-        </is>
-      </c>
-      <c r="H290" t="inlineStr">
-        <is>
-          <t>public/images/recipes/kinch-mosara/featured.jpg</t>
-        </is>
-      </c>
-      <c r="I290" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="291">
-      <c r="A291" t="n">
-        <v>290</v>
-      </c>
-      <c r="B291" t="inlineStr">
-        <is>
-          <t>Vegetarian Cooking Tips - Gap Fill</t>
-        </is>
-      </c>
-      <c r="C291" t="inlineStr">
-        <is>
-          <t>pirattu-kari</t>
-        </is>
-      </c>
-      <c r="D291" t="inlineStr">
-        <is>
-          <t>Pirattu Kari (Braised Mutton)</t>
-        </is>
-      </c>
-      <c r="E291" t="inlineStr">
-        <is>
-          <t>பிறட்டுக்கறி</t>
-        </is>
-      </c>
-      <c r="F291" t="inlineStr">
-        <is>
-          <t>curry</t>
-        </is>
-      </c>
-      <c r="G291" t="inlineStr">
-        <is>
-          <t>A close-up photorealistic food photo of dark reddish-brown braised mutton pieces in a thick, dry-ish onion masala coating, glistening slightly with oil, served in a steel bowl garnished with curry leaves, warm dramatic lighting, shallow depth of field.</t>
-        </is>
-      </c>
-      <c r="H291" t="inlineStr">
-        <is>
-          <t>public/images/recipes/pirattu-kari/featured.jpg</t>
-        </is>
-      </c>
-      <c r="I291" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="292">
-      <c r="A292" t="n">
-        <v>291</v>
-      </c>
-      <c r="B292" t="inlineStr">
-        <is>
-          <t>Vegetarian Cooking Tips - Gap Fill</t>
-        </is>
-      </c>
-      <c r="C292" t="inlineStr">
-        <is>
-          <t>chinese-sooce</t>
-        </is>
-      </c>
-      <c r="D292" t="inlineStr">
-        <is>
-          <t>Chinese Sooce (Cashew-Date Bars)</t>
-        </is>
-      </c>
-      <c r="E292" t="inlineStr">
-        <is>
-          <t>சைனீஸ் சூஸ்</t>
-        </is>
-      </c>
-      <c r="F292" t="inlineStr">
-        <is>
-          <t>sweet</t>
-        </is>
-      </c>
-      <c r="G292" t="inlineStr">
-        <is>
-          <t>A close-up photorealistic food photo of rectangular golden-brown baked bars studded with chopped cashews and dates, dusted with white icing sugar, stacked on a plate, soft natural lighting, shallow depth of field.</t>
-        </is>
-      </c>
-      <c r="H292" t="inlineStr">
-        <is>
-          <t>public/images/recipes/chinese-sooce/featured.jpg</t>
-        </is>
-      </c>
-      <c r="I292" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="293">
-      <c r="A293" t="n">
-        <v>292</v>
-      </c>
-      <c r="B293" t="inlineStr">
-        <is>
-          <t>Vegetarian Cooking Tips - Gap Fill</t>
-        </is>
-      </c>
-      <c r="C293" t="inlineStr">
-        <is>
-          <t>boat-egg</t>
-        </is>
-      </c>
-      <c r="D293" t="inlineStr">
-        <is>
-          <t>Boat Egg</t>
-        </is>
-      </c>
-      <c r="E293" t="inlineStr">
-        <is>
-          <t>படகு முட்டை</t>
-        </is>
-      </c>
-      <c r="F293" t="inlineStr">
-        <is>
-          <t>snack</t>
-        </is>
-      </c>
-      <c r="G293" t="inlineStr">
-        <is>
-          <t>A close-up photorealistic food photo of small boiled-egg-white boat shapes arranged on a platter, each filled with pale yellow mashed egg yolk and topped with a small triangular bread-slice sail propped upright, playful party-snack styling, bright even lighting.</t>
-        </is>
-      </c>
-      <c r="H293" t="inlineStr">
-        <is>
-          <t>public/images/recipes/boat-egg/featured.jpg</t>
-        </is>
-      </c>
-      <c r="I293" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="294">
-      <c r="A294" t="n">
-        <v>293</v>
-      </c>
-      <c r="B294" t="inlineStr">
-        <is>
-          <t>Vegetarian Cooking Tips - Gap Fill</t>
-        </is>
-      </c>
-      <c r="C294" t="inlineStr">
-        <is>
-          <t>fish-fry-roast</t>
-        </is>
-      </c>
-      <c r="D294" t="inlineStr">
-        <is>
-          <t>Fish Fry Roast</t>
-        </is>
-      </c>
-      <c r="E294" t="inlineStr">
-        <is>
-          <t>மீன் ஃபிராஸ்ட்</t>
-        </is>
-      </c>
-      <c r="F294" t="inlineStr">
-        <is>
-          <t>curry</t>
-        </is>
-      </c>
-      <c r="G294" t="inlineStr">
-        <is>
-          <t>A close-up photorealistic food photo of golden-brown shallow-fried fish steaks on a steel plate, a red-orange spice crust visible on the surface, garnished with sliced onion, coriander leaves, and a lemon wedge, warm kitchen lighting, shallow depth of field.</t>
-        </is>
-      </c>
-      <c r="H294" t="inlineStr">
-        <is>
-          <t>public/images/recipes/fish-fry-roast/featured.jpg</t>
-        </is>
-      </c>
-      <c r="I294" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
fix(tracker): restore batch-2 image prompts lost in previous revert
The batch-2 71-row Gemini prompt addition (S.No 202-272) had never been
committed on its own -- it was sitting as an uncommitted change and got
folded into the "21 gap-fill recipes" commit together with the new rows.
Reverting that commit therefore also wiped out the batch-2 prompts.
Restores just S.No 1-272, keeping the gap-fill rows (273-293) out.
</commit_message>
<xml_diff>
--- a/docs/recipe-image-tracker.xlsx
+++ b/docs/recipe-image-tracker.xlsx
@@ -496,7 +496,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K202"/>
+  <dimension ref="A1:K273"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -11423,6 +11423,3201 @@
         </is>
       </c>
       <c r="K202" s="15" t="n"/>
+    </row>
+    <row r="203">
+      <c r="A203" t="n">
+        <v>202</v>
+      </c>
+      <c r="B203" t="inlineStr">
+        <is>
+          <t>Vegetarian</t>
+        </is>
+      </c>
+      <c r="C203" t="inlineStr">
+        <is>
+          <t>banana-cutlets</t>
+        </is>
+      </c>
+      <c r="D203" t="inlineStr">
+        <is>
+          <t>Banana Cutlets</t>
+        </is>
+      </c>
+      <c r="E203" t="inlineStr">
+        <is>
+          <t>வாழைக்காய் கட்லெட்</t>
+        </is>
+      </c>
+      <c r="F203" t="inlineStr">
+        <is>
+          <t>cutlet</t>
+        </is>
+      </c>
+      <c r="G203" t="inlineStr">
+        <is>
+          <t>A close-up photorealistic food photo of golden-brown oval cutlets with a crisp breadcrumb crust, plated on a white ceramic plate, garnished with a wedge of lemon and a small bowl of tomato ketchup, one cutlet broken open to reveal a soft reddish-brown banana-potato filling flecked with green coriander, warm natural lighting, shallow depth of field.</t>
+        </is>
+      </c>
+      <c r="H203" t="inlineStr">
+        <is>
+          <t>public/images/recipes/banana-cutlets/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I203" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" t="n">
+        <v>203</v>
+      </c>
+      <c r="B204" t="inlineStr">
+        <is>
+          <t>Vegetarian</t>
+        </is>
+      </c>
+      <c r="C204" t="inlineStr">
+        <is>
+          <t>vegetable-sizzlers</t>
+        </is>
+      </c>
+      <c r="D204" t="inlineStr">
+        <is>
+          <t>Vegetable Sizzlers</t>
+        </is>
+      </c>
+      <c r="E204" t="inlineStr">
+        <is>
+          <t>வெஜிடபிள் சிஸ்லர்ஸ்</t>
+        </is>
+      </c>
+      <c r="F204" t="inlineStr">
+        <is>
+          <t>fusion</t>
+        </is>
+      </c>
+      <c r="G204" t="inlineStr">
+        <is>
+          <t>A dramatic photorealistic photo of a cast-iron sizzler plate on a wooden board, visibly smoking with steam rising, holding a golden fried cutlet in the center surrounded by charred grilled carrot rounds, cabbage wedges, capsicum rings, and potato slices, glossy with butter and reddish sauce, dark moody restaurant lighting.</t>
+        </is>
+      </c>
+      <c r="H204" t="inlineStr">
+        <is>
+          <t>public/images/recipes/vegetable-sizzlers/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I204" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" t="n">
+        <v>204</v>
+      </c>
+      <c r="B205" t="inlineStr">
+        <is>
+          <t>Vegetarian</t>
+        </is>
+      </c>
+      <c r="C205" t="inlineStr">
+        <is>
+          <t>vegetable-burgers</t>
+        </is>
+      </c>
+      <c r="D205" t="inlineStr">
+        <is>
+          <t>Vegetable Burgers</t>
+        </is>
+      </c>
+      <c r="E205" t="inlineStr">
+        <is>
+          <t>வெஜிடபிள் பர்கர்ஸ்</t>
+        </is>
+      </c>
+      <c r="F205" t="inlineStr">
+        <is>
+          <t>fusion</t>
+        </is>
+      </c>
+      <c r="G205" t="inlineStr">
+        <is>
+          <t>A photorealistic close-up of a round golden-brown vegetable burger patty inside a soft bun, layered with a crisp cabbage leaf, thin onion rings, beetroot slices, and tomato, skewered with a small toothpick, plated with crinkle-cut potato fries and ketchup, bright appetizing lighting.</t>
+        </is>
+      </c>
+      <c r="H205" t="inlineStr">
+        <is>
+          <t>public/images/recipes/vegetable-burgers/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I205" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" t="n">
+        <v>205</v>
+      </c>
+      <c r="B206" t="inlineStr">
+        <is>
+          <t>Vegetarian</t>
+        </is>
+      </c>
+      <c r="C206" t="inlineStr">
+        <is>
+          <t>sago-bonda</t>
+        </is>
+      </c>
+      <c r="D206" t="inlineStr">
+        <is>
+          <t>Sago Bonda</t>
+        </is>
+      </c>
+      <c r="E206" t="inlineStr">
+        <is>
+          <t>ஜவ்வரிசி போண்டா</t>
+        </is>
+      </c>
+      <c r="F206" t="inlineStr">
+        <is>
+          <t>bonda</t>
+        </is>
+      </c>
+      <c r="G206" t="inlineStr">
+        <is>
+          <t>A photorealistic close-up of small round golden-brown bondas with a translucent, pearly, slightly bumpy sago texture visible on the fried crust, piled on a steel plate lined with paper, garnished with coriander leaves, a small bowl of green chutney beside them, warm kitchen lighting.</t>
+        </is>
+      </c>
+      <c r="H206" t="inlineStr">
+        <is>
+          <t>public/images/recipes/sago-bonda/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I206" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" t="n">
+        <v>206</v>
+      </c>
+      <c r="B207" t="inlineStr">
+        <is>
+          <t>Vegetarian</t>
+        </is>
+      </c>
+      <c r="C207" t="inlineStr">
+        <is>
+          <t>vegetable-bonda</t>
+        </is>
+      </c>
+      <c r="D207" t="inlineStr">
+        <is>
+          <t>Vegetable Bonda</t>
+        </is>
+      </c>
+      <c r="E207" t="inlineStr">
+        <is>
+          <t>வெஜிடபிள் போண்டா</t>
+        </is>
+      </c>
+      <c r="F207" t="inlineStr">
+        <is>
+          <t>bonda</t>
+        </is>
+      </c>
+      <c r="G207" t="inlineStr">
+        <is>
+          <t>A photorealistic photo of golden fried round bondas with a slightly bumpy, craggy batter surface, one bonda broken in half to show a moist mixed-vegetable filling of carrot, peas, and potato, served on a steel plate with mint chutney and tomato sauce, natural daylight.</t>
+        </is>
+      </c>
+      <c r="H207" t="inlineStr">
+        <is>
+          <t>public/images/recipes/vegetable-bonda/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I207" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" t="n">
+        <v>207</v>
+      </c>
+      <c r="B208" t="inlineStr">
+        <is>
+          <t>Vegetarian</t>
+        </is>
+      </c>
+      <c r="C208" t="inlineStr">
+        <is>
+          <t>aloo-bonda</t>
+        </is>
+      </c>
+      <c r="D208" t="inlineStr">
+        <is>
+          <t>Aloo Bonda</t>
+        </is>
+      </c>
+      <c r="E208" t="inlineStr">
+        <is>
+          <t>உருளைக்கிழங்கு போண்டா</t>
+        </is>
+      </c>
+      <c r="F208" t="inlineStr">
+        <is>
+          <t>bonda</t>
+        </is>
+      </c>
+      <c r="G208" t="inlineStr">
+        <is>
+          <t>A photorealistic image of golden-brown round bondas with a smooth thin batter coating, arranged on a banana leaf, one cut open to reveal a soft yellow mashed-potato filling flecked with onion and coriander, served with coconut chutney, warm South Indian tea-stall lighting.</t>
+        </is>
+      </c>
+      <c r="H208" t="inlineStr">
+        <is>
+          <t>public/images/recipes/aloo-bonda/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I208" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" t="n">
+        <v>208</v>
+      </c>
+      <c r="B209" t="inlineStr">
+        <is>
+          <t>Vegetarian</t>
+        </is>
+      </c>
+      <c r="C209" t="inlineStr">
+        <is>
+          <t>mysore-bonda</t>
+        </is>
+      </c>
+      <c r="D209" t="inlineStr">
+        <is>
+          <t>Mysore Bonda</t>
+        </is>
+      </c>
+      <c r="E209" t="inlineStr">
+        <is>
+          <t>மைசூர் போண்டா</t>
+        </is>
+      </c>
+      <c r="F209" t="inlineStr">
+        <is>
+          <t>bonda</t>
+        </is>
+      </c>
+      <c r="G209" t="inlineStr">
+        <is>
+          <t>A photorealistic close-up of fluffy, irregularly round golden-brown bondas with a light, airy fried crust, stacked in a steel plate, one broken open showing a soft white lentil interior studded with coconut bits, served with coconut chutney in a small bowl, bright natural light.</t>
+        </is>
+      </c>
+      <c r="H209" t="inlineStr">
+        <is>
+          <t>public/images/recipes/mysore-bonda/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I209" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" t="n">
+        <v>209</v>
+      </c>
+      <c r="B210" t="inlineStr">
+        <is>
+          <t>Vegetarian</t>
+        </is>
+      </c>
+      <c r="C210" t="inlineStr">
+        <is>
+          <t>pullani-vunta</t>
+        </is>
+      </c>
+      <c r="D210" t="inlineStr">
+        <is>
+          <t>Pullani Vunta</t>
+        </is>
+      </c>
+      <c r="E210" t="inlineStr">
+        <is>
+          <t>தோசைமாவு போண்டா</t>
+        </is>
+      </c>
+      <c r="F210" t="inlineStr">
+        <is>
+          <t>bonda</t>
+        </is>
+      </c>
+      <c r="G210" t="inlineStr">
+        <is>
+          <t>A photorealistic photo of small irregular golden-brown fried dumplings made from fermented dosa batter, slightly craggy surface with visible onion and coriander flecks, piled on a steel plate with coconut chutney on the side, cozy kitchen lighting.</t>
+        </is>
+      </c>
+      <c r="H210" t="inlineStr">
+        <is>
+          <t>public/images/recipes/pullani-vunta/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I210" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" t="n">
+        <v>210</v>
+      </c>
+      <c r="B211" t="inlineStr">
+        <is>
+          <t>Vegetarian</t>
+        </is>
+      </c>
+      <c r="C211" t="inlineStr">
+        <is>
+          <t>mangalore-bonda</t>
+        </is>
+      </c>
+      <c r="D211" t="inlineStr">
+        <is>
+          <t>Mangalore Bonda</t>
+        </is>
+      </c>
+      <c r="E211" t="inlineStr">
+        <is>
+          <t>மங்களூர் போண்டா</t>
+        </is>
+      </c>
+      <c r="F211" t="inlineStr">
+        <is>
+          <t>bonda</t>
+        </is>
+      </c>
+      <c r="G211" t="inlineStr">
+        <is>
+          <t>A photorealistic close-up of soft, puffy golden-brown fried bondas with a slightly wrinkled curd-based batter texture, arranged on a plate, one broken open to reveal a soft white interior, served with coconut chutney, warm ambient lighting.</t>
+        </is>
+      </c>
+      <c r="H211" t="inlineStr">
+        <is>
+          <t>public/images/recipes/mangalore-bonda/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I211" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" t="n">
+        <v>211</v>
+      </c>
+      <c r="B212" t="inlineStr">
+        <is>
+          <t>Vegetarian</t>
+        </is>
+      </c>
+      <c r="C212" t="inlineStr">
+        <is>
+          <t>cheese-bonda</t>
+        </is>
+      </c>
+      <c r="D212" t="inlineStr">
+        <is>
+          <t>Cheese Bonda</t>
+        </is>
+      </c>
+      <c r="E212" t="inlineStr">
+        <is>
+          <t>சீஸ் போண்டா</t>
+        </is>
+      </c>
+      <c r="F212" t="inlineStr">
+        <is>
+          <t>bonda</t>
+        </is>
+      </c>
+      <c r="G212" t="inlineStr">
+        <is>
+          <t>A photorealistic close-up of small golden fried bondas glistening with oil, one cut in half to reveal a stretchy, melted golden-yellow cheese pull, plated on a white dish, steam rising, cozy warm lighting.</t>
+        </is>
+      </c>
+      <c r="H212" t="inlineStr">
+        <is>
+          <t>public/images/recipes/cheese-bonda/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I212" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" t="n">
+        <v>212</v>
+      </c>
+      <c r="B213" t="inlineStr">
+        <is>
+          <t>Vegetarian</t>
+        </is>
+      </c>
+      <c r="C213" t="inlineStr">
+        <is>
+          <t>palak-dumplings</t>
+        </is>
+      </c>
+      <c r="D213" t="inlineStr">
+        <is>
+          <t>Palak Dumplings</t>
+        </is>
+      </c>
+      <c r="E213" t="inlineStr">
+        <is>
+          <t>பாலக் மெதுபக்கோடா</t>
+        </is>
+      </c>
+      <c r="F213" t="inlineStr">
+        <is>
+          <t>fried-snack</t>
+        </is>
+      </c>
+      <c r="G213" t="inlineStr">
+        <is>
+          <t>A photorealistic photo of small dark-green-flecked golden fried dumplings, irregular round shape, piled on a plate, showing visible bits of dark green spinach and chili in the crisp fried crust, served with ketchup, natural daylight.</t>
+        </is>
+      </c>
+      <c r="H213" t="inlineStr">
+        <is>
+          <t>public/images/recipes/palak-dumplings/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I213" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" t="n">
+        <v>213</v>
+      </c>
+      <c r="B214" t="inlineStr">
+        <is>
+          <t>Vegetarian</t>
+        </is>
+      </c>
+      <c r="C214" t="inlineStr">
+        <is>
+          <t>ridge-gourd-dumplings</t>
+        </is>
+      </c>
+      <c r="D214" t="inlineStr">
+        <is>
+          <t>Ridge Gourd Dumplings</t>
+        </is>
+      </c>
+      <c r="E214" t="inlineStr">
+        <is>
+          <t>பீர்க்கங்காய் மெதுபக்கோடா</t>
+        </is>
+      </c>
+      <c r="F214" t="inlineStr">
+        <is>
+          <t>fried-snack</t>
+        </is>
+      </c>
+      <c r="G214" t="inlineStr">
+        <is>
+          <t>A photorealistic close-up of small golden fried dumplings with pale green ridge-gourd flecks visible through the thin gram-flour crust, piled on a steel plate, served hot with tomato sauce, warm kitchen lighting.</t>
+        </is>
+      </c>
+      <c r="H214" t="inlineStr">
+        <is>
+          <t>public/images/recipes/ridge-gourd-dumplings/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I214" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" t="n">
+        <v>214</v>
+      </c>
+      <c r="B215" t="inlineStr">
+        <is>
+          <t>Vegetarian</t>
+        </is>
+      </c>
+      <c r="C215" t="inlineStr">
+        <is>
+          <t>mint-pakodas</t>
+        </is>
+      </c>
+      <c r="D215" t="inlineStr">
+        <is>
+          <t>Mint Pakodas</t>
+        </is>
+      </c>
+      <c r="E215" t="inlineStr">
+        <is>
+          <t>புதினா பக்கோடா</t>
+        </is>
+      </c>
+      <c r="F215" t="inlineStr">
+        <is>
+          <t>bajji</t>
+        </is>
+      </c>
+      <c r="G215" t="inlineStr">
+        <is>
+          <t>A photorealistic photo of dark green-brown irregular fried pakodas with visible mint and coriander leaf flecks throughout the crumbly, coarse lentil texture, piled high on a plate, steam rising, natural light.</t>
+        </is>
+      </c>
+      <c r="H215" t="inlineStr">
+        <is>
+          <t>public/images/recipes/mint-pakodas/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I215" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" t="n">
+        <v>215</v>
+      </c>
+      <c r="B216" t="inlineStr">
+        <is>
+          <t>Vegetarian</t>
+        </is>
+      </c>
+      <c r="C216" t="inlineStr">
+        <is>
+          <t>potato-nest</t>
+        </is>
+      </c>
+      <c r="D216" t="inlineStr">
+        <is>
+          <t>Potato Nest</t>
+        </is>
+      </c>
+      <c r="E216" t="inlineStr">
+        <is>
+          <t>உருளைக்கிழங்கு கூடுகள்</t>
+        </is>
+      </c>
+      <c r="F216" t="inlineStr">
+        <is>
+          <t>fried-snack</t>
+        </is>
+      </c>
+      <c r="G216" t="inlineStr">
+        <is>
+          <t>A photorealistic close-up of round golden fried balls coated entirely in crisp, spiky strands of fried vermicelli giving a bird's-nest texture, one cut in half to reveal a bright yellow mashed-potato interior with green peas, plated elegantly with lettuce and tomato sauce, bright studio food photography lighting.</t>
+        </is>
+      </c>
+      <c r="H216" t="inlineStr">
+        <is>
+          <t>public/images/recipes/potato-nest/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I216" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" t="n">
+        <v>216</v>
+      </c>
+      <c r="B217" t="inlineStr">
+        <is>
+          <t>Vegetarian</t>
+        </is>
+      </c>
+      <c r="C217" t="inlineStr">
+        <is>
+          <t>garam-pakodas</t>
+        </is>
+      </c>
+      <c r="D217" t="inlineStr">
+        <is>
+          <t>Garam Pakodas</t>
+        </is>
+      </c>
+      <c r="E217" t="inlineStr">
+        <is>
+          <t>வெங்காய பக்கோடா</t>
+        </is>
+      </c>
+      <c r="F217" t="inlineStr">
+        <is>
+          <t>bajji</t>
+        </is>
+      </c>
+      <c r="G217" t="inlineStr">
+        <is>
+          <t>A photorealistic photo of a heaping pile of irregular, craggy, deep-golden fried pakoda chunks with visible long strands of onion and green chili baked into the crisp crust, on a steel plate, chai glass beside it, warm evening tea-stall lighting.</t>
+        </is>
+      </c>
+      <c r="H217" t="inlineStr">
+        <is>
+          <t>public/images/recipes/garam-pakodas/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I217" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" t="n">
+        <v>217</v>
+      </c>
+      <c r="B218" t="inlineStr">
+        <is>
+          <t>Vegetarian</t>
+        </is>
+      </c>
+      <c r="C218" t="inlineStr">
+        <is>
+          <t>paneer-pakodas</t>
+        </is>
+      </c>
+      <c r="D218" t="inlineStr">
+        <is>
+          <t>Paneer Pakodas</t>
+        </is>
+      </c>
+      <c r="E218" t="inlineStr">
+        <is>
+          <t>பனீர் பக்கோடா</t>
+        </is>
+      </c>
+      <c r="F218" t="inlineStr">
+        <is>
+          <t>bajji</t>
+        </is>
+      </c>
+      <c r="G218" t="inlineStr">
+        <is>
+          <t>A photorealistic close-up of irregular golden fried pakoda chunks with visible crumbly white paneer and pink cashew pieces embedded in the crust, piled on a plate with mint garnish, warm kitchen lighting.</t>
+        </is>
+      </c>
+      <c r="H218" t="inlineStr">
+        <is>
+          <t>public/images/recipes/paneer-pakodas/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I218" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" t="n">
+        <v>218</v>
+      </c>
+      <c r="B219" t="inlineStr">
+        <is>
+          <t>Vegetarian</t>
+        </is>
+      </c>
+      <c r="C219" t="inlineStr">
+        <is>
+          <t>bread-pakodas</t>
+        </is>
+      </c>
+      <c r="D219" t="inlineStr">
+        <is>
+          <t>Bread Pakodas</t>
+        </is>
+      </c>
+      <c r="E219" t="inlineStr">
+        <is>
+          <t>பிரட் பக்கோடா</t>
+        </is>
+      </c>
+      <c r="F219" t="inlineStr">
+        <is>
+          <t>bajji</t>
+        </is>
+      </c>
+      <c r="G219" t="inlineStr">
+        <is>
+          <t>A photorealistic photo of golden-brown irregular fried pakoda pieces with a soft doughy bread interior visible at the torn edges, piled on a plate, served with tomato ketchup, natural daylight.</t>
+        </is>
+      </c>
+      <c r="H219" t="inlineStr">
+        <is>
+          <t>public/images/recipes/bread-pakodas/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I219" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" t="n">
+        <v>219</v>
+      </c>
+      <c r="B220" t="inlineStr">
+        <is>
+          <t>Vegetarian</t>
+        </is>
+      </c>
+      <c r="C220" t="inlineStr">
+        <is>
+          <t>vermicelli-pakodas</t>
+        </is>
+      </c>
+      <c r="D220" t="inlineStr">
+        <is>
+          <t>Vermicelli Pakodas</t>
+        </is>
+      </c>
+      <c r="E220" t="inlineStr">
+        <is>
+          <t>சேமியா பக்கோடா</t>
+        </is>
+      </c>
+      <c r="F220" t="inlineStr">
+        <is>
+          <t>bajji</t>
+        </is>
+      </c>
+      <c r="G220" t="inlineStr">
+        <is>
+          <t>A photorealistic close-up of golden fried pakodas with fine strands of crisp vermicelli visible on the textured surface, piled on a steel plate with mint chutney, warm ambient lighting.</t>
+        </is>
+      </c>
+      <c r="H220" t="inlineStr">
+        <is>
+          <t>public/images/recipes/vermicelli-pakodas/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I220" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" t="n">
+        <v>220</v>
+      </c>
+      <c r="B221" t="inlineStr">
+        <is>
+          <t>Vegetarian</t>
+        </is>
+      </c>
+      <c r="C221" t="inlineStr">
+        <is>
+          <t>layered-sandwich-bajji</t>
+        </is>
+      </c>
+      <c r="D221" t="inlineStr">
+        <is>
+          <t>Layered Sandwich Bajji</t>
+        </is>
+      </c>
+      <c r="E221" t="inlineStr">
+        <is>
+          <t>பிரட் சாண்ட்விட்ச் பஜ்ஜி</t>
+        </is>
+      </c>
+      <c r="F221" t="inlineStr">
+        <is>
+          <t>bajji,sandwich</t>
+        </is>
+      </c>
+      <c r="G221" t="inlineStr">
+        <is>
+          <t>A photorealistic close-up of a golden fried rectangular sandwich bajji cut in half, showing three layers of white bread with visible green mint chutney and red tomato chutney filling between the layers, crisp golden batter coating on the outside, served with tomato sauce, bright natural lighting.</t>
+        </is>
+      </c>
+      <c r="H221" t="inlineStr">
+        <is>
+          <t>public/images/recipes/layered-sandwich-bajji/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I221" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" t="n">
+        <v>221</v>
+      </c>
+      <c r="B222" t="inlineStr">
+        <is>
+          <t>Vegetarian</t>
+        </is>
+      </c>
+      <c r="C222" t="inlineStr">
+        <is>
+          <t>capsicum-bajji</t>
+        </is>
+      </c>
+      <c r="D222" t="inlineStr">
+        <is>
+          <t>Capsicum Bajji</t>
+        </is>
+      </c>
+      <c r="E222" t="inlineStr">
+        <is>
+          <t>குடமிளகாய் பஜ்ஜி</t>
+        </is>
+      </c>
+      <c r="F222" t="inlineStr">
+        <is>
+          <t>bajji</t>
+        </is>
+      </c>
+      <c r="G222" t="inlineStr">
+        <is>
+          <t>A photorealistic photo of whole small green capsicums coated in a golden fried batter, one sliced open at the top showing chopped onion tucked inside with a wedge of lemon on the side, plated attractively, warm lighting.</t>
+        </is>
+      </c>
+      <c r="H222" t="inlineStr">
+        <is>
+          <t>public/images/recipes/capsicum-bajji/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I222" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" t="n">
+        <v>222</v>
+      </c>
+      <c r="B223" t="inlineStr">
+        <is>
+          <t>Vegetarian</t>
+        </is>
+      </c>
+      <c r="C223" t="inlineStr">
+        <is>
+          <t>stuffed-chilli-bajji</t>
+        </is>
+      </c>
+      <c r="D223" t="inlineStr">
+        <is>
+          <t>Stuffed Chilli Bajji</t>
+        </is>
+      </c>
+      <c r="E223" t="inlineStr">
+        <is>
+          <t>மிளகாய் பஜ்ஜி</t>
+        </is>
+      </c>
+      <c r="F223" t="inlineStr">
+        <is>
+          <t>bajji</t>
+        </is>
+      </c>
+      <c r="G223" t="inlineStr">
+        <is>
+          <t>A photorealistic close-up of long green bajji chilies coated in golden fried batter, one split open lengthwise to reveal a pale coconut-and-gram filling inside, garnished with chopped onion and a drizzle of sweet brown chutney, plated on a steel dish, warm tea-stall lighting.</t>
+        </is>
+      </c>
+      <c r="H223" t="inlineStr">
+        <is>
+          <t>public/images/recipes/stuffed-chilli-bajji/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I223" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" t="n">
+        <v>223</v>
+      </c>
+      <c r="B224" t="inlineStr">
+        <is>
+          <t>Vegetarian</t>
+        </is>
+      </c>
+      <c r="C224" t="inlineStr">
+        <is>
+          <t>lasania</t>
+        </is>
+      </c>
+      <c r="D224" t="inlineStr">
+        <is>
+          <t>Lasania (Stuffed Potato Bajji)</t>
+        </is>
+      </c>
+      <c r="E224" t="inlineStr">
+        <is>
+          <t>உருளைகிழங்கு ஸ்டப் பஜ்ஜி</t>
+        </is>
+      </c>
+      <c r="F224" t="inlineStr">
+        <is>
+          <t>bajji</t>
+        </is>
+      </c>
+      <c r="G224" t="inlineStr">
+        <is>
+          <t>A photorealistic photo of small whole potatoes coated in golden fried batter, one sliced partway open showing a reddish garlic-spice paste inside, piled on a plate, warm lighting.</t>
+        </is>
+      </c>
+      <c r="H224" t="inlineStr">
+        <is>
+          <t>public/images/recipes/lasania/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I224" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" t="n">
+        <v>224</v>
+      </c>
+      <c r="B225" t="inlineStr">
+        <is>
+          <t>Vegetarian</t>
+        </is>
+      </c>
+      <c r="C225" t="inlineStr">
+        <is>
+          <t>medu-vadai</t>
+        </is>
+      </c>
+      <c r="D225" t="inlineStr">
+        <is>
+          <t>Medu Vadai</t>
+        </is>
+      </c>
+      <c r="E225" t="inlineStr">
+        <is>
+          <t>மெதுவடை</t>
+        </is>
+      </c>
+      <c r="F225" t="inlineStr">
+        <is>
+          <t>vadai</t>
+        </is>
+      </c>
+      <c r="G225" t="inlineStr">
+        <is>
+          <t>A photorealistic close-up of classic golden-brown ring-shaped vadais with a lacy, crisp textured surface, stacked on a banana leaf, served with sambar in a small steel bowl and coconut chutney, warm South Indian breakfast table lighting.</t>
+        </is>
+      </c>
+      <c r="H225" t="inlineStr">
+        <is>
+          <t>public/images/recipes/medu-vadai/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I225" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" t="n">
+        <v>225</v>
+      </c>
+      <c r="B226" t="inlineStr">
+        <is>
+          <t>Vegetarian</t>
+        </is>
+      </c>
+      <c r="C226" t="inlineStr">
+        <is>
+          <t>curd-vadai</t>
+        </is>
+      </c>
+      <c r="D226" t="inlineStr">
+        <is>
+          <t>Thair Vadai</t>
+        </is>
+      </c>
+      <c r="E226" t="inlineStr">
+        <is>
+          <t>தயிர் வடை</t>
+        </is>
+      </c>
+      <c r="F226" t="inlineStr">
+        <is>
+          <t>vadai</t>
+        </is>
+      </c>
+      <c r="G226" t="inlineStr">
+        <is>
+          <t>A photorealistic close-up of soft, pale golden vadais submerged in thick white curd on a steel plate, garnished with a drizzle of tempered mustard seeds, chopped coriander leaves, and a light dusting of red chili powder on top, bright natural lighting.</t>
+        </is>
+      </c>
+      <c r="H226" t="inlineStr">
+        <is>
+          <t>public/images/recipes/curd-vadai/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I226" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" t="n">
+        <v>226</v>
+      </c>
+      <c r="B227" t="inlineStr">
+        <is>
+          <t>Vegetarian</t>
+        </is>
+      </c>
+      <c r="C227" t="inlineStr">
+        <is>
+          <t>special-curd-vadai-1</t>
+        </is>
+      </c>
+      <c r="D227" t="inlineStr">
+        <is>
+          <t>Special Curd Vadai 1</t>
+        </is>
+      </c>
+      <c r="E227" t="inlineStr">
+        <is>
+          <t>ஸ்பெஷல் தயிர் வடை (1)</t>
+        </is>
+      </c>
+      <c r="F227" t="inlineStr">
+        <is>
+          <t>vadai</t>
+        </is>
+      </c>
+      <c r="G227" t="inlineStr">
+        <is>
+          <t>A photorealistic close-up of a curd-soaked vadai cut open on a plate revealing a colorful filling of chopped cashews, almonds, raisins, and coconut inside the soft white lentil dough, surrounded by thick curd, garnished with fried spicy boondi on top, bright lighting.</t>
+        </is>
+      </c>
+      <c r="H227" t="inlineStr">
+        <is>
+          <t>public/images/recipes/special-curd-vadai-1/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I227" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" t="n">
+        <v>227</v>
+      </c>
+      <c r="B228" t="inlineStr">
+        <is>
+          <t>Vegetarian</t>
+        </is>
+      </c>
+      <c r="C228" t="inlineStr">
+        <is>
+          <t>special-curd-vadai-2</t>
+        </is>
+      </c>
+      <c r="D228" t="inlineStr">
+        <is>
+          <t>Special Curd Vadai 2</t>
+        </is>
+      </c>
+      <c r="E228" t="inlineStr">
+        <is>
+          <t>ஸ்பெஷல் தயிர் வடை (2)</t>
+        </is>
+      </c>
+      <c r="F228" t="inlineStr">
+        <is>
+          <t>vadai</t>
+        </is>
+      </c>
+      <c r="G228" t="inlineStr">
+        <is>
+          <t>A photorealistic close-up of a half-moon, samosa-shaped curd vadai on a plate, soaked in white curd, with visible green herb flecks along the folded edge, garnished with grated carrot and coriander, natural lighting.</t>
+        </is>
+      </c>
+      <c r="H228" t="inlineStr">
+        <is>
+          <t>public/images/recipes/special-curd-vadai-2/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I228" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" t="n">
+        <v>228</v>
+      </c>
+      <c r="B229" t="inlineStr">
+        <is>
+          <t>Vegetarian</t>
+        </is>
+      </c>
+      <c r="C229" t="inlineStr">
+        <is>
+          <t>pattani-curd-vadai</t>
+        </is>
+      </c>
+      <c r="D229" t="inlineStr">
+        <is>
+          <t>Pattani Curd Vadai</t>
+        </is>
+      </c>
+      <c r="E229" t="inlineStr">
+        <is>
+          <t>பட்டாணி தயிர் வடை</t>
+        </is>
+      </c>
+      <c r="F229" t="inlineStr">
+        <is>
+          <t>vadai</t>
+        </is>
+      </c>
+      <c r="G229" t="inlineStr">
+        <is>
+          <t>A photorealistic close-up of a curd-soaked vadai cut in half showing a bright green mashed-pea filling inside the soft white lentil exterior, surrounded by thick curd on a steel plate, garnished with coriander, natural lighting.</t>
+        </is>
+      </c>
+      <c r="H229" t="inlineStr">
+        <is>
+          <t>public/images/recipes/pattani-curd-vadai/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I229" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" t="n">
+        <v>229</v>
+      </c>
+      <c r="B230" t="inlineStr">
+        <is>
+          <t>Vegetarian</t>
+        </is>
+      </c>
+      <c r="C230" t="inlineStr">
+        <is>
+          <t>mor-kuzhambu-vadai</t>
+        </is>
+      </c>
+      <c r="D230" t="inlineStr">
+        <is>
+          <t>Mor Kuzhambu Vadai</t>
+        </is>
+      </c>
+      <c r="E230" t="inlineStr">
+        <is>
+          <t>மோர்க்குழம்பு வடை</t>
+        </is>
+      </c>
+      <c r="F230" t="inlineStr">
+        <is>
+          <t>vadai</t>
+        </is>
+      </c>
+      <c r="G230" t="inlineStr">
+        <is>
+          <t>A photorealistic close-up of pale golden vadais submerged in a thick, pale-yellow spiced buttermilk gravy flecked with coconut and curry leaves, served in a steel bowl, garnished with coriander leaves, warm home-style lighting.</t>
+        </is>
+      </c>
+      <c r="H230" t="inlineStr">
+        <is>
+          <t>public/images/recipes/mor-kuzhambu-vadai/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I230" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" t="n">
+        <v>230</v>
+      </c>
+      <c r="B231" t="inlineStr">
+        <is>
+          <t>Vegetarian</t>
+        </is>
+      </c>
+      <c r="C231" t="inlineStr">
+        <is>
+          <t>aamai-vadai</t>
+        </is>
+      </c>
+      <c r="D231" t="inlineStr">
+        <is>
+          <t>Aamai Vadai</t>
+        </is>
+      </c>
+      <c r="E231" t="inlineStr">
+        <is>
+          <t>ஆமை வடை</t>
+        </is>
+      </c>
+      <c r="F231" t="inlineStr">
+        <is>
+          <t>vadai</t>
+        </is>
+      </c>
+      <c r="G231" t="inlineStr">
+        <is>
+          <t>A photorealistic photo of torn half-moon pieces of coarse-textured urad-toor dal vadai, soaked briefly in curd, plated with a light garnish, rustic table lighting.</t>
+        </is>
+      </c>
+      <c r="H231" t="inlineStr">
+        <is>
+          <t>public/images/recipes/aamai-vadai/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I231" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" t="n">
+        <v>231</v>
+      </c>
+      <c r="B232" t="inlineStr">
+        <is>
+          <t>Vegetarian</t>
+        </is>
+      </c>
+      <c r="C232" t="inlineStr">
+        <is>
+          <t>bread-dahi-vadai</t>
+        </is>
+      </c>
+      <c r="D232" t="inlineStr">
+        <is>
+          <t>Bread Dahi Vadai</t>
+        </is>
+      </c>
+      <c r="E232" t="inlineStr">
+        <is>
+          <t>திடீர் பிரட் தயிர்வடை</t>
+        </is>
+      </c>
+      <c r="F232" t="inlineStr">
+        <is>
+          <t>vadai</t>
+        </is>
+      </c>
+      <c r="G232" t="inlineStr">
+        <is>
+          <t>A photorealistic close-up of small round bread-dough vadais topped generously with white curd, dusted with black salt, roasted cumin powder, and red chili powder, drizzled with brown sweet chutney and garnished with coriander leaves, bright appetizing lighting.</t>
+        </is>
+      </c>
+      <c r="H232" t="inlineStr">
+        <is>
+          <t>public/images/recipes/bread-dahi-vadai/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I232" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" t="n">
+        <v>232</v>
+      </c>
+      <c r="B233" t="inlineStr">
+        <is>
+          <t>Vegetarian</t>
+        </is>
+      </c>
+      <c r="C233" t="inlineStr">
+        <is>
+          <t>moong-dhal-curd-pakoda</t>
+        </is>
+      </c>
+      <c r="D233" t="inlineStr">
+        <is>
+          <t>Moong Dhal Curd Pakoda</t>
+        </is>
+      </c>
+      <c r="E233" t="inlineStr">
+        <is>
+          <t>பயத்தம் பருப்பு தயிர் பக்கோடா</t>
+        </is>
+      </c>
+      <c r="F233" t="inlineStr">
+        <is>
+          <t>bajji</t>
+        </is>
+      </c>
+      <c r="G233" t="inlineStr">
+        <is>
+          <t>A photorealistic close-up of small golden fried lentil pakodas arranged on a plate, topped with a generous pour of white whisked curd, dusted with a dark spice powder and tomato sauce drizzle, bright lighting.</t>
+        </is>
+      </c>
+      <c r="H233" t="inlineStr">
+        <is>
+          <t>public/images/recipes/moong-dhal-curd-pakoda/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I233" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" t="n">
+        <v>233</v>
+      </c>
+      <c r="B234" t="inlineStr">
+        <is>
+          <t>Vegetarian</t>
+        </is>
+      </c>
+      <c r="C234" t="inlineStr">
+        <is>
+          <t>mysore-vadai</t>
+        </is>
+      </c>
+      <c r="D234" t="inlineStr">
+        <is>
+          <t>Mysore Vadai</t>
+        </is>
+      </c>
+      <c r="E234" t="inlineStr">
+        <is>
+          <t>மைசூர் வடை</t>
+        </is>
+      </c>
+      <c r="F234" t="inlineStr">
+        <is>
+          <t>vadai</t>
+        </is>
+      </c>
+      <c r="G234" t="inlineStr">
+        <is>
+          <t>A photorealistic close-up of textured, coarse golden-brown vadais studded with visible cashew pieces and melon seeds, stacked on a plate, served with thokku, warm lighting.</t>
+        </is>
+      </c>
+      <c r="H234" t="inlineStr">
+        <is>
+          <t>public/images/recipes/mysore-vadai/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I234" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" t="n">
+        <v>234</v>
+      </c>
+      <c r="B235" t="inlineStr">
+        <is>
+          <t>Vegetarian</t>
+        </is>
+      </c>
+      <c r="C235" t="inlineStr">
+        <is>
+          <t>madhur-vadai</t>
+        </is>
+      </c>
+      <c r="D235" t="inlineStr">
+        <is>
+          <t>Madhur Vadai</t>
+        </is>
+      </c>
+      <c r="E235" t="inlineStr">
+        <is>
+          <t>மதுர் வடை</t>
+        </is>
+      </c>
+      <c r="F235" t="inlineStr">
+        <is>
+          <t>vadai</t>
+        </is>
+      </c>
+      <c r="G235" t="inlineStr">
+        <is>
+          <t>A photorealistic photo of thin, flat, deep reddish-brown crispy discs with visible onion flecks, stacked in a glass jar and also arranged on a plate, matte crunchy texture, natural light.</t>
+        </is>
+      </c>
+      <c r="H235" t="inlineStr">
+        <is>
+          <t>public/images/recipes/madhur-vadai/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I235" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" t="n">
+        <v>235</v>
+      </c>
+      <c r="B236" t="inlineStr">
+        <is>
+          <t>Vegetarian</t>
+        </is>
+      </c>
+      <c r="C236" t="inlineStr">
+        <is>
+          <t>masal-vadai</t>
+        </is>
+      </c>
+      <c r="D236" t="inlineStr">
+        <is>
+          <t>Masal Vadai</t>
+        </is>
+      </c>
+      <c r="E236" t="inlineStr">
+        <is>
+          <t>மசால் வடை</t>
+        </is>
+      </c>
+      <c r="F236" t="inlineStr">
+        <is>
+          <t>vadai</t>
+        </is>
+      </c>
+      <c r="G236" t="inlineStr">
+        <is>
+          <t>A photorealistic close-up of flat, coarse-textured golden-brown vadais with visible chana dal grains, onion, and curry leaf flecks, stacked on a banana leaf, served with coconut chutney, warm lighting.</t>
+        </is>
+      </c>
+      <c r="H236" t="inlineStr">
+        <is>
+          <t>public/images/recipes/masal-vadai/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I236" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" t="n">
+        <v>236</v>
+      </c>
+      <c r="B237" t="inlineStr">
+        <is>
+          <t>Vegetarian</t>
+        </is>
+      </c>
+      <c r="C237" t="inlineStr">
+        <is>
+          <t>gherugu-vadai</t>
+        </is>
+      </c>
+      <c r="D237" t="inlineStr">
+        <is>
+          <t>Gherugu Vadai</t>
+        </is>
+      </c>
+      <c r="E237" t="inlineStr">
+        <is>
+          <t>கெருகு வடை</t>
+        </is>
+      </c>
+      <c r="F237" t="inlineStr">
+        <is>
+          <t>vadai</t>
+        </is>
+      </c>
+      <c r="G237" t="inlineStr">
+        <is>
+          <t>A photorealistic photo of thin, flat, pale golden crispy discs with a slightly speckled sesame-seed texture, stacked on a plate, rustic homely lighting.</t>
+        </is>
+      </c>
+      <c r="H237" t="inlineStr">
+        <is>
+          <t>public/images/recipes/gherugu-vadai/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I237" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238" t="n">
+        <v>237</v>
+      </c>
+      <c r="B238" t="inlineStr">
+        <is>
+          <t>Vegetarian</t>
+        </is>
+      </c>
+      <c r="C238" t="inlineStr">
+        <is>
+          <t>mullangi-vadai</t>
+        </is>
+      </c>
+      <c r="D238" t="inlineStr">
+        <is>
+          <t>Mullangi Vadai</t>
+        </is>
+      </c>
+      <c r="E238" t="inlineStr">
+        <is>
+          <t>முள்ளங்கி வடை</t>
+        </is>
+      </c>
+      <c r="F238" t="inlineStr">
+        <is>
+          <t>vadai</t>
+        </is>
+      </c>
+      <c r="G238" t="inlineStr">
+        <is>
+          <t>A photorealistic close-up of thin, flat, pale golden-brown vadais with visible shreds of white radish embedded in the crisp exterior, stacked on a steel plate, natural daylight.</t>
+        </is>
+      </c>
+      <c r="H238" t="inlineStr">
+        <is>
+          <t>public/images/recipes/mullangi-vadai/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I238" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" t="n">
+        <v>238</v>
+      </c>
+      <c r="B239" t="inlineStr">
+        <is>
+          <t>Vegetarian</t>
+        </is>
+      </c>
+      <c r="C239" t="inlineStr">
+        <is>
+          <t>pulusu-vadai</t>
+        </is>
+      </c>
+      <c r="D239" t="inlineStr">
+        <is>
+          <t>Pulusu Vadai</t>
+        </is>
+      </c>
+      <c r="E239" t="inlineStr">
+        <is>
+          <t>புளி வடை அல்லது புலுசு வடை</t>
+        </is>
+      </c>
+      <c r="F239" t="inlineStr">
+        <is>
+          <t>vadai</t>
+        </is>
+      </c>
+      <c r="G239" t="inlineStr">
+        <is>
+          <t>A photorealistic photo of flat reddish-orange vadais with a speckled texture from ground red chili and pumpkin, stacked on a plate, tangy glossy sheen, warm lighting.</t>
+        </is>
+      </c>
+      <c r="H239" t="inlineStr">
+        <is>
+          <t>public/images/recipes/pulusu-vadai/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I239" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" t="n">
+        <v>239</v>
+      </c>
+      <c r="B240" t="inlineStr">
+        <is>
+          <t>Vegetarian</t>
+        </is>
+      </c>
+      <c r="C240" t="inlineStr">
+        <is>
+          <t>milagu-vadai</t>
+        </is>
+      </c>
+      <c r="D240" t="inlineStr">
+        <is>
+          <t>Milagu Vadai</t>
+        </is>
+      </c>
+      <c r="E240" t="inlineStr">
+        <is>
+          <t>மிளகு வடை</t>
+        </is>
+      </c>
+      <c r="F240" t="inlineStr">
+        <is>
+          <t>vadai</t>
+        </is>
+      </c>
+      <c r="G240" t="inlineStr">
+        <is>
+          <t>A photorealistic close-up of small pale golden vadais with visible flecks of cracked black pepper, some strung together on a thread like a garland, others piled on a plate, temple-offering style presentation, warm devotional lighting.</t>
+        </is>
+      </c>
+      <c r="H240" t="inlineStr">
+        <is>
+          <t>public/images/recipes/milagu-vadai/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I240" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="241">
+      <c r="A241" t="n">
+        <v>240</v>
+      </c>
+      <c r="B241" t="inlineStr">
+        <is>
+          <t>Vegetarian</t>
+        </is>
+      </c>
+      <c r="C241" t="inlineStr">
+        <is>
+          <t>drumstick-vadai</t>
+        </is>
+      </c>
+      <c r="D241" t="inlineStr">
+        <is>
+          <t>Drumstick Vadai</t>
+        </is>
+      </c>
+      <c r="E241" t="inlineStr">
+        <is>
+          <t>முருங்கைக்காய் வடை</t>
+        </is>
+      </c>
+      <c r="F241" t="inlineStr">
+        <is>
+          <t>vadai</t>
+        </is>
+      </c>
+      <c r="G241" t="inlineStr">
+        <is>
+          <t>A photorealistic close-up of coarse, flat golden-brown vadais with a slightly speckled surface, stacked on a plate, served with vinegar-tossed onion rings on the side, warm lighting.</t>
+        </is>
+      </c>
+      <c r="H241" t="inlineStr">
+        <is>
+          <t>public/images/recipes/drumstick-vadai/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I241" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="242">
+      <c r="A242" t="n">
+        <v>241</v>
+      </c>
+      <c r="B242" t="inlineStr">
+        <is>
+          <t>Vegetarian</t>
+        </is>
+      </c>
+      <c r="C242" t="inlineStr">
+        <is>
+          <t>perugu-vadai</t>
+        </is>
+      </c>
+      <c r="D242" t="inlineStr">
+        <is>
+          <t>Perugu Vadai</t>
+        </is>
+      </c>
+      <c r="E242" t="inlineStr">
+        <is>
+          <t>பெருகு வடை</t>
+        </is>
+      </c>
+      <c r="F242" t="inlineStr">
+        <is>
+          <t>vadai</t>
+        </is>
+      </c>
+      <c r="G242" t="inlineStr">
+        <is>
+          <t>A photorealistic photo of soft, pale, lightly golden flat discs with a matte soft surface (not deeply fried), stacked on a plate, gentle lighting emphasizing their softness.</t>
+        </is>
+      </c>
+      <c r="H242" t="inlineStr">
+        <is>
+          <t>public/images/recipes/perugu-vadai/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I242" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="243">
+      <c r="A243" t="n">
+        <v>242</v>
+      </c>
+      <c r="B243" t="inlineStr">
+        <is>
+          <t>Vegetarian</t>
+        </is>
+      </c>
+      <c r="C243" t="inlineStr">
+        <is>
+          <t>moong-dhal-toast</t>
+        </is>
+      </c>
+      <c r="D243" t="inlineStr">
+        <is>
+          <t>Moong Dhal Toast</t>
+        </is>
+      </c>
+      <c r="E243" t="inlineStr">
+        <is>
+          <t>பயத்தம்பருப்பு டோஸ்ட்</t>
+        </is>
+      </c>
+      <c r="F243" t="inlineStr">
+        <is>
+          <t>sandwich</t>
+        </is>
+      </c>
+      <c r="G243" t="inlineStr">
+        <is>
+          <t>A photorealistic close-up of a golden-brown fried bread toast cut diagonally, showing a thin green mint chutney layer and a yellow lentil paste layer between the crisp bread surface and the crust, plated with tomato sauce, bright lighting.</t>
+        </is>
+      </c>
+      <c r="H243" t="inlineStr">
+        <is>
+          <t>public/images/recipes/moong-dhal-toast/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I243" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="244">
+      <c r="A244" t="n">
+        <v>243</v>
+      </c>
+      <c r="B244" t="inlineStr">
+        <is>
+          <t>Vegetarian</t>
+        </is>
+      </c>
+      <c r="C244" t="inlineStr">
+        <is>
+          <t>masala-toast</t>
+        </is>
+      </c>
+      <c r="D244" t="inlineStr">
+        <is>
+          <t>Masala Toast</t>
+        </is>
+      </c>
+      <c r="E244" t="inlineStr">
+        <is>
+          <t>மசாலா டோஸ்ட்</t>
+        </is>
+      </c>
+      <c r="F244" t="inlineStr">
+        <is>
+          <t>sandwich</t>
+        </is>
+      </c>
+      <c r="G244" t="inlineStr">
+        <is>
+          <t>A photorealistic photo of golden-brown toasted bread slices with a thin reddish-brown spice chutney visible on the surface, griddle-toasted with light char marks, stacked on a plate, warm lighting.</t>
+        </is>
+      </c>
+      <c r="H244" t="inlineStr">
+        <is>
+          <t>public/images/recipes/masala-toast/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I244" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="245">
+      <c r="A245" t="n">
+        <v>244</v>
+      </c>
+      <c r="B245" t="inlineStr">
+        <is>
+          <t>Vegetarian</t>
+        </is>
+      </c>
+      <c r="C245" t="inlineStr">
+        <is>
+          <t>tomato-toast</t>
+        </is>
+      </c>
+      <c r="D245" t="inlineStr">
+        <is>
+          <t>Tomato Toast</t>
+        </is>
+      </c>
+      <c r="E245" t="inlineStr">
+        <is>
+          <t>தக்காளி டோஸ்ட்</t>
+        </is>
+      </c>
+      <c r="F245" t="inlineStr">
+        <is>
+          <t>sandwich</t>
+        </is>
+      </c>
+      <c r="G245" t="inlineStr">
+        <is>
+          <t>A photorealistic close-up of a golden-toasted bread slice topped with a glossy reddish-orange cooked tomato-onion masala spread evenly across the surface, slightly caramelized edges, plated hot, warm kitchen lighting.</t>
+        </is>
+      </c>
+      <c r="H245" t="inlineStr">
+        <is>
+          <t>public/images/recipes/tomato-toast/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I245" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="246">
+      <c r="A246" t="n">
+        <v>245</v>
+      </c>
+      <c r="B246" t="inlineStr">
+        <is>
+          <t>Vegetarian</t>
+        </is>
+      </c>
+      <c r="C246" t="inlineStr">
+        <is>
+          <t>potato-sandwich</t>
+        </is>
+      </c>
+      <c r="D246" t="inlineStr">
+        <is>
+          <t>Potato Sandwich</t>
+        </is>
+      </c>
+      <c r="E246" t="inlineStr">
+        <is>
+          <t>உருளைக்கிழங்கு பிரட் சாண்ட்விச்</t>
+        </is>
+      </c>
+      <c r="F246" t="inlineStr">
+        <is>
+          <t>sandwich</t>
+        </is>
+      </c>
+      <c r="G246" t="inlineStr">
+        <is>
+          <t>A photorealistic close-up of a golden-brown griddle-fried sandwich cut diagonally, showing a thick yellow spiced-potato filling coated in crisp bread crumbs between the toasted bread layers, plated with ketchup, bright appetizing lighting.</t>
+        </is>
+      </c>
+      <c r="H246" t="inlineStr">
+        <is>
+          <t>public/images/recipes/potato-sandwich/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I246" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="247">
+      <c r="A247" t="n">
+        <v>246</v>
+      </c>
+      <c r="B247" t="inlineStr">
+        <is>
+          <t>Vegetarian</t>
+        </is>
+      </c>
+      <c r="C247" t="inlineStr">
+        <is>
+          <t>corn-sandwich</t>
+        </is>
+      </c>
+      <c r="D247" t="inlineStr">
+        <is>
+          <t>Corn Sandwich</t>
+        </is>
+      </c>
+      <c r="E247" t="inlineStr">
+        <is>
+          <t>மக்காச்சோள சாண்ட்விச்</t>
+        </is>
+      </c>
+      <c r="F247" t="inlineStr">
+        <is>
+          <t>sandwich</t>
+        </is>
+      </c>
+      <c r="G247" t="inlineStr">
+        <is>
+          <t>A photorealistic photo of an open-faced toast topped with golden corn kernels mixed with cream, and a layer of melted golden cheese bubbling on top, baked and lightly browned, warm oven-fresh lighting.</t>
+        </is>
+      </c>
+      <c r="H247" t="inlineStr">
+        <is>
+          <t>public/images/recipes/corn-sandwich/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I247" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="248">
+      <c r="A248" t="n">
+        <v>247</v>
+      </c>
+      <c r="B248" t="inlineStr">
+        <is>
+          <t>Vegetarian</t>
+        </is>
+      </c>
+      <c r="C248" t="inlineStr">
+        <is>
+          <t>tomato-ketchup</t>
+        </is>
+      </c>
+      <c r="D248" t="inlineStr">
+        <is>
+          <t>Tomato Ketchup</t>
+        </is>
+      </c>
+      <c r="E248" t="inlineStr">
+        <is>
+          <t>தக்காளி கெட்ச்அப்</t>
+        </is>
+      </c>
+      <c r="F248" t="inlineStr">
+        <is>
+          <t>chutney</t>
+        </is>
+      </c>
+      <c r="G248" t="inlineStr">
+        <is>
+          <t>A photorealistic close-up of a clear glass bottle filled with thick, deep-red glossy homemade tomato ketchup, a spoonful pooled beside it on a white plate showing its smooth, thick consistency, bright clean lighting.</t>
+        </is>
+      </c>
+      <c r="H248" t="inlineStr">
+        <is>
+          <t>public/images/recipes/tomato-ketchup/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I248" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="249">
+      <c r="A249" t="n">
+        <v>248</v>
+      </c>
+      <c r="B249" t="inlineStr">
+        <is>
+          <t>Vegetarian</t>
+        </is>
+      </c>
+      <c r="C249" t="inlineStr">
+        <is>
+          <t>vegetable-sandwich</t>
+        </is>
+      </c>
+      <c r="D249" t="inlineStr">
+        <is>
+          <t>Vegetable Sandwich</t>
+        </is>
+      </c>
+      <c r="E249" t="inlineStr">
+        <is>
+          <t>காய்கறி சாண்ட்விச்</t>
+        </is>
+      </c>
+      <c r="F249" t="inlineStr">
+        <is>
+          <t>sandwich</t>
+        </is>
+      </c>
+      <c r="G249" t="inlineStr">
+        <is>
+          <t>A photorealistic close-up of a triangle-cut sandwich showing distinct colorful layers of thin cucumber, carrot, tomato, and onion rounds between green mint-chutney-spread bread, fresh and vibrant, natural bright lighting.</t>
+        </is>
+      </c>
+      <c r="H249" t="inlineStr">
+        <is>
+          <t>public/images/recipes/vegetable-sandwich/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I249" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="250">
+      <c r="A250" t="n">
+        <v>249</v>
+      </c>
+      <c r="B250" t="inlineStr">
+        <is>
+          <t>Vegetarian</t>
+        </is>
+      </c>
+      <c r="C250" t="inlineStr">
+        <is>
+          <t>chilli-cheese-sandwich</t>
+        </is>
+      </c>
+      <c r="D250" t="inlineStr">
+        <is>
+          <t>Chilli Cheese Sandwich</t>
+        </is>
+      </c>
+      <c r="E250" t="inlineStr">
+        <is>
+          <t>சில்லி சீஸ் சாண்ட்விச்</t>
+        </is>
+      </c>
+      <c r="F250" t="inlineStr">
+        <is>
+          <t>sandwich</t>
+        </is>
+      </c>
+      <c r="G250" t="inlineStr">
+        <is>
+          <t>A photorealistic close-up of a golden toasted sandwich cut in half, oozing melted golden cheese mixed with visible flecks of green chili and onion between the crisp bread layers, warm appetizing lighting.</t>
+        </is>
+      </c>
+      <c r="H250" t="inlineStr">
+        <is>
+          <t>public/images/recipes/chilli-cheese-sandwich/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I250" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="251">
+      <c r="A251" t="n">
+        <v>250</v>
+      </c>
+      <c r="B251" t="inlineStr">
+        <is>
+          <t>Vegetarian</t>
+        </is>
+      </c>
+      <c r="C251" t="inlineStr">
+        <is>
+          <t>paneer-sandwich</t>
+        </is>
+      </c>
+      <c r="D251" t="inlineStr">
+        <is>
+          <t>Paneer Sandwich</t>
+        </is>
+      </c>
+      <c r="E251" t="inlineStr">
+        <is>
+          <t>பாலாடைக்கட்டி சாண்ட்விச்</t>
+        </is>
+      </c>
+      <c r="F251" t="inlineStr">
+        <is>
+          <t>sandwich</t>
+        </is>
+      </c>
+      <c r="G251" t="inlineStr">
+        <is>
+          <t>A photorealistic close-up of a golden toasted sandwich cut diagonally, showing a crumbly white paneer filling studded with green sprouts and herbs between the bread layers, plated with ketchup, bright lighting.</t>
+        </is>
+      </c>
+      <c r="H251" t="inlineStr">
+        <is>
+          <t>public/images/recipes/paneer-sandwich/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I251" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="252">
+      <c r="A252" t="n">
+        <v>251</v>
+      </c>
+      <c r="B252" t="inlineStr">
+        <is>
+          <t>Vegetarian</t>
+        </is>
+      </c>
+      <c r="C252" t="inlineStr">
+        <is>
+          <t>sandwich-roll</t>
+        </is>
+      </c>
+      <c r="D252" t="inlineStr">
+        <is>
+          <t>Sandwich Roll</t>
+        </is>
+      </c>
+      <c r="E252" t="inlineStr">
+        <is>
+          <t>சாண்ட்விட்ச் ரோல்</t>
+        </is>
+      </c>
+      <c r="F252" t="inlineStr">
+        <is>
+          <t>sandwich</t>
+        </is>
+      </c>
+      <c r="G252" t="inlineStr">
+        <is>
+          <t>A photorealistic close-up of pinwheel-shaped bread roll slices arranged on a plate, showing a spiral of white bread with thin green and red chutney swirls visible in the layers, elegant party-platter presentation, bright clean lighting.</t>
+        </is>
+      </c>
+      <c r="H252" t="inlineStr">
+        <is>
+          <t>public/images/recipes/sandwich-roll/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I252" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="253">
+      <c r="A253" t="n">
+        <v>252</v>
+      </c>
+      <c r="B253" t="inlineStr">
+        <is>
+          <t>Vegetarian</t>
+        </is>
+      </c>
+      <c r="C253" t="inlineStr">
+        <is>
+          <t>aloo-chat-1</t>
+        </is>
+      </c>
+      <c r="D253" t="inlineStr">
+        <is>
+          <t>Aloo Chat 1</t>
+        </is>
+      </c>
+      <c r="E253" t="inlineStr">
+        <is>
+          <t>ஆலு சாட் - 1</t>
+        </is>
+      </c>
+      <c r="F253" t="inlineStr">
+        <is>
+          <t>chaat</t>
+        </is>
+      </c>
+      <c r="G253" t="inlineStr">
+        <is>
+          <t>A photorealistic close-up of a boiled potato stuffed and topped generously with white whisked curd, drizzled with dark brown tangy tamarind sauce, dusted with red chili powder and dark chat masala, garnished with coriander leaves, served on a decorative plate, vibrant street-food lighting.</t>
+        </is>
+      </c>
+      <c r="H253" t="inlineStr">
+        <is>
+          <t>public/images/recipes/aloo-chat-1/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I253" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="254">
+      <c r="A254" t="n">
+        <v>253</v>
+      </c>
+      <c r="B254" t="inlineStr">
+        <is>
+          <t>Vegetarian</t>
+        </is>
+      </c>
+      <c r="C254" t="inlineStr">
+        <is>
+          <t>aloo-chat-2</t>
+        </is>
+      </c>
+      <c r="D254" t="inlineStr">
+        <is>
+          <t>Aloo Chat 2</t>
+        </is>
+      </c>
+      <c r="E254" t="inlineStr">
+        <is>
+          <t>ஆலு சாட் - 2</t>
+        </is>
+      </c>
+      <c r="F254" t="inlineStr">
+        <is>
+          <t>chaat</t>
+        </is>
+      </c>
+      <c r="G254" t="inlineStr">
+        <is>
+          <t>A photorealistic photo of diced potato mixed with golden fried diamond-shaped crisps, tossed in a chat bowl with dark tangy sauce, chopped onion, and a scattering of thin crispy sev on top, colorful street-food presentation, bright lighting.</t>
+        </is>
+      </c>
+      <c r="H254" t="inlineStr">
+        <is>
+          <t>public/images/recipes/aloo-chat-2/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I254" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="255">
+      <c r="A255" t="n">
+        <v>254</v>
+      </c>
+      <c r="B255" t="inlineStr">
+        <is>
+          <t>Vegetarian</t>
+        </is>
+      </c>
+      <c r="C255" t="inlineStr">
+        <is>
+          <t>chat-masala-powder</t>
+        </is>
+      </c>
+      <c r="D255" t="inlineStr">
+        <is>
+          <t>Chat Masala Powder</t>
+        </is>
+      </c>
+      <c r="E255" t="inlineStr">
+        <is>
+          <t>சாட் மசாலா பவுடர்</t>
+        </is>
+      </c>
+      <c r="F255" t="inlineStr">
+        <is>
+          <t>chaat</t>
+        </is>
+      </c>
+      <c r="G255" t="inlineStr">
+        <is>
+          <t>A photorealistic close-up of a small glass jar filled with reddish-brown aromatic spice powder, a small mound of the powder spilled beside it on a wooden surface with whole dried red chilies and cardamom pods scattered around, warm spice-market lighting.</t>
+        </is>
+      </c>
+      <c r="H255" t="inlineStr">
+        <is>
+          <t>public/images/recipes/chat-masala-powder/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I255" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="256">
+      <c r="A256" t="n">
+        <v>255</v>
+      </c>
+      <c r="B256" t="inlineStr">
+        <is>
+          <t>Vegetarian</t>
+        </is>
+      </c>
+      <c r="C256" t="inlineStr">
+        <is>
+          <t>aloo-pappad-chat</t>
+        </is>
+      </c>
+      <c r="D256" t="inlineStr">
+        <is>
+          <t>Aloo Pappad Chat</t>
+        </is>
+      </c>
+      <c r="E256" t="inlineStr">
+        <is>
+          <t>ஆலு பப்பட் சாட்</t>
+        </is>
+      </c>
+      <c r="F256" t="inlineStr">
+        <is>
+          <t>chaat</t>
+        </is>
+      </c>
+      <c r="G256" t="inlineStr">
+        <is>
+          <t>A photorealistic close-up of a plate layered with crushed golden fried papad pieces, topped with diced potato, a generous pour of white curd, dark brown sweet chutney drizzle, and a dusting of spices with fresh coriander on top, vibrant street-food lighting.</t>
+        </is>
+      </c>
+      <c r="H256" t="inlineStr">
+        <is>
+          <t>public/images/recipes/aloo-pappad-chat/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I256" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="257">
+      <c r="A257" t="n">
+        <v>256</v>
+      </c>
+      <c r="B257" t="inlineStr">
+        <is>
+          <t>Vegetarian</t>
+        </is>
+      </c>
+      <c r="C257" t="inlineStr">
+        <is>
+          <t>mattar-chat</t>
+        </is>
+      </c>
+      <c r="D257" t="inlineStr">
+        <is>
+          <t>Mattar Chat</t>
+        </is>
+      </c>
+      <c r="E257" t="inlineStr">
+        <is>
+          <t>பச்சைப் பட்டாணி சாட்</t>
+        </is>
+      </c>
+      <c r="F257" t="inlineStr">
+        <is>
+          <t>chaat</t>
+        </is>
+      </c>
+      <c r="G257" t="inlineStr">
+        <is>
+          <t>A photorealistic close-up of a bowl of cooked green peas topped with crushed golden puri pieces, white curd, dark tamarind chutney, chopped onion, and fine crispy sev, colorful layered presentation, bright lighting.</t>
+        </is>
+      </c>
+      <c r="H257" t="inlineStr">
+        <is>
+          <t>public/images/recipes/mattar-chat/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I257" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="258">
+      <c r="A258" t="n">
+        <v>257</v>
+      </c>
+      <c r="B258" t="inlineStr">
+        <is>
+          <t>Vegetarian</t>
+        </is>
+      </c>
+      <c r="C258" t="inlineStr">
+        <is>
+          <t>fruit-vegetable-chat</t>
+        </is>
+      </c>
+      <c r="D258" t="inlineStr">
+        <is>
+          <t>Fruit &amp; Vegetable Chat</t>
+        </is>
+      </c>
+      <c r="E258" t="inlineStr">
+        <is>
+          <t>காய்கறி, பழக்கலவை சாட்</t>
+        </is>
+      </c>
+      <c r="F258" t="inlineStr">
+        <is>
+          <t>chaat</t>
+        </is>
+      </c>
+      <c r="G258" t="inlineStr">
+        <is>
+          <t>A photorealistic photo of a colorful bowl mix of diced banana, orange segments, tomato, potato, and guava tossed together, garnished with coriander leaves and a light dusting of chat masala, fresh and vibrant, bright natural lighting.</t>
+        </is>
+      </c>
+      <c r="H258" t="inlineStr">
+        <is>
+          <t>public/images/recipes/fruit-vegetable-chat/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I258" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="259">
+      <c r="A259" t="n">
+        <v>258</v>
+      </c>
+      <c r="B259" t="inlineStr">
+        <is>
+          <t>Vegetarian</t>
+        </is>
+      </c>
+      <c r="C259" t="inlineStr">
+        <is>
+          <t>finger-chips</t>
+        </is>
+      </c>
+      <c r="D259" t="inlineStr">
+        <is>
+          <t>Finger Chips</t>
+        </is>
+      </c>
+      <c r="E259" t="inlineStr">
+        <is>
+          <t>ஃபிங்கர் சிப்ஸ்</t>
+        </is>
+      </c>
+      <c r="F259" t="inlineStr">
+        <is>
+          <t>snack</t>
+        </is>
+      </c>
+      <c r="G259" t="inlineStr">
+        <is>
+          <t>A photorealistic close-up of golden-brown crispy potato finger chips piled high on a plate, lightly dusted with salt and pepper, served with tomato ketchup, bright appetizing lighting.</t>
+        </is>
+      </c>
+      <c r="H259" t="inlineStr">
+        <is>
+          <t>public/images/recipes/finger-chips/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I259" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="260">
+      <c r="A260" t="n">
+        <v>259</v>
+      </c>
+      <c r="B260" t="inlineStr">
+        <is>
+          <t>Vegetarian</t>
+        </is>
+      </c>
+      <c r="C260" t="inlineStr">
+        <is>
+          <t>crisp-groundnuts</t>
+        </is>
+      </c>
+      <c r="D260" t="inlineStr">
+        <is>
+          <t>Crisp Groundnuts</t>
+        </is>
+      </c>
+      <c r="E260" t="inlineStr">
+        <is>
+          <t>வறுகடலை</t>
+        </is>
+      </c>
+      <c r="F260" t="inlineStr">
+        <is>
+          <t>snack</t>
+        </is>
+      </c>
+      <c r="G260" t="inlineStr">
+        <is>
+          <t>A photorealistic close-up of small glossy, deep golden-brown fried groundnuts piled in a bowl, with a visible shiny sheen, some scattered on a napkin, warm snack-time lighting.</t>
+        </is>
+      </c>
+      <c r="H260" t="inlineStr">
+        <is>
+          <t>public/images/recipes/crisp-groundnuts/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I260" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="261">
+      <c r="A261" t="n">
+        <v>260</v>
+      </c>
+      <c r="B261" t="inlineStr">
+        <is>
+          <t>Vegetarian</t>
+        </is>
+      </c>
+      <c r="C261" t="inlineStr">
+        <is>
+          <t>pop-corn</t>
+        </is>
+      </c>
+      <c r="D261" t="inlineStr">
+        <is>
+          <t>Pop Corn</t>
+        </is>
+      </c>
+      <c r="E261" t="inlineStr">
+        <is>
+          <t>பாப் கார்ன்</t>
+        </is>
+      </c>
+      <c r="F261" t="inlineStr">
+        <is>
+          <t>snack</t>
+        </is>
+      </c>
+      <c r="G261" t="inlineStr">
+        <is>
+          <t>A photorealistic close-up of a bowl overflowing with fluffy white popcorn lightly dusted with orange-red spice seasoning, warm cozy lighting.</t>
+        </is>
+      </c>
+      <c r="H261" t="inlineStr">
+        <is>
+          <t>public/images/recipes/pop-corn/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I261" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="262">
+      <c r="A262" t="n">
+        <v>261</v>
+      </c>
+      <c r="B262" t="inlineStr">
+        <is>
+          <t>Vegetarian</t>
+        </is>
+      </c>
+      <c r="C262" t="inlineStr">
+        <is>
+          <t>masala-pori-1</t>
+        </is>
+      </c>
+      <c r="D262" t="inlineStr">
+        <is>
+          <t>Masala Pori 1 (Instant Bhel)</t>
+        </is>
+      </c>
+      <c r="E262" t="inlineStr">
+        <is>
+          <t>மசாலா பொரி - 1</t>
+        </is>
+      </c>
+      <c r="F262" t="inlineStr">
+        <is>
+          <t>chaat</t>
+        </is>
+      </c>
+      <c r="G262" t="inlineStr">
+        <is>
+          <t>A photorealistic photo of a colorful bowl of puffed rice mixed with roasted gram, small dice of mango, tomato, carrot, and beetroot, garnished with coriander leaves, bright vibrant street-food lighting.</t>
+        </is>
+      </c>
+      <c r="H262" t="inlineStr">
+        <is>
+          <t>public/images/recipes/masala-pori-1/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I262" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="263">
+      <c r="A263" t="n">
+        <v>262</v>
+      </c>
+      <c r="B263" t="inlineStr">
+        <is>
+          <t>Vegetarian</t>
+        </is>
+      </c>
+      <c r="C263" t="inlineStr">
+        <is>
+          <t>masala-pori-2</t>
+        </is>
+      </c>
+      <c r="D263" t="inlineStr">
+        <is>
+          <t>Masala Pori 2 (Instant Bhel)</t>
+        </is>
+      </c>
+      <c r="E263" t="inlineStr">
+        <is>
+          <t>மசாலா பொரி - 2</t>
+        </is>
+      </c>
+      <c r="F263" t="inlineStr">
+        <is>
+          <t>chaat</t>
+        </is>
+      </c>
+      <c r="G263" t="inlineStr">
+        <is>
+          <t>A photorealistic photo of a bowl of puffed rice mixed with roasted gram and groundnuts, tossed with pink-tinged marinated onion and a drizzle of dark green chutney, colorful and fresh, bright lighting.</t>
+        </is>
+      </c>
+      <c r="H263" t="inlineStr">
+        <is>
+          <t>public/images/recipes/masala-pori-2/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I263" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="264">
+      <c r="A264" t="n">
+        <v>263</v>
+      </c>
+      <c r="B264" t="inlineStr">
+        <is>
+          <t>Vegetarian</t>
+        </is>
+      </c>
+      <c r="C264" t="inlineStr">
+        <is>
+          <t>mint-coriander-chutney-cutlets</t>
+        </is>
+      </c>
+      <c r="D264" t="inlineStr">
+        <is>
+          <t>Mint-Coriander Chutney (for Cutlets)</t>
+        </is>
+      </c>
+      <c r="E264" t="inlineStr">
+        <is>
+          <t>புதினா, கொத்தமல்லி சட்னி (கட்லெட்டிற்கு)</t>
+        </is>
+      </c>
+      <c r="F264" t="inlineStr">
+        <is>
+          <t>chutney</t>
+        </is>
+      </c>
+      <c r="G264" t="inlineStr">
+        <is>
+          <t>A photorealistic close-up of a small bowl of smooth, vivid green chutney with a glossy sheen, served beside golden fried cutlets, garnished with a mint sprig, bright fresh lighting.</t>
+        </is>
+      </c>
+      <c r="H264" t="inlineStr">
+        <is>
+          <t>public/images/recipes/mint-coriander-chutney-cutlets/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I264" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="265">
+      <c r="A265" t="n">
+        <v>264</v>
+      </c>
+      <c r="B265" t="inlineStr">
+        <is>
+          <t>Vegetarian</t>
+        </is>
+      </c>
+      <c r="C265" t="inlineStr">
+        <is>
+          <t>mint-chutney-cutlets</t>
+        </is>
+      </c>
+      <c r="D265" t="inlineStr">
+        <is>
+          <t>Mint Chutney (for Cutlets)</t>
+        </is>
+      </c>
+      <c r="E265" t="inlineStr">
+        <is>
+          <t>புதினா சட்னி (கட்லெட்டிற்கு)</t>
+        </is>
+      </c>
+      <c r="F265" t="inlineStr">
+        <is>
+          <t>chutney</t>
+        </is>
+      </c>
+      <c r="G265" t="inlineStr">
+        <is>
+          <t>A photorealistic close-up of a small bowl of dark green, thick chutney with a tempered mustard-seed garnish floating on top, bright natural lighting.</t>
+        </is>
+      </c>
+      <c r="H265" t="inlineStr">
+        <is>
+          <t>public/images/recipes/mint-chutney-cutlets/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I265" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="266">
+      <c r="A266" t="n">
+        <v>265</v>
+      </c>
+      <c r="B266" t="inlineStr">
+        <is>
+          <t>Vegetarian</t>
+        </is>
+      </c>
+      <c r="C266" t="inlineStr">
+        <is>
+          <t>mint-onion-chutney</t>
+        </is>
+      </c>
+      <c r="D266" t="inlineStr">
+        <is>
+          <t>Mint-Onion Chutney</t>
+        </is>
+      </c>
+      <c r="E266" t="inlineStr">
+        <is>
+          <t>புதினா வெங்காயச் சட்னி</t>
+        </is>
+      </c>
+      <c r="F266" t="inlineStr">
+        <is>
+          <t>chutney</t>
+        </is>
+      </c>
+      <c r="G266" t="inlineStr">
+        <is>
+          <t>A photorealistic close-up of a bowl of textured dark green chutney flecked with white coconut, garnished with a tempering of mustard seeds and curry leaves on top, warm lighting.</t>
+        </is>
+      </c>
+      <c r="H266" t="inlineStr">
+        <is>
+          <t>public/images/recipes/mint-onion-chutney/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I266" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="267">
+      <c r="A267" t="n">
+        <v>266</v>
+      </c>
+      <c r="B267" t="inlineStr">
+        <is>
+          <t>Vegetarian</t>
+        </is>
+      </c>
+      <c r="C267" t="inlineStr">
+        <is>
+          <t>coriander-chutney-sandwiches</t>
+        </is>
+      </c>
+      <c r="D267" t="inlineStr">
+        <is>
+          <t>Coriander Chutney (for Sandwiches)</t>
+        </is>
+      </c>
+      <c r="E267" t="inlineStr">
+        <is>
+          <t>கொத்தமல்லி சட்னி (சாண்ட்விச்சிற்கு)</t>
+        </is>
+      </c>
+      <c r="F267" t="inlineStr">
+        <is>
+          <t>chutney</t>
+        </is>
+      </c>
+      <c r="G267" t="inlineStr">
+        <is>
+          <t>A photorealistic close-up of a small bowl of deep green-red chutney with a thick, spreadable texture, a butter knife resting beside it with chutney on the blade, bright kitchen lighting.</t>
+        </is>
+      </c>
+      <c r="H267" t="inlineStr">
+        <is>
+          <t>public/images/recipes/coriander-chutney-sandwiches/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I267" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="268">
+      <c r="A268" t="n">
+        <v>267</v>
+      </c>
+      <c r="B268" t="inlineStr">
+        <is>
+          <t>Vegetarian</t>
+        </is>
+      </c>
+      <c r="C268" t="inlineStr">
+        <is>
+          <t>garlic-chutney-sandwiches</t>
+        </is>
+      </c>
+      <c r="D268" t="inlineStr">
+        <is>
+          <t>Garlic Chutney (for Sandwiches)</t>
+        </is>
+      </c>
+      <c r="E268" t="inlineStr">
+        <is>
+          <t>பூண்டு சட்னி (சாண்ட்விச்சிற்கு)</t>
+        </is>
+      </c>
+      <c r="F268" t="inlineStr">
+        <is>
+          <t>chutney</t>
+        </is>
+      </c>
+      <c r="G268" t="inlineStr">
+        <is>
+          <t>A photorealistic close-up of a bowl of reddish-brown chutney with visible garlic and chili flecks, thick and glossy, served beside buttered bread slices, warm lighting.</t>
+        </is>
+      </c>
+      <c r="H268" t="inlineStr">
+        <is>
+          <t>public/images/recipes/garlic-chutney-sandwiches/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I268" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="269">
+      <c r="A269" t="n">
+        <v>268</v>
+      </c>
+      <c r="B269" t="inlineStr">
+        <is>
+          <t>Vegetarian</t>
+        </is>
+      </c>
+      <c r="C269" t="inlineStr">
+        <is>
+          <t>coconut-ginger-chutney-sandwiches</t>
+        </is>
+      </c>
+      <c r="D269" t="inlineStr">
+        <is>
+          <t>Coconut-Ginger Chutney (for Sandwiches)</t>
+        </is>
+      </c>
+      <c r="E269" t="inlineStr">
+        <is>
+          <t>தேங்காய், இஞ்சி சட்னி (சாண்ட்விச்சிற்கு)</t>
+        </is>
+      </c>
+      <c r="F269" t="inlineStr">
+        <is>
+          <t>chutney</t>
+        </is>
+      </c>
+      <c r="G269" t="inlineStr">
+        <is>
+          <t>A photorealistic close-up of a bowl of coarse, off-white coconut chutney with visible ginger and red chili flecks, glossy texture, natural bright lighting.</t>
+        </is>
+      </c>
+      <c r="H269" t="inlineStr">
+        <is>
+          <t>public/images/recipes/coconut-ginger-chutney-sandwiches/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I269" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="270">
+      <c r="A270" t="n">
+        <v>269</v>
+      </c>
+      <c r="B270" t="inlineStr">
+        <is>
+          <t>Vegetarian</t>
+        </is>
+      </c>
+      <c r="C270" t="inlineStr">
+        <is>
+          <t>mint-chutney-sandwiches</t>
+        </is>
+      </c>
+      <c r="D270" t="inlineStr">
+        <is>
+          <t>Mint Chutney (for Sandwiches)</t>
+        </is>
+      </c>
+      <c r="E270" t="inlineStr">
+        <is>
+          <t>புதினா சட்னி (சாண்ட்விச்சிற்கு)</t>
+        </is>
+      </c>
+      <c r="F270" t="inlineStr">
+        <is>
+          <t>chutney</t>
+        </is>
+      </c>
+      <c r="G270" t="inlineStr">
+        <is>
+          <t>A photorealistic close-up of a small bowl of smooth bright green mint chutney, glossy sheen, served beside a stack of white bread slices, fresh vibrant lighting.</t>
+        </is>
+      </c>
+      <c r="H270" t="inlineStr">
+        <is>
+          <t>public/images/recipes/mint-chutney-sandwiches/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I270" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="271">
+      <c r="A271" t="n">
+        <v>270</v>
+      </c>
+      <c r="B271" t="inlineStr">
+        <is>
+          <t>Vegetarian</t>
+        </is>
+      </c>
+      <c r="C271" t="inlineStr">
+        <is>
+          <t>onion-bajji</t>
+        </is>
+      </c>
+      <c r="D271" t="inlineStr">
+        <is>
+          <t>Onion Bajji</t>
+        </is>
+      </c>
+      <c r="E271" t="inlineStr">
+        <is>
+          <t>வெங்காயப் பஜ்ஜி</t>
+        </is>
+      </c>
+      <c r="F271" t="inlineStr">
+        <is>
+          <t>bajji</t>
+        </is>
+      </c>
+      <c r="G271" t="inlineStr">
+        <is>
+          <t>A photorealistic close-up of golden fried onion bajjis with a distinctive ring-shaped, batter-coated onion visible inside the crisp fried coating, piled on a plate, served with coconut chutney, warm tea-stall lighting.</t>
+        </is>
+      </c>
+      <c r="H271" t="inlineStr">
+        <is>
+          <t>public/images/recipes/onion-bajji/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I271" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="272">
+      <c r="A272" t="n">
+        <v>271</v>
+      </c>
+      <c r="B272" t="inlineStr">
+        <is>
+          <t>Vegetarian</t>
+        </is>
+      </c>
+      <c r="C272" t="inlineStr">
+        <is>
+          <t>vendaikkai-pakoda</t>
+        </is>
+      </c>
+      <c r="D272" t="inlineStr">
+        <is>
+          <t>Deep Fried Ladies Fingers</t>
+        </is>
+      </c>
+      <c r="E272" t="inlineStr">
+        <is>
+          <t>வெண்டைக்காய் பக்கோடா</t>
+        </is>
+      </c>
+      <c r="F272" t="inlineStr">
+        <is>
+          <t>bajji</t>
+        </is>
+      </c>
+      <c r="G272" t="inlineStr">
+        <is>
+          <t>A photorealistic close-up of whole okra pieces coated in a crisp golden fried batter with visible bread-crumb texture, arranged on a plate with tomato sauce, natural daylight.</t>
+        </is>
+      </c>
+      <c r="H272" t="inlineStr">
+        <is>
+          <t>public/images/recipes/vendaikkai-pakoda/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I272" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="273">
+      <c r="A273" t="n">
+        <v>272</v>
+      </c>
+      <c r="B273" t="inlineStr">
+        <is>
+          <t>Vegetarian</t>
+        </is>
+      </c>
+      <c r="C273" t="inlineStr">
+        <is>
+          <t>carrot-sandwich</t>
+        </is>
+      </c>
+      <c r="D273" t="inlineStr">
+        <is>
+          <t>Carrot Sandwich</t>
+        </is>
+      </c>
+      <c r="E273" t="inlineStr">
+        <is>
+          <t>கேரட் சாண்ட்விச்</t>
+        </is>
+      </c>
+      <c r="F273" t="inlineStr">
+        <is>
+          <t>sandwich</t>
+        </is>
+      </c>
+      <c r="G273" t="inlineStr">
+        <is>
+          <t>A photorealistic close-up of a pressed golden-toasted sandwich cut in half, showing a bright orange sauteed carrot-tomato filling between the bread layers, plated with tomato sauce, warm appetizing lighting.</t>
+        </is>
+      </c>
+      <c r="H273" t="inlineStr">
+        <is>
+          <t>public/images/recipes/carrot-sandwich/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I273" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
docs(tracker): rewrite batch-2 image prompts to structured template
Match the "Professional food photography of ... an Indian X: ..." format
with explicit camera angle, lighting, and negative constraints (no text/
watermark/logo/people/packaging), applied to all 71 batch-2 rows
(S.No 202-272).
</commit_message>
<xml_diff>
--- a/docs/recipe-image-tracker.xlsx
+++ b/docs/recipe-image-tracker.xlsx
@@ -11455,7 +11455,7 @@
       </c>
       <c r="G203" t="inlineStr">
         <is>
-          <t>A close-up photorealistic food photo of golden-brown oval cutlets with a crisp breadcrumb crust, plated on a white ceramic plate, garnished with a wedge of lemon and a small bowl of tomato ketchup, one cutlet broken open to reveal a soft reddish-brown banana-potato filling flecked with green coriander, warm natural lighting, shallow depth of field.</t>
+          <t>Professional food photography of "Banana Cutlets" (வாழைக்காய் கட்லெட்), an Indian snack: golden-brown oval cutlets with a crisp breadcrumb crust, one cutlet broken open to reveal a soft reddish-brown banana-potato filling flecked with green coriander, arranged on a plate with a wedge of lemon and a small bowl of tomato ketchup. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
         </is>
       </c>
       <c r="H203" t="inlineStr">
@@ -11500,7 +11500,7 @@
       </c>
       <c r="G204" t="inlineStr">
         <is>
-          <t>A dramatic photorealistic photo of a cast-iron sizzler plate on a wooden board, visibly smoking with steam rising, holding a golden fried cutlet in the center surrounded by charred grilled carrot rounds, cabbage wedges, capsicum rings, and potato slices, glossy with butter and reddish sauce, dark moody restaurant lighting.</t>
+          <t>Professional food photography of "Vegetable Sizzlers" (வெஜிடபிள் சிஸ்லர்ஸ்), an Indian fusion dish: a cast-iron sizzler plate visibly smoking with steam rising, a golden fried cutlet in the center surrounded by charred grilled carrot rounds, cabbage wedges, capsicum rings, and potato slices, glossy with butter and reddish sauce. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
         </is>
       </c>
       <c r="H204" t="inlineStr">
@@ -11545,7 +11545,7 @@
       </c>
       <c r="G205" t="inlineStr">
         <is>
-          <t>A photorealistic close-up of a round golden-brown vegetable burger patty inside a soft bun, layered with a crisp cabbage leaf, thin onion rings, beetroot slices, and tomato, skewered with a small toothpick, plated with crinkle-cut potato fries and ketchup, bright appetizing lighting.</t>
+          <t>Professional food photography of "Vegetable Burgers" (வெஜிடபிள் பர்கர்ஸ்), an Indian fusion snack: a round golden-brown vegetable burger patty inside a soft bun, layered with a crisp cabbage leaf, thin onion rings, beetroot slices, and tomato, skewered with a small toothpick, plated with crinkle-cut potato fries and ketchup. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
         </is>
       </c>
       <c r="H205" t="inlineStr">
@@ -11590,7 +11590,7 @@
       </c>
       <c r="G206" t="inlineStr">
         <is>
-          <t>A photorealistic close-up of small round golden-brown bondas with a translucent, pearly, slightly bumpy sago texture visible on the fried crust, piled on a steel plate lined with paper, garnished with coriander leaves, a small bowl of green chutney beside them, warm kitchen lighting.</t>
+          <t>Professional food photography of "Sago Bonda" (ஜவ்வரிசி போண்டா), an Indian snack: small round golden-brown bondas with a translucent, pearly, slightly bumpy sago texture on the fried crust, piled on a plate lined with paper, garnished with coriander leaves, a small bowl of green chutney beside them. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
         </is>
       </c>
       <c r="H206" t="inlineStr">
@@ -11635,7 +11635,7 @@
       </c>
       <c r="G207" t="inlineStr">
         <is>
-          <t>A photorealistic photo of golden fried round bondas with a slightly bumpy, craggy batter surface, one bonda broken in half to show a moist mixed-vegetable filling of carrot, peas, and potato, served on a steel plate with mint chutney and tomato sauce, natural daylight.</t>
+          <t>Professional food photography of "Vegetable Bonda" (வெஜிடபிள் போண்டா), an Indian snack: golden fried round bondas with a slightly bumpy, craggy batter surface, one bonda broken in half to show a moist mixed-vegetable filling of carrot, peas, and potato, served with mint chutney and tomato sauce. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
         </is>
       </c>
       <c r="H207" t="inlineStr">
@@ -11680,7 +11680,7 @@
       </c>
       <c r="G208" t="inlineStr">
         <is>
-          <t>A photorealistic image of golden-brown round bondas with a smooth thin batter coating, arranged on a banana leaf, one cut open to reveal a soft yellow mashed-potato filling flecked with onion and coriander, served with coconut chutney, warm South Indian tea-stall lighting.</t>
+          <t>Professional food photography of "Aloo Bonda" (உருளைக்கிழங்கு போண்டா), an Indian snack: golden-brown round bondas with a smooth thin batter coating, arranged on a banana leaf, one cut open to reveal a soft yellow mashed-potato filling flecked with onion and coriander, served with coconut chutney. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
         </is>
       </c>
       <c r="H208" t="inlineStr">
@@ -11725,7 +11725,7 @@
       </c>
       <c r="G209" t="inlineStr">
         <is>
-          <t>A photorealistic close-up of fluffy, irregularly round golden-brown bondas with a light, airy fried crust, stacked in a steel plate, one broken open showing a soft white lentil interior studded with coconut bits, served with coconut chutney in a small bowl, bright natural light.</t>
+          <t>Professional food photography of "Mysore Bonda" (மைசூர் போண்டா), an Indian snack: fluffy, irregularly round golden-brown bondas with a light, airy fried crust, stacked on a plate, one broken open showing a soft white lentil interior studded with coconut bits, served with coconut chutney. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
         </is>
       </c>
       <c r="H209" t="inlineStr">
@@ -11770,7 +11770,7 @@
       </c>
       <c r="G210" t="inlineStr">
         <is>
-          <t>A photorealistic photo of small irregular golden-brown fried dumplings made from fermented dosa batter, slightly craggy surface with visible onion and coriander flecks, piled on a steel plate with coconut chutney on the side, cozy kitchen lighting.</t>
+          <t>Professional food photography of "Pullani Vunta" (தோசைமாவு போண்டா), an Indian snack: small irregular golden-brown fried dumplings made from fermented dosa batter, a slightly craggy surface with visible onion and coriander flecks, piled on a plate with coconut chutney on the side. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
         </is>
       </c>
       <c r="H210" t="inlineStr">
@@ -11815,7 +11815,7 @@
       </c>
       <c r="G211" t="inlineStr">
         <is>
-          <t>A photorealistic close-up of soft, puffy golden-brown fried bondas with a slightly wrinkled curd-based batter texture, arranged on a plate, one broken open to reveal a soft white interior, served with coconut chutney, warm ambient lighting.</t>
+          <t>Professional food photography of "Mangalore Bonda" (மங்களூர் போண்டா), an Indian snack: soft, puffy golden-brown fried bondas with a slightly wrinkled curd-based batter texture, arranged on a plate, one broken open to reveal a soft white interior, served with coconut chutney. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
         </is>
       </c>
       <c r="H211" t="inlineStr">
@@ -11860,7 +11860,7 @@
       </c>
       <c r="G212" t="inlineStr">
         <is>
-          <t>A photorealistic close-up of small golden fried bondas glistening with oil, one cut in half to reveal a stretchy, melted golden-yellow cheese pull, plated on a white dish, steam rising, cozy warm lighting.</t>
+          <t>Professional food photography of "Cheese Bonda" (சீஸ் போண்டா), an Indian snack: small golden fried bondas glistening with oil, one cut in half to reveal a stretchy, melted golden-yellow cheese pull, plated with steam rising. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
         </is>
       </c>
       <c r="H212" t="inlineStr">
@@ -11905,7 +11905,7 @@
       </c>
       <c r="G213" t="inlineStr">
         <is>
-          <t>A photorealistic photo of small dark-green-flecked golden fried dumplings, irregular round shape, piled on a plate, showing visible bits of dark green spinach and chili in the crisp fried crust, served with ketchup, natural daylight.</t>
+          <t>Professional food photography of "Palak Dumplings" (பாலக் மெதுபக்கோடா), an Indian snack: small dark-green-flecked golden fried dumplings, irregular round shape, piled on a plate, showing visible bits of dark green spinach and chili in the crisp fried crust, served with ketchup. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
         </is>
       </c>
       <c r="H213" t="inlineStr">
@@ -11950,7 +11950,7 @@
       </c>
       <c r="G214" t="inlineStr">
         <is>
-          <t>A photorealistic close-up of small golden fried dumplings with pale green ridge-gourd flecks visible through the thin gram-flour crust, piled on a steel plate, served hot with tomato sauce, warm kitchen lighting.</t>
+          <t>Professional food photography of "Ridge Gourd Dumplings" (பீர்க்கங்காய் மெதுபக்கோடா), an Indian snack: small golden fried dumplings with pale green ridge-gourd flecks visible through the thin gram-flour crust, piled on a plate, served hot with tomato sauce. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
         </is>
       </c>
       <c r="H214" t="inlineStr">
@@ -11995,7 +11995,7 @@
       </c>
       <c r="G215" t="inlineStr">
         <is>
-          <t>A photorealistic photo of dark green-brown irregular fried pakodas with visible mint and coriander leaf flecks throughout the crumbly, coarse lentil texture, piled high on a plate, steam rising, natural light.</t>
+          <t>Professional food photography of "Mint Pakodas" (புதினா பக்கோடா), an Indian snack: dark green-brown irregular fried pakodas with visible mint and coriander leaf flecks throughout the crumbly, coarse lentil texture, piled high on a plate, steam rising. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
         </is>
       </c>
       <c r="H215" t="inlineStr">
@@ -12040,7 +12040,7 @@
       </c>
       <c r="G216" t="inlineStr">
         <is>
-          <t>A photorealistic close-up of round golden fried balls coated entirely in crisp, spiky strands of fried vermicelli giving a bird's-nest texture, one cut in half to reveal a bright yellow mashed-potato interior with green peas, plated elegantly with lettuce and tomato sauce, bright studio food photography lighting.</t>
+          <t>Professional food photography of "Potato Nest" (உருளைக்கிழங்கு கூடுகள்), an Indian snack: round golden fried balls coated entirely in crisp, spiky strands of fried vermicelli giving a bird's-nest texture, one cut in half to reveal a bright yellow mashed-potato interior with green peas, plated elegantly with lettuce and tomato sauce. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
         </is>
       </c>
       <c r="H216" t="inlineStr">
@@ -12085,7 +12085,7 @@
       </c>
       <c r="G217" t="inlineStr">
         <is>
-          <t>A photorealistic photo of a heaping pile of irregular, craggy, deep-golden fried pakoda chunks with visible long strands of onion and green chili baked into the crisp crust, on a steel plate, chai glass beside it, warm evening tea-stall lighting.</t>
+          <t>Professional food photography of "Garam Pakodas" (வெங்காய பக்கோடா), an Indian snack: a heaping pile of irregular, craggy, deep-golden fried pakoda chunks with visible long strands of onion and green chili baked into the crisp crust, on a plate, with a chai glass beside it. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
         </is>
       </c>
       <c r="H217" t="inlineStr">
@@ -12130,7 +12130,7 @@
       </c>
       <c r="G218" t="inlineStr">
         <is>
-          <t>A photorealistic close-up of irregular golden fried pakoda chunks with visible crumbly white paneer and pink cashew pieces embedded in the crust, piled on a plate with mint garnish, warm kitchen lighting.</t>
+          <t>Professional food photography of "Paneer Pakodas" (பனீர் பக்கோடா), an Indian snack: irregular golden fried pakoda chunks with visible crumbly white paneer and pink cashew pieces embedded in the crust, piled on a plate with mint garnish. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
         </is>
       </c>
       <c r="H218" t="inlineStr">
@@ -12175,7 +12175,7 @@
       </c>
       <c r="G219" t="inlineStr">
         <is>
-          <t>A photorealistic photo of golden-brown irregular fried pakoda pieces with a soft doughy bread interior visible at the torn edges, piled on a plate, served with tomato ketchup, natural daylight.</t>
+          <t>Professional food photography of "Bread Pakodas" (பிரட் பக்கோடா), an Indian snack: golden-brown irregular fried pakoda pieces with a soft doughy bread interior visible at the torn edges, piled on a plate, served with tomato ketchup. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
         </is>
       </c>
       <c r="H219" t="inlineStr">
@@ -12220,7 +12220,7 @@
       </c>
       <c r="G220" t="inlineStr">
         <is>
-          <t>A photorealistic close-up of golden fried pakodas with fine strands of crisp vermicelli visible on the textured surface, piled on a steel plate with mint chutney, warm ambient lighting.</t>
+          <t>Professional food photography of "Vermicelli Pakodas" (சேமியா பக்கோடா), an Indian snack: golden fried pakodas with fine strands of crisp vermicelli visible on the textured surface, piled on a plate with mint chutney. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
         </is>
       </c>
       <c r="H220" t="inlineStr">
@@ -12265,7 +12265,7 @@
       </c>
       <c r="G221" t="inlineStr">
         <is>
-          <t>A photorealistic close-up of a golden fried rectangular sandwich bajji cut in half, showing three layers of white bread with visible green mint chutney and red tomato chutney filling between the layers, crisp golden batter coating on the outside, served with tomato sauce, bright natural lighting.</t>
+          <t>Professional food photography of "Layered Sandwich Bajji" (பிரட் சாண்ட்விட்ச் பஜ்ஜி), an Indian snack: a golden fried rectangular sandwich bajji cut in half, showing three layers of white bread with visible green mint chutney and red tomato chutney filling between the layers, a crisp golden batter coating on the outside, served with tomato sauce. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
         </is>
       </c>
       <c r="H221" t="inlineStr">
@@ -12310,7 +12310,7 @@
       </c>
       <c r="G222" t="inlineStr">
         <is>
-          <t>A photorealistic photo of whole small green capsicums coated in a golden fried batter, one sliced open at the top showing chopped onion tucked inside with a wedge of lemon on the side, plated attractively, warm lighting.</t>
+          <t>Professional food photography of "Capsicum Bajji" (குடமிளகாய் பஜ்ஜி), an Indian snack: whole small green capsicums coated in a golden fried batter, one sliced open at the top showing chopped onion tucked inside with a wedge of lemon on the side. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
         </is>
       </c>
       <c r="H222" t="inlineStr">
@@ -12355,7 +12355,7 @@
       </c>
       <c r="G223" t="inlineStr">
         <is>
-          <t>A photorealistic close-up of long green bajji chilies coated in golden fried batter, one split open lengthwise to reveal a pale coconut-and-gram filling inside, garnished with chopped onion and a drizzle of sweet brown chutney, plated on a steel dish, warm tea-stall lighting.</t>
+          <t>Professional food photography of "Stuffed Chilli Bajji" (மிளகாய் பஜ்ஜி), an Indian snack: long green bajji chilies coated in golden fried batter, one split open lengthwise to reveal a pale coconut-and-gram filling inside, garnished with chopped onion and a drizzle of sweet brown chutney. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
         </is>
       </c>
       <c r="H223" t="inlineStr">
@@ -12400,7 +12400,7 @@
       </c>
       <c r="G224" t="inlineStr">
         <is>
-          <t>A photorealistic photo of small whole potatoes coated in golden fried batter, one sliced partway open showing a reddish garlic-spice paste inside, piled on a plate, warm lighting.</t>
+          <t>Professional food photography of "Lasania (Stuffed Potato Bajji)" (உருளைகிழங்கு ஸ்டப் பஜ்ஜி), an Indian snack: small whole potatoes coated in golden fried batter, one sliced partway open showing a reddish garlic-spice paste inside, piled on a plate. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
         </is>
       </c>
       <c r="H224" t="inlineStr">
@@ -12445,7 +12445,7 @@
       </c>
       <c r="G225" t="inlineStr">
         <is>
-          <t>A photorealistic close-up of classic golden-brown ring-shaped vadais with a lacy, crisp textured surface, stacked on a banana leaf, served with sambar in a small steel bowl and coconut chutney, warm South Indian breakfast table lighting.</t>
+          <t>Professional food photography of "Medu Vadai" (மெதுவடை), an Indian snack: classic golden-brown ring-shaped vadais with a lacy, crisp textured surface, stacked on a banana leaf, served with sambar in a small bowl and coconut chutney. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
         </is>
       </c>
       <c r="H225" t="inlineStr">
@@ -12490,7 +12490,7 @@
       </c>
       <c r="G226" t="inlineStr">
         <is>
-          <t>A photorealistic close-up of soft, pale golden vadais submerged in thick white curd on a steel plate, garnished with a drizzle of tempered mustard seeds, chopped coriander leaves, and a light dusting of red chili powder on top, bright natural lighting.</t>
+          <t>Professional food photography of "Thair Vadai" (தயிர் வடை), an Indian snack: soft, pale golden vadais submerged in thick white curd on a plate, garnished with a drizzle of tempered mustard seeds, chopped coriander leaves, and a light dusting of red chili powder on top. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
         </is>
       </c>
       <c r="H226" t="inlineStr">
@@ -12535,7 +12535,7 @@
       </c>
       <c r="G227" t="inlineStr">
         <is>
-          <t>A photorealistic close-up of a curd-soaked vadai cut open on a plate revealing a colorful filling of chopped cashews, almonds, raisins, and coconut inside the soft white lentil dough, surrounded by thick curd, garnished with fried spicy boondi on top, bright lighting.</t>
+          <t>Professional food photography of "Special Curd Vadai 1" (ஸ்பெஷல் தயிர் வடை (1)), an Indian snack: a curd-soaked vadai cut open on a plate revealing a colorful filling of chopped cashews, almonds, raisins, and coconut inside the soft white lentil dough, surrounded by thick curd, garnished with fried spicy boondi on top. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
         </is>
       </c>
       <c r="H227" t="inlineStr">
@@ -12580,7 +12580,7 @@
       </c>
       <c r="G228" t="inlineStr">
         <is>
-          <t>A photorealistic close-up of a half-moon, samosa-shaped curd vadai on a plate, soaked in white curd, with visible green herb flecks along the folded edge, garnished with grated carrot and coriander, natural lighting.</t>
+          <t>Professional food photography of "Special Curd Vadai 2" (ஸ்பெஷல் தயிர் வடை (2)), an Indian snack: a half-moon, samosa-shaped curd vadai on a plate, soaked in white curd, with visible green herb flecks along the folded edge, garnished with grated carrot and coriander. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
         </is>
       </c>
       <c r="H228" t="inlineStr">
@@ -12625,7 +12625,7 @@
       </c>
       <c r="G229" t="inlineStr">
         <is>
-          <t>A photorealistic close-up of a curd-soaked vadai cut in half showing a bright green mashed-pea filling inside the soft white lentil exterior, surrounded by thick curd on a steel plate, garnished with coriander, natural lighting.</t>
+          <t>Professional food photography of "Pattani Curd Vadai" (பட்டாணி தயிர் வடை), an Indian snack: a curd-soaked vadai cut in half showing a bright green mashed-pea filling inside the soft white lentil exterior, surrounded by thick curd on a plate, garnished with coriander. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
         </is>
       </c>
       <c r="H229" t="inlineStr">
@@ -12670,7 +12670,7 @@
       </c>
       <c r="G230" t="inlineStr">
         <is>
-          <t>A photorealistic close-up of pale golden vadais submerged in a thick, pale-yellow spiced buttermilk gravy flecked with coconut and curry leaves, served in a steel bowl, garnished with coriander leaves, warm home-style lighting.</t>
+          <t>Professional food photography of "Mor Kuzhambu Vadai" (மோர்க்குழம்பு வடை), an Indian snack: pale golden vadais submerged in a thick, pale-yellow spiced buttermilk gravy flecked with coconut and curry leaves, served in a bowl, garnished with coriander leaves. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
         </is>
       </c>
       <c r="H230" t="inlineStr">
@@ -12715,7 +12715,7 @@
       </c>
       <c r="G231" t="inlineStr">
         <is>
-          <t>A photorealistic photo of torn half-moon pieces of coarse-textured urad-toor dal vadai, soaked briefly in curd, plated with a light garnish, rustic table lighting.</t>
+          <t>Professional food photography of "Aamai Vadai" (ஆமை வடை), an Indian snack: torn half-moon pieces of coarse-textured urad-toor dal vadai, soaked briefly in curd, plated with a light garnish. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
         </is>
       </c>
       <c r="H231" t="inlineStr">
@@ -12760,7 +12760,7 @@
       </c>
       <c r="G232" t="inlineStr">
         <is>
-          <t>A photorealistic close-up of small round bread-dough vadais topped generously with white curd, dusted with black salt, roasted cumin powder, and red chili powder, drizzled with brown sweet chutney and garnished with coriander leaves, bright appetizing lighting.</t>
+          <t>Professional food photography of "Bread Dahi Vadai" (திடீர் பிரட் தயிர்வடை), an Indian snack: small round bread-dough vadais topped generously with white curd, dusted with black salt, roasted cumin powder, and red chili powder, drizzled with brown sweet chutney and garnished with coriander leaves. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
         </is>
       </c>
       <c r="H232" t="inlineStr">
@@ -12805,7 +12805,7 @@
       </c>
       <c r="G233" t="inlineStr">
         <is>
-          <t>A photorealistic close-up of small golden fried lentil pakodas arranged on a plate, topped with a generous pour of white whisked curd, dusted with a dark spice powder and tomato sauce drizzle, bright lighting.</t>
+          <t>Professional food photography of "Moong Dhal Curd Pakoda" (பயத்தம் பருப்பு தயிர் பக்கோடா), an Indian snack: small golden fried lentil pakodas arranged on a plate, topped with a generous pour of white whisked curd, dusted with a dark spice powder and a tomato sauce drizzle. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
         </is>
       </c>
       <c r="H233" t="inlineStr">
@@ -12850,7 +12850,7 @@
       </c>
       <c r="G234" t="inlineStr">
         <is>
-          <t>A photorealistic close-up of textured, coarse golden-brown vadais studded with visible cashew pieces and melon seeds, stacked on a plate, served with thokku, warm lighting.</t>
+          <t>Professional food photography of "Mysore Vadai" (மைசூர் வடை), an Indian snack: textured, coarse golden-brown vadais studded with visible cashew pieces and melon seeds, stacked on a plate, served with thokku. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
         </is>
       </c>
       <c r="H234" t="inlineStr">
@@ -12895,7 +12895,7 @@
       </c>
       <c r="G235" t="inlineStr">
         <is>
-          <t>A photorealistic photo of thin, flat, deep reddish-brown crispy discs with visible onion flecks, stacked in a glass jar and also arranged on a plate, matte crunchy texture, natural light.</t>
+          <t>Professional food photography of "Madhur Vadai" (மதுர் வடை), an Indian snack: thin, flat, deep reddish-brown crispy discs with visible onion flecks, stacked in a glass jar and also arranged on a plate, a matte crunchy texture. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
         </is>
       </c>
       <c r="H235" t="inlineStr">
@@ -12940,7 +12940,7 @@
       </c>
       <c r="G236" t="inlineStr">
         <is>
-          <t>A photorealistic close-up of flat, coarse-textured golden-brown vadais with visible chana dal grains, onion, and curry leaf flecks, stacked on a banana leaf, served with coconut chutney, warm lighting.</t>
+          <t>Professional food photography of "Masal Vadai" (மசால் வடை), an Indian snack: flat, coarse-textured golden-brown vadais with visible chana dal grains, onion, and curry leaf flecks, stacked on a banana leaf, served with coconut chutney. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
         </is>
       </c>
       <c r="H236" t="inlineStr">
@@ -12985,7 +12985,7 @@
       </c>
       <c r="G237" t="inlineStr">
         <is>
-          <t>A photorealistic photo of thin, flat, pale golden crispy discs with a slightly speckled sesame-seed texture, stacked on a plate, rustic homely lighting.</t>
+          <t>Professional food photography of "Gherugu Vadai" (கெருகு வடை), an Indian snack: thin, flat, pale golden crispy discs with a slightly speckled sesame-seed texture, stacked on a plate. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
         </is>
       </c>
       <c r="H237" t="inlineStr">
@@ -13030,7 +13030,7 @@
       </c>
       <c r="G238" t="inlineStr">
         <is>
-          <t>A photorealistic close-up of thin, flat, pale golden-brown vadais with visible shreds of white radish embedded in the crisp exterior, stacked on a steel plate, natural daylight.</t>
+          <t>Professional food photography of "Mullangi Vadai" (முள்ளங்கி வடை), an Indian snack: thin, flat, pale golden-brown vadais with visible shreds of white radish embedded in the crisp exterior, stacked on a plate. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
         </is>
       </c>
       <c r="H238" t="inlineStr">
@@ -13075,7 +13075,7 @@
       </c>
       <c r="G239" t="inlineStr">
         <is>
-          <t>A photorealistic photo of flat reddish-orange vadais with a speckled texture from ground red chili and pumpkin, stacked on a plate, tangy glossy sheen, warm lighting.</t>
+          <t>Professional food photography of "Pulusu Vadai" (புளி வடை அல்லது புலுசு வடை), an Indian snack: flat reddish-orange vadais with a speckled texture from ground red chili and pumpkin, stacked on a plate, a tangy glossy sheen. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
         </is>
       </c>
       <c r="H239" t="inlineStr">
@@ -13120,7 +13120,7 @@
       </c>
       <c r="G240" t="inlineStr">
         <is>
-          <t>A photorealistic close-up of small pale golden vadais with visible flecks of cracked black pepper, some strung together on a thread like a garland, others piled on a plate, temple-offering style presentation, warm devotional lighting.</t>
+          <t>Professional food photography of "Milagu Vadai" (மிளகு வடை), an Indian snack: small pale golden vadais with visible flecks of cracked black pepper, some strung together on a thread like a garland, others piled on a plate, a temple-offering style presentation. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
         </is>
       </c>
       <c r="H240" t="inlineStr">
@@ -13165,7 +13165,7 @@
       </c>
       <c r="G241" t="inlineStr">
         <is>
-          <t>A photorealistic close-up of coarse, flat golden-brown vadais with a slightly speckled surface, stacked on a plate, served with vinegar-tossed onion rings on the side, warm lighting.</t>
+          <t>Professional food photography of "Drumstick Vadai" (முருங்கைக்காய் வடை), an Indian snack: coarse, flat golden-brown vadais with a slightly speckled surface, stacked on a plate, served with vinegar-tossed onion rings on the side. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
         </is>
       </c>
       <c r="H241" t="inlineStr">
@@ -13210,7 +13210,7 @@
       </c>
       <c r="G242" t="inlineStr">
         <is>
-          <t>A photorealistic photo of soft, pale, lightly golden flat discs with a matte soft surface (not deeply fried), stacked on a plate, gentle lighting emphasizing their softness.</t>
+          <t>Professional food photography of "Perugu Vadai" (பெருகு வடை), an Indian snack: soft, pale, lightly golden flat discs with a matte soft surface, not deeply fried, stacked on a plate. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
         </is>
       </c>
       <c r="H242" t="inlineStr">
@@ -13255,7 +13255,7 @@
       </c>
       <c r="G243" t="inlineStr">
         <is>
-          <t>A photorealistic close-up of a golden-brown fried bread toast cut diagonally, showing a thin green mint chutney layer and a yellow lentil paste layer between the crisp bread surface and the crust, plated with tomato sauce, bright lighting.</t>
+          <t>Professional food photography of "Moong Dhal Toast" (பயத்தம்பருப்பு டோஸ்ட்), an Indian sandwich: a golden-brown fried bread toast cut diagonally, showing a thin green mint chutney layer and a yellow lentil paste layer between the crisp bread surface and the crust, plated with tomato sauce. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
         </is>
       </c>
       <c r="H243" t="inlineStr">
@@ -13300,7 +13300,7 @@
       </c>
       <c r="G244" t="inlineStr">
         <is>
-          <t>A photorealistic photo of golden-brown toasted bread slices with a thin reddish-brown spice chutney visible on the surface, griddle-toasted with light char marks, stacked on a plate, warm lighting.</t>
+          <t>Professional food photography of "Masala Toast" (மசாலா டோஸ்ட்), an Indian sandwich: golden-brown toasted bread slices with a thin reddish-brown spice chutney visible on the surface, griddle-toasted with light char marks, stacked on a plate. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
         </is>
       </c>
       <c r="H244" t="inlineStr">
@@ -13345,7 +13345,7 @@
       </c>
       <c r="G245" t="inlineStr">
         <is>
-          <t>A photorealistic close-up of a golden-toasted bread slice topped with a glossy reddish-orange cooked tomato-onion masala spread evenly across the surface, slightly caramelized edges, plated hot, warm kitchen lighting.</t>
+          <t>Professional food photography of "Tomato Toast" (தக்காளி டோஸ்ட்), an Indian sandwich: a golden-toasted bread slice topped with a glossy reddish-orange cooked tomato-onion masala spread evenly across the surface, slightly caramelized edges, plated hot. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
         </is>
       </c>
       <c r="H245" t="inlineStr">
@@ -13390,7 +13390,7 @@
       </c>
       <c r="G246" t="inlineStr">
         <is>
-          <t>A photorealistic close-up of a golden-brown griddle-fried sandwich cut diagonally, showing a thick yellow spiced-potato filling coated in crisp bread crumbs between the toasted bread layers, plated with ketchup, bright appetizing lighting.</t>
+          <t>Professional food photography of "Potato Sandwich" (உருளைக்கிழங்கு பிரட் சாண்ட்விச்), an Indian sandwich: a golden-brown griddle-fried sandwich cut diagonally, showing a thick yellow spiced-potato filling coated in crisp bread crumbs between the toasted bread layers, plated with ketchup. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
         </is>
       </c>
       <c r="H246" t="inlineStr">
@@ -13435,7 +13435,7 @@
       </c>
       <c r="G247" t="inlineStr">
         <is>
-          <t>A photorealistic photo of an open-faced toast topped with golden corn kernels mixed with cream, and a layer of melted golden cheese bubbling on top, baked and lightly browned, warm oven-fresh lighting.</t>
+          <t>Professional food photography of "Corn Sandwich" (மக்காச்சோள சாண்ட்விச்), an Indian sandwich: an open-faced toast topped with golden corn kernels mixed with cream, and a layer of melted golden cheese bubbling on top, baked and lightly browned. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
         </is>
       </c>
       <c r="H247" t="inlineStr">
@@ -13480,7 +13480,7 @@
       </c>
       <c r="G248" t="inlineStr">
         <is>
-          <t>A photorealistic close-up of a clear glass bottle filled with thick, deep-red glossy homemade tomato ketchup, a spoonful pooled beside it on a white plate showing its smooth, thick consistency, bright clean lighting.</t>
+          <t>Professional food photography of "Tomato Ketchup" (தக்காளி கெட்ச்அப்), an Indian condiment: a clear glass bottle filled with thick, deep-red glossy homemade tomato ketchup, a spoonful pooled beside it on a white plate showing its smooth, thick consistency. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
         </is>
       </c>
       <c r="H248" t="inlineStr">
@@ -13525,7 +13525,7 @@
       </c>
       <c r="G249" t="inlineStr">
         <is>
-          <t>A photorealistic close-up of a triangle-cut sandwich showing distinct colorful layers of thin cucumber, carrot, tomato, and onion rounds between green mint-chutney-spread bread, fresh and vibrant, natural bright lighting.</t>
+          <t>Professional food photography of "Vegetable Sandwich" (காய்கறி சாண்ட்விச்), an Indian sandwich: a triangle-cut sandwich showing distinct colorful layers of thin cucumber, carrot, tomato, and onion rounds between green mint-chutney-spread bread, fresh and vibrant. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
         </is>
       </c>
       <c r="H249" t="inlineStr">
@@ -13570,7 +13570,7 @@
       </c>
       <c r="G250" t="inlineStr">
         <is>
-          <t>A photorealistic close-up of a golden toasted sandwich cut in half, oozing melted golden cheese mixed with visible flecks of green chili and onion between the crisp bread layers, warm appetizing lighting.</t>
+          <t>Professional food photography of "Chilli Cheese Sandwich" (சில்லி சீஸ் சாண்ட்விச்), an Indian sandwich: a golden toasted sandwich cut in half, oozing melted golden cheese mixed with visible flecks of green chili and onion between the crisp bread layers. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
         </is>
       </c>
       <c r="H250" t="inlineStr">
@@ -13615,7 +13615,7 @@
       </c>
       <c r="G251" t="inlineStr">
         <is>
-          <t>A photorealistic close-up of a golden toasted sandwich cut diagonally, showing a crumbly white paneer filling studded with green sprouts and herbs between the bread layers, plated with ketchup, bright lighting.</t>
+          <t>Professional food photography of "Paneer Sandwich" (பாலாடைக்கட்டி சாண்ட்விச்), an Indian sandwich: a golden toasted sandwich cut diagonally, showing a crumbly white paneer filling studded with green sprouts and herbs between the bread layers, plated with ketchup. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
         </is>
       </c>
       <c r="H251" t="inlineStr">
@@ -13660,7 +13660,7 @@
       </c>
       <c r="G252" t="inlineStr">
         <is>
-          <t>A photorealistic close-up of pinwheel-shaped bread roll slices arranged on a plate, showing a spiral of white bread with thin green and red chutney swirls visible in the layers, elegant party-platter presentation, bright clean lighting.</t>
+          <t>Professional food photography of "Sandwich Roll" (சாண்ட்விட்ச் ரோல்), an Indian sandwich: pinwheel-shaped bread roll slices arranged on a plate, showing a spiral of white bread with thin green and red chutney swirls visible in the layers, an elegant party-platter presentation. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
         </is>
       </c>
       <c r="H252" t="inlineStr">
@@ -13705,7 +13705,7 @@
       </c>
       <c r="G253" t="inlineStr">
         <is>
-          <t>A photorealistic close-up of a boiled potato stuffed and topped generously with white whisked curd, drizzled with dark brown tangy tamarind sauce, dusted with red chili powder and dark chat masala, garnished with coriander leaves, served on a decorative plate, vibrant street-food lighting.</t>
+          <t>Professional food photography of "Aloo Chat 1" (ஆலு சாட் - 1), an Indian street food: a boiled potato stuffed and topped generously with white whisked curd, drizzled with dark brown tangy tamarind sauce, dusted with red chili powder and dark chat masala, garnished with coriander leaves, served on a decorative plate. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
         </is>
       </c>
       <c r="H253" t="inlineStr">
@@ -13750,7 +13750,7 @@
       </c>
       <c r="G254" t="inlineStr">
         <is>
-          <t>A photorealistic photo of diced potato mixed with golden fried diamond-shaped crisps, tossed in a chat bowl with dark tangy sauce, chopped onion, and a scattering of thin crispy sev on top, colorful street-food presentation, bright lighting.</t>
+          <t>Professional food photography of "Aloo Chat 2" (ஆலு சாட் - 2), an Indian street food: diced potato mixed with golden fried diamond-shaped crisps, tossed in a bowl with dark tangy sauce, chopped onion, and a scattering of thin crispy sev on top. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
         </is>
       </c>
       <c r="H254" t="inlineStr">
@@ -13795,7 +13795,7 @@
       </c>
       <c r="G255" t="inlineStr">
         <is>
-          <t>A photorealistic close-up of a small glass jar filled with reddish-brown aromatic spice powder, a small mound of the powder spilled beside it on a wooden surface with whole dried red chilies and cardamom pods scattered around, warm spice-market lighting.</t>
+          <t>Professional food photography of "Chat Masala Powder" (சாட் மசாலா பவுடர்), an Indian spice blend: a small glass jar filled with reddish-brown aromatic spice powder, a small mound of the powder spilled beside it on a wooden surface with whole dried red chilies and cardamom pods scattered around. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
         </is>
       </c>
       <c r="H255" t="inlineStr">
@@ -13840,7 +13840,7 @@
       </c>
       <c r="G256" t="inlineStr">
         <is>
-          <t>A photorealistic close-up of a plate layered with crushed golden fried papad pieces, topped with diced potato, a generous pour of white curd, dark brown sweet chutney drizzle, and a dusting of spices with fresh coriander on top, vibrant street-food lighting.</t>
+          <t>Professional food photography of "Aloo Pappad Chat" (ஆலு பப்பட் சாட்), an Indian street food: a plate layered with crushed golden fried papad pieces, topped with diced potato, a generous pour of white curd, a dark brown sweet chutney drizzle, and a dusting of spices with fresh coriander on top. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
         </is>
       </c>
       <c r="H256" t="inlineStr">
@@ -13885,7 +13885,7 @@
       </c>
       <c r="G257" t="inlineStr">
         <is>
-          <t>A photorealistic close-up of a bowl of cooked green peas topped with crushed golden puri pieces, white curd, dark tamarind chutney, chopped onion, and fine crispy sev, colorful layered presentation, bright lighting.</t>
+          <t>Professional food photography of "Mattar Chat" (பச்சைப் பட்டாணி சாட்), an Indian street food: a bowl of cooked green peas topped with crushed golden puri pieces, white curd, dark tamarind chutney, chopped onion, and fine crispy sev, a colorful layered presentation. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
         </is>
       </c>
       <c r="H257" t="inlineStr">
@@ -13930,7 +13930,7 @@
       </c>
       <c r="G258" t="inlineStr">
         <is>
-          <t>A photorealistic photo of a colorful bowl mix of diced banana, orange segments, tomato, potato, and guava tossed together, garnished with coriander leaves and a light dusting of chat masala, fresh and vibrant, bright natural lighting.</t>
+          <t>Professional food photography of "Fruit &amp; Vegetable Chat" (காய்கறி, பழக்கலவை சாட்), an Indian street food: a colorful bowl mix of diced banana, orange segments, tomato, potato, and guava tossed together, garnished with coriander leaves and a light dusting of chat masala. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
         </is>
       </c>
       <c r="H258" t="inlineStr">
@@ -13975,7 +13975,7 @@
       </c>
       <c r="G259" t="inlineStr">
         <is>
-          <t>A photorealistic close-up of golden-brown crispy potato finger chips piled high on a plate, lightly dusted with salt and pepper, served with tomato ketchup, bright appetizing lighting.</t>
+          <t>Professional food photography of "Finger Chips" (ஃபிங்கர் சிப்ஸ்), an Indian snack: golden-brown crispy potato finger chips piled high on a plate, lightly dusted with salt and pepper, served with tomato ketchup. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
         </is>
       </c>
       <c r="H259" t="inlineStr">
@@ -14020,7 +14020,7 @@
       </c>
       <c r="G260" t="inlineStr">
         <is>
-          <t>A photorealistic close-up of small glossy, deep golden-brown fried groundnuts piled in a bowl, with a visible shiny sheen, some scattered on a napkin, warm snack-time lighting.</t>
+          <t>Professional food photography of "Crisp Groundnuts" (வறுகடலை), an Indian snack: small glossy, deep golden-brown fried groundnuts piled in a bowl, with a visible shiny sheen, some scattered on a napkin. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
         </is>
       </c>
       <c r="H260" t="inlineStr">
@@ -14065,7 +14065,7 @@
       </c>
       <c r="G261" t="inlineStr">
         <is>
-          <t>A photorealistic close-up of a bowl overflowing with fluffy white popcorn lightly dusted with orange-red spice seasoning, warm cozy lighting.</t>
+          <t>Professional food photography of "Pop Corn" (பாப் கார்ன்), an Indian snack: a bowl overflowing with fluffy white popcorn lightly dusted with orange-red spice seasoning. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
         </is>
       </c>
       <c r="H261" t="inlineStr">
@@ -14110,7 +14110,7 @@
       </c>
       <c r="G262" t="inlineStr">
         <is>
-          <t>A photorealistic photo of a colorful bowl of puffed rice mixed with roasted gram, small dice of mango, tomato, carrot, and beetroot, garnished with coriander leaves, bright vibrant street-food lighting.</t>
+          <t>Professional food photography of "Masala Pori 1 (Instant Bhel)" (மசாலா பொரி - 1), an Indian street food: a colorful bowl of puffed rice mixed with roasted gram, small dice of mango, tomato, carrot, and beetroot, garnished with coriander leaves. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
         </is>
       </c>
       <c r="H262" t="inlineStr">
@@ -14155,7 +14155,7 @@
       </c>
       <c r="G263" t="inlineStr">
         <is>
-          <t>A photorealistic photo of a bowl of puffed rice mixed with roasted gram and groundnuts, tossed with pink-tinged marinated onion and a drizzle of dark green chutney, colorful and fresh, bright lighting.</t>
+          <t>Professional food photography of "Masala Pori 2 (Instant Bhel)" (மசாலா பொரி - 2), an Indian street food: a bowl of puffed rice mixed with roasted gram and groundnuts, tossed with pink-tinged marinated onion and a drizzle of dark green chutney, colorful and fresh. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
         </is>
       </c>
       <c r="H263" t="inlineStr">
@@ -14200,7 +14200,7 @@
       </c>
       <c r="G264" t="inlineStr">
         <is>
-          <t>A photorealistic close-up of a small bowl of smooth, vivid green chutney with a glossy sheen, served beside golden fried cutlets, garnished with a mint sprig, bright fresh lighting.</t>
+          <t>Professional food photography of "Mint-Coriander Chutney (for Cutlets)" (புதினா, கொத்தமல்லி சட்னி (கட்லெட்டிற்கு)), an Indian condiment: a small bowl of smooth, vivid green chutney with a glossy sheen, served beside golden fried cutlets, garnished with a mint sprig. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
         </is>
       </c>
       <c r="H264" t="inlineStr">
@@ -14245,7 +14245,7 @@
       </c>
       <c r="G265" t="inlineStr">
         <is>
-          <t>A photorealistic close-up of a small bowl of dark green, thick chutney with a tempered mustard-seed garnish floating on top, bright natural lighting.</t>
+          <t>Professional food photography of "Mint Chutney (for Cutlets)" (புதினா சட்னி (கட்லெட்டிற்கு)), an Indian condiment: a small bowl of dark green, thick chutney with a tempered mustard-seed garnish floating on top. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
         </is>
       </c>
       <c r="H265" t="inlineStr">
@@ -14290,7 +14290,7 @@
       </c>
       <c r="G266" t="inlineStr">
         <is>
-          <t>A photorealistic close-up of a bowl of textured dark green chutney flecked with white coconut, garnished with a tempering of mustard seeds and curry leaves on top, warm lighting.</t>
+          <t>Professional food photography of "Mint-Onion Chutney" (புதினா வெங்காயச் சட்னி), an Indian condiment: a bowl of textured dark green chutney flecked with white coconut, garnished with a tempering of mustard seeds and curry leaves on top. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
         </is>
       </c>
       <c r="H266" t="inlineStr">
@@ -14335,7 +14335,7 @@
       </c>
       <c r="G267" t="inlineStr">
         <is>
-          <t>A photorealistic close-up of a small bowl of deep green-red chutney with a thick, spreadable texture, a butter knife resting beside it with chutney on the blade, bright kitchen lighting.</t>
+          <t>Professional food photography of "Coriander Chutney (for Sandwiches)" (கொத்தமல்லி சட்னி (சாண்ட்விச்சிற்கு)), an Indian condiment: a small bowl of deep green-red chutney with a thick, spreadable texture, a butter knife resting beside it with chutney on the blade. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
         </is>
       </c>
       <c r="H267" t="inlineStr">
@@ -14380,7 +14380,7 @@
       </c>
       <c r="G268" t="inlineStr">
         <is>
-          <t>A photorealistic close-up of a bowl of reddish-brown chutney with visible garlic and chili flecks, thick and glossy, served beside buttered bread slices, warm lighting.</t>
+          <t>Professional food photography of "Garlic Chutney (for Sandwiches)" (பூண்டு சட்னி (சாண்ட்விச்சிற்கு)), an Indian condiment: a bowl of reddish-brown chutney with visible garlic and chili flecks, thick and glossy, served beside buttered bread slices. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
         </is>
       </c>
       <c r="H268" t="inlineStr">
@@ -14425,7 +14425,7 @@
       </c>
       <c r="G269" t="inlineStr">
         <is>
-          <t>A photorealistic close-up of a bowl of coarse, off-white coconut chutney with visible ginger and red chili flecks, glossy texture, natural bright lighting.</t>
+          <t>Professional food photography of "Coconut-Ginger Chutney (for Sandwiches)" (தேங்காய், இஞ்சி சட்னி (சாண்ட்விச்சிற்கு)), an Indian condiment: a bowl of coarse, off-white coconut chutney with visible ginger and red chili flecks, a glossy texture. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
         </is>
       </c>
       <c r="H269" t="inlineStr">
@@ -14470,7 +14470,7 @@
       </c>
       <c r="G270" t="inlineStr">
         <is>
-          <t>A photorealistic close-up of a small bowl of smooth bright green mint chutney, glossy sheen, served beside a stack of white bread slices, fresh vibrant lighting.</t>
+          <t>Professional food photography of "Mint Chutney (for Sandwiches)" (புதினா சட்னி (சாண்ட்விச்சிற்கு)), an Indian condiment: a small bowl of smooth bright green mint chutney with a glossy sheen, served beside a stack of white bread slices. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
         </is>
       </c>
       <c r="H270" t="inlineStr">
@@ -14515,7 +14515,7 @@
       </c>
       <c r="G271" t="inlineStr">
         <is>
-          <t>A photorealistic close-up of golden fried onion bajjis with a distinctive ring-shaped, batter-coated onion visible inside the crisp fried coating, piled on a plate, served with coconut chutney, warm tea-stall lighting.</t>
+          <t>Professional food photography of "Onion Bajji" (வெங்காயப் பஜ்ஜி), an Indian snack: golden fried onion bajjis with a distinctive ring-shaped, batter-coated onion visible inside the crisp fried coating, piled on a plate, served with coconut chutney. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
         </is>
       </c>
       <c r="H271" t="inlineStr">
@@ -14560,7 +14560,7 @@
       </c>
       <c r="G272" t="inlineStr">
         <is>
-          <t>A photorealistic close-up of whole okra pieces coated in a crisp golden fried batter with visible bread-crumb texture, arranged on a plate with tomato sauce, natural daylight.</t>
+          <t>Professional food photography of "Deep Fried Ladies Fingers" (வெண்டைக்காய் பக்கோடா), an Indian snack: whole okra pieces coated in a crisp golden fried batter with visible bread-crumb texture, arranged on a plate with tomato sauce. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
         </is>
       </c>
       <c r="H272" t="inlineStr">
@@ -14605,7 +14605,7 @@
       </c>
       <c r="G273" t="inlineStr">
         <is>
-          <t>A photorealistic close-up of a pressed golden-toasted sandwich cut in half, showing a bright orange sauteed carrot-tomato filling between the bread layers, plated with tomato sauce, warm appetizing lighting.</t>
+          <t>Professional food photography of "Carrot Sandwich" (கேரட் சாண்ட்விச்), an Indian sandwich: a pressed golden-toasted sandwich cut in half, showing a bright orange sauteed carrot-tomato filling between the bread layers, plated with tomato sauce. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
         </is>
       </c>
       <c r="H273" t="inlineStr">

</xml_diff>

<commit_message>
docs(tracker): ensure named ingredients are visually verifiable in prompts
Several batch-2 prompts named an ingredient (moong dal, radish, pumpkin,
drumstick, onion) that gets fully blended into a fried batter or ground
chutney and wouldn't actually render as a visible cue. Added a cross-
section reveal or a raw-ingredient side garnish to each so the generated
photo matches the recipe: moong-dhal-curd-pakoda, mullangi-vadai,
pulusu-vadai, drumstick-vadai, mint-onion-chutney.
</commit_message>
<xml_diff>
--- a/docs/recipe-image-tracker.xlsx
+++ b/docs/recipe-image-tracker.xlsx
@@ -11465,7 +11465,12 @@
       </c>
       <c r="I203" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J203" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
         </is>
       </c>
     </row>
@@ -11510,7 +11515,12 @@
       </c>
       <c r="I204" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J204" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
         </is>
       </c>
     </row>
@@ -11555,7 +11565,12 @@
       </c>
       <c r="I205" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J205" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
         </is>
       </c>
     </row>
@@ -11600,7 +11615,12 @@
       </c>
       <c r="I206" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J206" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
         </is>
       </c>
     </row>
@@ -11645,7 +11665,12 @@
       </c>
       <c r="I207" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J207" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
         </is>
       </c>
     </row>
@@ -11690,7 +11715,12 @@
       </c>
       <c r="I208" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J208" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
         </is>
       </c>
     </row>
@@ -11735,7 +11765,12 @@
       </c>
       <c r="I209" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J209" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
         </is>
       </c>
     </row>
@@ -11780,7 +11815,12 @@
       </c>
       <c r="I210" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J210" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
         </is>
       </c>
     </row>
@@ -11825,7 +11865,12 @@
       </c>
       <c r="I211" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J211" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
         </is>
       </c>
     </row>
@@ -11870,7 +11915,12 @@
       </c>
       <c r="I212" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J212" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
         </is>
       </c>
     </row>
@@ -11915,7 +11965,12 @@
       </c>
       <c r="I213" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J213" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
         </is>
       </c>
     </row>
@@ -11960,7 +12015,12 @@
       </c>
       <c r="I214" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J214" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
         </is>
       </c>
     </row>
@@ -12005,7 +12065,12 @@
       </c>
       <c r="I215" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J215" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
         </is>
       </c>
     </row>
@@ -12050,7 +12115,12 @@
       </c>
       <c r="I216" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J216" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
         </is>
       </c>
     </row>
@@ -12095,7 +12165,12 @@
       </c>
       <c r="I217" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J217" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
         </is>
       </c>
     </row>
@@ -12140,7 +12215,12 @@
       </c>
       <c r="I218" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J218" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
         </is>
       </c>
     </row>
@@ -12185,7 +12265,12 @@
       </c>
       <c r="I219" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J219" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
         </is>
       </c>
     </row>
@@ -12230,7 +12315,12 @@
       </c>
       <c r="I220" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J220" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
         </is>
       </c>
     </row>
@@ -12275,7 +12365,12 @@
       </c>
       <c r="I221" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J221" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
         </is>
       </c>
     </row>
@@ -12320,7 +12415,12 @@
       </c>
       <c r="I222" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J222" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
         </is>
       </c>
     </row>
@@ -12365,7 +12465,12 @@
       </c>
       <c r="I223" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J223" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
         </is>
       </c>
     </row>
@@ -12410,7 +12515,12 @@
       </c>
       <c r="I224" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J224" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
         </is>
       </c>
     </row>
@@ -12455,7 +12565,12 @@
       </c>
       <c r="I225" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J225" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
         </is>
       </c>
     </row>
@@ -12500,7 +12615,12 @@
       </c>
       <c r="I226" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J226" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
         </is>
       </c>
     </row>
@@ -12545,7 +12665,12 @@
       </c>
       <c r="I227" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J227" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
         </is>
       </c>
     </row>
@@ -12590,7 +12715,12 @@
       </c>
       <c r="I228" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J228" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
         </is>
       </c>
     </row>
@@ -12635,7 +12765,12 @@
       </c>
       <c r="I229" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J229" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
         </is>
       </c>
     </row>
@@ -12680,7 +12815,12 @@
       </c>
       <c r="I230" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J230" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
         </is>
       </c>
     </row>
@@ -12725,7 +12865,12 @@
       </c>
       <c r="I231" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J231" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
         </is>
       </c>
     </row>
@@ -12770,7 +12915,12 @@
       </c>
       <c r="I232" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J232" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
         </is>
       </c>
     </row>
@@ -12805,7 +12955,7 @@
       </c>
       <c r="G233" t="inlineStr">
         <is>
-          <t>Professional food photography of "Moong Dhal Curd Pakoda" (பயத்தம் பருப்பு தயிர் பக்கோடா), an Indian snack: small golden fried lentil pakodas arranged on a plate, topped with a generous pour of white whisked curd, dusted with a dark spice powder and a tomato sauce drizzle. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
+          <t>Professional food photography of "Moong Dhal Curd Pakoda" (பயத்தம் பருப்பு தயிர் பக்கோடா), an Indian snack: small golden fried pakodas made from a pale yellow moong dal batter, one pakoda broken open to reveal the coarse, grainy moong dal texture inside, the pakodas topped with a generous pour of white whisked curd and dusted with a dark spice powder and a tomato sauce drizzle, a small mound of whole yellow moong dal placed beside the plate as a visual cue. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
         </is>
       </c>
       <c r="H233" t="inlineStr">
@@ -13030,7 +13180,7 @@
       </c>
       <c r="G238" t="inlineStr">
         <is>
-          <t>Professional food photography of "Mullangi Vadai" (முள்ளங்கி வடை), an Indian snack: thin, flat, pale golden-brown vadais with visible shreds of white radish embedded in the crisp exterior, stacked on a plate. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
+          <t>Professional food photography of "Mullangi Vadai" (முள்ளங்கி வடை), an Indian snack: thin, flat, pale golden-brown lentil vadais with clearly visible white and pale-green shredded radish pieces studded throughout the crisp, speckled surface, one vadai broken in half to show radish shreds inside the crumb, stacked on a plate next to a small mound of raw grated radish as a visual cue. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
         </is>
       </c>
       <c r="H238" t="inlineStr">
@@ -13075,7 +13225,7 @@
       </c>
       <c r="G239" t="inlineStr">
         <is>
-          <t>Professional food photography of "Pulusu Vadai" (புளி வடை அல்லது புலுசு வடை), an Indian snack: flat reddish-orange vadais with a speckled texture from ground red chili and pumpkin, stacked on a plate, a tangy glossy sheen. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
+          <t>Professional food photography of "Pulusu Vadai" (புளி வடை அல்லது புலுசு வடை), an Indian snack: flat reddish-orange vadais with visible small orange pumpkin flecks embedded in the speckled batter, one vadai broken open to show the pumpkin pieces inside, a tangy glossy sheen, stacked on a plate next to a small wedge of raw orange pumpkin as a visual cue. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
         </is>
       </c>
       <c r="H239" t="inlineStr">
@@ -13165,7 +13315,7 @@
       </c>
       <c r="G241" t="inlineStr">
         <is>
-          <t>Professional food photography of "Drumstick Vadai" (முருங்கைக்காய் வடை), an Indian snack: coarse, flat golden-brown vadais with a slightly speckled surface, stacked on a plate, served with vinegar-tossed onion rings on the side. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
+          <t>Professional food photography of "Drumstick Vadai" (முருங்கைக்காய் வடை), an Indian snack: coarse, flat golden-brown vadais with visible pale green shredded drumstick (moringa) pulp embedded in the speckled surface, one vadai broken open to show the drumstick fiber inside, stacked on a plate with vinegar-tossed onion rings on the side and a whole raw drumstick pod placed beside the plate as a visual cue. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
         </is>
       </c>
       <c r="H241" t="inlineStr">
@@ -14290,7 +14440,7 @@
       </c>
       <c r="G266" t="inlineStr">
         <is>
-          <t>Professional food photography of "Mint-Onion Chutney" (புதினா வெங்காயச் சட்னி), an Indian condiment: a bowl of textured dark green chutney flecked with white coconut, garnished with a tempering of mustard seeds and curry leaves on top. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
+          <t>Professional food photography of "Mint-Onion Chutney" (புதினா வெங்காயச் சட்னி), an Indian condiment: a bowl of textured dark green chutney flecked with visible white coconut and small translucent pieces of chopped onion throughout, garnished with a tempering of mustard seeds and curry leaves on top, a few raw onion slices placed beside the bowl as a visual cue. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
         </is>
       </c>
       <c r="H266" t="inlineStr">

</xml_diff>

<commit_message>
docs(tracker): add scene-variation and anti-watermark constraints for batch 232-241
Generated images for this batch all shared an identical background prop
setup (same tumbler, lamp, jars) plus a visible checkered rendering
artifact and a sparkle watermark glyph. Strengthened prompts to demand a
unique composition per dish and an explicitly artifact/watermark-free
result.
</commit_message>
<xml_diff>
--- a/docs/recipe-image-tracker.xlsx
+++ b/docs/recipe-image-tracker.xlsx
@@ -12955,7 +12955,7 @@
       </c>
       <c r="G233" t="inlineStr">
         <is>
-          <t>Professional food photography of "Moong Dhal Curd Pakoda" (பயத்தம் பருப்பு தயிர் பக்கோடா), an Indian snack: small golden fried pakodas made from a pale yellow moong dal batter, one pakoda broken open to reveal the coarse, grainy moong dal texture inside, the pakodas topped with a generous pour of white whisked curd and dusted with a dark spice powder and a tomato sauce drizzle, a small mound of whole yellow moong dal placed beside the plate as a visual cue. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
+          <t>Professional food photography of "Moong Dhal Curd Pakoda" (பயத்தம் பருப்பு தயிர் பக்கோடா), an Indian snack: small golden fried pakodas made from a pale yellow moong dal batter, one pakoda broken open to reveal the coarse, grainy moong dal texture inside, the pakodas topped with a generous pour of white whisked curd and dusted with a dark spice powder and a tomato sauce drizzle, a small mound of whole yellow moong dal placed beside the plate as a visual cue. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging, Use a fresh, unique table setting and prop arrangement for this shot -- do not reuse the composition, background objects, or camera framing from any other photo. Absolutely no watermark, logo, sparkle icon, brand mark, or any repeating overlay pattern/texture anywhere in the image; the surface and background must be clean and artifact-free.</t>
         </is>
       </c>
       <c r="H233" t="inlineStr">
@@ -13000,7 +13000,7 @@
       </c>
       <c r="G234" t="inlineStr">
         <is>
-          <t>Professional food photography of "Mysore Vadai" (மைசூர் வடை), an Indian snack: textured, coarse golden-brown vadais studded with visible cashew pieces and melon seeds, stacked on a plate, served with thokku. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
+          <t>Professional food photography of "Mysore Vadai" (மைசூர் வடை), an Indian snack: textured, coarse golden-brown vadais studded with visible cashew pieces and melon seeds, stacked on a plate, served with thokku. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging, Use a fresh, unique table setting and prop arrangement for this shot -- do not reuse the composition, background objects, or camera framing from any other photo. Absolutely no watermark, logo, sparkle icon, brand mark, or any repeating overlay pattern/texture anywhere in the image; the surface and background must be clean and artifact-free.</t>
         </is>
       </c>
       <c r="H234" t="inlineStr">
@@ -13045,7 +13045,7 @@
       </c>
       <c r="G235" t="inlineStr">
         <is>
-          <t>Professional food photography of "Madhur Vadai" (மதுர் வடை), an Indian snack: thin, flat, deep reddish-brown crispy discs with visible onion flecks, stacked in a glass jar and also arranged on a plate, a matte crunchy texture. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
+          <t>Professional food photography of "Madhur Vadai" (மதுர் வடை), an Indian snack: thin, flat, deep reddish-brown crispy discs with visible onion flecks, stacked in a glass jar and also arranged on a plate, a matte crunchy texture. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging, Use a fresh, unique table setting and prop arrangement for this shot -- do not reuse the composition, background objects, or camera framing from any other photo. Absolutely no watermark, logo, sparkle icon, brand mark, or any repeating overlay pattern/texture anywhere in the image; the surface and background must be clean and artifact-free.</t>
         </is>
       </c>
       <c r="H235" t="inlineStr">
@@ -13090,7 +13090,7 @@
       </c>
       <c r="G236" t="inlineStr">
         <is>
-          <t>Professional food photography of "Masal Vadai" (மசால் வடை), an Indian snack: flat, coarse-textured golden-brown vadais with visible chana dal grains, onion, and curry leaf flecks, stacked on a banana leaf, served with coconut chutney. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
+          <t>Professional food photography of "Masal Vadai" (மசால் வடை), an Indian snack: flat, coarse-textured golden-brown vadais with visible chana dal grains, onion, and curry leaf flecks, stacked on a banana leaf, served with coconut chutney. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging, Use a fresh, unique table setting and prop arrangement for this shot -- do not reuse the composition, background objects, or camera framing from any other photo. Absolutely no watermark, logo, sparkle icon, brand mark, or any repeating overlay pattern/texture anywhere in the image; the surface and background must be clean and artifact-free.</t>
         </is>
       </c>
       <c r="H236" t="inlineStr">
@@ -13135,7 +13135,7 @@
       </c>
       <c r="G237" t="inlineStr">
         <is>
-          <t>Professional food photography of "Gherugu Vadai" (கெருகு வடை), an Indian snack: thin, flat, pale golden crispy discs with a slightly speckled sesame-seed texture, stacked on a plate. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
+          <t>Professional food photography of "Gherugu Vadai" (கெருகு வடை), an Indian snack: thin, flat, pale golden crispy discs with a slightly speckled sesame-seed texture, stacked on a plate. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging, Use a fresh, unique table setting and prop arrangement for this shot -- do not reuse the composition, background objects, or camera framing from any other photo. Absolutely no watermark, logo, sparkle icon, brand mark, or any repeating overlay pattern/texture anywhere in the image; the surface and background must be clean and artifact-free.</t>
         </is>
       </c>
       <c r="H237" t="inlineStr">
@@ -13180,7 +13180,7 @@
       </c>
       <c r="G238" t="inlineStr">
         <is>
-          <t>Professional food photography of "Mullangi Vadai" (முள்ளங்கி வடை), an Indian snack: thin, flat, pale golden-brown lentil vadais with clearly visible white and pale-green shredded radish pieces studded throughout the crisp, speckled surface, one vadai broken in half to show radish shreds inside the crumb, stacked on a plate next to a small mound of raw grated radish as a visual cue. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
+          <t>Professional food photography of "Mullangi Vadai" (முள்ளங்கி வடை), an Indian snack: thin, flat, pale golden-brown lentil vadais with clearly visible fine white shredded radish threads studded throughout the crisp surface, one vadai broken in half to show the white radish shreds inside the crumb, stacked on a plate, with one whole fresh white radish root (its own green leafy top still attached, bulbous white body, clearly root-vegetable shaped) resting prominently in the foreground next to the plate for scale and identification. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging, Use a fresh, unique table setting and prop arrangement for this shot -- do not reuse the composition, background objects, or camera framing from any other photo. Absolutely no watermark, logo, sparkle icon, brand mark, or any repeating overlay pattern/texture anywhere in the image; the surface and background must be clean and artifact-free.</t>
         </is>
       </c>
       <c r="H238" t="inlineStr">
@@ -13225,7 +13225,7 @@
       </c>
       <c r="G239" t="inlineStr">
         <is>
-          <t>Professional food photography of "Pulusu Vadai" (புளி வடை அல்லது புலுசு வடை), an Indian snack: flat reddish-orange vadais with visible small orange pumpkin flecks embedded in the speckled batter, one vadai broken open to show the pumpkin pieces inside, a tangy glossy sheen, stacked on a plate next to a small wedge of raw orange pumpkin as a visual cue. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
+          <t>Professional food photography of "Pulusu Vadai" (புளி வடை அல்லது புலுசு வடை), an Indian snack: flat reddish-orange vadais with visible small orange pumpkin flecks embedded in the speckled batter, one vadai broken open to show the pumpkin pieces inside, a tangy glossy sheen, stacked on a plate next to a small wedge of raw orange pumpkin as a visual cue. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging, Use a fresh, unique table setting and prop arrangement for this shot -- do not reuse the composition, background objects, or camera framing from any other photo. Absolutely no watermark, logo, sparkle icon, brand mark, or any repeating overlay pattern/texture anywhere in the image; the surface and background must be clean and artifact-free.</t>
         </is>
       </c>
       <c r="H239" t="inlineStr">
@@ -13270,7 +13270,7 @@
       </c>
       <c r="G240" t="inlineStr">
         <is>
-          <t>Professional food photography of "Milagu Vadai" (மிளகு வடை), an Indian snack: small pale golden vadais with visible flecks of cracked black pepper, some strung together on a thread like a garland, others piled on a plate, a temple-offering style presentation. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
+          <t>Professional food photography of "Milagu Vadai" (மிளகு வடை), an Indian snack: small pale golden vadais with visible flecks of cracked black pepper, some strung together on a thread like a garland, others piled on a plate, a temple-offering style presentation. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging, Use a fresh, unique table setting and prop arrangement for this shot -- do not reuse the composition, background objects, or camera framing from any other photo. Absolutely no watermark, logo, sparkle icon, brand mark, or any repeating overlay pattern/texture anywhere in the image; the surface and background must be clean and artifact-free.</t>
         </is>
       </c>
       <c r="H240" t="inlineStr">
@@ -13315,7 +13315,7 @@
       </c>
       <c r="G241" t="inlineStr">
         <is>
-          <t>Professional food photography of "Drumstick Vadai" (முருங்கைக்காய் வடை), an Indian snack: coarse, flat golden-brown vadais with visible pale green shredded drumstick (moringa) pulp embedded in the speckled surface, one vadai broken open to show the drumstick fiber inside, stacked on a plate with vinegar-tossed onion rings on the side and a whole raw drumstick pod placed beside the plate as a visual cue. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
+          <t>Professional food photography of "Drumstick Vadai" (முருங்கைக்காய் வடை), an Indian snack: coarse, flat golden-brown vadais with a faint green tint and visible pale green fibrous drumstick pulp embedded in the speckled surface, one vadai broken open to show the stringy green drumstick fiber inside, stacked on a plate with vinegar-tossed onion rings on the side, and two whole raw drumstick (moringa) pods -- long, slender, deeply ridged green pods about a foot long, unmistakably different from any root vegetable -- laid diagonally across the foreground of the scene for scale and identification. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging, Use a fresh, unique table setting and prop arrangement for this shot -- do not reuse the composition, background objects, or camera framing from any other photo. Absolutely no watermark, logo, sparkle icon, brand mark, or any repeating overlay pattern/texture anywhere in the image; the surface and background must be clean and artifact-free.</t>
         </is>
       </c>
       <c r="H241" t="inlineStr">
@@ -13360,7 +13360,7 @@
       </c>
       <c r="G242" t="inlineStr">
         <is>
-          <t>Professional food photography of "Perugu Vadai" (பெருகு வடை), an Indian snack: soft, pale, lightly golden flat discs with a matte soft surface, not deeply fried, stacked on a plate. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
+          <t>Professional food photography of "Perugu Vadai" (பெருகு வடை), an Indian snack: plain soft, pale golden flat rice-flour discs with a smooth matte soft surface and no visible vegetable pieces or flecks of any kind, lightly pan-fried (not deep-fried, not crisp), stacked on a plate on their own with no garnish and no side vegetables. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging, no drumstick, no moringa, no radish, no other vegetables in the frame. Use a fresh, unique table setting and prop arrangement for this shot -- do not reuse the composition, background objects, or camera framing from any other photo. Absolutely no watermark, logo, sparkle icon, brand mark, or any repeating overlay pattern/texture anywhere in the image; the surface and background must be clean and artifact-free.</t>
         </is>
       </c>
       <c r="H242" t="inlineStr">

</xml_diff>

<commit_message>
content(images): wire featured images for street-food batch 2 (71 recipes)
Add Gemini-generated featured.jpg for all 71 remaining street-food/snack
recipes (S.No 202-272 in the tracker), wired into featured_image_url/
alt_ta/alt_en. Update the image tracker to Done for all of them. Batch 1
(50 recipes) already had photos; the full 121-recipe street-food cookbook
now has images end to end.
</commit_message>
<xml_diff>
--- a/docs/recipe-image-tracker.xlsx
+++ b/docs/recipe-image-tracker.xlsx
@@ -12965,7 +12965,12 @@
       </c>
       <c r="I233" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J233" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
         </is>
       </c>
     </row>
@@ -13010,7 +13015,12 @@
       </c>
       <c r="I234" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J234" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
         </is>
       </c>
     </row>
@@ -13055,7 +13065,12 @@
       </c>
       <c r="I235" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J235" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
         </is>
       </c>
     </row>
@@ -13100,7 +13115,12 @@
       </c>
       <c r="I236" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J236" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
         </is>
       </c>
     </row>
@@ -13145,7 +13165,12 @@
       </c>
       <c r="I237" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J237" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
         </is>
       </c>
     </row>
@@ -13190,7 +13215,12 @@
       </c>
       <c r="I238" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J238" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
         </is>
       </c>
     </row>
@@ -13235,7 +13265,12 @@
       </c>
       <c r="I239" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J239" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
         </is>
       </c>
     </row>
@@ -13280,7 +13315,12 @@
       </c>
       <c r="I240" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J240" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
         </is>
       </c>
     </row>
@@ -13325,7 +13365,12 @@
       </c>
       <c r="I241" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J241" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
         </is>
       </c>
     </row>
@@ -13370,7 +13415,12 @@
       </c>
       <c r="I242" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J242" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
         </is>
       </c>
     </row>
@@ -13405,7 +13455,7 @@
       </c>
       <c r="G243" t="inlineStr">
         <is>
-          <t>Professional food photography of "Moong Dhal Toast" (பயத்தம்பருப்பு டோஸ்ட்), an Indian sandwich: a golden-brown fried bread toast cut diagonally, showing a thin green mint chutney layer and a yellow lentil paste layer between the crisp bread surface and the crust, plated with tomato sauce. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
+          <t>Professional food photography of "Moong Dhal Toast" (பயத்தம்பருப்பு டோஸ்ட்), an Indian sandwich: a golden-brown fried bread toast cut diagonally, showing a thin green mint chutney layer and a yellow lentil paste layer between the crisp bread surface and the crust, plated with tomato sauce. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging, Use a fresh, unique table setting and prop arrangement for this shot -- do not reuse the composition, background objects, or camera framing from any other photo.</t>
         </is>
       </c>
       <c r="H243" t="inlineStr">
@@ -13415,7 +13465,12 @@
       </c>
       <c r="I243" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J243" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
         </is>
       </c>
     </row>
@@ -13450,7 +13505,7 @@
       </c>
       <c r="G244" t="inlineStr">
         <is>
-          <t>Professional food photography of "Masala Toast" (மசாலா டோஸ்ட்), an Indian sandwich: golden-brown toasted bread slices with a thin reddish-brown spice chutney visible on the surface, griddle-toasted with light char marks, stacked on a plate. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
+          <t>Professional food photography of "Masala Toast" (மசாலா டோஸ்ட்), an Indian sandwich: golden-brown toasted bread slices with a thin reddish-brown spice chutney visible on the surface, griddle-toasted with light char marks, stacked on a plate. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging, Use a fresh, unique table setting and prop arrangement for this shot -- do not reuse the composition, background objects, or camera framing from any other photo.</t>
         </is>
       </c>
       <c r="H244" t="inlineStr">
@@ -13460,7 +13515,12 @@
       </c>
       <c r="I244" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J244" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
         </is>
       </c>
     </row>
@@ -13495,7 +13555,7 @@
       </c>
       <c r="G245" t="inlineStr">
         <is>
-          <t>Professional food photography of "Tomato Toast" (தக்காளி டோஸ்ட்), an Indian sandwich: a golden-toasted bread slice topped with a glossy reddish-orange cooked tomato-onion masala spread evenly across the surface, slightly caramelized edges, plated hot. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
+          <t>Professional food photography of "Tomato Toast" (தக்காளி டோஸ்ட்), an Indian sandwich: a golden-toasted bread slice topped with a glossy reddish-orange cooked tomato-onion masala spread evenly across the surface, slightly caramelized edges, plated hot. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging, Use a fresh, unique table setting and prop arrangement for this shot -- do not reuse the composition, background objects, or camera framing from any other photo.</t>
         </is>
       </c>
       <c r="H245" t="inlineStr">
@@ -13505,7 +13565,12 @@
       </c>
       <c r="I245" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J245" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
         </is>
       </c>
     </row>
@@ -13540,7 +13605,7 @@
       </c>
       <c r="G246" t="inlineStr">
         <is>
-          <t>Professional food photography of "Potato Sandwich" (உருளைக்கிழங்கு பிரட் சாண்ட்விச்), an Indian sandwich: a golden-brown griddle-fried sandwich cut diagonally, showing a thick yellow spiced-potato filling coated in crisp bread crumbs between the toasted bread layers, plated with ketchup. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
+          <t>Professional food photography of "Potato Sandwich" (உருளைக்கிழங்கு பிரட் சாண்ட்விச்), an Indian sandwich: a golden-brown griddle-fried sandwich cut diagonally, showing a thick yellow spiced-potato filling coated in crisp bread crumbs between the toasted bread layers, plated with ketchup. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging, Use a fresh, unique table setting and prop arrangement for this shot -- do not reuse the composition, background objects, or camera framing from any other photo.</t>
         </is>
       </c>
       <c r="H246" t="inlineStr">
@@ -13550,7 +13615,12 @@
       </c>
       <c r="I246" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J246" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
         </is>
       </c>
     </row>
@@ -13585,7 +13655,7 @@
       </c>
       <c r="G247" t="inlineStr">
         <is>
-          <t>Professional food photography of "Corn Sandwich" (மக்காச்சோள சாண்ட்விச்), an Indian sandwich: an open-faced toast topped with golden corn kernels mixed with cream, and a layer of melted golden cheese bubbling on top, baked and lightly browned. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
+          <t>Professional food photography of "Corn Sandwich" (மக்காச்சோள சாண்ட்விச்), an Indian sandwich: an open-faced toast topped with golden corn kernels mixed with cream, and a layer of melted golden cheese bubbling on top, baked and lightly browned. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging, Use a fresh, unique table setting and prop arrangement for this shot -- do not reuse the composition, background objects, or camera framing from any other photo.</t>
         </is>
       </c>
       <c r="H247" t="inlineStr">
@@ -13595,7 +13665,12 @@
       </c>
       <c r="I247" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J247" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
         </is>
       </c>
     </row>
@@ -13630,7 +13705,7 @@
       </c>
       <c r="G248" t="inlineStr">
         <is>
-          <t>Professional food photography of "Tomato Ketchup" (தக்காளி கெட்ச்அப்), an Indian condiment: a clear glass bottle filled with thick, deep-red glossy homemade tomato ketchup, a spoonful pooled beside it on a white plate showing its smooth, thick consistency. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
+          <t>Professional food photography of "Tomato Ketchup" (தக்காளி கெட்ச்அப்), an Indian condiment: a clear glass bottle filled with thick, deep-red glossy homemade tomato ketchup, a spoonful pooled beside it on a white plate showing its smooth, thick consistency. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging, Use a fresh, unique table setting and prop arrangement for this shot -- do not reuse the composition, background objects, or camera framing from any other photo.</t>
         </is>
       </c>
       <c r="H248" t="inlineStr">
@@ -13640,7 +13715,12 @@
       </c>
       <c r="I248" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J248" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
         </is>
       </c>
     </row>
@@ -13675,7 +13755,7 @@
       </c>
       <c r="G249" t="inlineStr">
         <is>
-          <t>Professional food photography of "Vegetable Sandwich" (காய்கறி சாண்ட்விச்), an Indian sandwich: a triangle-cut sandwich showing distinct colorful layers of thin cucumber, carrot, tomato, and onion rounds between green mint-chutney-spread bread, fresh and vibrant. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
+          <t>Professional food photography of "Vegetable Sandwich" (காய்கறி சாண்ட்விச்), an Indian sandwich: a triangle-cut sandwich showing distinct colorful layers of thin cucumber, carrot, tomato, and onion rounds between green mint-chutney-spread bread, fresh and vibrant. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging, Use a fresh, unique table setting and prop arrangement for this shot -- do not reuse the composition, background objects, or camera framing from any other photo.</t>
         </is>
       </c>
       <c r="H249" t="inlineStr">
@@ -13685,7 +13765,12 @@
       </c>
       <c r="I249" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J249" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
         </is>
       </c>
     </row>
@@ -13720,7 +13805,7 @@
       </c>
       <c r="G250" t="inlineStr">
         <is>
-          <t>Professional food photography of "Chilli Cheese Sandwich" (சில்லி சீஸ் சாண்ட்விச்), an Indian sandwich: a golden toasted sandwich cut in half, oozing melted golden cheese mixed with visible flecks of green chili and onion between the crisp bread layers. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
+          <t>Professional food photography of "Chilli Cheese Sandwich" (சில்லி சீஸ் சாண்ட்விச்), an Indian sandwich: a golden toasted sandwich cut in half, oozing melted golden cheese mixed with visible flecks of green chili and onion between the crisp bread layers. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging, Use a fresh, unique table setting and prop arrangement for this shot -- do not reuse the composition, background objects, or camera framing from any other photo.</t>
         </is>
       </c>
       <c r="H250" t="inlineStr">
@@ -13730,7 +13815,12 @@
       </c>
       <c r="I250" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J250" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
         </is>
       </c>
     </row>
@@ -13765,7 +13855,7 @@
       </c>
       <c r="G251" t="inlineStr">
         <is>
-          <t>Professional food photography of "Paneer Sandwich" (பாலாடைக்கட்டி சாண்ட்விச்), an Indian sandwich: a golden toasted sandwich cut diagonally, showing a crumbly white paneer filling studded with green sprouts and herbs between the bread layers, plated with ketchup. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
+          <t>Professional food photography of "Paneer Sandwich" (பாலாடைக்கட்டி சாண்ட்விச்), an Indian sandwich: a golden toasted sandwich cut diagonally, showing a crumbly white paneer filling studded with green sprouts and herbs between the bread layers, plated with ketchup. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging, Use a fresh, unique table setting and prop arrangement for this shot -- do not reuse the composition, background objects, or camera framing from any other photo.</t>
         </is>
       </c>
       <c r="H251" t="inlineStr">
@@ -13775,7 +13865,12 @@
       </c>
       <c r="I251" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J251" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
         </is>
       </c>
     </row>
@@ -13810,7 +13905,7 @@
       </c>
       <c r="G252" t="inlineStr">
         <is>
-          <t>Professional food photography of "Sandwich Roll" (சாண்ட்விட்ச் ரோல்), an Indian sandwich: pinwheel-shaped bread roll slices arranged on a plate, showing a spiral of white bread with thin green and red chutney swirls visible in the layers, an elegant party-platter presentation. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
+          <t>Professional food photography of "Sandwich Roll" (சாண்ட்விட்ச் ரோல்), an Indian sandwich: pinwheel-shaped bread roll slices arranged on a plate, showing a spiral of white bread with thin green and red chutney swirls visible in the layers, an elegant party-platter presentation. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging, Use a fresh, unique table setting and prop arrangement for this shot -- do not reuse the composition, background objects, or camera framing from any other photo.</t>
         </is>
       </c>
       <c r="H252" t="inlineStr">
@@ -13820,7 +13915,12 @@
       </c>
       <c r="I252" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J252" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
         </is>
       </c>
     </row>
@@ -13855,7 +13955,7 @@
       </c>
       <c r="G253" t="inlineStr">
         <is>
-          <t>Professional food photography of "Aloo Chat 1" (ஆலு சாட் - 1), an Indian street food: a boiled potato stuffed and topped generously with white whisked curd, drizzled with dark brown tangy tamarind sauce, dusted with red chili powder and dark chat masala, garnished with coriander leaves, served on a decorative plate. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
+          <t>Professional food photography of "Aloo Chat 1" (ஆலு சாட் - 1), an Indian street food: a boiled potato stuffed and topped generously with white whisked curd, drizzled with dark brown tangy tamarind sauce, dusted with red chili powder and dark chat masala, garnished with coriander leaves, served on a decorative plate. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging, Use a fresh, unique table setting and prop arrangement for this shot -- do not reuse the composition, background objects, or camera framing from any other photo.</t>
         </is>
       </c>
       <c r="H253" t="inlineStr">
@@ -13865,7 +13965,12 @@
       </c>
       <c r="I253" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J253" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
         </is>
       </c>
     </row>
@@ -13900,7 +14005,7 @@
       </c>
       <c r="G254" t="inlineStr">
         <is>
-          <t>Professional food photography of "Aloo Chat 2" (ஆலு சாட் - 2), an Indian street food: diced potato mixed with golden fried diamond-shaped crisps, tossed in a bowl with dark tangy sauce, chopped onion, and a scattering of thin crispy sev on top. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
+          <t>Professional food photography of "Aloo Chat 2" (ஆலு சாட் - 2), an Indian street food: diced potato mixed with golden fried diamond-shaped crisps, tossed in a bowl with dark tangy sauce, chopped onion, and a scattering of thin crispy sev on top. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging, Use a fresh, unique table setting and prop arrangement for this shot -- do not reuse the composition, background objects, or camera framing from any other photo.</t>
         </is>
       </c>
       <c r="H254" t="inlineStr">
@@ -13910,7 +14015,12 @@
       </c>
       <c r="I254" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J254" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
         </is>
       </c>
     </row>
@@ -13945,7 +14055,7 @@
       </c>
       <c r="G255" t="inlineStr">
         <is>
-          <t>Professional food photography of "Chat Masala Powder" (சாட் மசாலா பவுடர்), an Indian spice blend: a small glass jar filled with reddish-brown aromatic spice powder, a small mound of the powder spilled beside it on a wooden surface with whole dried red chilies and cardamom pods scattered around. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
+          <t>Professional food photography of "Chat Masala Powder" (சாட் மசாலா பவுடர்), an Indian spice blend: a small glass jar filled with reddish-brown aromatic spice powder, a small mound of the powder spilled beside it on a wooden surface with whole dried red chilies and cardamom pods scattered around. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging, Use a fresh, unique table setting and prop arrangement for this shot -- do not reuse the composition, background objects, or camera framing from any other photo.</t>
         </is>
       </c>
       <c r="H255" t="inlineStr">
@@ -13955,7 +14065,12 @@
       </c>
       <c r="I255" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J255" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
         </is>
       </c>
     </row>
@@ -13990,7 +14105,7 @@
       </c>
       <c r="G256" t="inlineStr">
         <is>
-          <t>Professional food photography of "Aloo Pappad Chat" (ஆலு பப்பட் சாட்), an Indian street food: a plate layered with crushed golden fried papad pieces, topped with diced potato, a generous pour of white curd, a dark brown sweet chutney drizzle, and a dusting of spices with fresh coriander on top. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
+          <t>Professional food photography of "Aloo Pappad Chat" (ஆலு பப்பட் சாட்), an Indian street food: a plate layered with crushed golden fried papad pieces, topped with diced potato, a generous pour of white curd, a dark brown sweet chutney drizzle, and a dusting of spices with fresh coriander on top. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging, Use a fresh, unique table setting and prop arrangement for this shot -- do not reuse the composition, background objects, or camera framing from any other photo.</t>
         </is>
       </c>
       <c r="H256" t="inlineStr">
@@ -14000,7 +14115,12 @@
       </c>
       <c r="I256" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J256" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
         </is>
       </c>
     </row>
@@ -14035,7 +14155,7 @@
       </c>
       <c r="G257" t="inlineStr">
         <is>
-          <t>Professional food photography of "Mattar Chat" (பச்சைப் பட்டாணி சாட்), an Indian street food: a bowl of cooked green peas topped with crushed golden puri pieces, white curd, dark tamarind chutney, chopped onion, and fine crispy sev, a colorful layered presentation. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
+          <t>Professional food photography of "Mattar Chat" (பச்சைப் பட்டாணி சாட்), an Indian street food: a bowl of cooked green peas topped with crushed golden puri pieces, white curd, dark tamarind chutney, chopped onion, and fine crispy sev, a colorful layered presentation. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging, Use a fresh, unique table setting and prop arrangement for this shot -- do not reuse the composition, background objects, or camera framing from any other photo.</t>
         </is>
       </c>
       <c r="H257" t="inlineStr">
@@ -14045,7 +14165,12 @@
       </c>
       <c r="I257" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J257" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
         </is>
       </c>
     </row>
@@ -14080,7 +14205,7 @@
       </c>
       <c r="G258" t="inlineStr">
         <is>
-          <t>Professional food photography of "Fruit &amp; Vegetable Chat" (காய்கறி, பழக்கலவை சாட்), an Indian street food: a colorful bowl mix of diced banana, orange segments, tomato, potato, and guava tossed together, garnished with coriander leaves and a light dusting of chat masala. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
+          <t>Professional food photography of "Fruit &amp; Vegetable Chat" (காய்கறி, பழக்கலவை சாட்), an Indian street food: a colorful bowl mix of diced banana, orange segments, tomato, potato, and guava tossed together, garnished with coriander leaves and a light dusting of chat masala. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging, Use a fresh, unique table setting and prop arrangement for this shot -- do not reuse the composition, background objects, or camera framing from any other photo.</t>
         </is>
       </c>
       <c r="H258" t="inlineStr">
@@ -14090,7 +14215,12 @@
       </c>
       <c r="I258" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J258" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
         </is>
       </c>
     </row>
@@ -14125,7 +14255,7 @@
       </c>
       <c r="G259" t="inlineStr">
         <is>
-          <t>Professional food photography of "Finger Chips" (ஃபிங்கர் சிப்ஸ்), an Indian snack: golden-brown crispy potato finger chips piled high on a plate, lightly dusted with salt and pepper, served with tomato ketchup. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
+          <t>Professional food photography of "Finger Chips" (ஃபிங்கர் சிப்ஸ்), an Indian snack: golden-brown crispy potato finger chips piled high on a plate, lightly dusted with salt and pepper, served with tomato ketchup. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging, Use a fresh, unique table setting and prop arrangement for this shot -- do not reuse the composition, background objects, or camera framing from any other photo.</t>
         </is>
       </c>
       <c r="H259" t="inlineStr">
@@ -14135,7 +14265,12 @@
       </c>
       <c r="I259" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J259" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
         </is>
       </c>
     </row>
@@ -14170,7 +14305,7 @@
       </c>
       <c r="G260" t="inlineStr">
         <is>
-          <t>Professional food photography of "Crisp Groundnuts" (வறுகடலை), an Indian snack: small glossy, deep golden-brown fried groundnuts piled in a bowl, with a visible shiny sheen, some scattered on a napkin. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
+          <t>Professional food photography of "Crisp Groundnuts" (வறுகடலை), an Indian snack: small glossy, deep golden-brown fried groundnuts piled in a bowl, with a visible shiny sheen, some scattered on a napkin. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging, Use a fresh, unique table setting and prop arrangement for this shot -- do not reuse the composition, background objects, or camera framing from any other photo.</t>
         </is>
       </c>
       <c r="H260" t="inlineStr">
@@ -14180,7 +14315,12 @@
       </c>
       <c r="I260" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J260" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
         </is>
       </c>
     </row>
@@ -14215,7 +14355,7 @@
       </c>
       <c r="G261" t="inlineStr">
         <is>
-          <t>Professional food photography of "Pop Corn" (பாப் கார்ன்), an Indian snack: a bowl overflowing with fluffy white popcorn lightly dusted with orange-red spice seasoning. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
+          <t>Professional food photography of "Pop Corn" (பாப் கார்ன்), an Indian snack: a bowl overflowing with fluffy white popcorn lightly dusted with orange-red spice seasoning. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging, Use a fresh, unique table setting and prop arrangement for this shot -- do not reuse the composition, background objects, or camera framing from any other photo.</t>
         </is>
       </c>
       <c r="H261" t="inlineStr">
@@ -14225,7 +14365,12 @@
       </c>
       <c r="I261" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J261" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
         </is>
       </c>
     </row>
@@ -14260,7 +14405,7 @@
       </c>
       <c r="G262" t="inlineStr">
         <is>
-          <t>Professional food photography of "Masala Pori 1 (Instant Bhel)" (மசாலா பொரி - 1), an Indian street food: a colorful bowl of puffed rice mixed with roasted gram, small dice of mango, tomato, carrot, and beetroot, garnished with coriander leaves. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
+          <t>Professional food photography of "Masala Pori 1 (Instant Bhel)" (மசாலா பொரி - 1), an Indian street food: a colorful bowl of puffed rice mixed with roasted gram, small dice of mango, tomato, carrot, and beetroot, garnished with coriander leaves. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging, Use a fresh, unique table setting and prop arrangement for this shot -- do not reuse the composition, background objects, or camera framing from any other photo.</t>
         </is>
       </c>
       <c r="H262" t="inlineStr">
@@ -14270,7 +14415,12 @@
       </c>
       <c r="I262" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J262" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
         </is>
       </c>
     </row>
@@ -14305,7 +14455,7 @@
       </c>
       <c r="G263" t="inlineStr">
         <is>
-          <t>Professional food photography of "Masala Pori 2 (Instant Bhel)" (மசாலா பொரி - 2), an Indian street food: a bowl of puffed rice mixed with roasted gram and groundnuts, tossed with pink-tinged marinated onion and a drizzle of dark green chutney, colorful and fresh. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
+          <t>Professional food photography of "Masala Pori 2 (Instant Bhel)" (மசாலா பொரி - 2), an Indian street food: a bowl of puffed rice mixed with roasted gram and groundnuts, tossed with pink-tinged marinated onion and a drizzle of dark green chutney, colorful and fresh. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging, Use a fresh, unique table setting and prop arrangement for this shot -- do not reuse the composition, background objects, or camera framing from any other photo.</t>
         </is>
       </c>
       <c r="H263" t="inlineStr">
@@ -14315,7 +14465,12 @@
       </c>
       <c r="I263" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J263" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
         </is>
       </c>
     </row>
@@ -14350,7 +14505,7 @@
       </c>
       <c r="G264" t="inlineStr">
         <is>
-          <t>Professional food photography of "Mint-Coriander Chutney (for Cutlets)" (புதினா, கொத்தமல்லி சட்னி (கட்லெட்டிற்கு)), an Indian condiment: a small bowl of smooth, vivid green chutney with a glossy sheen, served beside golden fried cutlets, garnished with a mint sprig. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
+          <t>Professional food photography of "Mint-Coriander Chutney (for Cutlets)" (புதினா, கொத்தமல்லி சட்னி (கட்லெட்டிற்கு)), an Indian condiment: a small bowl of smooth, vivid green chutney with a glossy sheen, served beside golden fried cutlets, garnished with a mint sprig. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging, Use a fresh, unique table setting and prop arrangement for this shot -- do not reuse the composition, background objects, or camera framing from any other photo.</t>
         </is>
       </c>
       <c r="H264" t="inlineStr">
@@ -14360,7 +14515,12 @@
       </c>
       <c r="I264" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J264" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
         </is>
       </c>
     </row>
@@ -14395,7 +14555,7 @@
       </c>
       <c r="G265" t="inlineStr">
         <is>
-          <t>Professional food photography of "Mint Chutney (for Cutlets)" (புதினா சட்னி (கட்லெட்டிற்கு)), an Indian condiment: a small bowl of dark green, thick chutney with a tempered mustard-seed garnish floating on top. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
+          <t>Professional food photography of "Mint Chutney (for Cutlets)" (புதினா சட்னி (கட்லெட்டிற்கு)), an Indian condiment: a small bowl of dark green, thick chutney with a tempered mustard-seed garnish floating on top. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging, Use a fresh, unique table setting and prop arrangement for this shot -- do not reuse the composition, background objects, or camera framing from any other photo.</t>
         </is>
       </c>
       <c r="H265" t="inlineStr">
@@ -14405,7 +14565,12 @@
       </c>
       <c r="I265" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J265" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
         </is>
       </c>
     </row>
@@ -14440,7 +14605,7 @@
       </c>
       <c r="G266" t="inlineStr">
         <is>
-          <t>Professional food photography of "Mint-Onion Chutney" (புதினா வெங்காயச் சட்னி), an Indian condiment: a bowl of textured dark green chutney flecked with visible white coconut and small translucent pieces of chopped onion throughout, garnished with a tempering of mustard seeds and curry leaves on top, a few raw onion slices placed beside the bowl as a visual cue. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
+          <t>Professional food photography of "Mint-Onion Chutney" (புதினா வெங்காயச் சட்னி), an Indian condiment: a bowl of textured dark green chutney flecked with visible white coconut and small translucent pieces of chopped onion throughout, garnished with a tempering of mustard seeds and curry leaves on top, a few raw onion slices placed beside the bowl as a visual cue. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging, Use a fresh, unique table setting and prop arrangement for this shot -- do not reuse the composition, background objects, or camera framing from any other photo.</t>
         </is>
       </c>
       <c r="H266" t="inlineStr">
@@ -14450,7 +14615,12 @@
       </c>
       <c r="I266" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J266" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
         </is>
       </c>
     </row>
@@ -14485,7 +14655,7 @@
       </c>
       <c r="G267" t="inlineStr">
         <is>
-          <t>Professional food photography of "Coriander Chutney (for Sandwiches)" (கொத்தமல்லி சட்னி (சாண்ட்விச்சிற்கு)), an Indian condiment: a small bowl of deep green-red chutney with a thick, spreadable texture, a butter knife resting beside it with chutney on the blade. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
+          <t>Professional food photography of "Coriander Chutney (for Sandwiches)" (கொத்தமல்லி சட்னி (சாண்ட்விச்சிற்கு)), an Indian condiment: a small bowl of deep green-red chutney with a thick, spreadable texture, a butter knife resting beside it with chutney on the blade. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging, Use a fresh, unique table setting and prop arrangement for this shot -- do not reuse the composition, background objects, or camera framing from any other photo.</t>
         </is>
       </c>
       <c r="H267" t="inlineStr">
@@ -14495,7 +14665,12 @@
       </c>
       <c r="I267" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J267" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
         </is>
       </c>
     </row>
@@ -14530,7 +14705,7 @@
       </c>
       <c r="G268" t="inlineStr">
         <is>
-          <t>Professional food photography of "Garlic Chutney (for Sandwiches)" (பூண்டு சட்னி (சாண்ட்விச்சிற்கு)), an Indian condiment: a bowl of reddish-brown chutney with visible garlic and chili flecks, thick and glossy, served beside buttered bread slices. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
+          <t>Professional food photography of "Garlic Chutney (for Sandwiches)" (பூண்டு சட்னி (சாண்ட்விச்சிற்கு)), an Indian condiment: a bowl of reddish-brown chutney with visible garlic and chili flecks, thick and glossy, served beside buttered bread slices. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging, Use a fresh, unique table setting and prop arrangement for this shot -- do not reuse the composition, background objects, or camera framing from any other photo.</t>
         </is>
       </c>
       <c r="H268" t="inlineStr">
@@ -14540,7 +14715,12 @@
       </c>
       <c r="I268" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J268" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
         </is>
       </c>
     </row>
@@ -14575,7 +14755,7 @@
       </c>
       <c r="G269" t="inlineStr">
         <is>
-          <t>Professional food photography of "Coconut-Ginger Chutney (for Sandwiches)" (தேங்காய், இஞ்சி சட்னி (சாண்ட்விச்சிற்கு)), an Indian condiment: a bowl of coarse, off-white coconut chutney with visible ginger and red chili flecks, a glossy texture. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
+          <t>Professional food photography of "Coconut-Ginger Chutney (for Sandwiches)" (தேங்காய், இஞ்சி சட்னி (சாண்ட்விச்சிற்கு)), an Indian condiment: a bowl of coarse, off-white coconut chutney with visible ginger and red chili flecks, a glossy texture. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging, Use a fresh, unique table setting and prop arrangement for this shot -- do not reuse the composition, background objects, or camera framing from any other photo.</t>
         </is>
       </c>
       <c r="H269" t="inlineStr">
@@ -14585,7 +14765,12 @@
       </c>
       <c r="I269" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J269" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
         </is>
       </c>
     </row>
@@ -14620,7 +14805,7 @@
       </c>
       <c r="G270" t="inlineStr">
         <is>
-          <t>Professional food photography of "Mint Chutney (for Sandwiches)" (புதினா சட்னி (சாண்ட்விச்சிற்கு)), an Indian condiment: a small bowl of smooth bright green mint chutney with a glossy sheen, served beside a stack of white bread slices. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
+          <t>Professional food photography of "Mint Chutney (for Sandwiches)" (புதினா சட்னி (சாண்ட்விச்சிற்கு)), an Indian condiment: a small bowl of smooth bright green mint chutney with a glossy sheen, served beside a stack of white bread slices. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging, Use a fresh, unique table setting and prop arrangement for this shot -- do not reuse the composition, background objects, or camera framing from any other photo.</t>
         </is>
       </c>
       <c r="H270" t="inlineStr">
@@ -14630,7 +14815,12 @@
       </c>
       <c r="I270" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J270" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
         </is>
       </c>
     </row>
@@ -14665,7 +14855,7 @@
       </c>
       <c r="G271" t="inlineStr">
         <is>
-          <t>Professional food photography of "Onion Bajji" (வெங்காயப் பஜ்ஜி), an Indian snack: golden fried onion bajjis with a distinctive ring-shaped, batter-coated onion visible inside the crisp fried coating, piled on a plate, served with coconut chutney. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
+          <t>Professional food photography of "Onion Bajji" (வெங்காயப் பஜ்ஜி), an Indian snack: golden fried onion bajjis with a distinctive ring-shaped, batter-coated onion visible inside the crisp fried coating, piled on a plate, served with coconut chutney. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging, Use a fresh, unique table setting and prop arrangement for this shot -- do not reuse the composition, background objects, or camera framing from any other photo.</t>
         </is>
       </c>
       <c r="H271" t="inlineStr">
@@ -14675,7 +14865,12 @@
       </c>
       <c r="I271" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J271" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
         </is>
       </c>
     </row>
@@ -14710,7 +14905,7 @@
       </c>
       <c r="G272" t="inlineStr">
         <is>
-          <t>Professional food photography of "Deep Fried Ladies Fingers" (வெண்டைக்காய் பக்கோடா), an Indian snack: whole okra pieces coated in a crisp golden fried batter with visible bread-crumb texture, arranged on a plate with tomato sauce. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
+          <t>Professional food photography of "Deep Fried Ladies Fingers" (வெண்டைக்காய் பக்கோடா), an Indian snack: whole okra pieces coated in a crisp golden fried batter with visible bread-crumb texture, arranged on a plate with tomato sauce. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging, Use a fresh, unique table setting and prop arrangement for this shot -- do not reuse the composition, background objects, or camera framing from any other photo.</t>
         </is>
       </c>
       <c r="H272" t="inlineStr">
@@ -14720,7 +14915,12 @@
       </c>
       <c r="I272" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J272" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
         </is>
       </c>
     </row>
@@ -14755,7 +14955,7 @@
       </c>
       <c r="G273" t="inlineStr">
         <is>
-          <t>Professional food photography of "Carrot Sandwich" (கேரட் சாண்ட்விச்), an Indian sandwich: a pressed golden-toasted sandwich cut in half, showing a bright orange sauteed carrot-tomato filling between the bread layers, plated with tomato sauce. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging.</t>
+          <t>Professional food photography of "Carrot Sandwich" (கேரட் சாண்ட்விச்), an Indian sandwich: a pressed golden-toasted sandwich cut in half, showing a bright orange sauteed carrot-tomato filling between the bread layers, plated with tomato sauce. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging, Use a fresh, unique table setting and prop arrangement for this shot -- do not reuse the composition, background objects, or camera framing from any other photo.</t>
         </is>
       </c>
       <c r="H273" t="inlineStr">
@@ -14765,7 +14965,12 @@
       </c>
       <c r="I273" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J273" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
content(images): wire featured images for the 21 restored recipes
Add Gemini-generated featured.jpg for all 21 recently-restored "Vegetarian
Cooking Tips" recipes, wired into featured_image_url/alt_ta/alt_en. Adds
matching rows (S.No 273-293) to the image tracker, marked Done. All 293
site recipes now have photos.
</commit_message>
<xml_diff>
--- a/docs/recipe-image-tracker.xlsx
+++ b/docs/recipe-image-tracker.xlsx
@@ -496,7 +496,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K273"/>
+  <dimension ref="A1:K294"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -14969,6 +14969,1056 @@
         </is>
       </c>
       <c r="J273" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="274">
+      <c r="A274" t="n">
+        <v>273</v>
+      </c>
+      <c r="B274" t="inlineStr">
+        <is>
+          <t>Vegetarian Cooking Tips - Gap Fill</t>
+        </is>
+      </c>
+      <c r="C274" t="inlineStr">
+        <is>
+          <t>egg-dosai</t>
+        </is>
+      </c>
+      <c r="D274" t="inlineStr">
+        <is>
+          <t>Egg Dosai</t>
+        </is>
+      </c>
+      <c r="E274" t="inlineStr">
+        <is>
+          <t>முட்டைத் தோசை</t>
+        </is>
+      </c>
+      <c r="F274" t="inlineStr">
+        <is>
+          <t>dosa</t>
+        </is>
+      </c>
+      <c r="G274" t="inlineStr">
+        <is>
+          <t>Professional food photography of "Egg Dosai" (முட்டைத் தோசை), an Indian breakfast dish: a thin golden-brown dosa on a griddle with a beaten egg spread across its surface and cooked in, giving it a mottled yellow-and-brown speckled texture, folded in half on a plate, sprinkled with chopped onion, served with coconut chutney. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging, Use a fresh, unique table setting and prop arrangement for this shot -- do not reuse the composition, background objects, or camera framing from any other photo.</t>
+        </is>
+      </c>
+      <c r="H274" t="inlineStr">
+        <is>
+          <t>public/images/recipes/egg-dosai/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I274" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J274" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="275">
+      <c r="A275" t="n">
+        <v>274</v>
+      </c>
+      <c r="B275" t="inlineStr">
+        <is>
+          <t>Vegetarian Cooking Tips - Gap Fill</t>
+        </is>
+      </c>
+      <c r="C275" t="inlineStr">
+        <is>
+          <t>masala-idli</t>
+        </is>
+      </c>
+      <c r="D275" t="inlineStr">
+        <is>
+          <t>Masala Idli</t>
+        </is>
+      </c>
+      <c r="E275" t="inlineStr">
+        <is>
+          <t>மசாலா இட்லி</t>
+        </is>
+      </c>
+      <c r="F275" t="inlineStr">
+        <is>
+          <t>idli</t>
+        </is>
+      </c>
+      <c r="G275" t="inlineStr">
+        <is>
+          <t>Professional food photography of "Masala Idli" (மசாலா இட்லி), an Indian steamed breakfast dish: a soft white idli cut in half on a plate, revealing a spiced reddish-orange vegetable filling layered through its center, steam rising, served with sambar and coconut chutney. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging, Use a fresh, unique table setting and prop arrangement for this shot -- do not reuse the composition, background objects, or camera framing from any other photo.</t>
+        </is>
+      </c>
+      <c r="H275" t="inlineStr">
+        <is>
+          <t>public/images/recipes/masala-idli/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I275" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J275" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="276">
+      <c r="A276" t="n">
+        <v>275</v>
+      </c>
+      <c r="B276" t="inlineStr">
+        <is>
+          <t>Vegetarian Cooking Tips - Gap Fill</t>
+        </is>
+      </c>
+      <c r="C276" t="inlineStr">
+        <is>
+          <t>vegetable-sambar</t>
+        </is>
+      </c>
+      <c r="D276" t="inlineStr">
+        <is>
+          <t>Vegetable Sambar</t>
+        </is>
+      </c>
+      <c r="E276" t="inlineStr">
+        <is>
+          <t>காய்கறி சாம்பார்</t>
+        </is>
+      </c>
+      <c r="F276" t="inlineStr">
+        <is>
+          <t>sambar</t>
+        </is>
+      </c>
+      <c r="G276" t="inlineStr">
+        <is>
+          <t>Professional food photography of "Vegetable Sambar" (காய்கறி சாம்பார்), an Indian lentil stew: steaming orange-yellow sambar in a bowl, chunks of drumstick and brinjal visible in the thick lentil gravy, a mustard-and-curry-leaf tempering glistening on top, garnished with fresh coriander leaves. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging, Use a fresh, unique table setting and prop arrangement for this shot -- do not reuse the composition, background objects, or camera framing from any other photo.</t>
+        </is>
+      </c>
+      <c r="H276" t="inlineStr">
+        <is>
+          <t>public/images/recipes/vegetable-sambar/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I276" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J276" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="277">
+      <c r="A277" t="n">
+        <v>276</v>
+      </c>
+      <c r="B277" t="inlineStr">
+        <is>
+          <t>Vegetarian Cooking Tips - Gap Fill</t>
+        </is>
+      </c>
+      <c r="C277" t="inlineStr">
+        <is>
+          <t>idiyappam</t>
+        </is>
+      </c>
+      <c r="D277" t="inlineStr">
+        <is>
+          <t>Idiyappam (String Hoppers)</t>
+        </is>
+      </c>
+      <c r="E277" t="inlineStr">
+        <is>
+          <t>இடியாப்பம்</t>
+        </is>
+      </c>
+      <c r="F277" t="inlineStr">
+        <is>
+          <t>steamed-tiffin</t>
+        </is>
+      </c>
+      <c r="G277" t="inlineStr">
+        <is>
+          <t>Professional food photography of "Idiyappam (String Hoppers)" (இடியாப்பம்), an Indian steamed rice-flour dish: a neat coiled disc of thin white string hoppers on a banana leaf, delicate steamed strands visible, served beside a small bowl of coconut milk and a wedge of lime. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging, Use a fresh, unique table setting and prop arrangement for this shot -- do not reuse the composition, background objects, or camera framing from any other photo.</t>
+        </is>
+      </c>
+      <c r="H277" t="inlineStr">
+        <is>
+          <t>public/images/recipes/idiyappam/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I277" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J277" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="278">
+      <c r="A278" t="n">
+        <v>277</v>
+      </c>
+      <c r="B278" t="inlineStr">
+        <is>
+          <t>Vegetarian Cooking Tips - Gap Fill</t>
+        </is>
+      </c>
+      <c r="C278" t="inlineStr">
+        <is>
+          <t>sweet-appam</t>
+        </is>
+      </c>
+      <c r="D278" t="inlineStr">
+        <is>
+          <t>Sweet Appam</t>
+        </is>
+      </c>
+      <c r="E278" t="inlineStr">
+        <is>
+          <t>இனிப்பு ஆப்பம்</t>
+        </is>
+      </c>
+      <c r="F278" t="inlineStr">
+        <is>
+          <t>steamed-tiffin, sweet</t>
+        </is>
+      </c>
+      <c r="G278" t="inlineStr">
+        <is>
+          <t>Professional food photography of "Sweet Appam" (இனிப்பு ஆப்பம்), an Indian sweet steamed dish: a golden caramel-toned bowl-shaped appam with a thick spongy center and lacy crisp edges, its jaggery-sweetened surface glistening slightly, resting on a plate. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging, Use a fresh, unique table setting and prop arrangement for this shot -- do not reuse the composition, background objects, or camera framing from any other photo.</t>
+        </is>
+      </c>
+      <c r="H278" t="inlineStr">
+        <is>
+          <t>public/images/recipes/sweet-appam/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I278" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J278" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="279">
+      <c r="A279" t="n">
+        <v>278</v>
+      </c>
+      <c r="B279" t="inlineStr">
+        <is>
+          <t>Vegetarian Cooking Tips - Gap Fill</t>
+        </is>
+      </c>
+      <c r="C279" t="inlineStr">
+        <is>
+          <t>chapati</t>
+        </is>
+      </c>
+      <c r="D279" t="inlineStr">
+        <is>
+          <t>Chapati</t>
+        </is>
+      </c>
+      <c r="E279" t="inlineStr">
+        <is>
+          <t>சப்பாத்தி</t>
+        </is>
+      </c>
+      <c r="F279" t="inlineStr">
+        <is>
+          <t>flatbread</t>
+        </is>
+      </c>
+      <c r="G279" t="inlineStr">
+        <is>
+          <t>Professional food photography of "Chapati" (சப்பாத்தி), an Indian flatbread: a puffed, golden-brown round chapati fresh off the griddle, a light sheen of ghee brushed on top, stacked with one leaning against the pile. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging, Use a fresh, unique table setting and prop arrangement for this shot -- do not reuse the composition, background objects, or camera framing from any other photo.</t>
+        </is>
+      </c>
+      <c r="H279" t="inlineStr">
+        <is>
+          <t>public/images/recipes/chapati/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I279" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J279" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="280">
+      <c r="A280" t="n">
+        <v>279</v>
+      </c>
+      <c r="B280" t="inlineStr">
+        <is>
+          <t>Vegetarian Cooking Tips - Gap Fill</t>
+        </is>
+      </c>
+      <c r="C280" t="inlineStr">
+        <is>
+          <t>patrora</t>
+        </is>
+      </c>
+      <c r="D280" t="inlineStr">
+        <is>
+          <t>Patrora (or Curd Poori)</t>
+        </is>
+      </c>
+      <c r="E280" t="inlineStr">
+        <is>
+          <t>பட்ரோரா (அல்லது) தயிர் பூரி</t>
+        </is>
+      </c>
+      <c r="F280" t="inlineStr">
+        <is>
+          <t>fried-bread</t>
+        </is>
+      </c>
+      <c r="G280" t="inlineStr">
+        <is>
+          <t>Professional food photography of "Patrora (or Curd Poori)" (பட்ரோரா (அல்லது) தயிர் பூரி), an Indian fried bread: a thick, golden-brown deep-fried round bread with a naan-like puffed thickness (noticeably thicker than a thin poori), served on a plate with a side of chana masala gravy. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging, Use a fresh, unique table setting and prop arrangement for this shot -- do not reuse the composition, background objects, or camera framing from any other photo.</t>
+        </is>
+      </c>
+      <c r="H280" t="inlineStr">
+        <is>
+          <t>public/images/recipes/patrora/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I280" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J280" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="281">
+      <c r="A281" t="n">
+        <v>280</v>
+      </c>
+      <c r="B281" t="inlineStr">
+        <is>
+          <t>Vegetarian Cooking Tips - Gap Fill</t>
+        </is>
+      </c>
+      <c r="C281" t="inlineStr">
+        <is>
+          <t>tomato-kurma</t>
+        </is>
+      </c>
+      <c r="D281" t="inlineStr">
+        <is>
+          <t>Tomato Kurma</t>
+        </is>
+      </c>
+      <c r="E281" t="inlineStr">
+        <is>
+          <t>தக்காளி குருமா</t>
+        </is>
+      </c>
+      <c r="F281" t="inlineStr">
+        <is>
+          <t>kuzhambu</t>
+        </is>
+      </c>
+      <c r="G281" t="inlineStr">
+        <is>
+          <t>Professional food photography of "Tomato Kurma" (தக்காளி குருமா), an Indian gravy: a thick reddish-orange tomato kurma in a bowl, chunks of potato visible in the glossy sauce, garnished with fresh coriander leaves. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging, Use a fresh, unique table setting and prop arrangement for this shot -- do not reuse the composition, background objects, or camera framing from any other photo.</t>
+        </is>
+      </c>
+      <c r="H281" t="inlineStr">
+        <is>
+          <t>public/images/recipes/tomato-kurma/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I281" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J281" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="282">
+      <c r="A282" t="n">
+        <v>281</v>
+      </c>
+      <c r="B282" t="inlineStr">
+        <is>
+          <t>Vegetarian Cooking Tips - Gap Fill</t>
+        </is>
+      </c>
+      <c r="C282" t="inlineStr">
+        <is>
+          <t>kathirikkai-kosu</t>
+        </is>
+      </c>
+      <c r="D282" t="inlineStr">
+        <is>
+          <t>Kathirikkai Kosu (Brinjal Kosu)</t>
+        </is>
+      </c>
+      <c r="E282" t="inlineStr">
+        <is>
+          <t>கத்தரிக்காய் கொச்சு</t>
+        </is>
+      </c>
+      <c r="F282" t="inlineStr">
+        <is>
+          <t>kuzhambu</t>
+        </is>
+      </c>
+      <c r="G282" t="inlineStr">
+        <is>
+          <t>Professional food photography of "Kathirikkai Kosu (Brinjal Kosu)" (கத்தரிக்காய் கொச்சு), an Indian side dish: a dark reddish-brown mashed brinjal side dish in a small bowl, thick and glossy with visible flecks of tempered mustard seeds, served beside plain rice. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging, Use a fresh, unique table setting and prop arrangement for this shot -- do not reuse the composition, background objects, or camera framing from any other photo.</t>
+        </is>
+      </c>
+      <c r="H282" t="inlineStr">
+        <is>
+          <t>public/images/recipes/kathirikkai-kosu/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I282" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J282" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="283">
+      <c r="A283" t="n">
+        <v>282</v>
+      </c>
+      <c r="B283" t="inlineStr">
+        <is>
+          <t>Vegetarian Cooking Tips - Gap Fill</t>
+        </is>
+      </c>
+      <c r="C283" t="inlineStr">
+        <is>
+          <t>masala-sundal</t>
+        </is>
+      </c>
+      <c r="D283" t="inlineStr">
+        <is>
+          <t>Masala Sundal</t>
+        </is>
+      </c>
+      <c r="E283" t="inlineStr">
+        <is>
+          <t>மசால் சுண்டல்</t>
+        </is>
+      </c>
+      <c r="F283" t="inlineStr">
+        <is>
+          <t>sundal</t>
+        </is>
+      </c>
+      <c r="G283" t="inlineStr">
+        <is>
+          <t>Professional food photography of "Masala Sundal" (மசால் சுண்டல்), an Indian spiced legume dish: a bowl of spiced chickpeas garnished generously with grated coconut and chopped coriander leaves, curry leaves visible throughout. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging, Use a fresh, unique table setting and prop arrangement for this shot -- do not reuse the composition, background objects, or camera framing from any other photo.</t>
+        </is>
+      </c>
+      <c r="H283" t="inlineStr">
+        <is>
+          <t>public/images/recipes/masala-sundal/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I283" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J283" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="284">
+      <c r="A284" t="n">
+        <v>283</v>
+      </c>
+      <c r="B284" t="inlineStr">
+        <is>
+          <t>Vegetarian Cooking Tips - Gap Fill</t>
+        </is>
+      </c>
+      <c r="C284" t="inlineStr">
+        <is>
+          <t>kuzhai-puttu</t>
+        </is>
+      </c>
+      <c r="D284" t="inlineStr">
+        <is>
+          <t>Kuzhai Puttu (Tube Puttu)</t>
+        </is>
+      </c>
+      <c r="E284" t="inlineStr">
+        <is>
+          <t>குழாய்ப்புட்டு</t>
+        </is>
+      </c>
+      <c r="F284" t="inlineStr">
+        <is>
+          <t>puttu, sweet</t>
+        </is>
+      </c>
+      <c r="G284" t="inlineStr">
+        <is>
+          <t>Professional food photography of "Kuzhai Puttu (Tube Puttu)" (குழாய்ப்புட்டு), an Indian steamed sweet dish: a cylindrical steamed puttu on a plate, cut into thick discs revealing alternating white rice-flour and grated-coconut-and-sugar layers, steam still rising. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging, Use a fresh, unique table setting and prop arrangement for this shot -- do not reuse the composition, background objects, or camera framing from any other photo.</t>
+        </is>
+      </c>
+      <c r="H284" t="inlineStr">
+        <is>
+          <t>public/images/recipes/kuzhai-puttu/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I284" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J284" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="285">
+      <c r="A285" t="n">
+        <v>284</v>
+      </c>
+      <c r="B285" t="inlineStr">
+        <is>
+          <t>Vegetarian Cooking Tips - Gap Fill</t>
+        </is>
+      </c>
+      <c r="C285" t="inlineStr">
+        <is>
+          <t>egg-pan-cake</t>
+        </is>
+      </c>
+      <c r="D285" t="inlineStr">
+        <is>
+          <t>Pan Cake</t>
+        </is>
+      </c>
+      <c r="E285" t="inlineStr">
+        <is>
+          <t>பான் கேக்</t>
+        </is>
+      </c>
+      <c r="F285" t="inlineStr">
+        <is>
+          <t>sweet</t>
+        </is>
+      </c>
+      <c r="G285" t="inlineStr">
+        <is>
+          <t>Professional food photography of "Pan Cake" (பான் கேக்), an Indian sweet pancake: a thin, pale golden egg-and-maida pancake folded in half on a plate, a slightly glossy surface from ghee, dusted lightly with sugar. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging, Use a fresh, unique table setting and prop arrangement for this shot -- do not reuse the composition, background objects, or camera framing from any other photo.</t>
+        </is>
+      </c>
+      <c r="H285" t="inlineStr">
+        <is>
+          <t>public/images/recipes/egg-pan-cake/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I285" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J285" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="286">
+      <c r="A286" t="n">
+        <v>285</v>
+      </c>
+      <c r="B286" t="inlineStr">
+        <is>
+          <t>Vegetarian Cooking Tips - Gap Fill</t>
+        </is>
+      </c>
+      <c r="C286" t="inlineStr">
+        <is>
+          <t>milk-basundi</t>
+        </is>
+      </c>
+      <c r="D286" t="inlineStr">
+        <is>
+          <t>Milk Basundi</t>
+        </is>
+      </c>
+      <c r="E286" t="inlineStr">
+        <is>
+          <t>பால் பாஸந்தி</t>
+        </is>
+      </c>
+      <c r="F286" t="inlineStr">
+        <is>
+          <t>sweet</t>
+        </is>
+      </c>
+      <c r="G286" t="inlineStr">
+        <is>
+          <t>Professional food photography of "Milk Basundi" (பால் பாஸந்தி), an Indian sweet: thick, creamy off-white basundi in a small bowl, slivers of pistachio and cashew scattered on top with a few golden saffron strands, condensation on the bowl suggesting it's chilled. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging, Use a fresh, unique table setting and prop arrangement for this shot -- do not reuse the composition, background objects, or camera framing from any other photo.</t>
+        </is>
+      </c>
+      <c r="H286" t="inlineStr">
+        <is>
+          <t>public/images/recipes/milk-basundi/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I286" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J286" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="287">
+      <c r="A287" t="n">
+        <v>286</v>
+      </c>
+      <c r="B287" t="inlineStr">
+        <is>
+          <t>Vegetarian Cooking Tips - Gap Fill</t>
+        </is>
+      </c>
+      <c r="C287" t="inlineStr">
+        <is>
+          <t>cashew-pakoda</t>
+        </is>
+      </c>
+      <c r="D287" t="inlineStr">
+        <is>
+          <t>Cashew Pakoda</t>
+        </is>
+      </c>
+      <c r="E287" t="inlineStr">
+        <is>
+          <t>முந்திரி பருப்பு பகோடா</t>
+        </is>
+      </c>
+      <c r="F287" t="inlineStr">
+        <is>
+          <t>bajji</t>
+        </is>
+      </c>
+      <c r="G287" t="inlineStr">
+        <is>
+          <t>Professional food photography of "Cashew Pakoda" (முந்திரி பருப்பு பகோடா), an Indian snack: golden-brown irregular-shaped fritters piled on a plate, whole cashew nuts and flecks of onion visible embedded in the crisp fried batter, a small bowl of ketchup beside it. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging, Use a fresh, unique table setting and prop arrangement for this shot -- do not reuse the composition, background objects, or camera framing from any other photo.</t>
+        </is>
+      </c>
+      <c r="H287" t="inlineStr">
+        <is>
+          <t>public/images/recipes/cashew-pakoda/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I287" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J287" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="288">
+      <c r="A288" t="n">
+        <v>287</v>
+      </c>
+      <c r="B288" t="inlineStr">
+        <is>
+          <t>Vegetarian Cooking Tips - Gap Fill</t>
+        </is>
+      </c>
+      <c r="C288" t="inlineStr">
+        <is>
+          <t>potato-chips</t>
+        </is>
+      </c>
+      <c r="D288" t="inlineStr">
+        <is>
+          <t>Potato Chips</t>
+        </is>
+      </c>
+      <c r="E288" t="inlineStr">
+        <is>
+          <t>உருளைக் கிழங்கு சிப்ஸ்</t>
+        </is>
+      </c>
+      <c r="F288" t="inlineStr">
+        <is>
+          <t>snack</t>
+        </is>
+      </c>
+      <c r="G288" t="inlineStr">
+        <is>
+          <t>Professional food photography of "Potato Chips" (உருளைக் கிழங்கு சிப்ஸ்), an Indian snack: thin, golden potato chip rounds piled in a bowl, dusted lightly with red chilli powder, glossy from frying oil. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging, Use a fresh, unique table setting and prop arrangement for this shot -- do not reuse the composition, background objects, or camera framing from any other photo.</t>
+        </is>
+      </c>
+      <c r="H288" t="inlineStr">
+        <is>
+          <t>public/images/recipes/potato-chips/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I288" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J288" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="289">
+      <c r="A289" t="n">
+        <v>288</v>
+      </c>
+      <c r="B289" t="inlineStr">
+        <is>
+          <t>Vegetarian Cooking Tips - Gap Fill</t>
+        </is>
+      </c>
+      <c r="C289" t="inlineStr">
+        <is>
+          <t>sweet-raw-mango</t>
+        </is>
+      </c>
+      <c r="D289" t="inlineStr">
+        <is>
+          <t>Sweet Raw Mango</t>
+        </is>
+      </c>
+      <c r="E289" t="inlineStr">
+        <is>
+          <t>இனிப்பு மாங்காய்</t>
+        </is>
+      </c>
+      <c r="F289" t="inlineStr">
+        <is>
+          <t>curry</t>
+        </is>
+      </c>
+      <c r="G289" t="inlineStr">
+        <is>
+          <t>Professional food photography of "Sweet Raw Mango" (இனிப்பு மாங்காய்), an Indian curry: a thick, glossy amber-colored mashed raw mango curry in a bowl, flecks of curry leaves and mustard seeds visible, served beside plain rice. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging, Use a fresh, unique table setting and prop arrangement for this shot -- do not reuse the composition, background objects, or camera framing from any other photo.</t>
+        </is>
+      </c>
+      <c r="H289" t="inlineStr">
+        <is>
+          <t>public/images/recipes/sweet-raw-mango/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I289" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J289" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="290">
+      <c r="A290" t="n">
+        <v>289</v>
+      </c>
+      <c r="B290" t="inlineStr">
+        <is>
+          <t>Vegetarian Cooking Tips - Gap Fill</t>
+        </is>
+      </c>
+      <c r="C290" t="inlineStr">
+        <is>
+          <t>kinch-mosara</t>
+        </is>
+      </c>
+      <c r="D290" t="inlineStr">
+        <is>
+          <t>Kinch Mosara (Stuffed Potato Cones)</t>
+        </is>
+      </c>
+      <c r="E290" t="inlineStr">
+        <is>
+          <t>கிஞ்ச மோசரா</t>
+        </is>
+      </c>
+      <c r="F290" t="inlineStr">
+        <is>
+          <t>fried-snack</t>
+        </is>
+      </c>
+      <c r="G290" t="inlineStr">
+        <is>
+          <t>Professional food photography of "Kinch Mosara (Stuffed Potato Cones)" (கிஞ்ச மோசரா), an Indian fried snack: golden-brown deep-fried cone-shaped pastries on a plate, one broken open to reveal a spiced mashed-potato-and-green-pea filling studded with raisins and cashews. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging, Use a fresh, unique table setting and prop arrangement for this shot -- do not reuse the composition, background objects, or camera framing from any other photo.</t>
+        </is>
+      </c>
+      <c r="H290" t="inlineStr">
+        <is>
+          <t>public/images/recipes/kinch-mosara/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I290" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J290" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="291">
+      <c r="A291" t="n">
+        <v>290</v>
+      </c>
+      <c r="B291" t="inlineStr">
+        <is>
+          <t>Vegetarian Cooking Tips - Gap Fill</t>
+        </is>
+      </c>
+      <c r="C291" t="inlineStr">
+        <is>
+          <t>pirattu-kari</t>
+        </is>
+      </c>
+      <c r="D291" t="inlineStr">
+        <is>
+          <t>Pirattu Kari (Braised Mutton)</t>
+        </is>
+      </c>
+      <c r="E291" t="inlineStr">
+        <is>
+          <t>பிறட்டுக்கறி</t>
+        </is>
+      </c>
+      <c r="F291" t="inlineStr">
+        <is>
+          <t>curry</t>
+        </is>
+      </c>
+      <c r="G291" t="inlineStr">
+        <is>
+          <t>Professional food photography of "Pirattu Kari (Braised Mutton)" (பிறட்டுக்கறி), an Indian curry: dark reddish-brown braised mutton pieces in a thick, dry-ish onion masala coating, glistening slightly with oil, served in a bowl garnished with curry leaves. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging, Use a fresh, unique table setting and prop arrangement for this shot -- do not reuse the composition, background objects, or camera framing from any other photo.</t>
+        </is>
+      </c>
+      <c r="H291" t="inlineStr">
+        <is>
+          <t>public/images/recipes/pirattu-kari/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I291" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J291" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="292">
+      <c r="A292" t="n">
+        <v>291</v>
+      </c>
+      <c r="B292" t="inlineStr">
+        <is>
+          <t>Vegetarian Cooking Tips - Gap Fill</t>
+        </is>
+      </c>
+      <c r="C292" t="inlineStr">
+        <is>
+          <t>chinese-sooce</t>
+        </is>
+      </c>
+      <c r="D292" t="inlineStr">
+        <is>
+          <t>Chinese Sooce (Cashew-Date Bars)</t>
+        </is>
+      </c>
+      <c r="E292" t="inlineStr">
+        <is>
+          <t>சைனீஸ் சூஸ்</t>
+        </is>
+      </c>
+      <c r="F292" t="inlineStr">
+        <is>
+          <t>sweet</t>
+        </is>
+      </c>
+      <c r="G292" t="inlineStr">
+        <is>
+          <t>Professional food photography of "Chinese Sooce (Cashew-Date Bars)" (சைனீஸ் சூஸ்), an Indian sweet: rectangular golden-brown baked bars studded with chopped cashews and dates, dusted with white icing sugar, stacked on a plate. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging, Use a fresh, unique table setting and prop arrangement for this shot -- do not reuse the composition, background objects, or camera framing from any other photo.</t>
+        </is>
+      </c>
+      <c r="H292" t="inlineStr">
+        <is>
+          <t>public/images/recipes/chinese-sooce/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I292" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J292" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="293">
+      <c r="A293" t="n">
+        <v>292</v>
+      </c>
+      <c r="B293" t="inlineStr">
+        <is>
+          <t>Vegetarian Cooking Tips - Gap Fill</t>
+        </is>
+      </c>
+      <c r="C293" t="inlineStr">
+        <is>
+          <t>boat-egg</t>
+        </is>
+      </c>
+      <c r="D293" t="inlineStr">
+        <is>
+          <t>Boat Egg</t>
+        </is>
+      </c>
+      <c r="E293" t="inlineStr">
+        <is>
+          <t>படகு முட்டை</t>
+        </is>
+      </c>
+      <c r="F293" t="inlineStr">
+        <is>
+          <t>snack</t>
+        </is>
+      </c>
+      <c r="G293" t="inlineStr">
+        <is>
+          <t>Professional food photography of "Boat Egg" (படகு முட்டை), an Indian snack: small boiled-egg-white boat shapes arranged on a platter, each filled with pale yellow mashed egg yolk and topped with a small triangular bread-slice sail propped upright. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging, Use a fresh, unique table setting and prop arrangement for this shot -- do not reuse the composition, background objects, or camera framing from any other photo.</t>
+        </is>
+      </c>
+      <c r="H293" t="inlineStr">
+        <is>
+          <t>public/images/recipes/boat-egg/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I293" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J293" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="294">
+      <c r="A294" t="n">
+        <v>293</v>
+      </c>
+      <c r="B294" t="inlineStr">
+        <is>
+          <t>Vegetarian Cooking Tips - Gap Fill</t>
+        </is>
+      </c>
+      <c r="C294" t="inlineStr">
+        <is>
+          <t>fish-fry-roast</t>
+        </is>
+      </c>
+      <c r="D294" t="inlineStr">
+        <is>
+          <t>Fish Fry Roast</t>
+        </is>
+      </c>
+      <c r="E294" t="inlineStr">
+        <is>
+          <t>மீன் ஃபிராஸ்ட்</t>
+        </is>
+      </c>
+      <c r="F294" t="inlineStr">
+        <is>
+          <t>curry</t>
+        </is>
+      </c>
+      <c r="G294" t="inlineStr">
+        <is>
+          <t>Professional food photography of "Fish Fry Roast" (மீன் ஃபிராஸ்ட்), an Indian curry: golden-brown shallow-fried fish steaks on a plate, a red-orange spice crust visible on the surface, garnished with sliced onion, coriander leaves, and a lemon wedge. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging, Use a fresh, unique table setting and prop arrangement for this shot -- do not reuse the composition, background objects, or camera framing from any other photo.</t>
+        </is>
+      </c>
+      <c r="H294" t="inlineStr">
+        <is>
+          <t>public/images/recipes/fish-fry-roast/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I294" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J294" t="inlineStr">
         <is>
           <t>2026-09-09</t>
         </is>

</xml_diff>

<commit_message>
feat(recipes): add Chicken Manchurian, the last held content gap
Book recipe #4 from the "Vegetarian Cooking Tips" cookbook's non-veg
section (source page 46-47). A finger in the source photo covered one
ingredient line; the user supplied the missing values (corn flour 50g,
egg 1, salt, water) directly rather than guessing. Includes a
Gemini-generated photo, wired in. All 294 site recipes now have photos.
</commit_message>
<xml_diff>
--- a/docs/recipe-image-tracker.xlsx
+++ b/docs/recipe-image-tracker.xlsx
@@ -496,7 +496,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K294"/>
+  <dimension ref="A1:K295"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -16019,6 +16019,56 @@
         </is>
       </c>
       <c r="J294" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="295">
+      <c r="A295" t="n">
+        <v>294</v>
+      </c>
+      <c r="B295" t="inlineStr">
+        <is>
+          <t>Vegetarian Cooking Tips - Gap Fill</t>
+        </is>
+      </c>
+      <c r="C295" t="inlineStr">
+        <is>
+          <t>chicken-manchurian</t>
+        </is>
+      </c>
+      <c r="D295" t="inlineStr">
+        <is>
+          <t>Chicken Manchurian</t>
+        </is>
+      </c>
+      <c r="E295" t="inlineStr">
+        <is>
+          <t>சிக்கன் மஞ்சூரியன்</t>
+        </is>
+      </c>
+      <c r="F295" t="inlineStr">
+        <is>
+          <t>curry</t>
+        </is>
+      </c>
+      <c r="G295" t="inlineStr">
+        <is>
+          <t>Professional food photography of "Chicken Manchurian" (சிக்கன் மஞ்சூரியன்), an Indian curry: golden-fried chicken pieces coated in a glossy dark brown Indo-Chinese gravy, chunks of green capsicum and translucent sauteed onion visible throughout the thick sauce, garnished with a few sesame seeds or spring onion greens on top, served in a bowl. Shot from a 45-degree angle with soft natural daylight, shallow depth of field, a rustic wooden table setting in the background, warm and appetizing color tones, photorealistic, high resolution, no text, no watermark, no logos, no people, no plastic packaging, Use a fresh, unique table setting and prop arrangement for this shot -- do not reuse the composition, background objects, or camera framing from any other photo.</t>
+        </is>
+      </c>
+      <c r="H295" t="inlineStr">
+        <is>
+          <t>public/images/recipes/chicken-manchurian/featured.jpg</t>
+        </is>
+      </c>
+      <c r="I295" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J295" t="inlineStr">
         <is>
           <t>2026-09-09</t>
         </is>

</xml_diff>